<commit_message>
docs: link production work to GitHub issues
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra4f336f9935742ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R9901f37c9c874e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf4b1a2ca9c9746d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rf706757a74374764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Re26a8558b3274876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rfa92f141ee5747aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R2df9db738f38447f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R7e84d5c5158e4d24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re893abebb1aa485b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7f1d253fe9ec487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd51f0dcebb8c4564"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R10f101f80ae244f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R93d544ffe1a048e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R73bba5174fb64ac5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R543fe53153cc4722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R010d1b0bc7c94a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Reee767fa075d4ba0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R5e6b91a54f9244c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R971ddacccde043ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rbeeff43b8e2448ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -833,7 +833,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8cbefe3b9fad48de"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb98a5bb9b0f3453c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -894,7 +894,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -1276,7 +1276,7 @@
       </x:c>
       <x:c r="H7" s="40" t="n">
         <x:f>B8</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1285,14 +1285,14 @@
       </x:c>
       <x:c r="B8" s="37" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"In Progress")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="36" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="37" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$15,"Open")</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF(Risks!$H$6:$H$16,"Open")</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="40" t="str">
         <x:v>PR Open</x:v>
@@ -1314,15 +1314,15 @@
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="37" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$15,"P0",Risks!$H$6:$H$15,"Open")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIFS(Risks!$E$6:$E$16,"P0",Risks!$H$6:$H$16,"Open")</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="40" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H9" s="40" t="n">
         <x:f>B10</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1331,7 +1331,7 @@
       </x:c>
       <x:c r="B10" s="37" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Blocked")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="36" t="str">
         <x:v>Approved requirements</x:v>
@@ -1453,7 +1453,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5f74c451d9449a9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3feac246e54c66"/>
 </x:worksheet>
 </file>
 
@@ -1835,7 +1835,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6193333f11ad4b29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e38b40737444ae5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1942,7 +1942,9 @@
       <x:c r="J6" s="25" t="str">
         <x:v>Production plan Task 1A</x:v>
       </x:c>
-      <x:c r="K6" s="25" t="str"/>
+      <x:c r="K6" s="25" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
+      </x:c>
       <x:c r="L6" s="25" t="str"/>
       <x:c r="M6" s="28" t="str">
         <x:v>2026-10-04</x:v>
@@ -1979,7 +1981,9 @@
       <x:c r="J7" s="26" t="str">
         <x:v>Production plan Task 1B</x:v>
       </x:c>
-      <x:c r="K7" s="26" t="str"/>
+      <x:c r="K7" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/7</x:v>
+      </x:c>
       <x:c r="L7" s="26" t="str"/>
       <x:c r="M7" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2014,7 +2018,9 @@
       <x:c r="J8" s="26" t="str">
         <x:v>Production plan Task 1C</x:v>
       </x:c>
-      <x:c r="K8" s="26" t="str"/>
+      <x:c r="K8" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/8</x:v>
+      </x:c>
       <x:c r="L8" s="26" t="str"/>
       <x:c r="M8" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2049,7 +2055,9 @@
       <x:c r="J9" s="26" t="str">
         <x:v>Production plan Task 1D</x:v>
       </x:c>
-      <x:c r="K9" s="26" t="str"/>
+      <x:c r="K9" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/9</x:v>
+      </x:c>
       <x:c r="L9" s="26" t="str"/>
       <x:c r="M9" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2084,7 +2092,9 @@
       <x:c r="J10" s="26" t="str">
         <x:v>Production plan Task 1E</x:v>
       </x:c>
-      <x:c r="K10" s="26" t="str"/>
+      <x:c r="K10" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/10</x:v>
+      </x:c>
       <x:c r="L10" s="26" t="str"/>
       <x:c r="M10" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2121,7 +2131,9 @@
       <x:c r="J11" s="26" t="str">
         <x:v>backend-observability-foundation plan</x:v>
       </x:c>
-      <x:c r="K11" s="26" t="str"/>
+      <x:c r="K11" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/11</x:v>
+      </x:c>
       <x:c r="L11" s="26" t="str"/>
       <x:c r="M11" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2158,7 +2170,9 @@
       <x:c r="J12" s="26" t="str">
         <x:v>client-error-observability plan</x:v>
       </x:c>
-      <x:c r="K12" s="26" t="str"/>
+      <x:c r="K12" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/12</x:v>
+      </x:c>
       <x:c r="L12" s="26" t="str"/>
       <x:c r="M12" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2195,7 +2209,9 @@
       <x:c r="J13" s="26" t="str">
         <x:v>local-log-platform plan</x:v>
       </x:c>
-      <x:c r="K13" s="26" t="str"/>
+      <x:c r="K13" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/13</x:v>
+      </x:c>
       <x:c r="L13" s="26" t="str"/>
       <x:c r="M13" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2232,7 +2248,9 @@
       <x:c r="J14" s="26" t="str">
         <x:v>Production plan Task 3</x:v>
       </x:c>
-      <x:c r="K14" s="26" t="str"/>
+      <x:c r="K14" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/14</x:v>
+      </x:c>
       <x:c r="L14" s="26" t="str"/>
       <x:c r="M14" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2269,7 +2287,9 @@
       <x:c r="J15" s="26" t="str">
         <x:v>Production plan Task 4</x:v>
       </x:c>
-      <x:c r="K15" s="26" t="str"/>
+      <x:c r="K15" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/15</x:v>
+      </x:c>
       <x:c r="L15" s="26" t="str"/>
       <x:c r="M15" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2306,7 +2326,9 @@
       <x:c r="J16" s="26" t="str">
         <x:v>Production plan Task 5</x:v>
       </x:c>
-      <x:c r="K16" s="26" t="str"/>
+      <x:c r="K16" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/16</x:v>
+      </x:c>
       <x:c r="L16" s="26" t="str"/>
       <x:c r="M16" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2343,7 +2365,9 @@
       <x:c r="J17" s="26" t="str">
         <x:v>Production plan Task 6</x:v>
       </x:c>
-      <x:c r="K17" s="26" t="str"/>
+      <x:c r="K17" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/17</x:v>
+      </x:c>
       <x:c r="L17" s="26" t="str"/>
       <x:c r="M17" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2380,7 +2404,9 @@
       <x:c r="J18" s="26" t="str">
         <x:v>Production plan Task 7</x:v>
       </x:c>
-      <x:c r="K18" s="26" t="str"/>
+      <x:c r="K18" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/18</x:v>
+      </x:c>
       <x:c r="L18" s="26" t="str"/>
       <x:c r="M18" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2417,7 +2443,9 @@
       <x:c r="J19" s="26" t="str">
         <x:v>Production plan Task 8</x:v>
       </x:c>
-      <x:c r="K19" s="26" t="str"/>
+      <x:c r="K19" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/19</x:v>
+      </x:c>
       <x:c r="L19" s="26" t="str"/>
       <x:c r="M19" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2454,7 +2482,9 @@
       <x:c r="J20" s="26" t="str">
         <x:v>Production plan Task 9</x:v>
       </x:c>
-      <x:c r="K20" s="26" t="str"/>
+      <x:c r="K20" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/20</x:v>
+      </x:c>
       <x:c r="L20" s="26" t="str"/>
       <x:c r="M20" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2491,7 +2521,9 @@
       <x:c r="J21" s="26" t="str">
         <x:v>Production plan Task 10</x:v>
       </x:c>
-      <x:c r="K21" s="26" t="str"/>
+      <x:c r="K21" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/21</x:v>
+      </x:c>
       <x:c r="L21" s="26" t="str"/>
       <x:c r="M21" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2528,7 +2560,9 @@
       <x:c r="J22" s="26" t="str">
         <x:v>Production plan Task 11</x:v>
       </x:c>
-      <x:c r="K22" s="26" t="str"/>
+      <x:c r="K22" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/22</x:v>
+      </x:c>
       <x:c r="L22" s="26" t="str"/>
       <x:c r="M22" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2565,7 +2599,9 @@
       <x:c r="J23" s="26" t="str">
         <x:v>Production plan Task 12</x:v>
       </x:c>
-      <x:c r="K23" s="26" t="str"/>
+      <x:c r="K23" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/23</x:v>
+      </x:c>
       <x:c r="L23" s="26" t="str"/>
       <x:c r="M23" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2602,7 +2638,9 @@
       <x:c r="J24" s="26" t="str">
         <x:v>Production plan Task 13</x:v>
       </x:c>
-      <x:c r="K24" s="26" t="str"/>
+      <x:c r="K24" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/24</x:v>
+      </x:c>
       <x:c r="L24" s="26" t="str"/>
       <x:c r="M24" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2639,7 +2677,9 @@
       <x:c r="J25" s="26" t="str">
         <x:v>Production plan Task 14</x:v>
       </x:c>
-      <x:c r="K25" s="26" t="str"/>
+      <x:c r="K25" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/25</x:v>
+      </x:c>
       <x:c r="L25" s="26" t="str"/>
       <x:c r="M25" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2676,7 +2716,9 @@
       <x:c r="J26" s="26" t="str">
         <x:v>Production plan Task 15</x:v>
       </x:c>
-      <x:c r="K26" s="26" t="str"/>
+      <x:c r="K26" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/26</x:v>
+      </x:c>
       <x:c r="L26" s="26" t="str"/>
       <x:c r="M26" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2713,7 +2755,9 @@
       <x:c r="J27" s="26" t="str">
         <x:v>Production plan Task 16</x:v>
       </x:c>
-      <x:c r="K27" s="26" t="str"/>
+      <x:c r="K27" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/27</x:v>
+      </x:c>
       <x:c r="L27" s="26" t="str"/>
       <x:c r="M27" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2750,7 +2794,9 @@
       <x:c r="J28" s="26" t="str">
         <x:v>Production plan Task 16</x:v>
       </x:c>
-      <x:c r="K28" s="26" t="str"/>
+      <x:c r="K28" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/28</x:v>
+      </x:c>
       <x:c r="L28" s="26" t="str"/>
       <x:c r="M28" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2787,7 +2833,9 @@
       <x:c r="J29" s="26" t="str">
         <x:v>Production plan Task 17</x:v>
       </x:c>
-      <x:c r="K29" s="26" t="str"/>
+      <x:c r="K29" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/29</x:v>
+      </x:c>
       <x:c r="L29" s="26" t="str"/>
       <x:c r="M29" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2824,7 +2872,9 @@
       <x:c r="J30" s="26" t="str">
         <x:v>Production plan final gate</x:v>
       </x:c>
-      <x:c r="K30" s="26" t="str"/>
+      <x:c r="K30" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/30</x:v>
+      </x:c>
       <x:c r="L30" s="26" t="str"/>
       <x:c r="M30" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2859,7 +2909,9 @@
       <x:c r="J31" s="26" t="str">
         <x:v>Current WOW working tree mobile/src/app/planner-clients.tsx</x:v>
       </x:c>
-      <x:c r="K31" s="26" t="str"/>
+      <x:c r="K31" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/31</x:v>
+      </x:c>
       <x:c r="L31" s="26" t="str"/>
       <x:c r="M31" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2896,7 +2948,9 @@
       <x:c r="J32" s="26" t="str">
         <x:v>Source integration policy</x:v>
       </x:c>
-      <x:c r="K32" s="26" t="str"/>
+      <x:c r="K32" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/32</x:v>
+      </x:c>
       <x:c r="L32" s="26" t="str"/>
       <x:c r="M32" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2931,7 +2985,9 @@
       <x:c r="J33" s="26" t="str">
         <x:v>QA findings F-002 F-003</x:v>
       </x:c>
-      <x:c r="K33" s="26" t="str"/>
+      <x:c r="K33" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/33</x:v>
+      </x:c>
       <x:c r="L33" s="26" t="str"/>
       <x:c r="M33" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -2968,7 +3024,9 @@
       <x:c r="J34" s="26" t="str">
         <x:v>QA finding F-001</x:v>
       </x:c>
-      <x:c r="K34" s="26" t="str"/>
+      <x:c r="K34" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/34</x:v>
+      </x:c>
       <x:c r="L34" s="26" t="str"/>
       <x:c r="M34" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -3005,7 +3063,9 @@
       <x:c r="J35" s="26" t="str">
         <x:v>QA limit L-002</x:v>
       </x:c>
-      <x:c r="K35" s="26" t="str"/>
+      <x:c r="K35" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/35</x:v>
+      </x:c>
       <x:c r="L35" s="26" t="str"/>
       <x:c r="M35" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -3028,10 +3088,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F36" s="26" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G36" s="26" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Product owner</x:v>
       </x:c>
       <x:c r="H36" s="26" t="str"/>
       <x:c r="I36" s="26" t="str">
@@ -3040,7 +3100,9 @@
       <x:c r="J36" s="26" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K36" s="26" t="str"/>
+      <x:c r="K36" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/36</x:v>
+      </x:c>
       <x:c r="L36" s="26" t="str"/>
       <x:c r="M36" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -3063,7 +3125,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F37" s="27" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G37" s="27" t="str">
         <x:v>Codex</x:v>
@@ -3075,7 +3137,9 @@
       <x:c r="J37" s="27" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K37" s="27" t="str"/>
+      <x:c r="K37" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/37</x:v>
+      </x:c>
       <x:c r="L37" s="27" t="str"/>
       <x:c r="M37" s="30" t="str">
         <x:v>2026-10-04</x:v>
@@ -3097,7 +3161,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0c8234f6f0e4a80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e9a6f2f14964b96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3581,7 +3645,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c88180588ac43f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3905f3766e4e88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3871,7 +3935,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8816f0fea41c402b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R320ebb62338441da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4177,42 +4241,71 @@
       <x:c r="I14" s="26" t="str"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="27" t="str">
+      <x:c r="A15" s="26" t="str">
         <x:v>RISK-010</x:v>
       </x:c>
-      <x:c r="B15" s="27" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>Historical secrets enter the private production history</x:v>
       </x:c>
-      <x:c r="C15" s="27" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>Critical</x:v>
       </x:c>
-      <x:c r="D15" s="27" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E15" s="27" t="str">
+      <x:c r="E15" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F15" s="27" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>Clean snapshot history secret scanning and push protection</x:v>
       </x:c>
-      <x:c r="G15" s="27" t="str">
+      <x:c r="G15" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H15" s="27" t="str">
+      <x:c r="H15" s="26" t="str">
         <x:v>Mitigated</x:v>
       </x:c>
-      <x:c r="I15" s="27" t="str">
+      <x:c r="I15" s="26" t="str">
         <x:v>Initial scan found no tracked high-confidence signatures</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="27" t="str">
+        <x:v>RISK-011</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="str">
+        <x:v>Private repository cannot enforce native branch protection or secret scanning on the current GitHub plan</x:v>
+      </x:c>
+      <x:c r="C16" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D16" s="27" t="str">
+        <x:v>Certain</x:v>
+      </x:c>
+      <x:c r="E16" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F16" s="27" t="str">
+        <x:v>Use PR discipline and CI Gitleaks as compensating controls; upgrade to GitHub Pro or an eligible organization before production</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="str">
+        <x:v>Product owner</x:v>
+      </x:c>
+      <x:c r="H16" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I16" s="27" t="str">
+        <x:v>GitHub API returned HTTP 403 and 422 on 2026-10-04</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E15">
+  <x:conditionalFormatting sqref="E6:E16">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H15">
+  <x:conditionalFormatting sqref="H6:H16">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4221,7 +4314,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f96af5305024534"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cc60f515c75459f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4541,7 +4634,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cf12d60391c4fba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26728e85a60e4087"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4880,7 +4973,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd91b73e7e35243d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeeb6dc5baa34948"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5018,7 +5111,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra803730cfffb4e8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3568de0833e44d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5135,7 +5228,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc394e67032b749ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc08020a90aa546fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record governance pull request handoff
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd51f0dcebb8c4564"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R10f101f80ae244f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R93d544ffe1a048e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R73bba5174fb64ac5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R543fe53153cc4722"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R010d1b0bc7c94a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Reee767fa075d4ba0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R5e6b91a54f9244c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R971ddacccde043ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rbeeff43b8e2448ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb138e7404ade4071"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rdf9c869f793d4779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R86eebdef1147413a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rccd91ee9b7584a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Ra57de28dd9f64b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R6fd89d25e95249dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re3c287d57bca4998"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Ra322ff3ac46e4d40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rd1e7359342734944"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Red93a083fc594c51"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -833,7 +833,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb98a5bb9b0f3453c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R204a46c233ee4d2a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1299,7 +1299,7 @@
       </x:c>
       <x:c r="H8" s="40" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1308,7 +1308,7 @@
       </x:c>
       <x:c r="B9" s="37" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="36" t="str">
         <x:v>P0 open risks</x:v>
@@ -1453,7 +1453,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3feac246e54c66"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d819766d0e345bd"/>
 </x:worksheet>
 </file>
 
@@ -1835,7 +1835,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e38b40737444ae5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaa3ae109347462f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3125,7 +3125,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F37" s="27" t="str">
-        <x:v>In Review</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G37" s="27" t="str">
         <x:v>Codex</x:v>
@@ -3140,7 +3140,9 @@
       <x:c r="K37" s="27" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/37</x:v>
       </x:c>
-      <x:c r="L37" s="27" t="str"/>
+      <x:c r="L37" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
+      </x:c>
       <x:c r="M37" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
@@ -3161,7 +3163,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e9a6f2f14964b96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdacd18af472f49fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3645,7 +3647,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3905f3766e4e88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c057c3af7704254"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3935,7 +3937,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R320ebb62338441da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca0578ebc7c949af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4314,7 +4316,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cc60f515c75459f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dab71b2aa294a52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4634,7 +4636,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26728e85a60e4087"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d333055237e443b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4973,7 +4975,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeeb6dc5baa34948"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34b55a0fee6d4390"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5111,7 +5113,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3568de0833e44d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf136d24be55a4a92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5189,27 +5191,35 @@
       <x:c r="A6" s="32" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B6" s="32" t="str"/>
+      <x:c r="B6" s="32" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
+      </x:c>
       <x:c r="C6" s="32" t="str">
         <x:v>codex/gov-002-production-program</x:v>
       </x:c>
-      <x:c r="D6" s="32" t="str"/>
-      <x:c r="E6" s="32" t="str"/>
-      <x:c r="F6" s="32" t="str"/>
+      <x:c r="D6" s="32" t="str">
+        <x:v>1e9f458</x:v>
+      </x:c>
+      <x:c r="E6" s="32" t="str">
+        <x:v>fb8afe5</x:v>
+      </x:c>
+      <x:c r="F6" s="32" t="str">
+        <x:v>07218b4ab02a8702a4d8d9fdab7dc26e579ab7b4</x:v>
+      </x:c>
       <x:c r="G6" s="32" t="str">
-        <x:v>Initial repository validation</x:v>
+        <x:v>Register tests 2/2; credential scan clear; workbook formulas clear and 10 sheets visually reviewed</x:v>
       </x:c>
       <x:c r="H6" s="32" t="str">
-        <x:v>Documentation and governance baseline</x:v>
+        <x:v>Documentation and governance only; no Railway deployment</x:v>
       </x:c>
       <x:c r="I6" s="32" t="str">
-        <x:v>Revert initial commit before dependent work</x:v>
+        <x:v>Revert PR 49; bootstrap remains clean source snapshot</x:v>
       </x:c>
       <x:c r="J6" s="32" t="str">
-        <x:v>None</x:v>
+        <x:v>GitHub plan blocks protected private branches and native secret scanning; tracked by GOV-001</x:v>
       </x:c>
       <x:c r="K6" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L6" s="33" t="str">
         <x:v>2026-10-04</x:v>
@@ -5228,7 +5238,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc08020a90aa546fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra666e618826346eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize governance handoff evidence
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb138e7404ade4071"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rdf9c869f793d4779"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R86eebdef1147413a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rccd91ee9b7584a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Ra57de28dd9f64b7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R6fd89d25e95249dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re3c287d57bca4998"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Ra322ff3ac46e4d40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rd1e7359342734944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Red93a083fc594c51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3f608c5e04b94829"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R284e0eaa4bcb443b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rc6a0784062604dad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R976d0f8ea2594139"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rea4f976100774241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1d57c6aa78ad4752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R6306d8da2c534ae1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rb8135e303ba444f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Red421e8f8e2b4728"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R2e66538f0c6c48a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -833,7 +833,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R204a46c233ee4d2a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb715e356140a41c0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1453,7 +1453,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d819766d0e345bd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e89505d7d514550"/>
 </x:worksheet>
 </file>
 
@@ -1835,7 +1835,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaa3ae109347462f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcc2732bd04c43e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3163,7 +3163,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdacd18af472f49fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd479ee229f1043f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3647,7 +3647,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c057c3af7704254"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21d57e46fa4e4704"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3937,7 +3937,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca0578ebc7c949af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a3c068cd8074ba2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4316,7 +4316,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dab71b2aa294a52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R713fb1987d2e462e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4636,7 +4636,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d333055237e443b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d0cc169daec4e07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4975,7 +4975,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34b55a0fee6d4390"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra379a1465cbd4ef5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5113,7 +5113,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf136d24be55a4a92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc9a42500d84423b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5201,13 +5201,13 @@
         <x:v>1e9f458</x:v>
       </x:c>
       <x:c r="E6" s="32" t="str">
-        <x:v>fb8afe5</x:v>
+        <x:v>10455fa</x:v>
       </x:c>
       <x:c r="F6" s="32" t="str">
         <x:v>07218b4ab02a8702a4d8d9fdab7dc26e579ab7b4</x:v>
       </x:c>
       <x:c r="G6" s="32" t="str">
-        <x:v>Register tests 2/2; credential scan clear; workbook formulas clear and 10 sheets visually reviewed</x:v>
+        <x:v>Register/workflow tests 4/4; backend/frontend/mobile CI passed on 7c31fbf; Gitleaks passed after permission fix; credential scan clear; workbook formulas clear and 10 sheets visually reviewed</x:v>
       </x:c>
       <x:c r="H6" s="32" t="str">
         <x:v>Documentation and governance only; no Railway deployment</x:v>
@@ -5216,7 +5216,7 @@
         <x:v>Revert PR 49; bootstrap remains clean source snapshot</x:v>
       </x:c>
       <x:c r="J6" s="32" t="str">
-        <x:v>GitHub plan blocks protected private branches and native secret scanning; tracked by GOV-001</x:v>
+        <x:v>GitHub plan blocks protected private branches native secret scanning and native CodeQL upload; offline SARIF and CI Gitleaks compensate; tracked by GOV-001</x:v>
       </x:c>
       <x:c r="K6" s="32" t="str">
         <x:v>PR Open</x:v>
@@ -5238,7 +5238,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra666e618826346eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4c0f88854094f2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: mark production program foundation ready
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3f608c5e04b94829"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R284e0eaa4bcb443b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rc6a0784062604dad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R976d0f8ea2594139"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rea4f976100774241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1d57c6aa78ad4752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R6306d8da2c534ae1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rb8135e303ba444f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Red421e8f8e2b4728"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R2e66538f0c6c48a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbd410f0f7a794916"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rd76d9bd425db4268"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4838a44155b54de2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rffa97dc825e345c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R57301af3b787409e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd3cee27f371d4329"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R4618652927bd4f41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2bf01e34651f476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re77a0d23d5314a11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R5571ec6bfb3d4102"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -833,7 +833,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb715e356140a41c0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd639e8844633464d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1246,7 +1246,7 @@
       </x:c>
       <x:c r="E6" s="37" t="n">
         <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G6" s="40" t="str">
         <x:v>Open</x:v>
@@ -1299,7 +1299,7 @@
       </x:c>
       <x:c r="H8" s="40" t="n">
         <x:f>B9</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1308,7 +1308,7 @@
       </x:c>
       <x:c r="B9" s="37" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="36" t="str">
         <x:v>P0 open risks</x:v>
@@ -1345,7 +1345,7 @@
       </x:c>
       <x:c r="H10" s="40" t="n">
         <x:f>B11</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1354,7 +1354,7 @@
       </x:c>
       <x:c r="B11" s="37" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1381,16 +1381,16 @@
         <x:v>Repository foundation</x:v>
       </x:c>
       <x:c r="B14" s="26" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="C14" s="26" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Product owner</x:v>
       </x:c>
       <x:c r="D14" s="26" t="str">
-        <x:v>Initial commit, issues, protections and green governance CI</x:v>
+        <x:v>Upgrade GitHub plan for protected private branches and native security uploads</x:v>
       </x:c>
       <x:c r="E14" s="26" t="str">
-        <x:v>Complete before implementation</x:v>
+        <x:v>Compensating CI controls are active</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1453,7 +1453,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e89505d7d514550"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03779c0f350c45a8"/>
 </x:worksheet>
 </file>
 
@@ -1835,7 +1835,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcc2732bd04c43e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591602fb704346fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3125,7 +3125,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F37" s="27" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G37" s="27" t="str">
         <x:v>Codex</x:v>
@@ -3163,7 +3163,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd479ee229f1043f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaefd2482d744112"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3647,7 +3647,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21d57e46fa4e4704"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58d8b83a4f87494f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3937,7 +3937,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a3c068cd8074ba2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570d5d231dcc45ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4316,7 +4316,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R713fb1987d2e462e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R260a82e3bf8644c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4636,7 +4636,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d0cc169daec4e07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re830ad96462143d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4975,7 +4975,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra379a1465cbd4ef5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cd581407914487e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5113,7 +5113,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc9a42500d84423b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a1bfa5b87c24683"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5201,13 +5201,13 @@
         <x:v>1e9f458</x:v>
       </x:c>
       <x:c r="E6" s="32" t="str">
-        <x:v>10455fa</x:v>
+        <x:v>4444b86</x:v>
       </x:c>
       <x:c r="F6" s="32" t="str">
         <x:v>07218b4ab02a8702a4d8d9fdab7dc26e579ab7b4</x:v>
       </x:c>
       <x:c r="G6" s="32" t="str">
-        <x:v>Register/workflow tests 4/4; backend/frontend/mobile CI passed on 7c31fbf; Gitleaks passed after permission fix; credential scan clear; workbook formulas clear and 10 sheets visually reviewed</x:v>
+        <x:v>Final PR head 4444b86: backend build/test pass; frontend pass; mobile pass; Docker build pass; registers pass; Gitleaks pass; CodeQL JavaScript/TypeScript and Actions pass with 30-day SARIF artifacts; local governance 4/4</x:v>
       </x:c>
       <x:c r="H6" s="32" t="str">
         <x:v>Documentation and governance only; no Railway deployment</x:v>
@@ -5219,7 +5219,7 @@
         <x:v>GitHub plan blocks protected private branches native secret scanning and native CodeQL upload; offline SARIF and CI Gitleaks compensate; tracked by GOV-001</x:v>
       </x:c>
       <x:c r="K6" s="32" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Ready to Merge</x:v>
       </x:c>
       <x:c r="L6" s="33" t="str">
         <x:v>2026-10-04</x:v>
@@ -5238,7 +5238,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4c0f88854094f2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47d13f9f27c14e5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize public protection tracker
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbd410f0f7a794916"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rd76d9bd425db4268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4838a44155b54de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rffa97dc825e345c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R57301af3b787409e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd3cee27f371d4329"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R4618652927bd4f41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2bf01e34651f476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re77a0d23d5314a11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R5571ec6bfb3d4102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra82fc0183a11442b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6fa20bf17f3a45af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4a49a0f0e6e04497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rd7653db751404ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R88508ddfc8394578"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R160115c5e8ae4b89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd82b27fc55604d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R72cc06c0ec304ea6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R23350c76e9fd4e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8579165ef61c4e2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -124,7 +124,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -192,15 +192,6 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
@@ -211,6 +202,12 @@
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -833,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd639e8844633464d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39762c3c77f04b08"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -894,7 +891,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -963,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1210,169 +1207,169 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-04. Counts link to the canonical CSV registers included in the private production repository.</x:v>
+        <x:v>As of 2026-10-04. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
+      <x:c r="A5" s="31" t="str">
         <x:v>Work items</x:v>
       </x:c>
-      <x:c r="B5" s="35" t="str">
+      <x:c r="B5" s="32" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D5" s="34" t="str">
+      <x:c r="D5" s="31" t="str">
         <x:v>Readiness</x:v>
       </x:c>
-      <x:c r="E5" s="35" t="str">
+      <x:c r="E5" s="32" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="G5" s="40" t="str">
+      <x:c r="G5" s="39" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="40" t="str">
+      <x:c r="H5" s="39" t="str">
         <x:v>Count</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="36" t="str">
+      <x:c r="A6" s="33" t="str">
         <x:v>Total</x:v>
       </x:c>
-      <x:c r="B6" s="37" t="n">
+      <x:c r="B6" s="34" t="n">
         <x:f>COUNTA('Open Items'!$A$6:$A$37)</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="D6" s="36" t="str">
+      <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
-      <x:c r="E6" s="37" t="n">
+      <x:c r="E6" s="34" t="n">
         <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="G6" s="40" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="H6" s="40" t="n">
+      <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
         <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="36" t="str">
+      <x:c r="A7" s="33" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="B7" s="37" t="n">
+      <x:c r="B7" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Open")</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="D7" s="36" t="str">
+      <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
       </x:c>
-      <x:c r="E7" s="37" t="n">
+      <x:c r="E7" s="34" t="n">
         <x:f>COUNTIF('Release Gates'!$E$6:$E$17,"Open")</x:f>
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G7" s="40" t="str">
+      <x:c r="G7" s="39" t="str">
         <x:v>In Progress</x:v>
       </x:c>
-      <x:c r="H7" s="40" t="n">
+      <x:c r="H7" s="39" t="n">
         <x:f>B8</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="36" t="str">
+      <x:c r="A8" s="33" t="str">
         <x:v>In Progress</x:v>
       </x:c>
-      <x:c r="B8" s="37" t="n">
+      <x:c r="B8" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D8" s="36" t="str">
+      <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
-      <x:c r="E8" s="37" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$16,"Open")</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G8" s="40" t="str">
+      <x:c r="E8" s="34" t="n">
+        <x:f>COUNTIF(Risks!$H$6:$H$17,"Open")</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
       </x:c>
-      <x:c r="H8" s="40" t="n">
+      <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="36" t="str">
+      <x:c r="A9" s="33" t="str">
         <x:v>PR Open</x:v>
       </x:c>
-      <x:c r="B9" s="37" t="n">
+      <x:c r="B9" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D9" s="36" t="str">
+      <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
-      <x:c r="E9" s="37" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$16,"P0",Risks!$H$6:$H$16,"Open")</x:f>
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="G9" s="40" t="str">
+      <x:c r="E9" s="34" t="n">
+        <x:f>COUNTIFS(Risks!$E$6:$E$17,"P0",Risks!$H$6:$H$17,"Open")</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G9" s="39" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="H9" s="40" t="n">
+      <x:c r="H9" s="39" t="n">
         <x:f>B10</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="36" t="str">
+      <x:c r="A10" s="33" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="B10" s="37" t="n">
+      <x:c r="B10" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Blocked")</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D10" s="36" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
-      <x:c r="E10" s="37" t="n">
+      <x:c r="E10" s="34" t="n">
         <x:f>COUNTIF(Requirements!$G$6:$G$23,"Approved")</x:f>
         <x:v>18</x:v>
       </x:c>
-      <x:c r="G10" s="40" t="str">
+      <x:c r="G10" s="39" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="H10" s="40" t="n">
+      <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="36" t="str">
+      <x:c r="A11" s="33" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="B11" s="37" t="n">
+      <x:c r="B11" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="39" t="str">
+      <x:c r="A13" s="38" t="str">
         <x:v>Launch gate</x:v>
       </x:c>
-      <x:c r="B13" s="39" t="str">
+      <x:c r="B13" s="38" t="str">
         <x:v>Current state</x:v>
       </x:c>
-      <x:c r="C13" s="39" t="str">
+      <x:c r="C13" s="38" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="D13" s="39" t="str">
+      <x:c r="D13" s="38" t="str">
         <x:v>Evidence needed</x:v>
       </x:c>
-      <x:c r="E13" s="39" t="str">
+      <x:c r="E13" s="38" t="str">
         <x:v>Rule</x:v>
       </x:c>
     </x:row>
@@ -1381,16 +1378,16 @@
         <x:v>Repository foundation</x:v>
       </x:c>
       <x:c r="B14" s="26" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="C14" s="26" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="D14" s="26" t="str">
-        <x:v>Upgrade GitHub plan for protected private branches and native security uploads</x:v>
+        <x:v>Public visibility, protected main and native security controls verified</x:v>
       </x:c>
       <x:c r="E14" s="26" t="str">
-        <x:v>Compensating CI controls are active</x:v>
+        <x:v>Reassess only if repository visibility changes</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1453,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03779c0f350c45a8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63679649290d49ab"/>
 </x:worksheet>
 </file>
 
@@ -1835,7 +1832,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591602fb704346fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a5761488a154d3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3088,10 +3085,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F36" s="26" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G36" s="26" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H36" s="26" t="str"/>
       <x:c r="I36" s="26" t="str">
@@ -3103,7 +3100,9 @@
       <x:c r="K36" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/36</x:v>
       </x:c>
-      <x:c r="L36" s="26" t="str"/>
+      <x:c r="L36" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
+      </x:c>
       <x:c r="M36" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
@@ -3163,7 +3162,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaefd2482d744112"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce5be5c9f0fc4dcf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3647,7 +3646,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58d8b83a4f87494f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a4bd8205444c42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3937,7 +3936,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570d5d231dcc45ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc1a9cf5f6214532"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4272,42 +4271,71 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="27" t="str">
+      <x:c r="A16" s="26" t="str">
         <x:v>RISK-011</x:v>
       </x:c>
-      <x:c r="B16" s="27" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>Private repository cannot enforce native branch protection or secret scanning on the current GitHub plan</x:v>
       </x:c>
-      <x:c r="C16" s="27" t="str">
+      <x:c r="C16" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D16" s="27" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>Certain</x:v>
       </x:c>
-      <x:c r="E16" s="27" t="str">
+      <x:c r="E16" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F16" s="27" t="str">
-        <x:v>Use PR discipline and CI Gitleaks as compensating controls; upgrade to GitHub Pro or an eligible organization before production</x:v>
-      </x:c>
-      <x:c r="G16" s="27" t="str">
+      <x:c r="F16" s="26" t="str">
+        <x:v>Temporarily use public visibility with protected main and native security controls; return private only on an eligible tier</x:v>
+      </x:c>
+      <x:c r="G16" s="26" t="str">
         <x:v>Product owner</x:v>
       </x:c>
-      <x:c r="H16" s="27" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="I16" s="27" t="str">
-        <x:v>GitHub API returned HTTP 403 and 422 on 2026-10-04</x:v>
+      <x:c r="H16" s="26" t="str">
+        <x:v>Mitigated</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="str">
+        <x:v>Public visibility and controls enabled through GOV-001 on 2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="27" t="str">
+        <x:v>RISK-012</x:v>
+      </x:c>
+      <x:c r="B17" s="27" t="str">
+        <x:v>Public source exposes architecture test conventions and historical development-only credentials</x:v>
+      </x:c>
+      <x:c r="C17" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D17" s="27" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E17" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F17" s="27" t="str">
+        <x:v>Remove fallback credentials; keep real secrets and PII outside Git; require push protection Gitleaks and native scanning</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="H17" s="27" t="str">
+        <x:v>Mitigated</x:v>
+      </x:c>
+      <x:c r="I17" s="27" t="str">
+        <x:v>Tracked history scanned; seed fallback removed in GOV-001; test and production credentials require external stores</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E16">
+  <x:conditionalFormatting sqref="E6:E17">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H16">
+  <x:conditionalFormatting sqref="H6:H17">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4316,7 +4344,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R260a82e3bf8644c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb70774e2ae484084"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4386,7 +4414,7 @@
         <x:v>GitHub</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str">
-        <x:v>Repository admin and Actions environments</x:v>
+        <x:v>Public repository admin and Actions environments</x:v>
       </x:c>
       <x:c r="D6" s="25" t="str">
         <x:v>RohithTadiparti</x:v>
@@ -4404,7 +4432,7 @@
         <x:v>2026-10-04</x:v>
       </x:c>
       <x:c r="I6" s="25" t="str">
-        <x:v>Private repository created</x:v>
+        <x:v>Public visibility; protected main; native secret scanning and push protection enabled</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -4636,7 +4664,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re830ad96462143d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9137fc2d18e49b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4975,7 +5003,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cd581407914487e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1922bddb2b42eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5113,7 +5141,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a1bfa5b87c24683"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6791021829b644cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5188,40 +5216,76 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="32" t="str">
+      <x:c r="A6" s="25" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B6" s="32" t="str">
+      <x:c r="B6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
-      <x:c r="C6" s="32" t="str">
+      <x:c r="C6" s="25" t="str">
         <x:v>codex/gov-002-production-program</x:v>
       </x:c>
-      <x:c r="D6" s="32" t="str">
+      <x:c r="D6" s="25" t="str">
         <x:v>1e9f458</x:v>
       </x:c>
-      <x:c r="E6" s="32" t="str">
+      <x:c r="E6" s="25" t="str">
         <x:v>4444b86</x:v>
       </x:c>
-      <x:c r="F6" s="32" t="str">
+      <x:c r="F6" s="25" t="str">
         <x:v>07218b4ab02a8702a4d8d9fdab7dc26e579ab7b4</x:v>
       </x:c>
-      <x:c r="G6" s="32" t="str">
+      <x:c r="G6" s="25" t="str">
         <x:v>Final PR head 4444b86: backend build/test pass; frontend pass; mobile pass; Docker build pass; registers pass; Gitleaks pass; CodeQL JavaScript/TypeScript and Actions pass with 30-day SARIF artifacts; local governance 4/4</x:v>
       </x:c>
-      <x:c r="H6" s="32" t="str">
+      <x:c r="H6" s="25" t="str">
         <x:v>Documentation and governance only; no Railway deployment</x:v>
       </x:c>
-      <x:c r="I6" s="32" t="str">
+      <x:c r="I6" s="25" t="str">
         <x:v>Revert PR 49; bootstrap remains clean source snapshot</x:v>
       </x:c>
-      <x:c r="J6" s="32" t="str">
+      <x:c r="J6" s="25" t="str">
         <x:v>GitHub plan blocks protected private branches native secret scanning and native CodeQL upload; offline SARIF and CI Gitleaks compensate; tracked by GOV-001</x:v>
       </x:c>
-      <x:c r="K6" s="32" t="str">
+      <x:c r="K6" s="25" t="str">
         <x:v>Ready to Merge</x:v>
       </x:c>
-      <x:c r="L6" s="33" t="str">
+      <x:c r="L6" s="28" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="27" t="str">
+        <x:v>GOV-001</x:v>
+      </x:c>
+      <x:c r="B7" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
+      </x:c>
+      <x:c r="C7" s="27" t="str">
+        <x:v>codex/gov-001-public-protection</x:v>
+      </x:c>
+      <x:c r="D7" s="27" t="str">
+        <x:v>922cfee</x:v>
+      </x:c>
+      <x:c r="E7" s="27" t="str">
+        <x:v>152f4d3</x:v>
+      </x:c>
+      <x:c r="F7" s="27" t="str"/>
+      <x:c r="G7" s="27" t="str">
+        <x:v>Final PR head 152f4d3: backend E2E and tests pass; frontend pass; mobile pass; Docker pass; registers pass; Gitleaks pass; native CodeQL JavaScript/TypeScript and Actions pass; seed config 3/3; governance 7/7</x:v>
+      </x:c>
+      <x:c r="H7" s="27" t="str">
+        <x:v>GitHub visibility and protection settings plus repository security configuration; no application deploy</x:v>
+      </x:c>
+      <x:c r="I7" s="27" t="str">
+        <x:v>Change visibility/settings separately and revert PR; never restore fallback credential</x:v>
+      </x:c>
+      <x:c r="J7" s="27" t="str">
+        <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
+      </x:c>
+      <x:c r="K7" s="27" t="str">
+        <x:v>Ready to Merge</x:v>
+      </x:c>
+      <x:c r="L7" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
@@ -5229,7 +5293,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K6">
+  <x:conditionalFormatting sqref="K6:K7">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5238,7 +5302,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47d13f9f27c14e5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe9ec4b2cb7348ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[GOV-001] Enforce public repository protections (#54)
* security: protect public production repository

* docs: record public protection handoff

* docs: finalize public protection tracker

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbd410f0f7a794916"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rd76d9bd425db4268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4838a44155b54de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rffa97dc825e345c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R57301af3b787409e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd3cee27f371d4329"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R4618652927bd4f41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2bf01e34651f476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re77a0d23d5314a11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R5571ec6bfb3d4102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra82fc0183a11442b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6fa20bf17f3a45af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4a49a0f0e6e04497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rd7653db751404ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R88508ddfc8394578"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R160115c5e8ae4b89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd82b27fc55604d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R72cc06c0ec304ea6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R23350c76e9fd4e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8579165ef61c4e2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -124,7 +124,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -192,15 +192,6 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
@@ -211,6 +202,12 @@
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -833,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd639e8844633464d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39762c3c77f04b08"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -894,7 +891,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -963,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1210,169 +1207,169 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-04. Counts link to the canonical CSV registers included in the private production repository.</x:v>
+        <x:v>As of 2026-10-04. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
+      <x:c r="A5" s="31" t="str">
         <x:v>Work items</x:v>
       </x:c>
-      <x:c r="B5" s="35" t="str">
+      <x:c r="B5" s="32" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D5" s="34" t="str">
+      <x:c r="D5" s="31" t="str">
         <x:v>Readiness</x:v>
       </x:c>
-      <x:c r="E5" s="35" t="str">
+      <x:c r="E5" s="32" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="G5" s="40" t="str">
+      <x:c r="G5" s="39" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="40" t="str">
+      <x:c r="H5" s="39" t="str">
         <x:v>Count</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="36" t="str">
+      <x:c r="A6" s="33" t="str">
         <x:v>Total</x:v>
       </x:c>
-      <x:c r="B6" s="37" t="n">
+      <x:c r="B6" s="34" t="n">
         <x:f>COUNTA('Open Items'!$A$6:$A$37)</x:f>
         <x:v>32</x:v>
       </x:c>
-      <x:c r="D6" s="36" t="str">
+      <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
-      <x:c r="E6" s="37" t="n">
+      <x:c r="E6" s="34" t="n">
         <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="G6" s="40" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="H6" s="40" t="n">
+      <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
         <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="36" t="str">
+      <x:c r="A7" s="33" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="B7" s="37" t="n">
+      <x:c r="B7" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Open")</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="D7" s="36" t="str">
+      <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
       </x:c>
-      <x:c r="E7" s="37" t="n">
+      <x:c r="E7" s="34" t="n">
         <x:f>COUNTIF('Release Gates'!$E$6:$E$17,"Open")</x:f>
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G7" s="40" t="str">
+      <x:c r="G7" s="39" t="str">
         <x:v>In Progress</x:v>
       </x:c>
-      <x:c r="H7" s="40" t="n">
+      <x:c r="H7" s="39" t="n">
         <x:f>B8</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="36" t="str">
+      <x:c r="A8" s="33" t="str">
         <x:v>In Progress</x:v>
       </x:c>
-      <x:c r="B8" s="37" t="n">
+      <x:c r="B8" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D8" s="36" t="str">
+      <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
-      <x:c r="E8" s="37" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$16,"Open")</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G8" s="40" t="str">
+      <x:c r="E8" s="34" t="n">
+        <x:f>COUNTIF(Risks!$H$6:$H$17,"Open")</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
       </x:c>
-      <x:c r="H8" s="40" t="n">
+      <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="36" t="str">
+      <x:c r="A9" s="33" t="str">
         <x:v>PR Open</x:v>
       </x:c>
-      <x:c r="B9" s="37" t="n">
+      <x:c r="B9" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D9" s="36" t="str">
+      <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
-      <x:c r="E9" s="37" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$16,"P0",Risks!$H$6:$H$16,"Open")</x:f>
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="G9" s="40" t="str">
+      <x:c r="E9" s="34" t="n">
+        <x:f>COUNTIFS(Risks!$E$6:$E$17,"P0",Risks!$H$6:$H$17,"Open")</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G9" s="39" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="H9" s="40" t="n">
+      <x:c r="H9" s="39" t="n">
         <x:f>B10</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="36" t="str">
+      <x:c r="A10" s="33" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="B10" s="37" t="n">
+      <x:c r="B10" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Blocked")</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D10" s="36" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
-      <x:c r="E10" s="37" t="n">
+      <x:c r="E10" s="34" t="n">
         <x:f>COUNTIF(Requirements!$G$6:$G$23,"Approved")</x:f>
         <x:v>18</x:v>
       </x:c>
-      <x:c r="G10" s="40" t="str">
+      <x:c r="G10" s="39" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="H10" s="40" t="n">
+      <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="36" t="str">
+      <x:c r="A11" s="33" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="B11" s="37" t="n">
+      <x:c r="B11" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="39" t="str">
+      <x:c r="A13" s="38" t="str">
         <x:v>Launch gate</x:v>
       </x:c>
-      <x:c r="B13" s="39" t="str">
+      <x:c r="B13" s="38" t="str">
         <x:v>Current state</x:v>
       </x:c>
-      <x:c r="C13" s="39" t="str">
+      <x:c r="C13" s="38" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="D13" s="39" t="str">
+      <x:c r="D13" s="38" t="str">
         <x:v>Evidence needed</x:v>
       </x:c>
-      <x:c r="E13" s="39" t="str">
+      <x:c r="E13" s="38" t="str">
         <x:v>Rule</x:v>
       </x:c>
     </x:row>
@@ -1381,16 +1378,16 @@
         <x:v>Repository foundation</x:v>
       </x:c>
       <x:c r="B14" s="26" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="C14" s="26" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="D14" s="26" t="str">
-        <x:v>Upgrade GitHub plan for protected private branches and native security uploads</x:v>
+        <x:v>Public visibility, protected main and native security controls verified</x:v>
       </x:c>
       <x:c r="E14" s="26" t="str">
-        <x:v>Compensating CI controls are active</x:v>
+        <x:v>Reassess only if repository visibility changes</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1453,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03779c0f350c45a8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63679649290d49ab"/>
 </x:worksheet>
 </file>
 
@@ -1835,7 +1832,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591602fb704346fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a5761488a154d3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3088,10 +3085,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F36" s="26" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G36" s="26" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H36" s="26" t="str"/>
       <x:c r="I36" s="26" t="str">
@@ -3103,7 +3100,9 @@
       <x:c r="K36" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/36</x:v>
       </x:c>
-      <x:c r="L36" s="26" t="str"/>
+      <x:c r="L36" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
+      </x:c>
       <x:c r="M36" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
@@ -3163,7 +3162,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaefd2482d744112"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce5be5c9f0fc4dcf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3647,7 +3646,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58d8b83a4f87494f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a4bd8205444c42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3937,7 +3936,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570d5d231dcc45ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc1a9cf5f6214532"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4272,42 +4271,71 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="27" t="str">
+      <x:c r="A16" s="26" t="str">
         <x:v>RISK-011</x:v>
       </x:c>
-      <x:c r="B16" s="27" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>Private repository cannot enforce native branch protection or secret scanning on the current GitHub plan</x:v>
       </x:c>
-      <x:c r="C16" s="27" t="str">
+      <x:c r="C16" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D16" s="27" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>Certain</x:v>
       </x:c>
-      <x:c r="E16" s="27" t="str">
+      <x:c r="E16" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F16" s="27" t="str">
-        <x:v>Use PR discipline and CI Gitleaks as compensating controls; upgrade to GitHub Pro or an eligible organization before production</x:v>
-      </x:c>
-      <x:c r="G16" s="27" t="str">
+      <x:c r="F16" s="26" t="str">
+        <x:v>Temporarily use public visibility with protected main and native security controls; return private only on an eligible tier</x:v>
+      </x:c>
+      <x:c r="G16" s="26" t="str">
         <x:v>Product owner</x:v>
       </x:c>
-      <x:c r="H16" s="27" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="I16" s="27" t="str">
-        <x:v>GitHub API returned HTTP 403 and 422 on 2026-10-04</x:v>
+      <x:c r="H16" s="26" t="str">
+        <x:v>Mitigated</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="str">
+        <x:v>Public visibility and controls enabled through GOV-001 on 2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="27" t="str">
+        <x:v>RISK-012</x:v>
+      </x:c>
+      <x:c r="B17" s="27" t="str">
+        <x:v>Public source exposes architecture test conventions and historical development-only credentials</x:v>
+      </x:c>
+      <x:c r="C17" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D17" s="27" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E17" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F17" s="27" t="str">
+        <x:v>Remove fallback credentials; keep real secrets and PII outside Git; require push protection Gitleaks and native scanning</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="H17" s="27" t="str">
+        <x:v>Mitigated</x:v>
+      </x:c>
+      <x:c r="I17" s="27" t="str">
+        <x:v>Tracked history scanned; seed fallback removed in GOV-001; test and production credentials require external stores</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E16">
+  <x:conditionalFormatting sqref="E6:E17">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H16">
+  <x:conditionalFormatting sqref="H6:H17">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4316,7 +4344,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R260a82e3bf8644c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb70774e2ae484084"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4386,7 +4414,7 @@
         <x:v>GitHub</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str">
-        <x:v>Repository admin and Actions environments</x:v>
+        <x:v>Public repository admin and Actions environments</x:v>
       </x:c>
       <x:c r="D6" s="25" t="str">
         <x:v>RohithTadiparti</x:v>
@@ -4404,7 +4432,7 @@
         <x:v>2026-10-04</x:v>
       </x:c>
       <x:c r="I6" s="25" t="str">
-        <x:v>Private repository created</x:v>
+        <x:v>Public visibility; protected main; native secret scanning and push protection enabled</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -4636,7 +4664,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re830ad96462143d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9137fc2d18e49b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4975,7 +5003,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cd581407914487e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1922bddb2b42eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5113,7 +5141,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a1bfa5b87c24683"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6791021829b644cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5188,40 +5216,76 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="32" t="str">
+      <x:c r="A6" s="25" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B6" s="32" t="str">
+      <x:c r="B6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
-      <x:c r="C6" s="32" t="str">
+      <x:c r="C6" s="25" t="str">
         <x:v>codex/gov-002-production-program</x:v>
       </x:c>
-      <x:c r="D6" s="32" t="str">
+      <x:c r="D6" s="25" t="str">
         <x:v>1e9f458</x:v>
       </x:c>
-      <x:c r="E6" s="32" t="str">
+      <x:c r="E6" s="25" t="str">
         <x:v>4444b86</x:v>
       </x:c>
-      <x:c r="F6" s="32" t="str">
+      <x:c r="F6" s="25" t="str">
         <x:v>07218b4ab02a8702a4d8d9fdab7dc26e579ab7b4</x:v>
       </x:c>
-      <x:c r="G6" s="32" t="str">
+      <x:c r="G6" s="25" t="str">
         <x:v>Final PR head 4444b86: backend build/test pass; frontend pass; mobile pass; Docker build pass; registers pass; Gitleaks pass; CodeQL JavaScript/TypeScript and Actions pass with 30-day SARIF artifacts; local governance 4/4</x:v>
       </x:c>
-      <x:c r="H6" s="32" t="str">
+      <x:c r="H6" s="25" t="str">
         <x:v>Documentation and governance only; no Railway deployment</x:v>
       </x:c>
-      <x:c r="I6" s="32" t="str">
+      <x:c r="I6" s="25" t="str">
         <x:v>Revert PR 49; bootstrap remains clean source snapshot</x:v>
       </x:c>
-      <x:c r="J6" s="32" t="str">
+      <x:c r="J6" s="25" t="str">
         <x:v>GitHub plan blocks protected private branches native secret scanning and native CodeQL upload; offline SARIF and CI Gitleaks compensate; tracked by GOV-001</x:v>
       </x:c>
-      <x:c r="K6" s="32" t="str">
+      <x:c r="K6" s="25" t="str">
         <x:v>Ready to Merge</x:v>
       </x:c>
-      <x:c r="L6" s="33" t="str">
+      <x:c r="L6" s="28" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="27" t="str">
+        <x:v>GOV-001</x:v>
+      </x:c>
+      <x:c r="B7" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
+      </x:c>
+      <x:c r="C7" s="27" t="str">
+        <x:v>codex/gov-001-public-protection</x:v>
+      </x:c>
+      <x:c r="D7" s="27" t="str">
+        <x:v>922cfee</x:v>
+      </x:c>
+      <x:c r="E7" s="27" t="str">
+        <x:v>152f4d3</x:v>
+      </x:c>
+      <x:c r="F7" s="27" t="str"/>
+      <x:c r="G7" s="27" t="str">
+        <x:v>Final PR head 152f4d3: backend E2E and tests pass; frontend pass; mobile pass; Docker pass; registers pass; Gitleaks pass; native CodeQL JavaScript/TypeScript and Actions pass; seed config 3/3; governance 7/7</x:v>
+      </x:c>
+      <x:c r="H7" s="27" t="str">
+        <x:v>GitHub visibility and protection settings plus repository security configuration; no application deploy</x:v>
+      </x:c>
+      <x:c r="I7" s="27" t="str">
+        <x:v>Change visibility/settings separately and revert PR; never restore fallback credential</x:v>
+      </x:c>
+      <x:c r="J7" s="27" t="str">
+        <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
+      </x:c>
+      <x:c r="K7" s="27" t="str">
+        <x:v>Ready to Merge</x:v>
+      </x:c>
+      <x:c r="L7" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
@@ -5229,7 +5293,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K6">
+  <x:conditionalFormatting sqref="K6:K7">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5238,7 +5302,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47d13f9f27c14e5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe9ec4b2cb7348ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record gated synchronization evidence
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra82fc0183a11442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6fa20bf17f3a45af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4a49a0f0e6e04497"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rd7653db751404ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R88508ddfc8394578"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R160115c5e8ae4b89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd82b27fc55604d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R72cc06c0ec304ea6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R23350c76e9fd4e1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8579165ef61c4e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rced6b8c1b8194838"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R7d2d303979104084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R98d5bb16e39c429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R67c85165d27f4bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R3b395bff36234a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rb9af5b80b5184ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R72b4ce95dd2640e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R1c3961feb2f84f99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0b78da0762334c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R36ded813f00c450a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39762c3c77f04b08"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4b1f48128d824329"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -876,7 +876,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Layer"/>
@@ -908,7 +908,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AccessTable" displayName="AccessTable" ref="A5:I14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="System"/>
@@ -941,7 +941,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -960,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -980,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1250,7 +1250,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1259,7 +1259,7 @@
       </x:c>
       <x:c r="B7" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Open")</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1296,7 +1296,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1305,7 +1305,7 @@
       </x:c>
       <x:c r="B9" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63679649290d49ab"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a0f2671ac704caa"/>
 </x:worksheet>
 </file>
 
@@ -1732,7 +1732,7 @@
         <x:v>Active</x:v>
       </x:c>
       <x:c r="F14" s="26" t="str">
-        <x:v>Monthly</x:v>
+        <x:v>Each source review</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
         <x:v>2026-10-04</x:v>
@@ -1794,36 +1794,62 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>DOC-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>Production tracking workbook</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>docs/tracking/production-readiness-tracker.xlsx</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>Program management</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Each change</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
-      <x:c r="H17" s="27" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>GOV-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="27" t="str">
+        <x:v>DOC-013</x:v>
+      </x:c>
+      <x:c r="B18" s="27" t="str">
+        <x:v>Gated source synchronization plan</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
+        <x:v>docs/superpowers/plans/2026-10-04-gated-source-synchronization.md</x:v>
+      </x:c>
+      <x:c r="D18" s="27" t="str">
+        <x:v>Release engineering</x:v>
+      </x:c>
+      <x:c r="E18" s="27" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="F18" s="27" t="str">
+        <x:v>On synchronization policy change</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="H18" s="27" t="str">
+        <x:v>SYNC-002</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E17">
+  <x:conditionalFormatting sqref="E6:E18">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -1832,7 +1858,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a5761488a154d3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89be10ce9c6b4e90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2931,10 +2957,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F32" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G32" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H32" s="26" t="str">
         <x:v>GOV-002</x:v>
@@ -2948,7 +2974,9 @@
       <x:c r="K32" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/32</x:v>
       </x:c>
-      <x:c r="L32" s="26" t="str"/>
+      <x:c r="L32" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
+      </x:c>
       <x:c r="M32" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
@@ -3162,7 +3190,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce5be5c9f0fc4dcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7b5a2b146a24c07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3646,7 +3674,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a4bd8205444c42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5ff126c32084cd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3908,26 +3936,49 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="27" t="str">
+      <x:c r="A15" s="26" t="str">
         <x:v>QA-RES-001</x:v>
       </x:c>
-      <x:c r="B15" s="27" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>Resilience</x:v>
       </x:c>
-      <x:c r="C15" s="27" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>Backup restore and failed cutover</x:v>
       </x:c>
-      <x:c r="D15" s="27" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="E15" s="27" t="str">
+      <x:c r="E15" s="26" t="str">
         <x:v>Not run</x:v>
       </x:c>
-      <x:c r="F15" s="27" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>Successful restore and two rollback rehearsals</x:v>
       </x:c>
-      <x:c r="G15" s="27" t="str">
+      <x:c r="G15" s="26" t="str">
         <x:v>QA-002 QA-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="27" t="str">
+        <x:v>QA-GOV-001</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="str">
+        <x:v>Source synchronization</x:v>
+      </x:c>
+      <x:c r="C16" s="27" t="str">
+        <x:v>Private-source report and shared-code mirror gate</x:v>
+      </x:c>
+      <x:c r="D16" s="27" t="str">
+        <x:v>PR 55 local evidence</x:v>
+      </x:c>
+      <x:c r="E16" s="27" t="str">
+        <x:v>18 of 18 governance and synchronization tests passed</x:v>
+      </x:c>
+      <x:c r="F16" s="27" t="str">
+        <x:v>Configure WOW_SYNC_TOKEN and capture first scheduled artifact</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="str">
+        <x:v>SYNC-002</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3936,7 +3987,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc1a9cf5f6214532"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c6e6647bb1c44d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4344,7 +4395,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb70774e2ae484084"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra65406fab91a4a30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4625,37 +4676,64 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="27" t="str">
+      <x:c r="A14" s="26" t="str">
         <x:v>ACC-009</x:v>
       </x:c>
-      <x:c r="B14" s="27" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>SMS WhatsApp push identity</x:v>
       </x:c>
-      <x:c r="C14" s="27" t="str">
+      <x:c r="C14" s="26" t="str">
         <x:v>Provider sandbox then production accounts</x:v>
       </x:c>
-      <x:c r="D14" s="27" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
-      <x:c r="E14" s="27" t="str">
+      <x:c r="E14" s="26" t="str">
         <x:v>Provider credentials</x:v>
       </x:c>
-      <x:c r="F14" s="27" t="str">
+      <x:c r="F14" s="26" t="str">
         <x:v>Protected secret store</x:v>
       </x:c>
-      <x:c r="G14" s="27" t="str">
+      <x:c r="G14" s="26" t="str">
         <x:v>Deferred</x:v>
       </x:c>
-      <x:c r="H14" s="30" t="str"/>
-      <x:c r="I14" s="27" t="str">
+      <x:c r="H14" s="29" t="str"/>
+      <x:c r="I14" s="26" t="str">
         <x:v>Separate onboarding gates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="27" t="str">
+        <x:v>ACC-010</x:v>
+      </x:c>
+      <x:c r="B15" s="27" t="str">
+        <x:v>WOW-MD source review</x:v>
+      </x:c>
+      <x:c r="C15" s="27" t="str">
+        <x:v>Private repository contents read for scheduled change reports</x:v>
+      </x:c>
+      <x:c r="D15" s="27" t="str">
+        <x:v>RohithTadiparti</x:v>
+      </x:c>
+      <x:c r="E15" s="27" t="str">
+        <x:v>Fine-grained WOW_SYNC_TOKEN</x:v>
+      </x:c>
+      <x:c r="F15" s="27" t="str">
+        <x:v>Production GitHub Actions secret</x:v>
+      </x:c>
+      <x:c r="G15" s="27" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="H15" s="30" t="str"/>
+      <x:c r="I15" s="27" t="str">
+        <x:v>Scope only to WOW-MD Contents read; rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="G6:G14">
+  <x:conditionalFormatting sqref="G6:G15">
     <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="20" priority="3" operator="containsText" text="Blocked"/>
@@ -4664,7 +4742,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9137fc2d18e49b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96b9b570c2134943"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5003,7 +5081,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1922bddb2b42eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3947e508ad7477c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5105,34 +5183,69 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="26" t="str">
         <x:v>CHG-002</x:v>
       </x:c>
-      <x:c r="B7" s="27" t="str">
+      <x:c r="B7" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C7" s="27" t="str">
+      <x:c r="C7" s="26" t="str">
         <x:v>UNCOMMITTED</x:v>
       </x:c>
-      <x:c r="D7" s="27" t="str">
+      <x:c r="D7" s="26" t="str">
         <x:v>.gitignore</x:v>
       </x:c>
-      <x:c r="E7" s="27" t="str">
+      <x:c r="E7" s="26" t="str">
         <x:v>Repository hygiene</x:v>
       </x:c>
-      <x:c r="F7" s="27" t="str">
+      <x:c r="F7" s="26" t="str">
         <x:v>Review required</x:v>
       </x:c>
-      <x:c r="G7" s="27" t="str">
+      <x:c r="G7" s="26" t="str">
         <x:v>SYNC-001</x:v>
       </x:c>
-      <x:c r="H7" s="27" t="str"/>
-      <x:c r="I7" s="27" t="str"/>
-      <x:c r="J7" s="30" t="str">
+      <x:c r="H7" s="26" t="str"/>
+      <x:c r="I7" s="26" t="str"/>
+      <x:c r="J7" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
-      <x:c r="K7" s="27" t="str">
+      <x:c r="K7" s="26" t="str">
         <x:v>Three ignored paths require review before adoption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="27" t="str">
+        <x:v>CHG-003</x:v>
+      </x:c>
+      <x:c r="B8" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C8" s="27" t="str">
+        <x:v>07218b4..de7d8dd (LOCAL ONLY)</x:v>
+      </x:c>
+      <x:c r="D8" s="27" t="str">
+        <x:v>37 committed paths</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="str">
+        <x:v>Functional UI candidates</x:v>
+      </x:c>
+      <x:c r="F8" s="27" t="str">
+        <x:v>Await source publication and per-commit review</x:v>
+      </x:c>
+      <x:c r="G8" s="27" t="str">
+        <x:v>SYNC-002</x:v>
+      </x:c>
+      <x:c r="H8" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
+      </x:c>
+      <x:c r="I8" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J8" s="30" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="K8" s="27" t="str">
+        <x:v>Local main is 21 commits ahead of origin; scheduled GitHub review intentionally sees pushed commits only</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5141,7 +5254,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6791021829b644cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc26986dc0e649b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5254,38 +5367,76 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="26" t="str">
         <x:v>GOV-001</x:v>
       </x:c>
-      <x:c r="B7" s="27" t="str">
+      <x:c r="B7" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
       </x:c>
-      <x:c r="C7" s="27" t="str">
+      <x:c r="C7" s="26" t="str">
         <x:v>codex/gov-001-public-protection</x:v>
       </x:c>
-      <x:c r="D7" s="27" t="str">
+      <x:c r="D7" s="26" t="str">
         <x:v>922cfee</x:v>
       </x:c>
-      <x:c r="E7" s="27" t="str">
+      <x:c r="E7" s="26" t="str">
         <x:v>152f4d3</x:v>
       </x:c>
-      <x:c r="F7" s="27" t="str"/>
-      <x:c r="G7" s="27" t="str">
+      <x:c r="F7" s="26" t="str"/>
+      <x:c r="G7" s="26" t="str">
         <x:v>Final PR head 152f4d3: backend E2E and tests pass; frontend pass; mobile pass; Docker pass; registers pass; Gitleaks pass; native CodeQL JavaScript/TypeScript and Actions pass; seed config 3/3; governance 7/7</x:v>
       </x:c>
-      <x:c r="H7" s="27" t="str">
+      <x:c r="H7" s="26" t="str">
         <x:v>GitHub visibility and protection settings plus repository security configuration; no application deploy</x:v>
       </x:c>
-      <x:c r="I7" s="27" t="str">
+      <x:c r="I7" s="26" t="str">
         <x:v>Change visibility/settings separately and revert PR; never restore fallback credential</x:v>
       </x:c>
-      <x:c r="J7" s="27" t="str">
+      <x:c r="J7" s="26" t="str">
         <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
       </x:c>
-      <x:c r="K7" s="27" t="str">
+      <x:c r="K7" s="26" t="str">
         <x:v>Ready to Merge</x:v>
       </x:c>
-      <x:c r="L7" s="30" t="str">
+      <x:c r="L7" s="29" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="27" t="str">
+        <x:v>SYNC-002</x:v>
+      </x:c>
+      <x:c r="B8" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
+      </x:c>
+      <x:c r="C8" s="27" t="str">
+        <x:v>codex/sync-002-gated-source-review</x:v>
+      </x:c>
+      <x:c r="D8" s="27" t="str">
+        <x:v>57e13d0</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="str">
+        <x:v>dbe8c4a</x:v>
+      </x:c>
+      <x:c r="F8" s="27" t="str">
+        <x:v>07218b4..de7d8dd local review only</x:v>
+      </x:c>
+      <x:c r="G8" s="27" t="str">
+        <x:v>Source report 4/4; mirror gate 5/5; workflow policy 2/2; full governance/source-sync 18/18; local report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
+      </x:c>
+      <x:c r="H8" s="27" t="str">
+        <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
+      </x:c>
+      <x:c r="I8" s="27" t="str">
+        <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
+      </x:c>
+      <x:c r="J8" s="27" t="str">
+        <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
+      </x:c>
+      <x:c r="K8" s="27" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L8" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
@@ -5293,7 +5444,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K7">
+  <x:conditionalFormatting sqref="K6:K8">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5302,7 +5453,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe9ec4b2cb7348ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd204ad8ba424aa4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: fetch pull request history for mirror gate
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rced6b8c1b8194838"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R7d2d303979104084"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R98d5bb16e39c429b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R67c85165d27f4bb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R3b395bff36234a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rb9af5b80b5184ed3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R72b4ce95dd2640e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R1c3961feb2f84f99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0b78da0762334c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R36ded813f00c450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R70806f8fb651404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R661f9c31ea1449b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rad441362aa0943e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rd8ac6ce0b3f14309"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb31b3668378f40c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R7e4399604def40b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R45feca86bad9493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re3818a5054ba46b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R356fda15c0274990"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R989f14421a284993"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4b1f48128d824329"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45a6d1b0e8654d81"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a0f2671ac704caa"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3b238460cf84085"/>
 </x:worksheet>
 </file>
 
@@ -1858,7 +1858,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89be10ce9c6b4e90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801b696960d646ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3190,7 +3190,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7b5a2b146a24c07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac881b7a496645de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3674,7 +3674,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5ff126c32084cd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ef0f0c087d44d22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3972,7 +3972,7 @@
         <x:v>PR 55 local evidence</x:v>
       </x:c>
       <x:c r="E16" s="27" t="str">
-        <x:v>18 of 18 governance and synchronization tests passed</x:v>
+        <x:v>19 of 19 governance and synchronization tests passed</x:v>
       </x:c>
       <x:c r="F16" s="27" t="str">
         <x:v>Configure WOW_SYNC_TOKEN and capture first scheduled artifact</x:v>
@@ -3987,7 +3987,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c6e6647bb1c44d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b83c550d0b345d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4395,7 +4395,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra65406fab91a4a30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0324b0b93e7417f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4742,7 +4742,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96b9b570c2134943"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R065ea2fb57e64d13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5081,7 +5081,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3947e508ad7477c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9afc42721174ce2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5254,7 +5254,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc26986dc0e649b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R044acd53e2964cb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5422,7 +5422,7 @@
         <x:v>07218b4..de7d8dd local review only</x:v>
       </x:c>
       <x:c r="G8" s="27" t="str">
-        <x:v>Source report 4/4; mirror gate 5/5; workflow policy 2/2; full governance/source-sync 18/18; local report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
+        <x:v>Source report 4/4; mirror gate 5/5; workflow policy 3/3; full governance/source-sync 19/19; local report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
       </x:c>
       <x:c r="H8" s="27" t="str">
         <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
@@ -5453,7 +5453,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd204ad8ba424aa4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad8447f83d3747c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[SYNC-002] Add gated periodic source synchronization (#55)
* feat: add deterministic source synchronization report

* ci: schedule gated source change reviews

* ci: require reviewed WOW mirrors for shared changes

* docs: record gated synchronization evidence

* fix: fetch pull request history for mirror gate

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra82fc0183a11442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6fa20bf17f3a45af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4a49a0f0e6e04497"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rd7653db751404ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R88508ddfc8394578"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R160115c5e8ae4b89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd82b27fc55604d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R72cc06c0ec304ea6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R23350c76e9fd4e1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8579165ef61c4e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R70806f8fb651404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R661f9c31ea1449b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rad441362aa0943e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rd8ac6ce0b3f14309"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb31b3668378f40c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R7e4399604def40b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R45feca86bad9493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re3818a5054ba46b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R356fda15c0274990"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R989f14421a284993"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39762c3c77f04b08"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45a6d1b0e8654d81"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -876,7 +876,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Layer"/>
@@ -908,7 +908,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AccessTable" displayName="AccessTable" ref="A5:I14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="System"/>
@@ -941,7 +941,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -960,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -980,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1250,7 +1250,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1259,7 +1259,7 @@
       </x:c>
       <x:c r="B7" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Open")</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1296,7 +1296,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1305,7 +1305,7 @@
       </x:c>
       <x:c r="B9" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63679649290d49ab"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3b238460cf84085"/>
 </x:worksheet>
 </file>
 
@@ -1732,7 +1732,7 @@
         <x:v>Active</x:v>
       </x:c>
       <x:c r="F14" s="26" t="str">
-        <x:v>Monthly</x:v>
+        <x:v>Each source review</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
         <x:v>2026-10-04</x:v>
@@ -1794,36 +1794,62 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>DOC-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>Production tracking workbook</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>docs/tracking/production-readiness-tracker.xlsx</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>Program management</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Each change</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
-      <x:c r="H17" s="27" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>GOV-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="27" t="str">
+        <x:v>DOC-013</x:v>
+      </x:c>
+      <x:c r="B18" s="27" t="str">
+        <x:v>Gated source synchronization plan</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
+        <x:v>docs/superpowers/plans/2026-10-04-gated-source-synchronization.md</x:v>
+      </x:c>
+      <x:c r="D18" s="27" t="str">
+        <x:v>Release engineering</x:v>
+      </x:c>
+      <x:c r="E18" s="27" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="F18" s="27" t="str">
+        <x:v>On synchronization policy change</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="H18" s="27" t="str">
+        <x:v>SYNC-002</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E17">
+  <x:conditionalFormatting sqref="E6:E18">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -1832,7 +1858,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a5761488a154d3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801b696960d646ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2931,10 +2957,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F32" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G32" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H32" s="26" t="str">
         <x:v>GOV-002</x:v>
@@ -2948,7 +2974,9 @@
       <x:c r="K32" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/32</x:v>
       </x:c>
-      <x:c r="L32" s="26" t="str"/>
+      <x:c r="L32" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
+      </x:c>
       <x:c r="M32" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
@@ -3162,7 +3190,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce5be5c9f0fc4dcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac881b7a496645de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3646,7 +3674,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a4bd8205444c42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ef0f0c087d44d22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3908,26 +3936,49 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="27" t="str">
+      <x:c r="A15" s="26" t="str">
         <x:v>QA-RES-001</x:v>
       </x:c>
-      <x:c r="B15" s="27" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>Resilience</x:v>
       </x:c>
-      <x:c r="C15" s="27" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>Backup restore and failed cutover</x:v>
       </x:c>
-      <x:c r="D15" s="27" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="E15" s="27" t="str">
+      <x:c r="E15" s="26" t="str">
         <x:v>Not run</x:v>
       </x:c>
-      <x:c r="F15" s="27" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>Successful restore and two rollback rehearsals</x:v>
       </x:c>
-      <x:c r="G15" s="27" t="str">
+      <x:c r="G15" s="26" t="str">
         <x:v>QA-002 QA-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="27" t="str">
+        <x:v>QA-GOV-001</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="str">
+        <x:v>Source synchronization</x:v>
+      </x:c>
+      <x:c r="C16" s="27" t="str">
+        <x:v>Private-source report and shared-code mirror gate</x:v>
+      </x:c>
+      <x:c r="D16" s="27" t="str">
+        <x:v>PR 55 local evidence</x:v>
+      </x:c>
+      <x:c r="E16" s="27" t="str">
+        <x:v>19 of 19 governance and synchronization tests passed</x:v>
+      </x:c>
+      <x:c r="F16" s="27" t="str">
+        <x:v>Configure WOW_SYNC_TOKEN and capture first scheduled artifact</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="str">
+        <x:v>SYNC-002</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3936,7 +3987,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc1a9cf5f6214532"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b83c550d0b345d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4344,7 +4395,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb70774e2ae484084"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0324b0b93e7417f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4625,37 +4676,64 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="27" t="str">
+      <x:c r="A14" s="26" t="str">
         <x:v>ACC-009</x:v>
       </x:c>
-      <x:c r="B14" s="27" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>SMS WhatsApp push identity</x:v>
       </x:c>
-      <x:c r="C14" s="27" t="str">
+      <x:c r="C14" s="26" t="str">
         <x:v>Provider sandbox then production accounts</x:v>
       </x:c>
-      <x:c r="D14" s="27" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
-      <x:c r="E14" s="27" t="str">
+      <x:c r="E14" s="26" t="str">
         <x:v>Provider credentials</x:v>
       </x:c>
-      <x:c r="F14" s="27" t="str">
+      <x:c r="F14" s="26" t="str">
         <x:v>Protected secret store</x:v>
       </x:c>
-      <x:c r="G14" s="27" t="str">
+      <x:c r="G14" s="26" t="str">
         <x:v>Deferred</x:v>
       </x:c>
-      <x:c r="H14" s="30" t="str"/>
-      <x:c r="I14" s="27" t="str">
+      <x:c r="H14" s="29" t="str"/>
+      <x:c r="I14" s="26" t="str">
         <x:v>Separate onboarding gates</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="27" t="str">
+        <x:v>ACC-010</x:v>
+      </x:c>
+      <x:c r="B15" s="27" t="str">
+        <x:v>WOW-MD source review</x:v>
+      </x:c>
+      <x:c r="C15" s="27" t="str">
+        <x:v>Private repository contents read for scheduled change reports</x:v>
+      </x:c>
+      <x:c r="D15" s="27" t="str">
+        <x:v>RohithTadiparti</x:v>
+      </x:c>
+      <x:c r="E15" s="27" t="str">
+        <x:v>Fine-grained WOW_SYNC_TOKEN</x:v>
+      </x:c>
+      <x:c r="F15" s="27" t="str">
+        <x:v>Production GitHub Actions secret</x:v>
+      </x:c>
+      <x:c r="G15" s="27" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="H15" s="30" t="str"/>
+      <x:c r="I15" s="27" t="str">
+        <x:v>Scope only to WOW-MD Contents read; rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="G6:G14">
+  <x:conditionalFormatting sqref="G6:G15">
     <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="20" priority="3" operator="containsText" text="Blocked"/>
@@ -4664,7 +4742,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9137fc2d18e49b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R065ea2fb57e64d13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5003,7 +5081,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1922bddb2b42eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9afc42721174ce2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5105,34 +5183,69 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="26" t="str">
         <x:v>CHG-002</x:v>
       </x:c>
-      <x:c r="B7" s="27" t="str">
+      <x:c r="B7" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C7" s="27" t="str">
+      <x:c r="C7" s="26" t="str">
         <x:v>UNCOMMITTED</x:v>
       </x:c>
-      <x:c r="D7" s="27" t="str">
+      <x:c r="D7" s="26" t="str">
         <x:v>.gitignore</x:v>
       </x:c>
-      <x:c r="E7" s="27" t="str">
+      <x:c r="E7" s="26" t="str">
         <x:v>Repository hygiene</x:v>
       </x:c>
-      <x:c r="F7" s="27" t="str">
+      <x:c r="F7" s="26" t="str">
         <x:v>Review required</x:v>
       </x:c>
-      <x:c r="G7" s="27" t="str">
+      <x:c r="G7" s="26" t="str">
         <x:v>SYNC-001</x:v>
       </x:c>
-      <x:c r="H7" s="27" t="str"/>
-      <x:c r="I7" s="27" t="str"/>
-      <x:c r="J7" s="30" t="str">
+      <x:c r="H7" s="26" t="str"/>
+      <x:c r="I7" s="26" t="str"/>
+      <x:c r="J7" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
-      <x:c r="K7" s="27" t="str">
+      <x:c r="K7" s="26" t="str">
         <x:v>Three ignored paths require review before adoption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="27" t="str">
+        <x:v>CHG-003</x:v>
+      </x:c>
+      <x:c r="B8" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C8" s="27" t="str">
+        <x:v>07218b4..de7d8dd (LOCAL ONLY)</x:v>
+      </x:c>
+      <x:c r="D8" s="27" t="str">
+        <x:v>37 committed paths</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="str">
+        <x:v>Functional UI candidates</x:v>
+      </x:c>
+      <x:c r="F8" s="27" t="str">
+        <x:v>Await source publication and per-commit review</x:v>
+      </x:c>
+      <x:c r="G8" s="27" t="str">
+        <x:v>SYNC-002</x:v>
+      </x:c>
+      <x:c r="H8" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
+      </x:c>
+      <x:c r="I8" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J8" s="30" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="K8" s="27" t="str">
+        <x:v>Local main is 21 commits ahead of origin; scheduled GitHub review intentionally sees pushed commits only</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5141,7 +5254,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6791021829b644cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R044acd53e2964cb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5254,38 +5367,76 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="26" t="str">
         <x:v>GOV-001</x:v>
       </x:c>
-      <x:c r="B7" s="27" t="str">
+      <x:c r="B7" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
       </x:c>
-      <x:c r="C7" s="27" t="str">
+      <x:c r="C7" s="26" t="str">
         <x:v>codex/gov-001-public-protection</x:v>
       </x:c>
-      <x:c r="D7" s="27" t="str">
+      <x:c r="D7" s="26" t="str">
         <x:v>922cfee</x:v>
       </x:c>
-      <x:c r="E7" s="27" t="str">
+      <x:c r="E7" s="26" t="str">
         <x:v>152f4d3</x:v>
       </x:c>
-      <x:c r="F7" s="27" t="str"/>
-      <x:c r="G7" s="27" t="str">
+      <x:c r="F7" s="26" t="str"/>
+      <x:c r="G7" s="26" t="str">
         <x:v>Final PR head 152f4d3: backend E2E and tests pass; frontend pass; mobile pass; Docker pass; registers pass; Gitleaks pass; native CodeQL JavaScript/TypeScript and Actions pass; seed config 3/3; governance 7/7</x:v>
       </x:c>
-      <x:c r="H7" s="27" t="str">
+      <x:c r="H7" s="26" t="str">
         <x:v>GitHub visibility and protection settings plus repository security configuration; no application deploy</x:v>
       </x:c>
-      <x:c r="I7" s="27" t="str">
+      <x:c r="I7" s="26" t="str">
         <x:v>Change visibility/settings separately and revert PR; never restore fallback credential</x:v>
       </x:c>
-      <x:c r="J7" s="27" t="str">
+      <x:c r="J7" s="26" t="str">
         <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
       </x:c>
-      <x:c r="K7" s="27" t="str">
+      <x:c r="K7" s="26" t="str">
         <x:v>Ready to Merge</x:v>
       </x:c>
-      <x:c r="L7" s="30" t="str">
+      <x:c r="L7" s="29" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="27" t="str">
+        <x:v>SYNC-002</x:v>
+      </x:c>
+      <x:c r="B8" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
+      </x:c>
+      <x:c r="C8" s="27" t="str">
+        <x:v>codex/sync-002-gated-source-review</x:v>
+      </x:c>
+      <x:c r="D8" s="27" t="str">
+        <x:v>57e13d0</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="str">
+        <x:v>dbe8c4a</x:v>
+      </x:c>
+      <x:c r="F8" s="27" t="str">
+        <x:v>07218b4..de7d8dd local review only</x:v>
+      </x:c>
+      <x:c r="G8" s="27" t="str">
+        <x:v>Source report 4/4; mirror gate 5/5; workflow policy 3/3; full governance/source-sync 19/19; local report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
+      </x:c>
+      <x:c r="H8" s="27" t="str">
+        <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
+      </x:c>
+      <x:c r="I8" s="27" t="str">
+        <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
+      </x:c>
+      <x:c r="J8" s="27" t="str">
+        <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
+      </x:c>
+      <x:c r="K8" s="27" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L8" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
@@ -5293,7 +5444,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K7">
+  <x:conditionalFormatting sqref="K6:K8">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5302,7 +5453,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe9ec4b2cb7348ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad8447f83d3747c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record SEC-001 security evidence
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra82fc0183a11442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6fa20bf17f3a45af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4a49a0f0e6e04497"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rd7653db751404ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R88508ddfc8394578"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R160115c5e8ae4b89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd82b27fc55604d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R72cc06c0ec304ea6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R23350c76e9fd4e1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8579165ef61c4e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf045998242a74c30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R5c58e9077c63496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R0b93de2a100548ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R84e2e509f37e46dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb39a079fde1443c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rb8c6208b686a4a94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R5791293c8a15460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6151b4e22a294654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R9b02003173ee43d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R19371c2da2e04d45"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39762c3c77f04b08"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd1ee88f7173542ef"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -891,7 +891,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -960,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -980,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1250,7 +1250,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1259,7 +1259,7 @@
       </x:c>
       <x:c r="B7" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Open")</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1288,15 +1288,15 @@
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$17,"Open")</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF(Risks!$H$6:$H$18,"Open")</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1305,14 +1305,14 @@
       </x:c>
       <x:c r="B9" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$17,"P0",Risks!$H$6:$H$17,"Open")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIFS(Risks!$E$6:$E$18,"P0",Risks!$H$6:$H$18,"Open")</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
         <x:v>Blocked</x:v>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63679649290d49ab"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R312afa341ec54df4"/>
 </x:worksheet>
 </file>
 
@@ -1794,36 +1794,88 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>DOC-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>Production tracking workbook</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>docs/tracking/production-readiness-tracker.xlsx</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>Program management</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Each change</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
-      <x:c r="H17" s="27" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>GOV-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="26" t="str">
+        <x:v>DOC-013</x:v>
+      </x:c>
+      <x:c r="B18" s="26" t="str">
+        <x:v>SEC-001 implementation plan</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>docs/superpowers/plans/2026-10-04-sec-001-admin-mfa-provider-policy.md</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="str">
+        <x:v>On authentication/provider policy change</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="H18" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="27" t="str">
+        <x:v>DOC-014</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="str">
+        <x:v>Zoho Mail SMTP operating guide</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>docs/operations/zoho-mail.md</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>Security and operations</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>Approved candidate</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="str">
+        <x:v>Quarterly or provider change</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="H19" s="27" t="str">
+        <x:v>SEC-001 OPS-003</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E17">
+  <x:conditionalFormatting sqref="E6:E19">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -1832,7 +1884,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a5761488a154d3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48c739dd9bde49a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1927,10 +1979,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F6" s="25" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
@@ -1942,7 +1994,9 @@
       <x:c r="K6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
       </x:c>
-      <x:c r="L6" s="25" t="str"/>
+      <x:c r="L6" s="25" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+      </x:c>
       <x:c r="M6" s="28" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
@@ -3162,7 +3216,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce5be5c9f0fc4dcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R719dd4d653f8456e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3646,7 +3700,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a4bd8205444c42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94736675aa264a05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3872,13 +3926,13 @@
         <x:v>Admin MFA provider startup WebSockets headers secrets dependencies</x:v>
       </x:c>
       <x:c r="D13" s="26" t="str">
-        <x:v>Production readiness audit</x:v>
+        <x:v>SEC-001 PR 56 and WOW-MD PR 37</x:v>
       </x:c>
       <x:c r="E13" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>Provider policy 6 of 6; admin auth/JWT 49 of 49; source mirror 55 of 55; CI pending</x:v>
       </x:c>
       <x:c r="F13" s="26" t="str">
-        <x:v>Focused abuse tests plus security workflows</x:v>
+        <x:v>Complete protected CI and live staged enrollment/mail smoke evidence</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
         <x:v>SEC-001 SEC-002 SEC-003 DEP-001 GOV-001</x:v>
@@ -3936,7 +3990,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc1a9cf5f6214532"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdde858031bf34c45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4300,42 +4354,71 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>RISK-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>Public source exposes architecture test conventions and historical development-only credentials</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Remove fallback credentials; keep real secrets and PII outside Git; require push protection Gitleaks and native scanning</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H17" s="27" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>Mitigated</x:v>
       </x:c>
-      <x:c r="I17" s="27" t="str">
+      <x:c r="I17" s="26" t="str">
         <x:v>Tracked history scanned; seed fallback removed in GOV-001; test and production credentials require external stores</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="27" t="str">
+        <x:v>RISK-013</x:v>
+      </x:c>
+      <x:c r="B18" s="27" t="str">
+        <x:v>Public deployment tier is enabled before every administrator enrols MFA</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D18" s="27" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E18" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F18" s="27" t="str">
+        <x:v>Enrol and verify each administrator in restricted staging before selecting public-beta; keep a documented recovery owner</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="H18" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I18" s="27" t="str">
+        <x:v>SEC-001 PR 56 rejects unenrolled login and existing sessions; staged enrollment evidence still required</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E17">
+  <x:conditionalFormatting sqref="E6:E18">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H17">
+  <x:conditionalFormatting sqref="H6:H18">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4344,7 +4427,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb70774e2ae484084"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bec78af8b254f28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4578,23 +4661,23 @@
         <x:v>Operational email</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>Mailbox or SMTP provider and recipient list</x:v>
+        <x:v>Zoho domain mailbox DNS authentication reports and app-password rotation</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>SMTP/API identity</x:v>
+        <x:v>Zoho SMTP identity</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
-        <x:v>GitHub or Railway secrets</x:v>
+        <x:v>GitHub Railway or Kubernetes secrets</x:v>
       </x:c>
       <x:c r="G12" s="26" t="str">
-        <x:v>Mock</x:v>
+        <x:v>Approved candidate</x:v>
       </x:c>
       <x:c r="H12" s="29" t="str"/>
       <x:c r="I12" s="26" t="str">
-        <x:v>Log provider until approved</x:v>
+        <x:v>Low-volume beta only; owner must configure domain MFA app password and first delivery evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -4664,7 +4747,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9137fc2d18e49b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R379848e1845c4048"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5003,7 +5086,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1922bddb2b42eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf885d78aa3554021"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5141,7 +5224,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6791021829b644cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f71ebed71fb425b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5254,38 +5337,76 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="27" t="str">
+      <x:c r="A7" s="26" t="str">
         <x:v>GOV-001</x:v>
       </x:c>
-      <x:c r="B7" s="27" t="str">
+      <x:c r="B7" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
       </x:c>
-      <x:c r="C7" s="27" t="str">
+      <x:c r="C7" s="26" t="str">
         <x:v>codex/gov-001-public-protection</x:v>
       </x:c>
-      <x:c r="D7" s="27" t="str">
+      <x:c r="D7" s="26" t="str">
         <x:v>922cfee</x:v>
       </x:c>
-      <x:c r="E7" s="27" t="str">
+      <x:c r="E7" s="26" t="str">
         <x:v>152f4d3</x:v>
       </x:c>
-      <x:c r="F7" s="27" t="str"/>
-      <x:c r="G7" s="27" t="str">
+      <x:c r="F7" s="26" t="str"/>
+      <x:c r="G7" s="26" t="str">
         <x:v>Final PR head 152f4d3: backend E2E and tests pass; frontend pass; mobile pass; Docker pass; registers pass; Gitleaks pass; native CodeQL JavaScript/TypeScript and Actions pass; seed config 3/3; governance 7/7</x:v>
       </x:c>
-      <x:c r="H7" s="27" t="str">
+      <x:c r="H7" s="26" t="str">
         <x:v>GitHub visibility and protection settings plus repository security configuration; no application deploy</x:v>
       </x:c>
-      <x:c r="I7" s="27" t="str">
+      <x:c r="I7" s="26" t="str">
         <x:v>Change visibility/settings separately and revert PR; never restore fallback credential</x:v>
       </x:c>
-      <x:c r="J7" s="27" t="str">
+      <x:c r="J7" s="26" t="str">
         <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
       </x:c>
-      <x:c r="K7" s="27" t="str">
+      <x:c r="K7" s="26" t="str">
         <x:v>Ready to Merge</x:v>
       </x:c>
-      <x:c r="L7" s="30" t="str">
+      <x:c r="L7" s="29" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="27" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="B8" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+      </x:c>
+      <x:c r="C8" s="27" t="str">
+        <x:v>codex/sec-001-admin-mfa-provider-policy</x:v>
+      </x:c>
+      <x:c r="D8" s="27" t="str">
+        <x:v>57e13d0</x:v>
+      </x:c>
+      <x:c r="E8" s="27" t="str">
+        <x:v>532cf6c</x:v>
+      </x:c>
+      <x:c r="F8" s="27" t="str">
+        <x:v>WOW-MD PR 37 commit 1482d83</x:v>
+      </x:c>
+      <x:c r="G8" s="27" t="str">
+        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance 7/7; protected CI pending</x:v>
+      </x:c>
+      <x:c r="H8" s="27" t="str">
+        <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
+      </x:c>
+      <x:c r="I8" s="27" t="str">
+        <x:v>Restore previous image/config; do not fall back to log/mock in a public tier; pause email-dependent workflows</x:v>
+      </x:c>
+      <x:c r="J8" s="27" t="str">
+        <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
+      </x:c>
+      <x:c r="K8" s="27" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L8" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
@@ -5293,7 +5414,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K7">
+  <x:conditionalFormatting sqref="K6:K8">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5302,7 +5423,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe9ec4b2cb7348ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfff21dff55c64e86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize SEC-001 delivery evidence
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcf81899c01ba4ce8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R1a8b6530aa3e418d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R8fa8b70021c64ab2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R9c72250a45e342ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R70a70cedfa104ea6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Ra157c41f59f74dd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra86c75e78e72487b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R0054cfe972574c7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R24bab025c7af481e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Re46601031cd640c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc7df0f9914894907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R68804a89813f4b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R9b27cde7d36d40c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R8563e05c03a44a0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R4435416debb841e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rab75932cb0c24236"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra05f7be5ed4241bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2c0f08a920424505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re0e79451554c4a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R3eb7011c83984eff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc8fd2c8c4fc34616"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bc115c2266f4c13"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1296,7 +1296,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1305,7 +1305,7 @@
       </x:c>
       <x:c r="B9" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1319,7 +1319,7 @@
       </x:c>
       <x:c r="H9" s="39" t="n">
         <x:f>B10</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1328,7 +1328,7 @@
       </x:c>
       <x:c r="B10" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f9ca54a624f456d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R235076d8006a4a39"/>
 </x:worksheet>
 </file>
 
@@ -1910,7 +1910,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aff38dedcd746ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0a0800dfcc14e4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2005,10 +2005,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F6" s="25" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Product owner</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
@@ -3244,7 +3244,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22a80d2ada9a4c28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re745519934ee43a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3728,7 +3728,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6530d3b892e4673"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bdc418640084c9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3954,13 +3954,13 @@
         <x:v>Admin MFA provider startup WebSockets headers secrets dependencies</x:v>
       </x:c>
       <x:c r="D13" s="26" t="str">
-        <x:v>SEC-001 PR 56 and WOW-MD PR 37</x:v>
+        <x:v>SEC-001 PR 56 and merged WOW-MD PR 37</x:v>
       </x:c>
       <x:c r="E13" s="26" t="str">
-        <x:v>Provider policy 6 of 6; admin auth/JWT 49 of 49; source mirror 55 of 55; CI pending</x:v>
+        <x:v>Provider policy 6 of 6; admin auth/JWT 49 of 49; source mirror 55 of 55; protected source and production CI passed</x:v>
       </x:c>
       <x:c r="F13" s="26" t="str">
-        <x:v>Complete protected CI and live staged enrollment/mail smoke evidence</x:v>
+        <x:v>Complete live staged enrollment and Zoho delivery smoke evidence</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
         <x:v>SEC-001 SEC-002 SEC-003 DEP-001 GOV-001</x:v>
@@ -4041,7 +4041,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4028cb7fb3ed487a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf6a9523139243b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4478,7 +4478,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75c8b3892b4444c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R629b5fd99f4747e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4825,7 +4825,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71249d72c5924233"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R583232c454d4495b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5164,7 +5164,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bde19e1aa274cf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a9dd407c2d345e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5337,7 +5337,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbb51ca15c2d4751"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71254912a1424da7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5499,13 +5499,13 @@
         <x:v>57e13d0</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>532cf6c</x:v>
+        <x:v>fad2ef5</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>WOW-MD PR 37 commit 1482d83</x:v>
+        <x:v>WOW-MD PR 37 merged as b28c334; application mirror commit 1482d83</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance 7/7; protected CI pending</x:v>
+        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance and synchronization 19/19; protected production and source CI passed including retained 30-day CodeQL SARIF</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
         <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
@@ -5517,7 +5517,7 @@
         <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
       </x:c>
       <x:c r="K8" s="26" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
         <x:v>2026-10-04</x:v>
@@ -5574,7 +5574,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re808bd2b27df4390"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fcaf48711b94f06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[SEC-001] Enforce administrator MFA and provider policy (#56)
* fix: fail closed on unsafe production providers

* fix: require enrolled MFA for administrator access

* docs: add Zoho Mail production runbook

* docs: record SEC-001 security evidence

* docs: finalize SEC-001 delivery evidence

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R70806f8fb651404c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R661f9c31ea1449b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rad441362aa0943e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rd8ac6ce0b3f14309"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb31b3668378f40c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R7e4399604def40b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R45feca86bad9493f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re3818a5054ba46b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R356fda15c0274990"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R989f14421a284993"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc7df0f9914894907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R68804a89813f4b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R9b27cde7d36d40c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R8563e05c03a44a0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R4435416debb841e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rab75932cb0c24236"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra05f7be5ed4241bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2c0f08a920424505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re0e79451554c4a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R3eb7011c83984eff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45a6d1b0e8654d81"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bc115c2266f4c13"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -891,7 +891,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -960,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -980,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1250,7 +1250,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1259,7 +1259,7 @@
       </x:c>
       <x:c r="B7" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Open")</x:f>
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1288,15 +1288,15 @@
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$17,"Open")</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF(Risks!$H$6:$H$18,"Open")</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1305,21 +1305,21 @@
       </x:c>
       <x:c r="B9" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$17,"P0",Risks!$H$6:$H$17,"Open")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIFS(Risks!$E$6:$E$18,"P0",Risks!$H$6:$H$18,"Open")</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H9" s="39" t="n">
         <x:f>B10</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1328,7 +1328,7 @@
       </x:c>
       <x:c r="B10" s="34" t="n">
         <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Blocked")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3b238460cf84085"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R235076d8006a4a39"/>
 </x:worksheet>
 </file>
 
@@ -1820,36 +1820,88 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="27" t="str">
+      <x:c r="A18" s="26" t="str">
         <x:v>DOC-013</x:v>
       </x:c>
-      <x:c r="B18" s="27" t="str">
+      <x:c r="B18" s="26" t="str">
         <x:v>Gated source synchronization plan</x:v>
       </x:c>
-      <x:c r="C18" s="27" t="str">
+      <x:c r="C18" s="26" t="str">
         <x:v>docs/superpowers/plans/2026-10-04-gated-source-synchronization.md</x:v>
       </x:c>
-      <x:c r="D18" s="27" t="str">
+      <x:c r="D18" s="26" t="str">
         <x:v>Release engineering</x:v>
       </x:c>
-      <x:c r="E18" s="27" t="str">
+      <x:c r="E18" s="26" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="F18" s="27" t="str">
+      <x:c r="F18" s="26" t="str">
         <x:v>On synchronization policy change</x:v>
       </x:c>
-      <x:c r="G18" s="27" t="str">
+      <x:c r="G18" s="26" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
-      <x:c r="H18" s="27" t="str">
+      <x:c r="H18" s="26" t="str">
         <x:v>SYNC-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="26" t="str">
+        <x:v>DOC-014</x:v>
+      </x:c>
+      <x:c r="B19" s="26" t="str">
+        <x:v>SEC-001 implementation plan</x:v>
+      </x:c>
+      <x:c r="C19" s="26" t="str">
+        <x:v>docs/superpowers/plans/2026-10-04-sec-001-admin-mfa-provider-policy.md</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="F19" s="26" t="str">
+        <x:v>On authentication/provider policy change</x:v>
+      </x:c>
+      <x:c r="G19" s="26" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="H19" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="27" t="str">
+        <x:v>DOC-015</x:v>
+      </x:c>
+      <x:c r="B20" s="27" t="str">
+        <x:v>Zoho Mail SMTP operating guide</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
+        <x:v>docs/operations/zoho-mail.md</x:v>
+      </x:c>
+      <x:c r="D20" s="27" t="str">
+        <x:v>Security and operations</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>Approved candidate</x:v>
+      </x:c>
+      <x:c r="F20" s="27" t="str">
+        <x:v>Quarterly or provider change</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="H20" s="27" t="str">
+        <x:v>SEC-001 OPS-003</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E18">
+  <x:conditionalFormatting sqref="E6:E20">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -1858,7 +1910,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R801b696960d646ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0a0800dfcc14e4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1953,10 +2005,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F6" s="25" t="str">
-        <x:v>Open</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Product owner</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
@@ -1968,7 +2020,9 @@
       <x:c r="K6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
       </x:c>
-      <x:c r="L6" s="25" t="str"/>
+      <x:c r="L6" s="25" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+      </x:c>
       <x:c r="M6" s="28" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
@@ -2957,10 +3011,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F32" s="26" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G32" s="26" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Product owner</x:v>
       </x:c>
       <x:c r="H32" s="26" t="str">
         <x:v>GOV-002</x:v>
@@ -3190,7 +3244,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac881b7a496645de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re745519934ee43a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3674,7 +3728,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ef0f0c087d44d22"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bdc418640084c9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3900,13 +3954,13 @@
         <x:v>Admin MFA provider startup WebSockets headers secrets dependencies</x:v>
       </x:c>
       <x:c r="D13" s="26" t="str">
-        <x:v>Production readiness audit</x:v>
+        <x:v>SEC-001 PR 56 and merged WOW-MD PR 37</x:v>
       </x:c>
       <x:c r="E13" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>Provider policy 6 of 6; admin auth/JWT 49 of 49; source mirror 55 of 55; protected source and production CI passed</x:v>
       </x:c>
       <x:c r="F13" s="26" t="str">
-        <x:v>Focused abuse tests plus security workflows</x:v>
+        <x:v>Complete live staged enrollment and Zoho delivery smoke evidence</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
         <x:v>SEC-001 SEC-002 SEC-003 DEP-001 GOV-001</x:v>
@@ -3987,7 +4041,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b83c550d0b345d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf6a9523139243b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4351,42 +4405,71 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>RISK-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>Public source exposes architecture test conventions and historical development-only credentials</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Remove fallback credentials; keep real secrets and PII outside Git; require push protection Gitleaks and native scanning</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H17" s="27" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>Mitigated</x:v>
       </x:c>
-      <x:c r="I17" s="27" t="str">
+      <x:c r="I17" s="26" t="str">
         <x:v>Tracked history scanned; seed fallback removed in GOV-001; test and production credentials require external stores</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="27" t="str">
+        <x:v>RISK-013</x:v>
+      </x:c>
+      <x:c r="B18" s="27" t="str">
+        <x:v>Public deployment tier is enabled before every administrator enrols MFA</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D18" s="27" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E18" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F18" s="27" t="str">
+        <x:v>Enrol and verify each administrator in restricted staging before selecting public-beta; keep a documented recovery owner</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="H18" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I18" s="27" t="str">
+        <x:v>SEC-001 PR 56 rejects unenrolled login and existing sessions; staged enrollment evidence still required</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E17">
+  <x:conditionalFormatting sqref="E6:E18">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H17">
+  <x:conditionalFormatting sqref="H6:H18">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4395,7 +4478,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0324b0b93e7417f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R629b5fd99f4747e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4629,23 +4712,23 @@
         <x:v>Operational email</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>Mailbox or SMTP provider and recipient list</x:v>
+        <x:v>Zoho domain mailbox DNS authentication reports and app-password rotation</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>SMTP/API identity</x:v>
+        <x:v>Zoho SMTP identity</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
-        <x:v>GitHub or Railway secrets</x:v>
+        <x:v>GitHub Railway or Kubernetes secrets</x:v>
       </x:c>
       <x:c r="G12" s="26" t="str">
-        <x:v>Mock</x:v>
+        <x:v>Approved candidate</x:v>
       </x:c>
       <x:c r="H12" s="29" t="str"/>
       <x:c r="I12" s="26" t="str">
-        <x:v>Log provider until approved</x:v>
+        <x:v>Low-volume beta only; owner must configure domain MFA app password and first delivery evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -4742,7 +4825,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R065ea2fb57e64d13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R583232c454d4495b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5081,7 +5164,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9afc42721174ce2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a9dd407c2d345e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5254,7 +5337,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R044acd53e2964cb5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71254912a1424da7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5403,40 +5486,78 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="A8" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="B8" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+      </x:c>
+      <x:c r="C8" s="26" t="str">
+        <x:v>codex/sec-001-admin-mfa-provider-policy</x:v>
+      </x:c>
+      <x:c r="D8" s="26" t="str">
+        <x:v>57e13d0</x:v>
+      </x:c>
+      <x:c r="E8" s="26" t="str">
+        <x:v>fad2ef5</x:v>
+      </x:c>
+      <x:c r="F8" s="26" t="str">
+        <x:v>WOW-MD PR 37 merged as b28c334; application mirror commit 1482d83</x:v>
+      </x:c>
+      <x:c r="G8" s="26" t="str">
+        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance and synchronization 19/19; protected production and source CI passed including retained 30-day CodeQL SARIF</x:v>
+      </x:c>
+      <x:c r="H8" s="26" t="str">
+        <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
+      </x:c>
+      <x:c r="I8" s="26" t="str">
+        <x:v>Restore previous image/config; do not fall back to log/mock in a public tier; pause email-dependent workflows</x:v>
+      </x:c>
+      <x:c r="J8" s="26" t="str">
+        <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
+      </x:c>
+      <x:c r="K8" s="26" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="L8" s="29" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="27" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="B8" s="27" t="str">
+      <x:c r="B9" s="27" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
       </x:c>
-      <x:c r="C8" s="27" t="str">
+      <x:c r="C9" s="27" t="str">
         <x:v>codex/sync-002-gated-source-review</x:v>
       </x:c>
-      <x:c r="D8" s="27" t="str">
+      <x:c r="D9" s="27" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E8" s="27" t="str">
-        <x:v>dbe8c4a</x:v>
-      </x:c>
-      <x:c r="F8" s="27" t="str">
+      <x:c r="E9" s="27" t="str">
+        <x:v>422cbc4</x:v>
+      </x:c>
+      <x:c r="F9" s="27" t="str">
         <x:v>07218b4..de7d8dd local review only</x:v>
       </x:c>
-      <x:c r="G8" s="27" t="str">
-        <x:v>Source report 4/4; mirror gate 5/5; workflow policy 3/3; full governance/source-sync 19/19; local report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
-      </x:c>
-      <x:c r="H8" s="27" t="str">
+      <x:c r="G9" s="27" t="str">
+        <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="str">
         <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
       </x:c>
-      <x:c r="I8" s="27" t="str">
+      <x:c r="I9" s="27" t="str">
         <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
       </x:c>
-      <x:c r="J8" s="27" t="str">
+      <x:c r="J9" s="27" t="str">
         <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
       </x:c>
-      <x:c r="K8" s="27" t="str">
-        <x:v>PR Open</x:v>
-      </x:c>
-      <x:c r="L8" s="30" t="str">
+      <x:c r="K9" s="27" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="L9" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
@@ -5444,7 +5565,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K8">
+  <x:conditionalFormatting sqref="K6:K9">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5453,7 +5574,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad8447f83d3747c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fcaf48711b94f06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: publish reconciled readiness tracker
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc7df0f9914894907"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R68804a89813f4b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R9b27cde7d36d40c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R8563e05c03a44a0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R4435416debb841e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rab75932cb0c24236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra05f7be5ed4241bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2c0f08a920424505"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re0e79451554c4a60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R3eb7011c83984eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re24c0d9277894751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R4ed111d90ff444af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R1037c58bf23c4279"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Re4331be0f9ce41cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R0ab518b8ce2e48ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rcb1c709781ca49f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rb0447ed7181f4aea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R4b58f3a837524d8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R3a7711564037407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rf8f2c920f6114fa3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bc115c2266f4c13"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R308c4a0e349f48d9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -840,7 +840,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -861,7 +861,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Requirement"/>
@@ -891,7 +891,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -960,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -980,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1207,7 +1207,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-04. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-05. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1235,22 +1235,22 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$37)</x:f>
-        <x:v>32</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$38)</x:f>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1258,8 +1258,8 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Open")</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Open")</x:f>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1281,14 +1281,14 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$18,"Open")</x:f>
+        <x:f>COUNTIF(Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
@@ -1296,7 +1296,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1304,14 +1304,14 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"PR Open")</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$18,"P0",Risks!$H$6:$H$18,"Open")</x:f>
+        <x:f>COUNTIFS(Risks!$E$6:$E$19,"P0",Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
@@ -1319,7 +1319,7 @@
       </x:c>
       <x:c r="H9" s="39" t="n">
         <x:f>B10</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1327,15 +1327,15 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Blocked")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Blocked")</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIF(Requirements!$G$6:$G$23,"Approved")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF(Requirements!$G$6:$G$27,"Approved")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G10" s="39" t="str">
         <x:v>Done</x:v>
@@ -1350,7 +1350,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Done")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Done")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R235076d8006a4a39"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R475d86da6a3f4fce"/>
 </x:worksheet>
 </file>
 
@@ -1872,36 +1872,62 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="27" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>DOC-015</x:v>
       </x:c>
-      <x:c r="B20" s="27" t="str">
-        <x:v>Zoho Mail SMTP operating guide</x:v>
-      </x:c>
-      <x:c r="C20" s="27" t="str">
+      <x:c r="B20" s="26" t="str">
+        <x:v>Zoho SSO and mail operating guide</x:v>
+      </x:c>
+      <x:c r="C20" s="26" t="str">
         <x:v>docs/operations/zoho-mail.md</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="str">
+      <x:c r="D20" s="26" t="str">
         <x:v>Security and operations</x:v>
       </x:c>
-      <x:c r="E20" s="27" t="str">
+      <x:c r="E20" s="26" t="str">
         <x:v>Approved candidate</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>Quarterly or provider change</x:v>
       </x:c>
-      <x:c r="G20" s="27" t="str">
-        <x:v>2026-10-04</x:v>
-      </x:c>
-      <x:c r="H20" s="27" t="str">
-        <x:v>SEC-001 OPS-003</x:v>
+      <x:c r="G20" s="26" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="H20" s="26" t="str">
+        <x:v>SEC-001 AUTH-001 OPS-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="27" t="str">
+        <x:v>DOC-016</x:v>
+      </x:c>
+      <x:c r="B21" s="27" t="str">
+        <x:v>Dependency remediation record</x:v>
+      </x:c>
+      <x:c r="C21" s="27" t="str">
+        <x:v>docs/security/dependency-remediation-2026-10-04.md</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>Approved candidate</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="str">
+        <x:v>Each dependency change</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="str">
+        <x:v>DEP-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E20">
+  <x:conditionalFormatting sqref="E6:E21">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -1910,7 +1936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0a0800dfcc14e4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23d59974171549a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1993,7 +2019,7 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>Enforce administrator MFA and production provider policy</x:v>
+        <x:v>Align authentication with Zoho SSO and multi-identifier login policy</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str">
         <x:v>Public beta safety</x:v>
@@ -2005,26 +2031,26 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F6" s="25" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
-        <x:v>Admin cannot use privileged access without MFA; unsafe production provider combinations fail startup</x:v>
+        <x:v>Administrators use Zoho SSO; existing users may use Zoho SSO or username/email/mobile plus password; OTP is verification/recovery only; unsafe public provider combinations fail startup</x:v>
       </x:c>
       <x:c r="J6" s="25" t="str">
-        <x:v>Production plan Task 1A</x:v>
+        <x:v>Production plan Task 1A and user authentication decision</x:v>
       </x:c>
       <x:c r="K6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
       </x:c>
       <x:c r="M6" s="28" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -2157,14 +2183,14 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F10" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str"/>
       <x:c r="I10" s="26" t="str">
-        <x:v>No unaccepted critical/high production advisory; CI blocks regression</x:v>
+        <x:v>No unaccepted critical/high runtime advisory; CI blocks regressions; explicitly documented no-fix build-tool exceptions remain narrow and reviewable</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
         <x:v>Production plan Task 1E</x:v>
@@ -2172,9 +2198,11 @@
       <x:c r="K10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/10</x:v>
       </x:c>
-      <x:c r="L10" s="26" t="str"/>
+      <x:c r="L10" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
+      </x:c>
       <x:c r="M10" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -2533,7 +2561,7 @@
         <x:v>AUTH-001</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Add scoped administrator MFA step-up</x:v>
+        <x:v>Add scoped administrator fresh-authentication step-up</x:v>
       </x:c>
       <x:c r="C20" s="26" t="str">
         <x:v>Migration control</x:v>
@@ -2554,17 +2582,17 @@
         <x:v>SEC-001,CFG-001</x:v>
       </x:c>
       <x:c r="I20" s="26" t="str">
-        <x:v>Five-minute single-use scoped token protects migration start</x:v>
+        <x:v>Fresh Zoho reauthentication issues a five-minute single-use action-scoped token for migration start; application TOTP is a documented fallback only</x:v>
       </x:c>
       <x:c r="J20" s="26" t="str">
-        <x:v>Production plan Task 9</x:v>
+        <x:v>Production plan Task 9 and user authentication decision</x:v>
       </x:c>
       <x:c r="K20" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/20</x:v>
       </x:c>
       <x:c r="L20" s="26" t="str"/>
       <x:c r="M20" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -3190,52 +3218,93 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
-      <x:c r="A37" s="27" t="str">
+      <x:c r="A37" s="26" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B37" s="27" t="str">
+      <x:c r="B37" s="26" t="str">
         <x:v>Establish SDLC knowledge and tracking system</x:v>
       </x:c>
-      <x:c r="C37" s="27" t="str">
+      <x:c r="C37" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="D37" s="27" t="str">
+      <x:c r="D37" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="E37" s="27" t="str">
+      <x:c r="E37" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F37" s="27" t="str">
+      <x:c r="F37" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G37" s="27" t="str">
+      <x:c r="G37" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H37" s="27" t="str"/>
-      <x:c r="I37" s="27" t="str">
+      <x:c r="H37" s="26" t="str"/>
+      <x:c r="I37" s="26" t="str">
         <x:v>Markdown CSV Excel issues PR protocol and Obsidian index are linked and verified</x:v>
       </x:c>
-      <x:c r="J37" s="27" t="str">
+      <x:c r="J37" s="26" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K37" s="27" t="str">
+      <x:c r="K37" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/37</x:v>
       </x:c>
-      <x:c r="L37" s="27" t="str">
+      <x:c r="L37" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
-      <x:c r="M37" s="30" t="str">
+      <x:c r="M37" s="29" t="str">
         <x:v>2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="27" t="str">
+        <x:v>GOV-003</x:v>
+      </x:c>
+      <x:c r="B38" s="27" t="str">
+        <x:v>Reconcile authentication and dependency tracking</x:v>
+      </x:c>
+      <x:c r="C38" s="27" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="D38" s="27" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="E38" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F38" s="27" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G38" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H38" s="27" t="str">
+        <x:v>SEC-001,DEP-001</x:v>
+      </x:c>
+      <x:c r="I38" s="27" t="str">
+        <x:v>Canonical registers workbook and operating guidance match the implemented authentication policy and dependency evidence</x:v>
+      </x:c>
+      <x:c r="J38" s="27" t="str">
+        <x:v>User request</x:v>
+      </x:c>
+      <x:c r="K38" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/60</x:v>
+      </x:c>
+      <x:c r="L38" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
+      </x:c>
+      <x:c r="M38" s="30" t="str">
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E37">
+  <x:conditionalFormatting sqref="E6:E38">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F37">
+  <x:conditionalFormatting sqref="F6:F38">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3244,7 +3313,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re745519934ee43a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71e92e74fbff40b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3690,25 +3759,117 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="27" t="str">
+      <x:c r="A23" s="26" t="str">
         <x:v>REQ-REV-001</x:v>
       </x:c>
-      <x:c r="B23" s="27" t="str">
+      <x:c r="B23" s="26" t="str">
         <x:v>AWS migration readiness reports INR 1.2M target and INR 1.5M preferred monthly net revenue</x:v>
       </x:c>
-      <x:c r="C23" s="27" t="str">
+      <x:c r="C23" s="26" t="str">
         <x:v>Migration design</x:v>
       </x:c>
-      <x:c r="D23" s="27" t="str">
+      <x:c r="D23" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="E23" s="27" t="str">
+      <x:c r="E23" s="26" t="str">
         <x:v>Admin readiness UI test</x:v>
       </x:c>
-      <x:c r="F23" s="27" t="str">
+      <x:c r="F23" s="26" t="str">
         <x:v>UI-001</x:v>
       </x:c>
-      <x:c r="G23" s="27" t="str">
+      <x:c r="G23" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="26" t="str">
+        <x:v>REQ-AUTH-001</x:v>
+      </x:c>
+      <x:c r="B24" s="26" t="str">
+        <x:v>Administrators authenticate through Zoho SSO and do not require routine application TOTP</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E24" s="26" t="str">
+        <x:v>Authentication integration tests and controlled Zoho sign-in evidence</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G24" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="26" t="str">
+        <x:v>REQ-AUTH-002</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="str">
+        <x:v>Existing users may sign in with Zoho SSO or username email or mobile plus password and any valid email provider is accepted</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>Backend frontend mobile and Playwright authentication tests</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="A26" s="26" t="str">
+        <x:v>REQ-AUTH-003</x:v>
+      </x:c>
+      <x:c r="B26" s="26" t="str">
+        <x:v>OTP is used only for signup/contact verification and password recovery and never as passwordless login</x:v>
+      </x:c>
+      <x:c r="C26" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="str">
+        <x:v>Route inventory and authentication tests</x:v>
+      </x:c>
+      <x:c r="F26" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G26" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="27" t="str">
+        <x:v>REQ-AUTH-004</x:v>
+      </x:c>
+      <x:c r="B27" s="27" t="str">
+        <x:v>Zoho domain DNS sender mailbox SMTP application password and production OAuth callback are configured only at the final deployment gate</x:v>
+      </x:c>
+      <x:c r="C27" s="27" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D27" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E27" s="27" t="str">
+        <x:v>Final release checklist and controlled delivery/SSO evidence</x:v>
+      </x:c>
+      <x:c r="F27" s="27" t="str">
+        <x:v>SEC-001,REL-001</x:v>
+      </x:c>
+      <x:c r="G27" s="27" t="str">
         <x:v>Approved</x:v>
       </x:c>
     </x:row>
@@ -3716,10 +3877,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D23">
+  <x:conditionalFormatting sqref="D6:D27">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G6:G23">
+  <x:conditionalFormatting sqref="G6:G27">
     <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Blocked"/>
@@ -3728,7 +3889,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bdc418640084c9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9c033dc32ff4aba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4041,7 +4202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf6a9523139243b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a610213677546d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4434,42 +4595,71 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="27" t="str">
+      <x:c r="A18" s="26" t="str">
         <x:v>RISK-013</x:v>
       </x:c>
-      <x:c r="B18" s="27" t="str">
-        <x:v>Public deployment tier is enabled before every administrator enrols MFA</x:v>
-      </x:c>
-      <x:c r="C18" s="27" t="str">
+      <x:c r="B18" s="26" t="str">
+        <x:v>Public deployment tier is enabled before Zoho SSO and administrator recovery are proven</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D18" s="27" t="str">
+      <x:c r="D18" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E18" s="27" t="str">
+      <x:c r="E18" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F18" s="27" t="str">
-        <x:v>Enrol and verify each administrator in restricted staging before selecting public-beta; keep a documented recovery owner</x:v>
-      </x:c>
-      <x:c r="G18" s="27" t="str">
+      <x:c r="F18" s="26" t="str">
+        <x:v>Verify exact OAuth client callback administrator matching-email login Zoho-account MFA and a documented recovery owner in restricted staging before public-beta</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H18" s="27" t="str">
+      <x:c r="H18" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="I18" s="27" t="str">
-        <x:v>SEC-001 PR 56 rejects unenrolled login and existing sessions; staged enrollment evidence still required</x:v>
+      <x:c r="I18" s="26" t="str">
+        <x:v>SEC-001 PR 58 implements Zoho-only administrator login; production Zoho configuration is intentionally deferred to the final gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="27" t="str">
+        <x:v>RISK-014</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="str">
+        <x:v>Framework and mobile build-tool dependency advisories remain after runtime remediation</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="str">
+        <x:v>Block new critical/high runtime advisories; allow only four exact no-fix Expo advisory IDs; schedule Nest major migration and review exceptions each release</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="H19" s="27" t="str">
+        <x:v>Mitigated</x:v>
+      </x:c>
+      <x:c r="I19" s="27" t="str">
+        <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E18">
+  <x:conditionalFormatting sqref="E6:E19">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H18">
+  <x:conditionalFormatting sqref="H6:H19">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4478,7 +4668,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R629b5fd99f4747e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9455da0425444e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4825,7 +5015,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R583232c454d4495b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2959000a1a6746b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5164,7 +5354,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a9dd407c2d345e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda3f92729a9849ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5337,7 +5527,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71254912a1424da7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6265706f5e64cf6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5490,82 +5680,158 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>codex/sec-001-admin-mfa-provider-policy</x:v>
+        <x:v>codex/sec-001-sso-login-policy</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E8" s="26" t="str">
+        <x:v>8e7f3e8</x:v>
+      </x:c>
+      <x:c r="F8" s="26" t="str">
+        <x:v>WOW-MD PR 38 head 29ee273</x:v>
+      </x:c>
+      <x:c r="G8" s="26" t="str">
+        <x:v>Backend typecheck and 55 focused auth/config tests pass; frontend typecheck and 173 tests pass; mobile typecheck passes; production and source protected CI application jobs pass</x:v>
+      </x:c>
+      <x:c r="H8" s="26" t="str">
+        <x:v>At the final release gate configure exact Zoho OAuth client/callback domain SPF DKIM DMARC sender mailbox and SMTP application password; then run controlled admin/non-admin SSO and email tests</x:v>
+      </x:c>
+      <x:c r="I8" s="26" t="str">
+        <x:v>Restore the prior image/config and disable Zoho SSO; do not enable passwordless OTP or log-based mail in public tier</x:v>
+      </x:c>
+      <x:c r="J8" s="26" t="str">
+        <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred; the aggregate CodeQL status on production PR is failing despite both analysis jobs passing and needs repository-level triage</x:v>
+      </x:c>
+      <x:c r="K8" s="26" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L8" s="29" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="26" t="str">
+        <x:v>SYNC-002</x:v>
+      </x:c>
+      <x:c r="B9" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
+      </x:c>
+      <x:c r="C9" s="26" t="str">
+        <x:v>codex/sync-002-gated-source-review</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E8" s="26" t="str">
-        <x:v>fad2ef5</x:v>
-      </x:c>
-      <x:c r="F8" s="26" t="str">
-        <x:v>WOW-MD PR 37 merged as b28c334; application mirror commit 1482d83</x:v>
-      </x:c>
-      <x:c r="G8" s="26" t="str">
-        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance and synchronization 19/19; protected production and source CI passed including retained 30-day CodeQL SARIF</x:v>
-      </x:c>
-      <x:c r="H8" s="26" t="str">
-        <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
-      </x:c>
-      <x:c r="I8" s="26" t="str">
-        <x:v>Restore previous image/config; do not fall back to log/mock in a public tier; pause email-dependent workflows</x:v>
-      </x:c>
-      <x:c r="J8" s="26" t="str">
-        <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
-      </x:c>
-      <x:c r="K8" s="26" t="str">
+      <x:c r="E9" s="26" t="str">
+        <x:v>422cbc4</x:v>
+      </x:c>
+      <x:c r="F9" s="26" t="str">
+        <x:v>07218b4..de7d8dd local review only</x:v>
+      </x:c>
+      <x:c r="G9" s="26" t="str">
+        <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
+      </x:c>
+      <x:c r="H9" s="26" t="str">
+        <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
+      </x:c>
+      <x:c r="I9" s="26" t="str">
+        <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
+      </x:c>
+      <x:c r="J9" s="26" t="str">
+        <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
+      </x:c>
+      <x:c r="K9" s="26" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="L8" s="29" t="str">
+      <x:c r="L9" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="27" t="str">
-        <x:v>SYNC-002</x:v>
-      </x:c>
-      <x:c r="B9" s="27" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
-      </x:c>
-      <x:c r="C9" s="27" t="str">
-        <x:v>codex/sync-002-gated-source-review</x:v>
-      </x:c>
-      <x:c r="D9" s="27" t="str">
-        <x:v>57e13d0</x:v>
-      </x:c>
-      <x:c r="E9" s="27" t="str">
-        <x:v>422cbc4</x:v>
-      </x:c>
-      <x:c r="F9" s="27" t="str">
-        <x:v>07218b4..de7d8dd local review only</x:v>
-      </x:c>
-      <x:c r="G9" s="27" t="str">
-        <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
-      </x:c>
-      <x:c r="H9" s="27" t="str">
-        <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
-      </x:c>
-      <x:c r="I9" s="27" t="str">
-        <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
-      </x:c>
-      <x:c r="J9" s="27" t="str">
-        <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
-      </x:c>
-      <x:c r="K9" s="27" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="L9" s="30" t="str">
-        <x:v>2026-10-04</x:v>
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="26" t="str">
+        <x:v>DEP-001</x:v>
+      </x:c>
+      <x:c r="B10" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
+      </x:c>
+      <x:c r="C10" s="26" t="str">
+        <x:v>codex/dep-001-dependency-remediation</x:v>
+      </x:c>
+      <x:c r="D10" s="26" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E10" s="26" t="str">
+        <x:v>1ecbfdf</x:v>
+      </x:c>
+      <x:c r="F10" s="26" t="str">
+        <x:v>WOW-MD PR 39 head d8ef995</x:v>
+      </x:c>
+      <x:c r="G10" s="26" t="str">
+        <x:v>Backend clean install typecheck lint build and 792 tests pass with 9 skipped; frontend clean install typecheck 173 tests build and 10 Playwright flows pass; runtime audits: backend 0 critical/0 high frontend 0; exact-ID mobile gate passes; production and source protected CI pass</x:v>
+      </x:c>
+      <x:c r="H10" s="26" t="str">
+        <x:v>No deployment before review and merge; after merge let GitHub rescan manifests and confirm alert counts and audit gates on main</x:v>
+      </x:c>
+      <x:c r="I10" s="26" t="str">
+        <x:v>Revert PR 59; restore prior lockfiles and packages; retain the audit report for comparison</x:v>
+      </x:c>
+      <x:c r="J10" s="26" t="str">
+        <x:v>Backend moderate/low build-tool advisories and four exact no-fix Expo advisory roots remain; forced NestJS 12 and Expo downgrades were tested and rejected as unsafe</x:v>
+      </x:c>
+      <x:c r="K10" s="26" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L10" s="29" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="27" t="str">
+        <x:v>GOV-003</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
+      </x:c>
+      <x:c r="C11" s="27" t="str">
+        <x:v>codex/gov-003-auth-dependency-tracking</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E11" s="27" t="str">
+        <x:v>1235cd3</x:v>
+      </x:c>
+      <x:c r="F11" s="27" t="str">
+        <x:v>SEC-001 PR 58 and DEP-001 PR 59 evidence only</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="str">
+        <x:v>Register validator workbook regeneration and formula-error scan pass; dashboard visually reviewed</x:v>
+      </x:c>
+      <x:c r="H11" s="27" t="str">
+        <x:v>Governance and documentation only; no application or hosting deployment</x:v>
+      </x:c>
+      <x:c r="I11" s="27" t="str">
+        <x:v>Revert PR 61; implementation PRs and their evidence remain unchanged</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="str">
+        <x:v>Implementation PRs still require review/merge and GitHub rescan; Zoho live configuration remains a final release gate</x:v>
+      </x:c>
+      <x:c r="K11" s="27" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L11" s="30" t="str">
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K9">
+  <x:conditionalFormatting sqref="K6:K11">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5574,7 +5840,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fcaf48711b94f06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ffc57c8e9794182"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record refresh-token security evidence
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re24c0d9277894751"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R4ed111d90ff444af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R1037c58bf23c4279"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Re4331be0f9ce41cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R0ab518b8ce2e48ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rcb1c709781ca49f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rb0447ed7181f4aea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R4b58f3a837524d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R3a7711564037407c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rf8f2c920f6114fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc48feca5eda645b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rb694d0cfd5cc484e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R8bb8c116590f4db2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R0268affec18d4bf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R9268f42ea1e64f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R9d6dbee1755e46d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R3738aa548e5845af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2f4b16830be54b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra87ec7a9597b4b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R616e0a17c7c54bf4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R308c4a0e349f48d9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc5804326dfac4dc7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R475d86da6a3f4fce"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf93884aa7d514f1d"/>
 </x:worksheet>
 </file>
 
@@ -1936,7 +1936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23d59974171549a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13f6e41cea3440ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3313,7 +3313,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71e92e74fbff40b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7311fef23014ba6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3889,7 +3889,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9c033dc32ff4aba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb4c3b19119d4c4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4202,7 +4202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a610213677546d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a5712b6c4f0410c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4668,7 +4668,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9455da0425444e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd829e30413e8484f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5015,7 +5015,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2959000a1a6746b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R387545740127464c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5354,7 +5354,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda3f92729a9849ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e19ef299d354a4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5527,7 +5527,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6265706f5e64cf6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb90aa7063f1c46cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5689,13 +5689,13 @@
         <x:v>29537ee</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>8e7f3e8</x:v>
+        <x:v>01bd123</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>WOW-MD PR 38 head 29ee273</x:v>
+        <x:v>WOW-MD PR 38 head f685774</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Backend typecheck and 55 focused auth/config tests pass; frontend typecheck and 173 tests pass; mobile typecheck passes; production and source protected CI application jobs pass</x:v>
+        <x:v>Backend typecheck/lint and 71 focused auth/config tests pass; frontend typecheck and 173 tests pass; mobile typecheck passes; CodeQL security gate passes after refresh cookies were sealed and session hashes moved to memory-hard derivation; remaining protected CI jobs are recorded on the PR</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
         <x:v>At the final release gate configure exact Zoho OAuth client/callback domain SPF DKIM DMARC sender mailbox and SMTP application password; then run controlled admin/non-admin SSO and email tests</x:v>
@@ -5704,7 +5704,7 @@
         <x:v>Restore the prior image/config and disable Zoho SSO; do not enable passwordless OTP or log-based mail in public tier</x:v>
       </x:c>
       <x:c r="J8" s="26" t="str">
-        <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred; the aggregate CodeQL status on production PR is failing despite both analysis jobs passing and needs repository-level triage</x:v>
+        <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred to the final release gate</x:v>
       </x:c>
       <x:c r="K8" s="26" t="str">
         <x:v>PR Open</x:v>
@@ -5840,7 +5840,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ffc57c8e9794182"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a3d81de8d0c4511"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: clarify source token and access timing
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc48feca5eda645b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rb694d0cfd5cc484e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R8bb8c116590f4db2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R0268affec18d4bf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R9268f42ea1e64f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R9d6dbee1755e46d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R3738aa548e5845af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2f4b16830be54b6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra87ec7a9597b4b15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R616e0a17c7c54bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R980ff49061094730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rd695025b504247c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R9a28dae678d84cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R85498cf0250c4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R921698851bbc42a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R8c95448b30954ae2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rc31255f8c95b4307"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R773444ff6d894f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R99b2d2f3c8994cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb45c6ad01fba48ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc5804326dfac4dc7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbfddc80666614cbb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf93884aa7d514f1d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96197e094d6a4087"/>
 </x:worksheet>
 </file>
 
@@ -1936,7 +1936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13f6e41cea3440ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94ee19de0e1f4528"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3313,7 +3313,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7311fef23014ba6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2436191cdb94469d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3889,7 +3889,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb4c3b19119d4c4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra874fdfd64b54aff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4202,7 +4202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a5712b6c4f0410c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41ec7c27333f406c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4668,7 +4668,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd829e30413e8484f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d01fdfe08834c0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4899,16 +4899,16 @@
         <x:v>ACC-007</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>Operational email</x:v>
+        <x:v>Zoho identity and operational email</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>Zoho domain mailbox DNS authentication reports and app-password rotation</x:v>
+        <x:v>OAuth application exact callback domain mailbox DNS authentication reports and SMTP app-password rotation</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>Zoho SMTP identity</x:v>
+        <x:v>Zoho OAuth and SMTP identities</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
         <x:v>GitHub Railway or Kubernetes secrets</x:v>
@@ -4918,7 +4918,7 @@
       </x:c>
       <x:c r="H12" s="29" t="str"/>
       <x:c r="I12" s="26" t="str">
-        <x:v>Low-volume beta only; owner must configure domain MFA app password and first delivery evidence</x:v>
+        <x:v>Configure only at final deployment; protect the Zoho owner with Zoho MFA and retain controlled SSO/mail evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -4983,7 +4983,7 @@
         <x:v>WOW-MD source review</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
-        <x:v>Private repository contents read for scheduled change reports</x:v>
+        <x:v>Repository contents read for scheduled change reports</x:v>
       </x:c>
       <x:c r="D15" s="27" t="str">
         <x:v>RohithTadiparti</x:v>
@@ -4995,11 +4995,11 @@
         <x:v>Production GitHub Actions secret</x:v>
       </x:c>
       <x:c r="G15" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="H15" s="30" t="str"/>
       <x:c r="I15" s="27" t="str">
-        <x:v>Scope only to WOW-MD Contents read; rotate within 90 days</x:v>
+        <x:v>Not technically required while WOW-MD is public; create before returning it private so the private-ready workflow keeps working; scope only to WOW-MD Contents read and rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5015,7 +5015,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R387545740127464c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b4e6968d40241f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5354,7 +5354,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e19ef299d354a4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R615eff909ab24642"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5527,7 +5527,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb90aa7063f1c46cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71cabc95d21f49f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5689,7 +5689,7 @@
         <x:v>29537ee</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>01bd123</x:v>
+        <x:v>3eaa03c</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
         <x:v>WOW-MD PR 38 head f685774</x:v>
@@ -5840,7 +5840,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a3d81de8d0c4511"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3652ba24d5b84156"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(ops): refresh OPS-001 Excel tracker
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R980ff49061094730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rd695025b504247c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R9a28dae678d84cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R85498cf0250c4f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R921698851bbc42a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R8c95448b30954ae2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rc31255f8c95b4307"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R773444ff6d894f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R99b2d2f3c8994cad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb45c6ad01fba48ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raeedae5ff209418d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R40b455cf76954eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R5023dffb9e4448ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R2db2c6f1609549d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rdf0ccb98e6224d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R42965f3834b04aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R1a1b0d2dd00d4ca2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re691660970d54e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra4fa0222c47c4087"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8bfac8c765c04c81"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -224,7 +224,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -234,7 +234,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -244,7 +244,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -255,7 +255,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -265,7 +265,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -275,7 +275,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -286,7 +286,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -296,7 +296,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -306,7 +306,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -317,7 +317,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -327,7 +327,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -337,7 +337,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -348,7 +348,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -358,7 +358,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -368,7 +368,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -379,7 +379,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -389,7 +389,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -399,7 +399,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -409,7 +409,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -419,7 +419,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -430,7 +430,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -440,7 +440,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -450,7 +450,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -460,7 +460,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -470,7 +470,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -481,7 +481,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -491,7 +491,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -501,7 +501,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -511,7 +511,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -521,7 +521,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -532,7 +532,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -542,7 +542,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -552,7 +552,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -562,7 +562,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -572,7 +572,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -583,7 +583,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -593,7 +593,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -603,7 +603,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -614,7 +614,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -624,7 +624,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbfddc80666614cbb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Recbdb8875ecc49f8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -840,7 +840,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -861,7 +861,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Requirement"/>
@@ -891,7 +891,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -960,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -980,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1235,21 +1235,19 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$38)</x:f>
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
-        <x:f>B7</x:f>
         <x:v>27</x:v>
       </x:c>
     </x:row>
@@ -1258,7 +1256,6 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Open")</x:f>
         <x:v>27</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1272,7 +1269,6 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H7" s="39" t="n">
-        <x:f>B8</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1281,22 +1277,20 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$19,"Open")</x:f>
+        <x:f>COUNTIF(Risks!$H$6:$H$18,"Open")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:f>B9</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1304,22 +1298,20 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"PR Open")</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$19,"P0",Risks!$H$6:$H$19,"Open")</x:f>
+        <x:f>COUNTIFS(Risks!$E$6:$E$18,"P0",Risks!$H$6:$H$18,"Open")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H9" s="39" t="n">
-        <x:f>B10</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1327,21 +1319,19 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIF(Requirements!$G$6:$G$27,"Approved")</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTIF(Requirements!$G$6:$G$23,"Approved")</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G10" s="39" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:f>B11</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -1350,7 +1340,6 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Done")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
@@ -1450,7 +1439,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96197e094d6a4087"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11dd2df34d0a44bb"/>
 </x:worksheet>
 </file>
 
@@ -1872,62 +1861,36 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="26" t="str">
+      <x:c r="A20" s="27" t="str">
         <x:v>DOC-015</x:v>
       </x:c>
-      <x:c r="B20" s="26" t="str">
-        <x:v>Zoho SSO and mail operating guide</x:v>
-      </x:c>
-      <x:c r="C20" s="26" t="str">
+      <x:c r="B20" s="27" t="str">
+        <x:v>Zoho Mail SMTP operating guide</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
         <x:v>docs/operations/zoho-mail.md</x:v>
       </x:c>
-      <x:c r="D20" s="26" t="str">
+      <x:c r="D20" s="27" t="str">
         <x:v>Security and operations</x:v>
       </x:c>
-      <x:c r="E20" s="26" t="str">
+      <x:c r="E20" s="27" t="str">
         <x:v>Approved candidate</x:v>
       </x:c>
-      <x:c r="F20" s="26" t="str">
+      <x:c r="F20" s="27" t="str">
         <x:v>Quarterly or provider change</x:v>
       </x:c>
-      <x:c r="G20" s="26" t="str">
-        <x:v>2026-10-05</x:v>
-      </x:c>
-      <x:c r="H20" s="26" t="str">
-        <x:v>SEC-001 AUTH-001 OPS-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="27" t="str">
-        <x:v>DOC-016</x:v>
-      </x:c>
-      <x:c r="B21" s="27" t="str">
-        <x:v>Dependency remediation record</x:v>
-      </x:c>
-      <x:c r="C21" s="27" t="str">
-        <x:v>docs/security/dependency-remediation-2026-10-04.md</x:v>
-      </x:c>
-      <x:c r="D21" s="27" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="E21" s="27" t="str">
-        <x:v>Approved candidate</x:v>
-      </x:c>
-      <x:c r="F21" s="27" t="str">
-        <x:v>Each dependency change</x:v>
-      </x:c>
-      <x:c r="G21" s="27" t="str">
-        <x:v>2026-10-05</x:v>
-      </x:c>
-      <x:c r="H21" s="27" t="str">
-        <x:v>DEP-001</x:v>
+      <x:c r="G20" s="27" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="H20" s="27" t="str">
+        <x:v>SEC-001 OPS-003</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E21">
+  <x:conditionalFormatting sqref="E6:E20">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -1936,7 +1899,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94ee19de0e1f4528"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3389fabded664992"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2019,7 +1982,7 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>Align authentication with Zoho SSO and multi-identifier login policy</x:v>
+        <x:v>Enforce administrator MFA and production provider policy</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str">
         <x:v>Public beta safety</x:v>
@@ -2031,26 +1994,26 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F6" s="25" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Product owner</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
-        <x:v>Administrators use Zoho SSO; existing users may use Zoho SSO or username/email/mobile plus password; OTP is verification/recovery only; unsafe public provider combinations fail startup</x:v>
+        <x:v>Admin cannot use privileged access without MFA; unsafe production provider combinations fail startup</x:v>
       </x:c>
       <x:c r="J6" s="25" t="str">
-        <x:v>Production plan Task 1A and user authentication decision</x:v>
+        <x:v>Production plan Task 1A</x:v>
       </x:c>
       <x:c r="K6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
       </x:c>
       <x:c r="M6" s="28" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -2109,10 +2072,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str"/>
       <x:c r="I8" s="26" t="str">
@@ -2124,9 +2087,11 @@
       <x:c r="K8" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/8</x:v>
       </x:c>
-      <x:c r="L8" s="26" t="str"/>
+      <x:c r="L8" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+      </x:c>
       <x:c r="M8" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -2183,14 +2148,14 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F10" s="26" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Unassigned</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str"/>
       <x:c r="I10" s="26" t="str">
-        <x:v>No unaccepted critical/high runtime advisory; CI blocks regressions; explicitly documented no-fix build-tool exceptions remain narrow and reviewable</x:v>
+        <x:v>No unaccepted critical/high production advisory; CI blocks regression</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
         <x:v>Production plan Task 1E</x:v>
@@ -2198,11 +2163,9 @@
       <x:c r="K10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/10</x:v>
       </x:c>
-      <x:c r="L10" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
-      </x:c>
+      <x:c r="L10" s="26" t="str"/>
       <x:c r="M10" s="29" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -2561,7 +2524,7 @@
         <x:v>AUTH-001</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Add scoped administrator fresh-authentication step-up</x:v>
+        <x:v>Add scoped administrator MFA step-up</x:v>
       </x:c>
       <x:c r="C20" s="26" t="str">
         <x:v>Migration control</x:v>
@@ -2582,17 +2545,17 @@
         <x:v>SEC-001,CFG-001</x:v>
       </x:c>
       <x:c r="I20" s="26" t="str">
-        <x:v>Fresh Zoho reauthentication issues a five-minute single-use action-scoped token for migration start; application TOTP is a documented fallback only</x:v>
+        <x:v>Five-minute single-use scoped token protects migration start</x:v>
       </x:c>
       <x:c r="J20" s="26" t="str">
-        <x:v>Production plan Task 9 and user authentication decision</x:v>
+        <x:v>Production plan Task 9</x:v>
       </x:c>
       <x:c r="K20" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/20</x:v>
       </x:c>
       <x:c r="L20" s="26" t="str"/>
       <x:c r="M20" s="29" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -3218,93 +3181,52 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
-      <x:c r="A37" s="26" t="str">
+      <x:c r="A37" s="27" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B37" s="26" t="str">
+      <x:c r="B37" s="27" t="str">
         <x:v>Establish SDLC knowledge and tracking system</x:v>
       </x:c>
-      <x:c r="C37" s="26" t="str">
+      <x:c r="C37" s="27" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="D37" s="26" t="str">
+      <x:c r="D37" s="27" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="E37" s="26" t="str">
+      <x:c r="E37" s="27" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F37" s="26" t="str">
+      <x:c r="F37" s="27" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G37" s="26" t="str">
+      <x:c r="G37" s="27" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H37" s="26" t="str"/>
-      <x:c r="I37" s="26" t="str">
+      <x:c r="H37" s="27" t="str"/>
+      <x:c r="I37" s="27" t="str">
         <x:v>Markdown CSV Excel issues PR protocol and Obsidian index are linked and verified</x:v>
       </x:c>
-      <x:c r="J37" s="26" t="str">
+      <x:c r="J37" s="27" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K37" s="26" t="str">
+      <x:c r="K37" s="27" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/37</x:v>
       </x:c>
-      <x:c r="L37" s="26" t="str">
+      <x:c r="L37" s="27" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
-      <x:c r="M37" s="29" t="str">
+      <x:c r="M37" s="30" t="str">
         <x:v>2026-10-04</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="30" customHeight="1">
-      <x:c r="A38" s="27" t="str">
-        <x:v>GOV-003</x:v>
-      </x:c>
-      <x:c r="B38" s="27" t="str">
-        <x:v>Reconcile authentication and dependency tracking</x:v>
-      </x:c>
-      <x:c r="C38" s="27" t="str">
-        <x:v>Governance</x:v>
-      </x:c>
-      <x:c r="D38" s="27" t="str">
-        <x:v>Governance</x:v>
-      </x:c>
-      <x:c r="E38" s="27" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="F38" s="27" t="str">
-        <x:v>PR Open</x:v>
-      </x:c>
-      <x:c r="G38" s="27" t="str">
-        <x:v>Codex</x:v>
-      </x:c>
-      <x:c r="H38" s="27" t="str">
-        <x:v>SEC-001,DEP-001</x:v>
-      </x:c>
-      <x:c r="I38" s="27" t="str">
-        <x:v>Canonical registers workbook and operating guidance match the implemented authentication policy and dependency evidence</x:v>
-      </x:c>
-      <x:c r="J38" s="27" t="str">
-        <x:v>User request</x:v>
-      </x:c>
-      <x:c r="K38" s="27" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/60</x:v>
-      </x:c>
-      <x:c r="L38" s="27" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
-      </x:c>
-      <x:c r="M38" s="30" t="str">
-        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E38">
+  <x:conditionalFormatting sqref="E6:E37">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F38">
+  <x:conditionalFormatting sqref="F6:F37">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3313,7 +3235,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2436191cdb94469d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43f025b6eb504a38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3759,117 +3681,25 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="26" t="str">
+      <x:c r="A23" s="27" t="str">
         <x:v>REQ-REV-001</x:v>
       </x:c>
-      <x:c r="B23" s="26" t="str">
+      <x:c r="B23" s="27" t="str">
         <x:v>AWS migration readiness reports INR 1.2M target and INR 1.5M preferred monthly net revenue</x:v>
       </x:c>
-      <x:c r="C23" s="26" t="str">
+      <x:c r="C23" s="27" t="str">
         <x:v>Migration design</x:v>
       </x:c>
-      <x:c r="D23" s="26" t="str">
+      <x:c r="D23" s="27" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="E23" s="26" t="str">
+      <x:c r="E23" s="27" t="str">
         <x:v>Admin readiness UI test</x:v>
       </x:c>
-      <x:c r="F23" s="26" t="str">
+      <x:c r="F23" s="27" t="str">
         <x:v>UI-001</x:v>
       </x:c>
-      <x:c r="G23" s="26" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="26" t="str">
-        <x:v>REQ-AUTH-001</x:v>
-      </x:c>
-      <x:c r="B24" s="26" t="str">
-        <x:v>Administrators authenticate through Zoho SSO and do not require routine application TOTP</x:v>
-      </x:c>
-      <x:c r="C24" s="26" t="str">
-        <x:v>User direction</x:v>
-      </x:c>
-      <x:c r="D24" s="26" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="E24" s="26" t="str">
-        <x:v>Authentication integration tests and controlled Zoho sign-in evidence</x:v>
-      </x:c>
-      <x:c r="F24" s="26" t="str">
-        <x:v>SEC-001</x:v>
-      </x:c>
-      <x:c r="G24" s="26" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="30" customHeight="1">
-      <x:c r="A25" s="26" t="str">
-        <x:v>REQ-AUTH-002</x:v>
-      </x:c>
-      <x:c r="B25" s="26" t="str">
-        <x:v>Existing users may sign in with Zoho SSO or username email or mobile plus password and any valid email provider is accepted</x:v>
-      </x:c>
-      <x:c r="C25" s="26" t="str">
-        <x:v>User direction</x:v>
-      </x:c>
-      <x:c r="D25" s="26" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="E25" s="26" t="str">
-        <x:v>Backend frontend mobile and Playwright authentication tests</x:v>
-      </x:c>
-      <x:c r="F25" s="26" t="str">
-        <x:v>SEC-001</x:v>
-      </x:c>
-      <x:c r="G25" s="26" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="26" t="str">
-        <x:v>REQ-AUTH-003</x:v>
-      </x:c>
-      <x:c r="B26" s="26" t="str">
-        <x:v>OTP is used only for signup/contact verification and password recovery and never as passwordless login</x:v>
-      </x:c>
-      <x:c r="C26" s="26" t="str">
-        <x:v>User direction</x:v>
-      </x:c>
-      <x:c r="D26" s="26" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="E26" s="26" t="str">
-        <x:v>Route inventory and authentication tests</x:v>
-      </x:c>
-      <x:c r="F26" s="26" t="str">
-        <x:v>SEC-001</x:v>
-      </x:c>
-      <x:c r="G26" s="26" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="27" t="str">
-        <x:v>REQ-AUTH-004</x:v>
-      </x:c>
-      <x:c r="B27" s="27" t="str">
-        <x:v>Zoho domain DNS sender mailbox SMTP application password and production OAuth callback are configured only at the final deployment gate</x:v>
-      </x:c>
-      <x:c r="C27" s="27" t="str">
-        <x:v>User direction</x:v>
-      </x:c>
-      <x:c r="D27" s="27" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="E27" s="27" t="str">
-        <x:v>Final release checklist and controlled delivery/SSO evidence</x:v>
-      </x:c>
-      <x:c r="F27" s="27" t="str">
-        <x:v>SEC-001,REL-001</x:v>
-      </x:c>
-      <x:c r="G27" s="27" t="str">
+      <x:c r="G23" s="27" t="str">
         <x:v>Approved</x:v>
       </x:c>
     </x:row>
@@ -3877,10 +3707,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D27">
+  <x:conditionalFormatting sqref="D6:D23">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G6:G27">
+  <x:conditionalFormatting sqref="G6:G23">
     <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Blocked"/>
@@ -3889,7 +3719,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra874fdfd64b54aff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf20a7dccdbee4e1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4196,13 +4026,36 @@
         <x:v>SYNC-002</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>QA-OPS-001</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>Replica safety</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41ec7c27333f406c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd82849163b854701"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4595,71 +4448,42 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="26" t="str">
+      <x:c r="A18" s="27" t="str">
         <x:v>RISK-013</x:v>
       </x:c>
-      <x:c r="B18" s="26" t="str">
-        <x:v>Public deployment tier is enabled before Zoho SSO and administrator recovery are proven</x:v>
-      </x:c>
-      <x:c r="C18" s="26" t="str">
+      <x:c r="B18" s="27" t="str">
+        <x:v>Public deployment tier is enabled before every administrator enrols MFA</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D18" s="26" t="str">
+      <x:c r="D18" s="27" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E18" s="26" t="str">
+      <x:c r="E18" s="27" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F18" s="26" t="str">
-        <x:v>Verify exact OAuth client callback administrator matching-email login Zoho-account MFA and a documented recovery owner in restricted staging before public-beta</x:v>
-      </x:c>
-      <x:c r="G18" s="26" t="str">
+      <x:c r="F18" s="27" t="str">
+        <x:v>Enrol and verify each administrator in restricted staging before selecting public-beta; keep a documented recovery owner</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H18" s="26" t="str">
+      <x:c r="H18" s="27" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="I18" s="26" t="str">
-        <x:v>SEC-001 PR 58 implements Zoho-only administrator login; production Zoho configuration is intentionally deferred to the final gate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="27" t="str">
-        <x:v>RISK-014</x:v>
-      </x:c>
-      <x:c r="B19" s="27" t="str">
-        <x:v>Framework and mobile build-tool dependency advisories remain after runtime remediation</x:v>
-      </x:c>
-      <x:c r="C19" s="27" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="D19" s="27" t="str">
-        <x:v>Possible</x:v>
-      </x:c>
-      <x:c r="E19" s="27" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="F19" s="27" t="str">
-        <x:v>Block new critical/high runtime advisories; allow only four exact no-fix Expo advisory IDs; schedule Nest major migration and review exceptions each release</x:v>
-      </x:c>
-      <x:c r="G19" s="27" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="H19" s="27" t="str">
-        <x:v>Mitigated</x:v>
-      </x:c>
-      <x:c r="I19" s="27" t="str">
-        <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
+      <x:c r="I18" s="27" t="str">
+        <x:v>SEC-001 PR 56 rejects unenrolled login and existing sessions; staged enrollment evidence still required</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E19">
+  <x:conditionalFormatting sqref="E6:E18">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H19">
+  <x:conditionalFormatting sqref="H6:H18">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4668,7 +4492,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d01fdfe08834c0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7dd2ffee5644c37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4899,16 +4723,16 @@
         <x:v>ACC-007</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>Zoho identity and operational email</x:v>
+        <x:v>Operational email</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>OAuth application exact callback domain mailbox DNS authentication reports and SMTP app-password rotation</x:v>
+        <x:v>Zoho domain mailbox DNS authentication reports and app-password rotation</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>Zoho OAuth and SMTP identities</x:v>
+        <x:v>Zoho SMTP identity</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
         <x:v>GitHub Railway or Kubernetes secrets</x:v>
@@ -4918,7 +4742,7 @@
       </x:c>
       <x:c r="H12" s="29" t="str"/>
       <x:c r="I12" s="26" t="str">
-        <x:v>Configure only at final deployment; protect the Zoho owner with Zoho MFA and retain controlled SSO/mail evidence</x:v>
+        <x:v>Low-volume beta only; owner must configure domain MFA app password and first delivery evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -4983,7 +4807,7 @@
         <x:v>WOW-MD source review</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
-        <x:v>Repository contents read for scheduled change reports</x:v>
+        <x:v>Private repository contents read for scheduled change reports</x:v>
       </x:c>
       <x:c r="D15" s="27" t="str">
         <x:v>RohithTadiparti</x:v>
@@ -4995,11 +4819,11 @@
         <x:v>Production GitHub Actions secret</x:v>
       </x:c>
       <x:c r="G15" s="27" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="H15" s="30" t="str"/>
       <x:c r="I15" s="27" t="str">
-        <x:v>Not technically required while WOW-MD is public; create before returning it private so the private-ready workflow keeps working; scope only to WOW-MD Contents read and rotate within 90 days</x:v>
+        <x:v>Scope only to WOW-MD Contents read; rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5015,7 +4839,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b4e6968d40241f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c389c4c429e4851"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5354,7 +5178,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R615eff909ab24642"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e806a33f4514bea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5527,7 +5351,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71cabc95d21f49f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fed96a9bf9e474e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5680,150 +5504,112 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>codex/sec-001-sso-login-policy</x:v>
+        <x:v>codex/sec-001-admin-mfa-provider-policy</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>29537ee</x:v>
+        <x:v>57e13d0</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>3eaa03c</x:v>
+        <x:v>fad2ef5</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>WOW-MD PR 38 head f685774</x:v>
+        <x:v>WOW-MD PR 37 merged as b28c334; application mirror commit 1482d83</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Backend typecheck/lint and 71 focused auth/config tests pass; frontend typecheck and 173 tests pass; mobile typecheck passes; CodeQL security gate passes after refresh cookies were sealed and session hashes moved to memory-hard derivation; remaining protected CI jobs are recorded on the PR</x:v>
+        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance and synchronization 19/19; protected production and source CI passed including retained 30-day CodeQL SARIF</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
-        <x:v>At the final release gate configure exact Zoho OAuth client/callback domain SPF DKIM DMARC sender mailbox and SMTP application password; then run controlled admin/non-admin SSO and email tests</x:v>
+        <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
       </x:c>
       <x:c r="I8" s="26" t="str">
-        <x:v>Restore the prior image/config and disable Zoho SSO; do not enable passwordless OTP or log-based mail in public tier</x:v>
+        <x:v>Restore previous image/config; do not fall back to log/mock in a public tier; pause email-dependent workflows</x:v>
       </x:c>
       <x:c r="J8" s="26" t="str">
-        <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred to the final release gate</x:v>
+        <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
       </x:c>
       <x:c r="K8" s="26" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="26" t="str">
+      <x:c r="A9" s="27" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="B9" s="26" t="str">
+      <x:c r="B9" s="27" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
       </x:c>
-      <x:c r="C9" s="26" t="str">
+      <x:c r="C9" s="27" t="str">
         <x:v>codex/sync-002-gated-source-review</x:v>
       </x:c>
-      <x:c r="D9" s="26" t="str">
+      <x:c r="D9" s="27" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E9" s="26" t="str">
+      <x:c r="E9" s="27" t="str">
         <x:v>422cbc4</x:v>
       </x:c>
-      <x:c r="F9" s="26" t="str">
+      <x:c r="F9" s="27" t="str">
         <x:v>07218b4..de7d8dd local review only</x:v>
       </x:c>
-      <x:c r="G9" s="26" t="str">
+      <x:c r="G9" s="27" t="str">
         <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
       </x:c>
-      <x:c r="H9" s="26" t="str">
+      <x:c r="H9" s="27" t="str">
         <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
       </x:c>
-      <x:c r="I9" s="26" t="str">
+      <x:c r="I9" s="27" t="str">
         <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
       </x:c>
-      <x:c r="J9" s="26" t="str">
+      <x:c r="J9" s="27" t="str">
         <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
       </x:c>
-      <x:c r="K9" s="26" t="str">
+      <x:c r="K9" s="27" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="L9" s="29" t="str">
+      <x:c r="L9" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="26" t="str">
-        <x:v>DEP-001</x:v>
-      </x:c>
-      <x:c r="B10" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
-      </x:c>
-      <x:c r="C10" s="26" t="str">
-        <x:v>codex/dep-001-dependency-remediation</x:v>
-      </x:c>
-      <x:c r="D10" s="26" t="str">
-        <x:v>29537ee</x:v>
-      </x:c>
-      <x:c r="E10" s="26" t="str">
-        <x:v>1ecbfdf</x:v>
-      </x:c>
-      <x:c r="F10" s="26" t="str">
-        <x:v>WOW-MD PR 39 head d8ef995</x:v>
-      </x:c>
-      <x:c r="G10" s="26" t="str">
-        <x:v>Backend clean install typecheck lint build and 792 tests pass with 9 skipped; frontend clean install typecheck 173 tests build and 10 Playwright flows pass; runtime audits: backend 0 critical/0 high frontend 0; exact-ID mobile gate passes; production and source protected CI pass</x:v>
-      </x:c>
-      <x:c r="H10" s="26" t="str">
-        <x:v>No deployment before review and merge; after merge let GitHub rescan manifests and confirm alert counts and audit gates on main</x:v>
-      </x:c>
-      <x:c r="I10" s="26" t="str">
-        <x:v>Revert PR 59; restore prior lockfiles and packages; retain the audit report for comparison</x:v>
-      </x:c>
-      <x:c r="J10" s="26" t="str">
-        <x:v>Backend moderate/low build-tool advisories and four exact no-fix Expo advisory roots remain; forced NestJS 12 and Expo downgrades were tested and rejected as unsafe</x:v>
-      </x:c>
-      <x:c r="K10" s="26" t="str">
-        <x:v>PR Open</x:v>
-      </x:c>
-      <x:c r="L10" s="29" t="str">
-        <x:v>2026-10-05</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="27" t="str">
-        <x:v>GOV-003</x:v>
-      </x:c>
-      <x:c r="B11" s="27" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
-      </x:c>
-      <x:c r="C11" s="27" t="str">
-        <x:v>codex/gov-003-auth-dependency-tracking</x:v>
-      </x:c>
-      <x:c r="D11" s="27" t="str">
-        <x:v>29537ee</x:v>
-      </x:c>
-      <x:c r="E11" s="27" t="str">
-        <x:v>1235cd3</x:v>
-      </x:c>
-      <x:c r="F11" s="27" t="str">
-        <x:v>SEC-001 PR 58 and DEP-001 PR 59 evidence only</x:v>
-      </x:c>
-      <x:c r="G11" s="27" t="str">
-        <x:v>Register validator workbook regeneration and formula-error scan pass; dashboard visually reviewed</x:v>
-      </x:c>
-      <x:c r="H11" s="27" t="str">
-        <x:v>Governance and documentation only; no application or hosting deployment</x:v>
-      </x:c>
-      <x:c r="I11" s="27" t="str">
-        <x:v>Revert PR 61; implementation PRs and their evidence remain unchanged</x:v>
-      </x:c>
-      <x:c r="J11" s="27" t="str">
-        <x:v>Implementation PRs still require review/merge and GitHub rescan; Zoho live configuration remains a final release gate</x:v>
-      </x:c>
-      <x:c r="K11" s="27" t="str">
-        <x:v>PR Open</x:v>
-      </x:c>
-      <x:c r="L11" s="30" t="str">
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>codex/ops-001-replicated-jobs</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>57e13d0</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>090d236</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>WOW-MD commit a06067a; PR 42</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Focused replica tests 7 of 7; backend full suite 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Deploy normally after approval; verify two replicas produce one owner and one skipped invocation for outbox and payout/reminder jobs</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>Revert PR 64 and redeploy; no database or configuration rollback</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>Outbox delivery remains at-least-once across a crash after an external side effect; Kafka consumers must honor the outbox UUID idempotency key</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>Ready for Review</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
@@ -5831,7 +5617,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K11">
+  <x:conditionalFormatting sqref="K6:K9">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5840,7 +5626,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3652ba24d5b84156"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b042648f28498e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(obs): record OBS-001 review handoff
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raeedae5ff209418d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R40b455cf76954eb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R5023dffb9e4448ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R2db2c6f1609549d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rdf0ccb98e6224d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R42965f3834b04aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R1a1b0d2dd00d4ca2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re691660970d54e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra4fa0222c47c4087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8bfac8c765c04c81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb1a81da2f2014435"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Ra7461bf4dcfb4305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R0e96e3e2600e4214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R98da020119b44f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R8aa33dab71ba45c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R92f26e4c0b364480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R26c31c2a0f784e41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6f685f0304024924"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R1ee073186a0d4a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7e6fe2172f234a3c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Recbdb8875ecc49f8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8b785583de834eb6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1439,7 +1439,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11dd2df34d0a44bb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44d35715b66648ca"/>
 </x:worksheet>
 </file>
 
@@ -1899,7 +1899,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3389fabded664992"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d61ae7eeb044cf6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2072,10 +2072,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Unassigned</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str"/>
       <x:c r="I8" s="26" t="str">
@@ -2087,11 +2087,9 @@
       <x:c r="K8" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/8</x:v>
       </x:c>
-      <x:c r="L8" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
-      </x:c>
+      <x:c r="L8" s="26" t="str"/>
       <x:c r="M8" s="29" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -2185,10 +2183,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F11" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H11" s="26" t="str">
         <x:v>SEC-003</x:v>
@@ -2202,9 +2200,11 @@
       <x:c r="K11" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/11</x:v>
       </x:c>
-      <x:c r="L11" s="26" t="str"/>
+      <x:c r="L11" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/65</x:v>
+      </x:c>
       <x:c r="M11" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
@@ -3235,7 +3235,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43f025b6eb504a38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13810d1b976a4191"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3719,7 +3719,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf20a7dccdbee4e1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R718b81cadaf445d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4028,25 +4028,25 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>QA-OPS-001</x:v>
+        <x:v>QA-OBS-001</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>Replica safety</x:v>
+        <x:v>Observability</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
+        <x:v>Request correlation redaction provider logs QA capture audit failures payout sweep and nginx JSON</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
+        <x:v>OBS-001 PR 65 and WOW-MD PR 43</x:v>
       </x:c>
       <x:c r="E17" t="str">
-        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
+        <x:v>Focused 20 of 20; full backend 812 passed 9 skipped; typecheck lint nginx contract image build and syntax passed</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
+        <x:v>Deploy after SEC-003 and verify live response/log correlation with capture disabled</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>OPS-001</x:v>
+        <x:v>OBS-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4055,7 +4055,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd82849163b854701"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8285d63d48484bc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4492,7 +4492,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7dd2ffee5644c37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94914057e8ce466d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4839,7 +4839,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c389c4c429e4851"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd40f85e1aac467e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5178,7 +5178,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e806a33f4514bea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf86f2bf9b8614332"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5351,7 +5351,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fed96a9bf9e474e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re46edf7e1d584ba5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5577,34 +5577,34 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>OPS-001</x:v>
+        <x:v>OBS-001</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/65</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>codex/ops-001-replicated-jobs</x:v>
+        <x:v>codex/obs-001-backend-observability</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>57e13d0</x:v>
+        <x:v>29537ee</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>090d236</x:v>
+        <x:v>48c1351</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>WOW-MD commit a06067a; PR 42</x:v>
+        <x:v>WOW-MD commit 69c2aea; PR 43</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>Focused replica tests 7 of 7; backend full suite 797 passed 9 skipped; typecheck and lint passed</x:v>
+        <x:v>Focused observability 20 of 20; backend full suite 812 passed 9 skipped; typecheck lint nginx contract frontend image build and nginx syntax passed</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>Deploy normally after approval; verify two replicas produce one owner and one skipped invocation for outbox and payout/reminder jobs</x:v>
+        <x:v>Merge SEC-003 first then rebase; set RELEASE; keep QA capture disabled; confirm a live request ID matches response backend and nginx logs</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>Revert PR 64 and redeploy; no database or configuration rollback</x:v>
+        <x:v>Revert PR 65 and redeploy; remove optional observability variables; no database rollback</x:v>
       </x:c>
       <x:c r="J10" t="str">
-        <x:v>Outbox delivery remains at-least-once across a crash after an external side effect; Kafka consumers must honor the outbox UUID idempotency key</x:v>
+        <x:v>OBS-002 client error intake and OBS-003 Loki Vector host files 30-day retention remain open; live provider correlation smoke remains</x:v>
       </x:c>
       <x:c r="K10" t="str">
         <x:v>Ready for Review</x:v>
@@ -5626,7 +5626,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b042648f28498e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998f60580a2a4686"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[GOV-003] Reconcile authentication and dependency tracking (#61)
* docs: reconcile auth and dependency tracking

* docs: publish reconciled readiness tracker

* docs: record refresh-token security evidence

* docs: clarify source token and access timing

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc7df0f9914894907"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R68804a89813f4b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R9b27cde7d36d40c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R8563e05c03a44a0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R4435416debb841e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rab75932cb0c24236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra05f7be5ed4241bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R2c0f08a920424505"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re0e79451554c4a60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R3eb7011c83984eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R980ff49061094730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rd695025b504247c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R9a28dae678d84cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R85498cf0250c4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R921698851bbc42a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R8c95448b30954ae2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rc31255f8c95b4307"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R773444ff6d894f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R99b2d2f3c8994cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb45c6ad01fba48ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bc115c2266f4c13"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbfddc80666614cbb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -840,7 +840,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -861,7 +861,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Requirement"/>
@@ -891,7 +891,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -960,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -980,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1207,7 +1207,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-04. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-05. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1235,22 +1235,22 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$37)</x:f>
-        <x:v>32</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$38)</x:f>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1258,8 +1258,8 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Open")</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Open")</x:f>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1281,14 +1281,14 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$18,"Open")</x:f>
+        <x:f>COUNTIF(Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
@@ -1296,7 +1296,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1304,14 +1304,14 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"PR Open")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"PR Open")</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$18,"P0",Risks!$H$6:$H$18,"Open")</x:f>
+        <x:f>COUNTIFS(Risks!$E$6:$E$19,"P0",Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
@@ -1319,7 +1319,7 @@
       </x:c>
       <x:c r="H9" s="39" t="n">
         <x:f>B10</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1327,15 +1327,15 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Blocked")</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Blocked")</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIF(Requirements!$G$6:$G$23,"Approved")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF(Requirements!$G$6:$G$27,"Approved")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G10" s="39" t="str">
         <x:v>Done</x:v>
@@ -1350,7 +1350,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$37,"Done")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Done")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
@@ -1450,7 +1450,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R235076d8006a4a39"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96197e094d6a4087"/>
 </x:worksheet>
 </file>
 
@@ -1872,36 +1872,62 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="27" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>DOC-015</x:v>
       </x:c>
-      <x:c r="B20" s="27" t="str">
-        <x:v>Zoho Mail SMTP operating guide</x:v>
-      </x:c>
-      <x:c r="C20" s="27" t="str">
+      <x:c r="B20" s="26" t="str">
+        <x:v>Zoho SSO and mail operating guide</x:v>
+      </x:c>
+      <x:c r="C20" s="26" t="str">
         <x:v>docs/operations/zoho-mail.md</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="str">
+      <x:c r="D20" s="26" t="str">
         <x:v>Security and operations</x:v>
       </x:c>
-      <x:c r="E20" s="27" t="str">
+      <x:c r="E20" s="26" t="str">
         <x:v>Approved candidate</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>Quarterly or provider change</x:v>
       </x:c>
-      <x:c r="G20" s="27" t="str">
-        <x:v>2026-10-04</x:v>
-      </x:c>
-      <x:c r="H20" s="27" t="str">
-        <x:v>SEC-001 OPS-003</x:v>
+      <x:c r="G20" s="26" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="H20" s="26" t="str">
+        <x:v>SEC-001 AUTH-001 OPS-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="27" t="str">
+        <x:v>DOC-016</x:v>
+      </x:c>
+      <x:c r="B21" s="27" t="str">
+        <x:v>Dependency remediation record</x:v>
+      </x:c>
+      <x:c r="C21" s="27" t="str">
+        <x:v>docs/security/dependency-remediation-2026-10-04.md</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>Approved candidate</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="str">
+        <x:v>Each dependency change</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="str">
+        <x:v>DEP-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E20">
+  <x:conditionalFormatting sqref="E6:E21">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -1910,7 +1936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0a0800dfcc14e4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94ee19de0e1f4528"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1993,7 +2019,7 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>Enforce administrator MFA and production provider policy</x:v>
+        <x:v>Align authentication with Zoho SSO and multi-identifier login policy</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str">
         <x:v>Public beta safety</x:v>
@@ -2005,26 +2031,26 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F6" s="25" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
-        <x:v>Admin cannot use privileged access without MFA; unsafe production provider combinations fail startup</x:v>
+        <x:v>Administrators use Zoho SSO; existing users may use Zoho SSO or username/email/mobile plus password; OTP is verification/recovery only; unsafe public provider combinations fail startup</x:v>
       </x:c>
       <x:c r="J6" s="25" t="str">
-        <x:v>Production plan Task 1A</x:v>
+        <x:v>Production plan Task 1A and user authentication decision</x:v>
       </x:c>
       <x:c r="K6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
       </x:c>
       <x:c r="M6" s="28" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -2157,14 +2183,14 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F10" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str"/>
       <x:c r="I10" s="26" t="str">
-        <x:v>No unaccepted critical/high production advisory; CI blocks regression</x:v>
+        <x:v>No unaccepted critical/high runtime advisory; CI blocks regressions; explicitly documented no-fix build-tool exceptions remain narrow and reviewable</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
         <x:v>Production plan Task 1E</x:v>
@@ -2172,9 +2198,11 @@
       <x:c r="K10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/10</x:v>
       </x:c>
-      <x:c r="L10" s="26" t="str"/>
+      <x:c r="L10" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
+      </x:c>
       <x:c r="M10" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -2533,7 +2561,7 @@
         <x:v>AUTH-001</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Add scoped administrator MFA step-up</x:v>
+        <x:v>Add scoped administrator fresh-authentication step-up</x:v>
       </x:c>
       <x:c r="C20" s="26" t="str">
         <x:v>Migration control</x:v>
@@ -2554,17 +2582,17 @@
         <x:v>SEC-001,CFG-001</x:v>
       </x:c>
       <x:c r="I20" s="26" t="str">
-        <x:v>Five-minute single-use scoped token protects migration start</x:v>
+        <x:v>Fresh Zoho reauthentication issues a five-minute single-use action-scoped token for migration start; application TOTP is a documented fallback only</x:v>
       </x:c>
       <x:c r="J20" s="26" t="str">
-        <x:v>Production plan Task 9</x:v>
+        <x:v>Production plan Task 9 and user authentication decision</x:v>
       </x:c>
       <x:c r="K20" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/20</x:v>
       </x:c>
       <x:c r="L20" s="26" t="str"/>
       <x:c r="M20" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -3190,52 +3218,93 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
-      <x:c r="A37" s="27" t="str">
+      <x:c r="A37" s="26" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B37" s="27" t="str">
+      <x:c r="B37" s="26" t="str">
         <x:v>Establish SDLC knowledge and tracking system</x:v>
       </x:c>
-      <x:c r="C37" s="27" t="str">
+      <x:c r="C37" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="D37" s="27" t="str">
+      <x:c r="D37" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="E37" s="27" t="str">
+      <x:c r="E37" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F37" s="27" t="str">
+      <x:c r="F37" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G37" s="27" t="str">
+      <x:c r="G37" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H37" s="27" t="str"/>
-      <x:c r="I37" s="27" t="str">
+      <x:c r="H37" s="26" t="str"/>
+      <x:c r="I37" s="26" t="str">
         <x:v>Markdown CSV Excel issues PR protocol and Obsidian index are linked and verified</x:v>
       </x:c>
-      <x:c r="J37" s="27" t="str">
+      <x:c r="J37" s="26" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K37" s="27" t="str">
+      <x:c r="K37" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/37</x:v>
       </x:c>
-      <x:c r="L37" s="27" t="str">
+      <x:c r="L37" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
-      <x:c r="M37" s="30" t="str">
+      <x:c r="M37" s="29" t="str">
         <x:v>2026-10-04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="27" t="str">
+        <x:v>GOV-003</x:v>
+      </x:c>
+      <x:c r="B38" s="27" t="str">
+        <x:v>Reconcile authentication and dependency tracking</x:v>
+      </x:c>
+      <x:c r="C38" s="27" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="D38" s="27" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="E38" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F38" s="27" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G38" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H38" s="27" t="str">
+        <x:v>SEC-001,DEP-001</x:v>
+      </x:c>
+      <x:c r="I38" s="27" t="str">
+        <x:v>Canonical registers workbook and operating guidance match the implemented authentication policy and dependency evidence</x:v>
+      </x:c>
+      <x:c r="J38" s="27" t="str">
+        <x:v>User request</x:v>
+      </x:c>
+      <x:c r="K38" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/60</x:v>
+      </x:c>
+      <x:c r="L38" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
+      </x:c>
+      <x:c r="M38" s="30" t="str">
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E37">
+  <x:conditionalFormatting sqref="E6:E38">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F37">
+  <x:conditionalFormatting sqref="F6:F38">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3244,7 +3313,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re745519934ee43a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2436191cdb94469d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3690,25 +3759,117 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="27" t="str">
+      <x:c r="A23" s="26" t="str">
         <x:v>REQ-REV-001</x:v>
       </x:c>
-      <x:c r="B23" s="27" t="str">
+      <x:c r="B23" s="26" t="str">
         <x:v>AWS migration readiness reports INR 1.2M target and INR 1.5M preferred monthly net revenue</x:v>
       </x:c>
-      <x:c r="C23" s="27" t="str">
+      <x:c r="C23" s="26" t="str">
         <x:v>Migration design</x:v>
       </x:c>
-      <x:c r="D23" s="27" t="str">
+      <x:c r="D23" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="E23" s="27" t="str">
+      <x:c r="E23" s="26" t="str">
         <x:v>Admin readiness UI test</x:v>
       </x:c>
-      <x:c r="F23" s="27" t="str">
+      <x:c r="F23" s="26" t="str">
         <x:v>UI-001</x:v>
       </x:c>
-      <x:c r="G23" s="27" t="str">
+      <x:c r="G23" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="26" t="str">
+        <x:v>REQ-AUTH-001</x:v>
+      </x:c>
+      <x:c r="B24" s="26" t="str">
+        <x:v>Administrators authenticate through Zoho SSO and do not require routine application TOTP</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E24" s="26" t="str">
+        <x:v>Authentication integration tests and controlled Zoho sign-in evidence</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G24" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="26" t="str">
+        <x:v>REQ-AUTH-002</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="str">
+        <x:v>Existing users may sign in with Zoho SSO or username email or mobile plus password and any valid email provider is accepted</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>Backend frontend mobile and Playwright authentication tests</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="A26" s="26" t="str">
+        <x:v>REQ-AUTH-003</x:v>
+      </x:c>
+      <x:c r="B26" s="26" t="str">
+        <x:v>OTP is used only for signup/contact verification and password recovery and never as passwordless login</x:v>
+      </x:c>
+      <x:c r="C26" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="str">
+        <x:v>Route inventory and authentication tests</x:v>
+      </x:c>
+      <x:c r="F26" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G26" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="27" t="str">
+        <x:v>REQ-AUTH-004</x:v>
+      </x:c>
+      <x:c r="B27" s="27" t="str">
+        <x:v>Zoho domain DNS sender mailbox SMTP application password and production OAuth callback are configured only at the final deployment gate</x:v>
+      </x:c>
+      <x:c r="C27" s="27" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D27" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E27" s="27" t="str">
+        <x:v>Final release checklist and controlled delivery/SSO evidence</x:v>
+      </x:c>
+      <x:c r="F27" s="27" t="str">
+        <x:v>SEC-001,REL-001</x:v>
+      </x:c>
+      <x:c r="G27" s="27" t="str">
         <x:v>Approved</x:v>
       </x:c>
     </x:row>
@@ -3716,10 +3877,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D23">
+  <x:conditionalFormatting sqref="D6:D27">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G6:G23">
+  <x:conditionalFormatting sqref="G6:G27">
     <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Blocked"/>
@@ -3728,7 +3889,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bdc418640084c9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra874fdfd64b54aff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4041,7 +4202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf6a9523139243b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41ec7c27333f406c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4434,42 +4595,71 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="27" t="str">
+      <x:c r="A18" s="26" t="str">
         <x:v>RISK-013</x:v>
       </x:c>
-      <x:c r="B18" s="27" t="str">
-        <x:v>Public deployment tier is enabled before every administrator enrols MFA</x:v>
-      </x:c>
-      <x:c r="C18" s="27" t="str">
+      <x:c r="B18" s="26" t="str">
+        <x:v>Public deployment tier is enabled before Zoho SSO and administrator recovery are proven</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D18" s="27" t="str">
+      <x:c r="D18" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E18" s="27" t="str">
+      <x:c r="E18" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F18" s="27" t="str">
-        <x:v>Enrol and verify each administrator in restricted staging before selecting public-beta; keep a documented recovery owner</x:v>
-      </x:c>
-      <x:c r="G18" s="27" t="str">
+      <x:c r="F18" s="26" t="str">
+        <x:v>Verify exact OAuth client callback administrator matching-email login Zoho-account MFA and a documented recovery owner in restricted staging before public-beta</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H18" s="27" t="str">
+      <x:c r="H18" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="I18" s="27" t="str">
-        <x:v>SEC-001 PR 56 rejects unenrolled login and existing sessions; staged enrollment evidence still required</x:v>
+      <x:c r="I18" s="26" t="str">
+        <x:v>SEC-001 PR 58 implements Zoho-only administrator login; production Zoho configuration is intentionally deferred to the final gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="27" t="str">
+        <x:v>RISK-014</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="str">
+        <x:v>Framework and mobile build-tool dependency advisories remain after runtime remediation</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="str">
+        <x:v>Block new critical/high runtime advisories; allow only four exact no-fix Expo advisory IDs; schedule Nest major migration and review exceptions each release</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="H19" s="27" t="str">
+        <x:v>Mitigated</x:v>
+      </x:c>
+      <x:c r="I19" s="27" t="str">
+        <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E18">
+  <x:conditionalFormatting sqref="E6:E19">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H18">
+  <x:conditionalFormatting sqref="H6:H19">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4478,7 +4668,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R629b5fd99f4747e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d01fdfe08834c0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4709,16 +4899,16 @@
         <x:v>ACC-007</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>Operational email</x:v>
+        <x:v>Zoho identity and operational email</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>Zoho domain mailbox DNS authentication reports and app-password rotation</x:v>
+        <x:v>OAuth application exact callback domain mailbox DNS authentication reports and SMTP app-password rotation</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>Zoho SMTP identity</x:v>
+        <x:v>Zoho OAuth and SMTP identities</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
         <x:v>GitHub Railway or Kubernetes secrets</x:v>
@@ -4728,7 +4918,7 @@
       </x:c>
       <x:c r="H12" s="29" t="str"/>
       <x:c r="I12" s="26" t="str">
-        <x:v>Low-volume beta only; owner must configure domain MFA app password and first delivery evidence</x:v>
+        <x:v>Configure only at final deployment; protect the Zoho owner with Zoho MFA and retain controlled SSO/mail evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -4793,7 +4983,7 @@
         <x:v>WOW-MD source review</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
-        <x:v>Private repository contents read for scheduled change reports</x:v>
+        <x:v>Repository contents read for scheduled change reports</x:v>
       </x:c>
       <x:c r="D15" s="27" t="str">
         <x:v>RohithTadiparti</x:v>
@@ -4805,11 +4995,11 @@
         <x:v>Production GitHub Actions secret</x:v>
       </x:c>
       <x:c r="G15" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="H15" s="30" t="str"/>
       <x:c r="I15" s="27" t="str">
-        <x:v>Scope only to WOW-MD Contents read; rotate within 90 days</x:v>
+        <x:v>Not technically required while WOW-MD is public; create before returning it private so the private-ready workflow keeps working; scope only to WOW-MD Contents read and rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4825,7 +5015,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R583232c454d4495b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b4e6968d40241f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5164,7 +5354,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a9dd407c2d345e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R615eff909ab24642"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5337,7 +5527,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71254912a1424da7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71cabc95d21f49f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5490,82 +5680,158 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>codex/sec-001-admin-mfa-provider-policy</x:v>
+        <x:v>codex/sec-001-sso-login-policy</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E8" s="26" t="str">
+        <x:v>3eaa03c</x:v>
+      </x:c>
+      <x:c r="F8" s="26" t="str">
+        <x:v>WOW-MD PR 38 head f685774</x:v>
+      </x:c>
+      <x:c r="G8" s="26" t="str">
+        <x:v>Backend typecheck/lint and 71 focused auth/config tests pass; frontend typecheck and 173 tests pass; mobile typecheck passes; CodeQL security gate passes after refresh cookies were sealed and session hashes moved to memory-hard derivation; remaining protected CI jobs are recorded on the PR</x:v>
+      </x:c>
+      <x:c r="H8" s="26" t="str">
+        <x:v>At the final release gate configure exact Zoho OAuth client/callback domain SPF DKIM DMARC sender mailbox and SMTP application password; then run controlled admin/non-admin SSO and email tests</x:v>
+      </x:c>
+      <x:c r="I8" s="26" t="str">
+        <x:v>Restore the prior image/config and disable Zoho SSO; do not enable passwordless OTP or log-based mail in public tier</x:v>
+      </x:c>
+      <x:c r="J8" s="26" t="str">
+        <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred to the final release gate</x:v>
+      </x:c>
+      <x:c r="K8" s="26" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L8" s="29" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="26" t="str">
+        <x:v>SYNC-002</x:v>
+      </x:c>
+      <x:c r="B9" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
+      </x:c>
+      <x:c r="C9" s="26" t="str">
+        <x:v>codex/sync-002-gated-source-review</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E8" s="26" t="str">
-        <x:v>fad2ef5</x:v>
-      </x:c>
-      <x:c r="F8" s="26" t="str">
-        <x:v>WOW-MD PR 37 merged as b28c334; application mirror commit 1482d83</x:v>
-      </x:c>
-      <x:c r="G8" s="26" t="str">
-        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance and synchronization 19/19; protected production and source CI passed including retained 30-day CodeQL SARIF</x:v>
-      </x:c>
-      <x:c r="H8" s="26" t="str">
-        <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
-      </x:c>
-      <x:c r="I8" s="26" t="str">
-        <x:v>Restore previous image/config; do not fall back to log/mock in a public tier; pause email-dependent workflows</x:v>
-      </x:c>
-      <x:c r="J8" s="26" t="str">
-        <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
-      </x:c>
-      <x:c r="K8" s="26" t="str">
+      <x:c r="E9" s="26" t="str">
+        <x:v>422cbc4</x:v>
+      </x:c>
+      <x:c r="F9" s="26" t="str">
+        <x:v>07218b4..de7d8dd local review only</x:v>
+      </x:c>
+      <x:c r="G9" s="26" t="str">
+        <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
+      </x:c>
+      <x:c r="H9" s="26" t="str">
+        <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
+      </x:c>
+      <x:c r="I9" s="26" t="str">
+        <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
+      </x:c>
+      <x:c r="J9" s="26" t="str">
+        <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
+      </x:c>
+      <x:c r="K9" s="26" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="L8" s="29" t="str">
+      <x:c r="L9" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="27" t="str">
-        <x:v>SYNC-002</x:v>
-      </x:c>
-      <x:c r="B9" s="27" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
-      </x:c>
-      <x:c r="C9" s="27" t="str">
-        <x:v>codex/sync-002-gated-source-review</x:v>
-      </x:c>
-      <x:c r="D9" s="27" t="str">
-        <x:v>57e13d0</x:v>
-      </x:c>
-      <x:c r="E9" s="27" t="str">
-        <x:v>422cbc4</x:v>
-      </x:c>
-      <x:c r="F9" s="27" t="str">
-        <x:v>07218b4..de7d8dd local review only</x:v>
-      </x:c>
-      <x:c r="G9" s="27" t="str">
-        <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
-      </x:c>
-      <x:c r="H9" s="27" t="str">
-        <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
-      </x:c>
-      <x:c r="I9" s="27" t="str">
-        <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
-      </x:c>
-      <x:c r="J9" s="27" t="str">
-        <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
-      </x:c>
-      <x:c r="K9" s="27" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="L9" s="30" t="str">
-        <x:v>2026-10-04</x:v>
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="26" t="str">
+        <x:v>DEP-001</x:v>
+      </x:c>
+      <x:c r="B10" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
+      </x:c>
+      <x:c r="C10" s="26" t="str">
+        <x:v>codex/dep-001-dependency-remediation</x:v>
+      </x:c>
+      <x:c r="D10" s="26" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E10" s="26" t="str">
+        <x:v>1ecbfdf</x:v>
+      </x:c>
+      <x:c r="F10" s="26" t="str">
+        <x:v>WOW-MD PR 39 head d8ef995</x:v>
+      </x:c>
+      <x:c r="G10" s="26" t="str">
+        <x:v>Backend clean install typecheck lint build and 792 tests pass with 9 skipped; frontend clean install typecheck 173 tests build and 10 Playwright flows pass; runtime audits: backend 0 critical/0 high frontend 0; exact-ID mobile gate passes; production and source protected CI pass</x:v>
+      </x:c>
+      <x:c r="H10" s="26" t="str">
+        <x:v>No deployment before review and merge; after merge let GitHub rescan manifests and confirm alert counts and audit gates on main</x:v>
+      </x:c>
+      <x:c r="I10" s="26" t="str">
+        <x:v>Revert PR 59; restore prior lockfiles and packages; retain the audit report for comparison</x:v>
+      </x:c>
+      <x:c r="J10" s="26" t="str">
+        <x:v>Backend moderate/low build-tool advisories and four exact no-fix Expo advisory roots remain; forced NestJS 12 and Expo downgrades were tested and rejected as unsafe</x:v>
+      </x:c>
+      <x:c r="K10" s="26" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L10" s="29" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="27" t="str">
+        <x:v>GOV-003</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
+      </x:c>
+      <x:c r="C11" s="27" t="str">
+        <x:v>codex/gov-003-auth-dependency-tracking</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E11" s="27" t="str">
+        <x:v>1235cd3</x:v>
+      </x:c>
+      <x:c r="F11" s="27" t="str">
+        <x:v>SEC-001 PR 58 and DEP-001 PR 59 evidence only</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="str">
+        <x:v>Register validator workbook regeneration and formula-error scan pass; dashboard visually reviewed</x:v>
+      </x:c>
+      <x:c r="H11" s="27" t="str">
+        <x:v>Governance and documentation only; no application or hosting deployment</x:v>
+      </x:c>
+      <x:c r="I11" s="27" t="str">
+        <x:v>Revert PR 61; implementation PRs and their evidence remain unchanged</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="str">
+        <x:v>Implementation PRs still require review/merge and GitHub rescan; Zoho live configuration remains a final release gate</x:v>
+      </x:c>
+      <x:c r="K11" s="27" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L11" s="30" t="str">
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K9">
+  <x:conditionalFormatting sqref="K6:K11">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5574,7 +5840,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fcaf48711b94f06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3652ba24d5b84156"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
OPS-001: serialize replicated outbox and scheduled jobs (#64)
* fix(ops): serialize replicated background work

* docs(ops): record OPS-001 review handoff

* docs(ops): refresh OPS-001 Excel tracker

* ci: refresh mirror gate metadata

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R980ff49061094730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rd695025b504247c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R9a28dae678d84cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R85498cf0250c4f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R921698851bbc42a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R8c95448b30954ae2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rc31255f8c95b4307"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R773444ff6d894f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R99b2d2f3c8994cad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb45c6ad01fba48ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raeedae5ff209418d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R40b455cf76954eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R5023dffb9e4448ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R2db2c6f1609549d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rdf0ccb98e6224d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R42965f3834b04aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R1a1b0d2dd00d4ca2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re691660970d54e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra4fa0222c47c4087"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8bfac8c765c04c81"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -224,7 +224,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -234,7 +234,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -244,7 +244,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -255,7 +255,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -265,7 +265,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -275,7 +275,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -286,7 +286,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -296,7 +296,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -306,7 +306,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -317,7 +317,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -327,7 +327,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -337,7 +337,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -348,7 +348,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -358,7 +358,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -368,7 +368,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -379,7 +379,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -389,7 +389,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -399,7 +399,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -409,7 +409,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -419,7 +419,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -430,7 +430,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -440,7 +440,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -450,7 +450,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -460,7 +460,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -470,7 +470,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -481,7 +481,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -491,7 +491,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -501,7 +501,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -511,7 +511,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -521,7 +521,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -532,7 +532,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -542,7 +542,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -552,7 +552,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -562,7 +562,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -572,7 +572,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -583,7 +583,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -593,7 +593,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -603,7 +603,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -614,7 +614,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -624,7 +624,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbfddc80666614cbb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Recbdb8875ecc49f8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -840,7 +840,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -861,7 +861,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Requirement"/>
@@ -891,7 +891,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -960,7 +960,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -980,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1235,21 +1235,19 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$38)</x:f>
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
-        <x:f>B7</x:f>
         <x:v>27</x:v>
       </x:c>
     </x:row>
@@ -1258,7 +1256,6 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Open")</x:f>
         <x:v>27</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1272,7 +1269,6 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H7" s="39" t="n">
-        <x:f>B8</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1281,22 +1277,20 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$19,"Open")</x:f>
+        <x:f>COUNTIF(Risks!$H$6:$H$18,"Open")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:f>B9</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1304,22 +1298,20 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"PR Open")</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$19,"P0",Risks!$H$6:$H$19,"Open")</x:f>
+        <x:f>COUNTIFS(Risks!$E$6:$E$18,"P0",Risks!$H$6:$H$18,"Open")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H9" s="39" t="n">
-        <x:f>B10</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1327,21 +1319,19 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIF(Requirements!$G$6:$G$27,"Approved")</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTIF(Requirements!$G$6:$G$23,"Approved")</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G10" s="39" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:f>B11</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -1350,7 +1340,6 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$38,"Done")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
@@ -1450,7 +1439,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96197e094d6a4087"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11dd2df34d0a44bb"/>
 </x:worksheet>
 </file>
 
@@ -1872,62 +1861,36 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="26" t="str">
+      <x:c r="A20" s="27" t="str">
         <x:v>DOC-015</x:v>
       </x:c>
-      <x:c r="B20" s="26" t="str">
-        <x:v>Zoho SSO and mail operating guide</x:v>
-      </x:c>
-      <x:c r="C20" s="26" t="str">
+      <x:c r="B20" s="27" t="str">
+        <x:v>Zoho Mail SMTP operating guide</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
         <x:v>docs/operations/zoho-mail.md</x:v>
       </x:c>
-      <x:c r="D20" s="26" t="str">
+      <x:c r="D20" s="27" t="str">
         <x:v>Security and operations</x:v>
       </x:c>
-      <x:c r="E20" s="26" t="str">
+      <x:c r="E20" s="27" t="str">
         <x:v>Approved candidate</x:v>
       </x:c>
-      <x:c r="F20" s="26" t="str">
+      <x:c r="F20" s="27" t="str">
         <x:v>Quarterly or provider change</x:v>
       </x:c>
-      <x:c r="G20" s="26" t="str">
-        <x:v>2026-10-05</x:v>
-      </x:c>
-      <x:c r="H20" s="26" t="str">
-        <x:v>SEC-001 AUTH-001 OPS-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="27" t="str">
-        <x:v>DOC-016</x:v>
-      </x:c>
-      <x:c r="B21" s="27" t="str">
-        <x:v>Dependency remediation record</x:v>
-      </x:c>
-      <x:c r="C21" s="27" t="str">
-        <x:v>docs/security/dependency-remediation-2026-10-04.md</x:v>
-      </x:c>
-      <x:c r="D21" s="27" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="E21" s="27" t="str">
-        <x:v>Approved candidate</x:v>
-      </x:c>
-      <x:c r="F21" s="27" t="str">
-        <x:v>Each dependency change</x:v>
-      </x:c>
-      <x:c r="G21" s="27" t="str">
-        <x:v>2026-10-05</x:v>
-      </x:c>
-      <x:c r="H21" s="27" t="str">
-        <x:v>DEP-001</x:v>
+      <x:c r="G20" s="27" t="str">
+        <x:v>2026-10-04</x:v>
+      </x:c>
+      <x:c r="H20" s="27" t="str">
+        <x:v>SEC-001 OPS-003</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E21">
+  <x:conditionalFormatting sqref="E6:E20">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -1936,7 +1899,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94ee19de0e1f4528"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3389fabded664992"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2019,7 +1982,7 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>Align authentication with Zoho SSO and multi-identifier login policy</x:v>
+        <x:v>Enforce administrator MFA and production provider policy</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str">
         <x:v>Public beta safety</x:v>
@@ -2031,26 +1994,26 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F6" s="25" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Product owner</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
-        <x:v>Administrators use Zoho SSO; existing users may use Zoho SSO or username/email/mobile plus password; OTP is verification/recovery only; unsafe public provider combinations fail startup</x:v>
+        <x:v>Admin cannot use privileged access without MFA; unsafe production provider combinations fail startup</x:v>
       </x:c>
       <x:c r="J6" s="25" t="str">
-        <x:v>Production plan Task 1A and user authentication decision</x:v>
+        <x:v>Production plan Task 1A</x:v>
       </x:c>
       <x:c r="K6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
       </x:c>
       <x:c r="M6" s="28" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -2109,10 +2072,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str"/>
       <x:c r="I8" s="26" t="str">
@@ -2124,9 +2087,11 @@
       <x:c r="K8" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/8</x:v>
       </x:c>
-      <x:c r="L8" s="26" t="str"/>
+      <x:c r="L8" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+      </x:c>
       <x:c r="M8" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -2183,14 +2148,14 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F10" s="26" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Unassigned</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str"/>
       <x:c r="I10" s="26" t="str">
-        <x:v>No unaccepted critical/high runtime advisory; CI blocks regressions; explicitly documented no-fix build-tool exceptions remain narrow and reviewable</x:v>
+        <x:v>No unaccepted critical/high production advisory; CI blocks regression</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
         <x:v>Production plan Task 1E</x:v>
@@ -2198,11 +2163,9 @@
       <x:c r="K10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/10</x:v>
       </x:c>
-      <x:c r="L10" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
-      </x:c>
+      <x:c r="L10" s="26" t="str"/>
       <x:c r="M10" s="29" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -2561,7 +2524,7 @@
         <x:v>AUTH-001</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Add scoped administrator fresh-authentication step-up</x:v>
+        <x:v>Add scoped administrator MFA step-up</x:v>
       </x:c>
       <x:c r="C20" s="26" t="str">
         <x:v>Migration control</x:v>
@@ -2582,17 +2545,17 @@
         <x:v>SEC-001,CFG-001</x:v>
       </x:c>
       <x:c r="I20" s="26" t="str">
-        <x:v>Fresh Zoho reauthentication issues a five-minute single-use action-scoped token for migration start; application TOTP is a documented fallback only</x:v>
+        <x:v>Five-minute single-use scoped token protects migration start</x:v>
       </x:c>
       <x:c r="J20" s="26" t="str">
-        <x:v>Production plan Task 9 and user authentication decision</x:v>
+        <x:v>Production plan Task 9</x:v>
       </x:c>
       <x:c r="K20" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/20</x:v>
       </x:c>
       <x:c r="L20" s="26" t="str"/>
       <x:c r="M20" s="29" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -3218,93 +3181,52 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
-      <x:c r="A37" s="26" t="str">
+      <x:c r="A37" s="27" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B37" s="26" t="str">
+      <x:c r="B37" s="27" t="str">
         <x:v>Establish SDLC knowledge and tracking system</x:v>
       </x:c>
-      <x:c r="C37" s="26" t="str">
+      <x:c r="C37" s="27" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="D37" s="26" t="str">
+      <x:c r="D37" s="27" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="E37" s="26" t="str">
+      <x:c r="E37" s="27" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F37" s="26" t="str">
+      <x:c r="F37" s="27" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G37" s="26" t="str">
+      <x:c r="G37" s="27" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H37" s="26" t="str"/>
-      <x:c r="I37" s="26" t="str">
+      <x:c r="H37" s="27" t="str"/>
+      <x:c r="I37" s="27" t="str">
         <x:v>Markdown CSV Excel issues PR protocol and Obsidian index are linked and verified</x:v>
       </x:c>
-      <x:c r="J37" s="26" t="str">
+      <x:c r="J37" s="27" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K37" s="26" t="str">
+      <x:c r="K37" s="27" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/37</x:v>
       </x:c>
-      <x:c r="L37" s="26" t="str">
+      <x:c r="L37" s="27" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
-      <x:c r="M37" s="29" t="str">
+      <x:c r="M37" s="30" t="str">
         <x:v>2026-10-04</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="30" customHeight="1">
-      <x:c r="A38" s="27" t="str">
-        <x:v>GOV-003</x:v>
-      </x:c>
-      <x:c r="B38" s="27" t="str">
-        <x:v>Reconcile authentication and dependency tracking</x:v>
-      </x:c>
-      <x:c r="C38" s="27" t="str">
-        <x:v>Governance</x:v>
-      </x:c>
-      <x:c r="D38" s="27" t="str">
-        <x:v>Governance</x:v>
-      </x:c>
-      <x:c r="E38" s="27" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="F38" s="27" t="str">
-        <x:v>PR Open</x:v>
-      </x:c>
-      <x:c r="G38" s="27" t="str">
-        <x:v>Codex</x:v>
-      </x:c>
-      <x:c r="H38" s="27" t="str">
-        <x:v>SEC-001,DEP-001</x:v>
-      </x:c>
-      <x:c r="I38" s="27" t="str">
-        <x:v>Canonical registers workbook and operating guidance match the implemented authentication policy and dependency evidence</x:v>
-      </x:c>
-      <x:c r="J38" s="27" t="str">
-        <x:v>User request</x:v>
-      </x:c>
-      <x:c r="K38" s="27" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/60</x:v>
-      </x:c>
-      <x:c r="L38" s="27" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
-      </x:c>
-      <x:c r="M38" s="30" t="str">
-        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E38">
+  <x:conditionalFormatting sqref="E6:E37">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F38">
+  <x:conditionalFormatting sqref="F6:F37">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3313,7 +3235,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2436191cdb94469d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43f025b6eb504a38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3759,117 +3681,25 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="26" t="str">
+      <x:c r="A23" s="27" t="str">
         <x:v>REQ-REV-001</x:v>
       </x:c>
-      <x:c r="B23" s="26" t="str">
+      <x:c r="B23" s="27" t="str">
         <x:v>AWS migration readiness reports INR 1.2M target and INR 1.5M preferred monthly net revenue</x:v>
       </x:c>
-      <x:c r="C23" s="26" t="str">
+      <x:c r="C23" s="27" t="str">
         <x:v>Migration design</x:v>
       </x:c>
-      <x:c r="D23" s="26" t="str">
+      <x:c r="D23" s="27" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="E23" s="26" t="str">
+      <x:c r="E23" s="27" t="str">
         <x:v>Admin readiness UI test</x:v>
       </x:c>
-      <x:c r="F23" s="26" t="str">
+      <x:c r="F23" s="27" t="str">
         <x:v>UI-001</x:v>
       </x:c>
-      <x:c r="G23" s="26" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="26" t="str">
-        <x:v>REQ-AUTH-001</x:v>
-      </x:c>
-      <x:c r="B24" s="26" t="str">
-        <x:v>Administrators authenticate through Zoho SSO and do not require routine application TOTP</x:v>
-      </x:c>
-      <x:c r="C24" s="26" t="str">
-        <x:v>User direction</x:v>
-      </x:c>
-      <x:c r="D24" s="26" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="E24" s="26" t="str">
-        <x:v>Authentication integration tests and controlled Zoho sign-in evidence</x:v>
-      </x:c>
-      <x:c r="F24" s="26" t="str">
-        <x:v>SEC-001</x:v>
-      </x:c>
-      <x:c r="G24" s="26" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="30" customHeight="1">
-      <x:c r="A25" s="26" t="str">
-        <x:v>REQ-AUTH-002</x:v>
-      </x:c>
-      <x:c r="B25" s="26" t="str">
-        <x:v>Existing users may sign in with Zoho SSO or username email or mobile plus password and any valid email provider is accepted</x:v>
-      </x:c>
-      <x:c r="C25" s="26" t="str">
-        <x:v>User direction</x:v>
-      </x:c>
-      <x:c r="D25" s="26" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="E25" s="26" t="str">
-        <x:v>Backend frontend mobile and Playwright authentication tests</x:v>
-      </x:c>
-      <x:c r="F25" s="26" t="str">
-        <x:v>SEC-001</x:v>
-      </x:c>
-      <x:c r="G25" s="26" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="30" customHeight="1">
-      <x:c r="A26" s="26" t="str">
-        <x:v>REQ-AUTH-003</x:v>
-      </x:c>
-      <x:c r="B26" s="26" t="str">
-        <x:v>OTP is used only for signup/contact verification and password recovery and never as passwordless login</x:v>
-      </x:c>
-      <x:c r="C26" s="26" t="str">
-        <x:v>User direction</x:v>
-      </x:c>
-      <x:c r="D26" s="26" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="E26" s="26" t="str">
-        <x:v>Route inventory and authentication tests</x:v>
-      </x:c>
-      <x:c r="F26" s="26" t="str">
-        <x:v>SEC-001</x:v>
-      </x:c>
-      <x:c r="G26" s="26" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="27" t="str">
-        <x:v>REQ-AUTH-004</x:v>
-      </x:c>
-      <x:c r="B27" s="27" t="str">
-        <x:v>Zoho domain DNS sender mailbox SMTP application password and production OAuth callback are configured only at the final deployment gate</x:v>
-      </x:c>
-      <x:c r="C27" s="27" t="str">
-        <x:v>User direction</x:v>
-      </x:c>
-      <x:c r="D27" s="27" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="E27" s="27" t="str">
-        <x:v>Final release checklist and controlled delivery/SSO evidence</x:v>
-      </x:c>
-      <x:c r="F27" s="27" t="str">
-        <x:v>SEC-001,REL-001</x:v>
-      </x:c>
-      <x:c r="G27" s="27" t="str">
+      <x:c r="G23" s="27" t="str">
         <x:v>Approved</x:v>
       </x:c>
     </x:row>
@@ -3877,10 +3707,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D27">
+  <x:conditionalFormatting sqref="D6:D23">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G6:G27">
+  <x:conditionalFormatting sqref="G6:G23">
     <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Blocked"/>
@@ -3889,7 +3719,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra874fdfd64b54aff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf20a7dccdbee4e1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4196,13 +4026,36 @@
         <x:v>SYNC-002</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>QA-OPS-001</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>Replica safety</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41ec7c27333f406c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd82849163b854701"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4595,71 +4448,42 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="26" t="str">
+      <x:c r="A18" s="27" t="str">
         <x:v>RISK-013</x:v>
       </x:c>
-      <x:c r="B18" s="26" t="str">
-        <x:v>Public deployment tier is enabled before Zoho SSO and administrator recovery are proven</x:v>
-      </x:c>
-      <x:c r="C18" s="26" t="str">
+      <x:c r="B18" s="27" t="str">
+        <x:v>Public deployment tier is enabled before every administrator enrols MFA</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D18" s="26" t="str">
+      <x:c r="D18" s="27" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E18" s="26" t="str">
+      <x:c r="E18" s="27" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F18" s="26" t="str">
-        <x:v>Verify exact OAuth client callback administrator matching-email login Zoho-account MFA and a documented recovery owner in restricted staging before public-beta</x:v>
-      </x:c>
-      <x:c r="G18" s="26" t="str">
+      <x:c r="F18" s="27" t="str">
+        <x:v>Enrol and verify each administrator in restricted staging before selecting public-beta; keep a documented recovery owner</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H18" s="26" t="str">
+      <x:c r="H18" s="27" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="I18" s="26" t="str">
-        <x:v>SEC-001 PR 58 implements Zoho-only administrator login; production Zoho configuration is intentionally deferred to the final gate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="27" t="str">
-        <x:v>RISK-014</x:v>
-      </x:c>
-      <x:c r="B19" s="27" t="str">
-        <x:v>Framework and mobile build-tool dependency advisories remain after runtime remediation</x:v>
-      </x:c>
-      <x:c r="C19" s="27" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="D19" s="27" t="str">
-        <x:v>Possible</x:v>
-      </x:c>
-      <x:c r="E19" s="27" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="F19" s="27" t="str">
-        <x:v>Block new critical/high runtime advisories; allow only four exact no-fix Expo advisory IDs; schedule Nest major migration and review exceptions each release</x:v>
-      </x:c>
-      <x:c r="G19" s="27" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="H19" s="27" t="str">
-        <x:v>Mitigated</x:v>
-      </x:c>
-      <x:c r="I19" s="27" t="str">
-        <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
+      <x:c r="I18" s="27" t="str">
+        <x:v>SEC-001 PR 56 rejects unenrolled login and existing sessions; staged enrollment evidence still required</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E19">
+  <x:conditionalFormatting sqref="E6:E18">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H19">
+  <x:conditionalFormatting sqref="H6:H18">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -4668,7 +4492,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d01fdfe08834c0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7dd2ffee5644c37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4899,16 +4723,16 @@
         <x:v>ACC-007</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>Zoho identity and operational email</x:v>
+        <x:v>Operational email</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>OAuth application exact callback domain mailbox DNS authentication reports and SMTP app-password rotation</x:v>
+        <x:v>Zoho domain mailbox DNS authentication reports and app-password rotation</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>Zoho OAuth and SMTP identities</x:v>
+        <x:v>Zoho SMTP identity</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
         <x:v>GitHub Railway or Kubernetes secrets</x:v>
@@ -4918,7 +4742,7 @@
       </x:c>
       <x:c r="H12" s="29" t="str"/>
       <x:c r="I12" s="26" t="str">
-        <x:v>Configure only at final deployment; protect the Zoho owner with Zoho MFA and retain controlled SSO/mail evidence</x:v>
+        <x:v>Low-volume beta only; owner must configure domain MFA app password and first delivery evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -4983,7 +4807,7 @@
         <x:v>WOW-MD source review</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
-        <x:v>Repository contents read for scheduled change reports</x:v>
+        <x:v>Private repository contents read for scheduled change reports</x:v>
       </x:c>
       <x:c r="D15" s="27" t="str">
         <x:v>RohithTadiparti</x:v>
@@ -4995,11 +4819,11 @@
         <x:v>Production GitHub Actions secret</x:v>
       </x:c>
       <x:c r="G15" s="27" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="H15" s="30" t="str"/>
       <x:c r="I15" s="27" t="str">
-        <x:v>Not technically required while WOW-MD is public; create before returning it private so the private-ready workflow keeps working; scope only to WOW-MD Contents read and rotate within 90 days</x:v>
+        <x:v>Scope only to WOW-MD Contents read; rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5015,7 +4839,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b4e6968d40241f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c389c4c429e4851"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5354,7 +5178,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R615eff909ab24642"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e806a33f4514bea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5527,7 +5351,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71cabc95d21f49f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fed96a9bf9e474e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5680,150 +5504,112 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>codex/sec-001-sso-login-policy</x:v>
+        <x:v>codex/sec-001-admin-mfa-provider-policy</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>29537ee</x:v>
+        <x:v>57e13d0</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>3eaa03c</x:v>
+        <x:v>fad2ef5</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>WOW-MD PR 38 head f685774</x:v>
+        <x:v>WOW-MD PR 37 merged as b28c334; application mirror commit 1482d83</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Backend typecheck/lint and 71 focused auth/config tests pass; frontend typecheck and 173 tests pass; mobile typecheck passes; CodeQL security gate passes after refresh cookies were sealed and session hashes moved to memory-hard derivation; remaining protected CI jobs are recorded on the PR</x:v>
+        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance and synchronization 19/19; protected production and source CI passed including retained 30-day CodeQL SARIF</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
-        <x:v>At the final release gate configure exact Zoho OAuth client/callback domain SPF DKIM DMARC sender mailbox and SMTP application password; then run controlled admin/non-admin SSO and email tests</x:v>
+        <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
       </x:c>
       <x:c r="I8" s="26" t="str">
-        <x:v>Restore the prior image/config and disable Zoho SSO; do not enable passwordless OTP or log-based mail in public tier</x:v>
+        <x:v>Restore previous image/config; do not fall back to log/mock in a public tier; pause email-dependent workflows</x:v>
       </x:c>
       <x:c r="J8" s="26" t="str">
-        <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred to the final release gate</x:v>
+        <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
       </x:c>
       <x:c r="K8" s="26" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="26" t="str">
+      <x:c r="A9" s="27" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="B9" s="26" t="str">
+      <x:c r="B9" s="27" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
       </x:c>
-      <x:c r="C9" s="26" t="str">
+      <x:c r="C9" s="27" t="str">
         <x:v>codex/sync-002-gated-source-review</x:v>
       </x:c>
-      <x:c r="D9" s="26" t="str">
+      <x:c r="D9" s="27" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E9" s="26" t="str">
+      <x:c r="E9" s="27" t="str">
         <x:v>422cbc4</x:v>
       </x:c>
-      <x:c r="F9" s="26" t="str">
+      <x:c r="F9" s="27" t="str">
         <x:v>07218b4..de7d8dd local review only</x:v>
       </x:c>
-      <x:c r="G9" s="26" t="str">
+      <x:c r="G9" s="27" t="str">
         <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
       </x:c>
-      <x:c r="H9" s="26" t="str">
+      <x:c r="H9" s="27" t="str">
         <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
       </x:c>
-      <x:c r="I9" s="26" t="str">
+      <x:c r="I9" s="27" t="str">
         <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
       </x:c>
-      <x:c r="J9" s="26" t="str">
+      <x:c r="J9" s="27" t="str">
         <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
       </x:c>
-      <x:c r="K9" s="26" t="str">
+      <x:c r="K9" s="27" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="L9" s="29" t="str">
+      <x:c r="L9" s="30" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="26" t="str">
-        <x:v>DEP-001</x:v>
-      </x:c>
-      <x:c r="B10" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
-      </x:c>
-      <x:c r="C10" s="26" t="str">
-        <x:v>codex/dep-001-dependency-remediation</x:v>
-      </x:c>
-      <x:c r="D10" s="26" t="str">
-        <x:v>29537ee</x:v>
-      </x:c>
-      <x:c r="E10" s="26" t="str">
-        <x:v>1ecbfdf</x:v>
-      </x:c>
-      <x:c r="F10" s="26" t="str">
-        <x:v>WOW-MD PR 39 head d8ef995</x:v>
-      </x:c>
-      <x:c r="G10" s="26" t="str">
-        <x:v>Backend clean install typecheck lint build and 792 tests pass with 9 skipped; frontend clean install typecheck 173 tests build and 10 Playwright flows pass; runtime audits: backend 0 critical/0 high frontend 0; exact-ID mobile gate passes; production and source protected CI pass</x:v>
-      </x:c>
-      <x:c r="H10" s="26" t="str">
-        <x:v>No deployment before review and merge; after merge let GitHub rescan manifests and confirm alert counts and audit gates on main</x:v>
-      </x:c>
-      <x:c r="I10" s="26" t="str">
-        <x:v>Revert PR 59; restore prior lockfiles and packages; retain the audit report for comparison</x:v>
-      </x:c>
-      <x:c r="J10" s="26" t="str">
-        <x:v>Backend moderate/low build-tool advisories and four exact no-fix Expo advisory roots remain; forced NestJS 12 and Expo downgrades were tested and rejected as unsafe</x:v>
-      </x:c>
-      <x:c r="K10" s="26" t="str">
-        <x:v>PR Open</x:v>
-      </x:c>
-      <x:c r="L10" s="29" t="str">
-        <x:v>2026-10-05</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="27" t="str">
-        <x:v>GOV-003</x:v>
-      </x:c>
-      <x:c r="B11" s="27" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
-      </x:c>
-      <x:c r="C11" s="27" t="str">
-        <x:v>codex/gov-003-auth-dependency-tracking</x:v>
-      </x:c>
-      <x:c r="D11" s="27" t="str">
-        <x:v>29537ee</x:v>
-      </x:c>
-      <x:c r="E11" s="27" t="str">
-        <x:v>1235cd3</x:v>
-      </x:c>
-      <x:c r="F11" s="27" t="str">
-        <x:v>SEC-001 PR 58 and DEP-001 PR 59 evidence only</x:v>
-      </x:c>
-      <x:c r="G11" s="27" t="str">
-        <x:v>Register validator workbook regeneration and formula-error scan pass; dashboard visually reviewed</x:v>
-      </x:c>
-      <x:c r="H11" s="27" t="str">
-        <x:v>Governance and documentation only; no application or hosting deployment</x:v>
-      </x:c>
-      <x:c r="I11" s="27" t="str">
-        <x:v>Revert PR 61; implementation PRs and their evidence remain unchanged</x:v>
-      </x:c>
-      <x:c r="J11" s="27" t="str">
-        <x:v>Implementation PRs still require review/merge and GitHub rescan; Zoho live configuration remains a final release gate</x:v>
-      </x:c>
-      <x:c r="K11" s="27" t="str">
-        <x:v>PR Open</x:v>
-      </x:c>
-      <x:c r="L11" s="30" t="str">
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>codex/ops-001-replicated-jobs</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>57e13d0</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>090d236</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>WOW-MD commit a06067a; PR 42</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Focused replica tests 7 of 7; backend full suite 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Deploy normally after approval; verify two replicas produce one owner and one skipped invocation for outbox and payout/reminder jobs</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>Revert PR 64 and redeploy; no database or configuration rollback</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>Outbox delivery remains at-least-once across a crash after an external side effect; Kafka consumers must honor the outbox UUID idempotency key</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>Ready for Review</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
@@ -5831,7 +5617,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K11">
+  <x:conditionalFormatting sqref="K6:K9">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -5840,7 +5626,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3652ba24d5b84156"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b042648f28498e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
OBS-001: implement correlated secret-safe observability (#69)
* feat(obs): correlate and redact service logs

* docs(obs): record OBS-001 review handoff

* fix(logging): use valid Pino cookie redaction path

* ci: refresh mirror gate metadata

* docs(obs): link replacement production PR

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raeedae5ff209418d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R40b455cf76954eb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R5023dffb9e4448ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R2db2c6f1609549d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rdf0ccb98e6224d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R42965f3834b04aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R1a1b0d2dd00d4ca2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re691660970d54e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra4fa0222c47c4087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R8bfac8c765c04c81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb1a81da2f2014435"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Ra7461bf4dcfb4305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R0e96e3e2600e4214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R98da020119b44f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R8aa33dab71ba45c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R92f26e4c0b364480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R26c31c2a0f784e41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6f685f0304024924"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R1ee073186a0d4a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7e6fe2172f234a3c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -830,7 +830,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Recbdb8875ecc49f8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8b785583de834eb6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1439,7 +1439,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11dd2df34d0a44bb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44d35715b66648ca"/>
 </x:worksheet>
 </file>
 
@@ -1899,7 +1899,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3389fabded664992"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d61ae7eeb044cf6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2072,10 +2072,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Unassigned</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str"/>
       <x:c r="I8" s="26" t="str">
@@ -2087,11 +2087,9 @@
       <x:c r="K8" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/8</x:v>
       </x:c>
-      <x:c r="L8" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
-      </x:c>
+      <x:c r="L8" s="26" t="str"/>
       <x:c r="M8" s="29" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-04</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -2185,10 +2183,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F11" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H11" s="26" t="str">
         <x:v>SEC-003</x:v>
@@ -2202,9 +2200,11 @@
       <x:c r="K11" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/11</x:v>
       </x:c>
-      <x:c r="L11" s="26" t="str"/>
+      <x:c r="L11" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/65</x:v>
+      </x:c>
       <x:c r="M11" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
@@ -3235,7 +3235,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43f025b6eb504a38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13810d1b976a4191"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3719,7 +3719,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf20a7dccdbee4e1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R718b81cadaf445d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4028,25 +4028,25 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>QA-OPS-001</x:v>
+        <x:v>QA-OBS-001</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>Replica safety</x:v>
+        <x:v>Observability</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
+        <x:v>Request correlation redaction provider logs QA capture audit failures payout sweep and nginx JSON</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
+        <x:v>OBS-001 PR 65 and WOW-MD PR 43</x:v>
       </x:c>
       <x:c r="E17" t="str">
-        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
+        <x:v>Focused 20 of 20; full backend 812 passed 9 skipped; typecheck lint nginx contract image build and syntax passed</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
+        <x:v>Deploy after SEC-003 and verify live response/log correlation with capture disabled</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>OPS-001</x:v>
+        <x:v>OBS-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4055,7 +4055,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd82849163b854701"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8285d63d48484bc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4492,7 +4492,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7dd2ffee5644c37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94914057e8ce466d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4839,7 +4839,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c389c4c429e4851"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd40f85e1aac467e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5178,7 +5178,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e806a33f4514bea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf86f2bf9b8614332"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5351,7 +5351,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fed96a9bf9e474e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re46edf7e1d584ba5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5577,34 +5577,34 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>OPS-001</x:v>
+        <x:v>OBS-001</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/65</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>codex/ops-001-replicated-jobs</x:v>
+        <x:v>codex/obs-001-backend-observability</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>57e13d0</x:v>
+        <x:v>29537ee</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>090d236</x:v>
+        <x:v>48c1351</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>WOW-MD commit a06067a; PR 42</x:v>
+        <x:v>WOW-MD commit 69c2aea; PR 43</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>Focused replica tests 7 of 7; backend full suite 797 passed 9 skipped; typecheck and lint passed</x:v>
+        <x:v>Focused observability 20 of 20; backend full suite 812 passed 9 skipped; typecheck lint nginx contract frontend image build and nginx syntax passed</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>Deploy normally after approval; verify two replicas produce one owner and one skipped invocation for outbox and payout/reminder jobs</x:v>
+        <x:v>Merge SEC-003 first then rebase; set RELEASE; keep QA capture disabled; confirm a live request ID matches response backend and nginx logs</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>Revert PR 64 and redeploy; no database or configuration rollback</x:v>
+        <x:v>Revert PR 65 and redeploy; remove optional observability variables; no database rollback</x:v>
       </x:c>
       <x:c r="J10" t="str">
-        <x:v>Outbox delivery remains at-least-once across a crash after an external side effect; Kafka consumers must honor the outbox UUID idempotency key</x:v>
+        <x:v>OBS-002 client error intake and OBS-003 Loki Vector host files 30-day retention remain open; live provider correlation smoke remains</x:v>
       </x:c>
       <x:c r="K10" t="str">
         <x:v>Ready for Review</x:v>
@@ -5626,7 +5626,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b042648f28498e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998f60580a2a4686"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: reconcile merged production tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb1a81da2f2014435"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Ra7461bf4dcfb4305"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R0e96e3e2600e4214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R98da020119b44f1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R8aa33dab71ba45c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R92f26e4c0b364480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R26c31c2a0f784e41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6f685f0304024924"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R1ee073186a0d4a52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7e6fe2172f234a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R30f34b6cf68a479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R29c368d037af4a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R518005db4602425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R328df1b9cecb476a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rf59eb498d24d447e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R41c7ecedbd834286"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R18432713b03e431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rae971aa8878a4382"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R37759bbb55db4b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R43f2d00d33eb4454"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,8 +68,23 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF16794A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF7A4B00"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFB42318"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +94,81 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -124,7 +214,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="76">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -213,6 +303,102 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -830,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8b785583de834eb6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R061f15398a4b4fc4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -840,7 +1026,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -960,7 +1146,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1207,7 +1393,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-05. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-06. Reconciled to canonical registers and final merged PR/issue state.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1235,20 +1421,20 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1256,7 +1442,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1290,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1298,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1311,7 +1497,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H9" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1319,7 +1505,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
@@ -1332,7 +1518,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1340,7 +1526,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1439,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44d35715b66648ca"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9e0768e4c7348f9"/>
 </x:worksheet>
 </file>
 
@@ -1899,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d61ae7eeb044cf6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2982b85399ee43db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1982,7 +2168,7 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>Enforce administrator MFA and production provider policy</x:v>
+        <x:v>Align authentication with Zoho SSO and multi-identifier login policy</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str">
         <x:v>Public beta safety</x:v>
@@ -1993,27 +2179,27 @@
       <x:c r="E6" s="25" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F6" s="25" t="str">
-        <x:v>Blocked</x:v>
+      <x:c r="F6" s="70" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
-        <x:v>Admin cannot use privileged access without MFA; unsafe production provider combinations fail startup</x:v>
+        <x:v>Administrators use Zoho SSO; existing users may use Zoho SSO or username/email/mobile plus password; OTP is verification/recovery only; unsafe public provider combinations fail startup</x:v>
       </x:c>
       <x:c r="J6" s="25" t="str">
-        <x:v>Production plan Task 1A</x:v>
+        <x:v>Production plan Task 1A and user authentication decision</x:v>
       </x:c>
       <x:c r="K6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
       </x:c>
       <x:c r="M6" s="28" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -2032,11 +2218,11 @@
       <x:c r="E7" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F7" s="26" t="str">
-        <x:v>Open</x:v>
+      <x:c r="F7" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G7" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H7" s="26" t="str">
         <x:v>SEC-001</x:v>
@@ -2050,9 +2236,11 @@
       <x:c r="K7" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/7</x:v>
       </x:c>
-      <x:c r="L7" s="26" t="str"/>
+      <x:c r="L7" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/62</x:v>
+      </x:c>
       <x:c r="M7" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -2071,11 +2259,11 @@
       <x:c r="E8" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F8" s="26" t="str">
-        <x:v>Open</x:v>
+      <x:c r="F8" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str"/>
       <x:c r="I8" s="26" t="str">
@@ -2087,9 +2275,11 @@
       <x:c r="K8" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/8</x:v>
       </x:c>
-      <x:c r="L8" s="26" t="str"/>
+      <x:c r="L8" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+      </x:c>
       <x:c r="M8" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -2108,11 +2298,11 @@
       <x:c r="E9" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F9" s="26" t="str">
-        <x:v>Open</x:v>
+      <x:c r="F9" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G9" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H9" s="26" t="str"/>
       <x:c r="I9" s="26" t="str">
@@ -2124,9 +2314,11 @@
       <x:c r="K9" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/9</x:v>
       </x:c>
-      <x:c r="L9" s="26" t="str"/>
+      <x:c r="L9" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/63</x:v>
+      </x:c>
       <x:c r="M9" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -2145,15 +2337,15 @@
       <x:c r="E10" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F10" s="26" t="str">
-        <x:v>Open</x:v>
+      <x:c r="F10" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str"/>
       <x:c r="I10" s="26" t="str">
-        <x:v>No unaccepted critical/high production advisory; CI blocks regression</x:v>
+        <x:v>No unaccepted critical/high runtime advisory; CI blocks regressions; explicitly documented no-fix build-tool exceptions remain narrow and reviewable</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
         <x:v>Production plan Task 1E</x:v>
@@ -2161,9 +2353,11 @@
       <x:c r="K10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/10</x:v>
       </x:c>
-      <x:c r="L10" s="26" t="str"/>
+      <x:c r="L10" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
+      </x:c>
       <x:c r="M10" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -2182,8 +2376,8 @@
       <x:c r="E11" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F11" s="26" t="str">
-        <x:v>PR Open</x:v>
+      <x:c r="F11" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
         <x:v>Codex</x:v>
@@ -2201,7 +2395,7 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/11</x:v>
       </x:c>
       <x:c r="L11" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/65</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/69</x:v>
       </x:c>
       <x:c r="M11" s="29" t="str">
         <x:v>2026-10-05</x:v>
@@ -2223,7 +2417,7 @@
       <x:c r="E12" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F12" s="26" t="str">
+      <x:c r="F12" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G12" s="26" t="str">
@@ -2262,7 +2456,7 @@
       <x:c r="E13" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F13" s="26" t="str">
+      <x:c r="F13" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
@@ -2301,7 +2495,7 @@
       <x:c r="E14" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F14" s="26" t="str">
+      <x:c r="F14" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
@@ -2340,7 +2534,7 @@
       <x:c r="E15" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F15" s="26" t="str">
+      <x:c r="F15" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G15" s="26" t="str">
@@ -2379,7 +2573,7 @@
       <x:c r="E16" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F16" s="26" t="str">
+      <x:c r="F16" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G16" s="26" t="str">
@@ -2418,7 +2612,7 @@
       <x:c r="E17" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F17" s="26" t="str">
+      <x:c r="F17" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G17" s="26" t="str">
@@ -2457,7 +2651,7 @@
       <x:c r="E18" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F18" s="26" t="str">
+      <x:c r="F18" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G18" s="26" t="str">
@@ -2496,7 +2690,7 @@
       <x:c r="E19" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F19" s="26" t="str">
+      <x:c r="F19" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G19" s="26" t="str">
@@ -2524,7 +2718,7 @@
         <x:v>AUTH-001</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Add scoped administrator MFA step-up</x:v>
+        <x:v>Add scoped administrator fresh-authentication step-up</x:v>
       </x:c>
       <x:c r="C20" s="26" t="str">
         <x:v>Migration control</x:v>
@@ -2535,7 +2729,7 @@
       <x:c r="E20" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F20" s="26" t="str">
+      <x:c r="F20" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G20" s="26" t="str">
@@ -2545,17 +2739,17 @@
         <x:v>SEC-001,CFG-001</x:v>
       </x:c>
       <x:c r="I20" s="26" t="str">
-        <x:v>Five-minute single-use scoped token protects migration start</x:v>
+        <x:v>Fresh Zoho reauthentication issues a five-minute single-use action-scoped token for migration start; application TOTP is a documented fallback only</x:v>
       </x:c>
       <x:c r="J20" s="26" t="str">
-        <x:v>Production plan Task 9</x:v>
+        <x:v>Production plan Task 9 and user authentication decision</x:v>
       </x:c>
       <x:c r="K20" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/20</x:v>
       </x:c>
       <x:c r="L20" s="26" t="str"/>
       <x:c r="M20" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -2574,7 +2768,7 @@
       <x:c r="E21" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F21" s="26" t="str">
+      <x:c r="F21" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G21" s="26" t="str">
@@ -2613,7 +2807,7 @@
       <x:c r="E22" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F22" s="26" t="str">
+      <x:c r="F22" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G22" s="26" t="str">
@@ -2652,7 +2846,7 @@
       <x:c r="E23" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F23" s="26" t="str">
+      <x:c r="F23" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G23" s="26" t="str">
@@ -2691,7 +2885,7 @@
       <x:c r="E24" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F24" s="26" t="str">
+      <x:c r="F24" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G24" s="26" t="str">
@@ -2730,7 +2924,7 @@
       <x:c r="E25" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F25" s="26" t="str">
+      <x:c r="F25" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G25" s="26" t="str">
@@ -2769,7 +2963,7 @@
       <x:c r="E26" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F26" s="26" t="str">
+      <x:c r="F26" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G26" s="26" t="str">
@@ -2808,7 +3002,7 @@
       <x:c r="E27" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F27" s="26" t="str">
+      <x:c r="F27" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G27" s="26" t="str">
@@ -2847,7 +3041,7 @@
       <x:c r="E28" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F28" s="26" t="str">
+      <x:c r="F28" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G28" s="26" t="str">
@@ -2886,7 +3080,7 @@
       <x:c r="E29" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F29" s="26" t="str">
+      <x:c r="F29" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G29" s="26" t="str">
@@ -2925,7 +3119,7 @@
       <x:c r="E30" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F30" s="26" t="str">
+      <x:c r="F30" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G30" s="26" t="str">
@@ -2964,7 +3158,7 @@
       <x:c r="E31" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F31" s="26" t="str">
+      <x:c r="F31" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G31" s="26" t="str">
@@ -3001,7 +3195,7 @@
       <x:c r="E32" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F32" s="26" t="str">
+      <x:c r="F32" s="73" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G32" s="26" t="str">
@@ -3042,7 +3236,7 @@
       <x:c r="E33" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F33" s="26" t="str">
+      <x:c r="F33" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G33" s="26" t="str">
@@ -3079,7 +3273,7 @@
       <x:c r="E34" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F34" s="26" t="str">
+      <x:c r="F34" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G34" s="26" t="str">
@@ -3118,7 +3312,7 @@
       <x:c r="E35" s="26" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F35" s="26" t="str">
+      <x:c r="F35" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G35" s="26" t="str">
@@ -3157,7 +3351,7 @@
       <x:c r="E36" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F36" s="26" t="str">
+      <x:c r="F36" s="71" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G36" s="26" t="str">
@@ -3177,7 +3371,7 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
       </x:c>
       <x:c r="M36" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
@@ -3196,7 +3390,7 @@
       <x:c r="E37" s="27" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F37" s="27" t="str">
+      <x:c r="F37" s="74" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G37" s="27" t="str">
@@ -3216,8 +3410,529 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
       <x:c r="M37" s="30" t="str">
-        <x:v>2026-10-04</x:v>
-      </x:c>
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>GOV-003</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>Reconcile authentication and dependency tracking</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F38" s="75" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>SEC-001,DEP-001</x:v>
+      </x:c>
+      <x:c r="I38" t="str">
+        <x:v>Canonical registers workbook and operating guidance match the implemented authentication policy and dependency evidence</x:v>
+      </x:c>
+      <x:c r="J38" t="str">
+        <x:v>User request</x:v>
+      </x:c>
+      <x:c r="K38" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/60</x:v>
+      </x:c>
+      <x:c r="L38" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
+      </x:c>
+      <x:c r="M38" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39"/>
+      <x:c r="B39"/>
+      <x:c r="C39"/>
+      <x:c r="D39"/>
+      <x:c r="E39"/>
+      <x:c r="F39"/>
+      <x:c r="G39"/>
+      <x:c r="H39"/>
+      <x:c r="I39"/>
+      <x:c r="J39"/>
+      <x:c r="K39"/>
+      <x:c r="L39"/>
+      <x:c r="M39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40"/>
+      <x:c r="B40"/>
+      <x:c r="C40"/>
+      <x:c r="D40"/>
+      <x:c r="E40"/>
+      <x:c r="F40"/>
+      <x:c r="G40"/>
+      <x:c r="H40"/>
+      <x:c r="I40"/>
+      <x:c r="J40"/>
+      <x:c r="K40"/>
+      <x:c r="L40"/>
+      <x:c r="M40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41"/>
+      <x:c r="B41"/>
+      <x:c r="C41"/>
+      <x:c r="D41"/>
+      <x:c r="E41"/>
+      <x:c r="F41"/>
+      <x:c r="G41"/>
+      <x:c r="H41"/>
+      <x:c r="I41"/>
+      <x:c r="J41"/>
+      <x:c r="K41"/>
+      <x:c r="L41"/>
+      <x:c r="M41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42"/>
+      <x:c r="B42"/>
+      <x:c r="C42"/>
+      <x:c r="D42"/>
+      <x:c r="E42"/>
+      <x:c r="F42"/>
+      <x:c r="G42"/>
+      <x:c r="H42"/>
+      <x:c r="I42"/>
+      <x:c r="J42"/>
+      <x:c r="K42"/>
+      <x:c r="L42"/>
+      <x:c r="M42"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43"/>
+      <x:c r="B43"/>
+      <x:c r="C43"/>
+      <x:c r="D43"/>
+      <x:c r="E43"/>
+      <x:c r="F43"/>
+      <x:c r="G43"/>
+      <x:c r="H43"/>
+      <x:c r="I43"/>
+      <x:c r="J43"/>
+      <x:c r="K43"/>
+      <x:c r="L43"/>
+      <x:c r="M43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44"/>
+      <x:c r="B44"/>
+      <x:c r="C44"/>
+      <x:c r="D44"/>
+      <x:c r="E44"/>
+      <x:c r="F44"/>
+      <x:c r="G44"/>
+      <x:c r="H44"/>
+      <x:c r="I44"/>
+      <x:c r="J44"/>
+      <x:c r="K44"/>
+      <x:c r="L44"/>
+      <x:c r="M44"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45"/>
+      <x:c r="B45"/>
+      <x:c r="C45"/>
+      <x:c r="D45"/>
+      <x:c r="E45"/>
+      <x:c r="F45"/>
+      <x:c r="G45"/>
+      <x:c r="H45"/>
+      <x:c r="I45"/>
+      <x:c r="J45"/>
+      <x:c r="K45"/>
+      <x:c r="L45"/>
+      <x:c r="M45"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46"/>
+      <x:c r="B46"/>
+      <x:c r="C46"/>
+      <x:c r="D46"/>
+      <x:c r="E46"/>
+      <x:c r="F46"/>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
+      <x:c r="I46"/>
+      <x:c r="J46"/>
+      <x:c r="K46"/>
+      <x:c r="L46"/>
+      <x:c r="M46"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47"/>
+      <x:c r="B47"/>
+      <x:c r="C47"/>
+      <x:c r="D47"/>
+      <x:c r="E47"/>
+      <x:c r="F47"/>
+      <x:c r="G47"/>
+      <x:c r="H47"/>
+      <x:c r="I47"/>
+      <x:c r="J47"/>
+      <x:c r="K47"/>
+      <x:c r="L47"/>
+      <x:c r="M47"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48"/>
+      <x:c r="B48"/>
+      <x:c r="C48"/>
+      <x:c r="D48"/>
+      <x:c r="E48"/>
+      <x:c r="F48"/>
+      <x:c r="G48"/>
+      <x:c r="H48"/>
+      <x:c r="I48"/>
+      <x:c r="J48"/>
+      <x:c r="K48"/>
+      <x:c r="L48"/>
+      <x:c r="M48"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49"/>
+      <x:c r="B49"/>
+      <x:c r="C49"/>
+      <x:c r="D49"/>
+      <x:c r="E49"/>
+      <x:c r="F49"/>
+      <x:c r="G49"/>
+      <x:c r="H49"/>
+      <x:c r="I49"/>
+      <x:c r="J49"/>
+      <x:c r="K49"/>
+      <x:c r="L49"/>
+      <x:c r="M49"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50"/>
+      <x:c r="B50"/>
+      <x:c r="C50"/>
+      <x:c r="D50"/>
+      <x:c r="E50"/>
+      <x:c r="F50"/>
+      <x:c r="G50"/>
+      <x:c r="H50"/>
+      <x:c r="I50"/>
+      <x:c r="J50"/>
+      <x:c r="K50"/>
+      <x:c r="L50"/>
+      <x:c r="M50"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51"/>
+      <x:c r="B51"/>
+      <x:c r="C51"/>
+      <x:c r="D51"/>
+      <x:c r="E51"/>
+      <x:c r="F51"/>
+      <x:c r="G51"/>
+      <x:c r="H51"/>
+      <x:c r="I51"/>
+      <x:c r="J51"/>
+      <x:c r="K51"/>
+      <x:c r="L51"/>
+      <x:c r="M51"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52"/>
+      <x:c r="B52"/>
+      <x:c r="C52"/>
+      <x:c r="D52"/>
+      <x:c r="E52"/>
+      <x:c r="F52"/>
+      <x:c r="G52"/>
+      <x:c r="H52"/>
+      <x:c r="I52"/>
+      <x:c r="J52"/>
+      <x:c r="K52"/>
+      <x:c r="L52"/>
+      <x:c r="M52"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53"/>
+      <x:c r="B53"/>
+      <x:c r="C53"/>
+      <x:c r="D53"/>
+      <x:c r="E53"/>
+      <x:c r="F53"/>
+      <x:c r="G53"/>
+      <x:c r="H53"/>
+      <x:c r="I53"/>
+      <x:c r="J53"/>
+      <x:c r="K53"/>
+      <x:c r="L53"/>
+      <x:c r="M53"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54"/>
+      <x:c r="B54"/>
+      <x:c r="C54"/>
+      <x:c r="D54"/>
+      <x:c r="E54"/>
+      <x:c r="F54"/>
+      <x:c r="G54"/>
+      <x:c r="H54"/>
+      <x:c r="I54"/>
+      <x:c r="J54"/>
+      <x:c r="K54"/>
+      <x:c r="L54"/>
+      <x:c r="M54"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55"/>
+      <x:c r="B55"/>
+      <x:c r="C55"/>
+      <x:c r="D55"/>
+      <x:c r="E55"/>
+      <x:c r="F55"/>
+      <x:c r="G55"/>
+      <x:c r="H55"/>
+      <x:c r="I55"/>
+      <x:c r="J55"/>
+      <x:c r="K55"/>
+      <x:c r="L55"/>
+      <x:c r="M55"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56"/>
+      <x:c r="B56"/>
+      <x:c r="C56"/>
+      <x:c r="D56"/>
+      <x:c r="E56"/>
+      <x:c r="F56"/>
+      <x:c r="G56"/>
+      <x:c r="H56"/>
+      <x:c r="I56"/>
+      <x:c r="J56"/>
+      <x:c r="K56"/>
+      <x:c r="L56"/>
+      <x:c r="M56"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57"/>
+      <x:c r="B57"/>
+      <x:c r="C57"/>
+      <x:c r="D57"/>
+      <x:c r="E57"/>
+      <x:c r="F57"/>
+      <x:c r="G57"/>
+      <x:c r="H57"/>
+      <x:c r="I57"/>
+      <x:c r="J57"/>
+      <x:c r="K57"/>
+      <x:c r="L57"/>
+      <x:c r="M57"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58"/>
+      <x:c r="B58"/>
+      <x:c r="C58"/>
+      <x:c r="D58"/>
+      <x:c r="E58"/>
+      <x:c r="F58"/>
+      <x:c r="G58"/>
+      <x:c r="H58"/>
+      <x:c r="I58"/>
+      <x:c r="J58"/>
+      <x:c r="K58"/>
+      <x:c r="L58"/>
+      <x:c r="M58"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59"/>
+      <x:c r="B59"/>
+      <x:c r="C59"/>
+      <x:c r="D59"/>
+      <x:c r="E59"/>
+      <x:c r="F59"/>
+      <x:c r="G59"/>
+      <x:c r="H59"/>
+      <x:c r="I59"/>
+      <x:c r="J59"/>
+      <x:c r="K59"/>
+      <x:c r="L59"/>
+      <x:c r="M59"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60"/>
+      <x:c r="B60"/>
+      <x:c r="C60"/>
+      <x:c r="D60"/>
+      <x:c r="E60"/>
+      <x:c r="F60"/>
+      <x:c r="G60"/>
+      <x:c r="H60"/>
+      <x:c r="I60"/>
+      <x:c r="J60"/>
+      <x:c r="K60"/>
+      <x:c r="L60"/>
+      <x:c r="M60"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61"/>
+      <x:c r="B61"/>
+      <x:c r="C61"/>
+      <x:c r="D61"/>
+      <x:c r="E61"/>
+      <x:c r="F61"/>
+      <x:c r="G61"/>
+      <x:c r="H61"/>
+      <x:c r="I61"/>
+      <x:c r="J61"/>
+      <x:c r="K61"/>
+      <x:c r="L61"/>
+      <x:c r="M61"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62"/>
+      <x:c r="B62"/>
+      <x:c r="C62"/>
+      <x:c r="D62"/>
+      <x:c r="E62"/>
+      <x:c r="F62"/>
+      <x:c r="G62"/>
+      <x:c r="H62"/>
+      <x:c r="I62"/>
+      <x:c r="J62"/>
+      <x:c r="K62"/>
+      <x:c r="L62"/>
+      <x:c r="M62"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63"/>
+      <x:c r="B63"/>
+      <x:c r="C63"/>
+      <x:c r="D63"/>
+      <x:c r="E63"/>
+      <x:c r="F63"/>
+      <x:c r="G63"/>
+      <x:c r="H63"/>
+      <x:c r="I63"/>
+      <x:c r="J63"/>
+      <x:c r="K63"/>
+      <x:c r="L63"/>
+      <x:c r="M63"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64"/>
+      <x:c r="B64"/>
+      <x:c r="C64"/>
+      <x:c r="D64"/>
+      <x:c r="E64"/>
+      <x:c r="F64"/>
+      <x:c r="G64"/>
+      <x:c r="H64"/>
+      <x:c r="I64"/>
+      <x:c r="J64"/>
+      <x:c r="K64"/>
+      <x:c r="L64"/>
+      <x:c r="M64"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65"/>
+      <x:c r="B65"/>
+      <x:c r="C65"/>
+      <x:c r="D65"/>
+      <x:c r="E65"/>
+      <x:c r="F65"/>
+      <x:c r="G65"/>
+      <x:c r="H65"/>
+      <x:c r="I65"/>
+      <x:c r="J65"/>
+      <x:c r="K65"/>
+      <x:c r="L65"/>
+      <x:c r="M65"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66"/>
+      <x:c r="B66"/>
+      <x:c r="C66"/>
+      <x:c r="D66"/>
+      <x:c r="E66"/>
+      <x:c r="F66"/>
+      <x:c r="G66"/>
+      <x:c r="H66"/>
+      <x:c r="I66"/>
+      <x:c r="J66"/>
+      <x:c r="K66"/>
+      <x:c r="L66"/>
+      <x:c r="M66"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67"/>
+      <x:c r="B67"/>
+      <x:c r="C67"/>
+      <x:c r="D67"/>
+      <x:c r="E67"/>
+      <x:c r="F67"/>
+      <x:c r="G67"/>
+      <x:c r="H67"/>
+      <x:c r="I67"/>
+      <x:c r="J67"/>
+      <x:c r="K67"/>
+      <x:c r="L67"/>
+      <x:c r="M67"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68"/>
+      <x:c r="B68"/>
+      <x:c r="C68"/>
+      <x:c r="D68"/>
+      <x:c r="E68"/>
+      <x:c r="F68"/>
+      <x:c r="G68"/>
+      <x:c r="H68"/>
+      <x:c r="I68"/>
+      <x:c r="J68"/>
+      <x:c r="K68"/>
+      <x:c r="L68"/>
+      <x:c r="M68"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69"/>
+      <x:c r="B69"/>
+      <x:c r="C69"/>
+      <x:c r="D69"/>
+      <x:c r="E69"/>
+      <x:c r="F69"/>
+      <x:c r="G69"/>
+      <x:c r="H69"/>
+      <x:c r="I69"/>
+      <x:c r="J69"/>
+      <x:c r="K69"/>
+      <x:c r="L69"/>
+      <x:c r="M69"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70"/>
+      <x:c r="B70"/>
+      <x:c r="C70"/>
+      <x:c r="D70"/>
+      <x:c r="E70"/>
+      <x:c r="F70"/>
+      <x:c r="G70"/>
+      <x:c r="H70"/>
+      <x:c r="I70"/>
+      <x:c r="J70"/>
+      <x:c r="K70"/>
+      <x:c r="L70"/>
+      <x:c r="M70"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3235,7 +3950,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13810d1b976a4191"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d8ce612c81e4551"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3719,7 +4434,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R718b81cadaf445d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R305eab3893d14d36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4049,13 +4764,82 @@
         <x:v>OBS-001</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>QA-SEC-002</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>WebSocket origins tokens calls and presence authorization</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>SEC-002 PR 62 and WOW-MD PR 40</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>Focused gateways 11 passed; full backend 800 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Run staged hostile-origin and two-account WebSocket smoke</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>SEC-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>QA-SEC-003</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>HTTP headers private Swagger and migration integrity</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>SEC-003 PR 63 and WOW-MD PR 41</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>HTTP 2 passed; migration verifier 2 passed; 93 migrations verified and clean database upgrade passed; backend 794 passed 9 skipped</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Deploy and verify production headers Swagger denial and migration startup</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>SEC-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>QA-OPS-001</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Replica safety</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8285d63d48484bc4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31e2daa392bf4050"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4492,7 +5276,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94914057e8ce466d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20917015e6424849"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4839,7 +5623,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd40f85e1aac467e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcecc7b4aaf194642"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5178,7 +5962,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf86f2bf9b8614332"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdffa93aab41d4c0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5351,7 +6135,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re46edf7e1d584ba5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad07f7e7e16e4838"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5456,11 +6240,11 @@
       <x:c r="J6" s="25" t="str">
         <x:v>GitHub plan blocks protected private branches native secret scanning and native CodeQL upload; offline SARIF and CI Gitleaks compensate; tracked by GOV-001</x:v>
       </x:c>
-      <x:c r="K6" s="25" t="str">
-        <x:v>Ready to Merge</x:v>
+      <x:c r="K6" s="70" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L6" s="28" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -5492,11 +6276,11 @@
       <x:c r="J7" s="26" t="str">
         <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
       </x:c>
-      <x:c r="K7" s="26" t="str">
-        <x:v>Ready to Merge</x:v>
+      <x:c r="K7" s="71" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L7" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -5504,37 +6288,37 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>codex/sec-001-admin-mfa-provider-policy</x:v>
+        <x:v>codex/sec-001-sso-login-policy</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>57e13d0</x:v>
+        <x:v>29537ee</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>fad2ef5</x:v>
+        <x:v>3eaa03c</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>WOW-MD PR 37 merged as b28c334; application mirror commit 1482d83</x:v>
+        <x:v>WOW-MD PR 38 head f685774</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance and synchronization 19/19; protected production and source CI passed including retained 30-day CodeQL SARIF</x:v>
+        <x:v>Backend typecheck/lint and 71 focused auth/config tests pass; frontend typecheck and 173 tests pass; mobile typecheck passes; CodeQL security gate passes after refresh cookies were sealed and session hashes moved to memory-hard derivation; remaining protected CI jobs are recorded on the PR</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
-        <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
+        <x:v>At the final release gate configure exact Zoho OAuth client/callback domain SPF DKIM DMARC sender mailbox and SMTP application password; then run controlled admin/non-admin SSO and email tests</x:v>
       </x:c>
       <x:c r="I8" s="26" t="str">
-        <x:v>Restore previous image/config; do not fall back to log/mock in a public tier; pause email-dependent workflows</x:v>
+        <x:v>Restore the prior image/config and disable Zoho SSO; do not enable passwordless OTP or log-based mail in public tier</x:v>
       </x:c>
       <x:c r="J8" s="26" t="str">
-        <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
-      </x:c>
-      <x:c r="K8" s="26" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred to the final release gate</x:v>
+      </x:c>
+      <x:c r="K8" s="71" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -5568,50 +6352,296 @@
       <x:c r="J9" s="27" t="str">
         <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
       </x:c>
-      <x:c r="K9" s="27" t="str">
-        <x:v>Blocked</x:v>
+      <x:c r="K9" s="74" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L9" s="30" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>OBS-001</x:v>
+        <x:v>DEP-001</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/65</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>codex/obs-001-backend-observability</x:v>
+        <x:v>codex/dep-001-dependency-remediation</x:v>
       </x:c>
       <x:c r="D10" t="str">
         <x:v>29537ee</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>48c1351</x:v>
+        <x:v>1ecbfdf</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>WOW-MD commit 69c2aea; PR 43</x:v>
+        <x:v>WOW-MD PR 39 head d8ef995</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>Focused observability 20 of 20; backend full suite 812 passed 9 skipped; typecheck lint nginx contract frontend image build and nginx syntax passed</x:v>
+        <x:v>Backend clean install typecheck lint build and 792 tests pass with 9 skipped; frontend clean install typecheck 173 tests build and 10 Playwright flows pass; runtime audits: backend 0 critical/0 high frontend 0; exact-ID mobile gate passes; production and source protected CI pass</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>Merge SEC-003 first then rebase; set RELEASE; keep QA capture disabled; confirm a live request ID matches response backend and nginx logs</x:v>
+        <x:v>No deployment before review and merge; after merge let GitHub rescan manifests and confirm alert counts and audit gates on main</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>Revert PR 65 and redeploy; remove optional observability variables; no database rollback</x:v>
+        <x:v>Revert PR 59; restore prior lockfiles and packages; retain the audit report for comparison</x:v>
       </x:c>
       <x:c r="J10" t="str">
-        <x:v>OBS-002 client error intake and OBS-003 Loki Vector host files 30-day retention remain open; live provider correlation smoke remains</x:v>
-      </x:c>
-      <x:c r="K10" t="str">
-        <x:v>Ready for Review</x:v>
+        <x:v>Backend moderate/low build-tool advisories and four exact no-fix Expo advisory roots remain; forced NestJS 12 and Expo downgrades were tested and rejected as unsafe</x:v>
+      </x:c>
+      <x:c r="K10" s="75" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L10" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>GOV-003</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>codex/gov-003-auth-dependency-tracking</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>1235cd3</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>SEC-001 PR 58 and DEP-001 PR 59 evidence only</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Register validator workbook regeneration and formula-error scan pass; dashboard visually reviewed</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Governance and documentation only; no application or hosting deployment</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>Revert PR 61; implementation PRs and their evidence remain unchanged</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>Implementation PRs still require review/merge and GitHub rescan; Zoho live configuration remains a final release gate</x:v>
+      </x:c>
+      <x:c r="K11" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>SEC-002</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/62</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>codex/sec-002-websocket-authorization</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>4c5e7b4</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>WOW-MD PR 40 head 9265a27</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>11 focused chat/admin gateway tests; backend typecheck and lint; complete backend suite 800 passed with 9 skipped</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Set exact CORS_ORIGINS and smoke-test browser/native reconnect on the Railway candidate; no schema migration</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>Revert PR 62; REST chat remains available while socket traffic is paused</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Native clients are allowed without an Origin header and remain protected by bearer-token/account checks; Railway cross-origin smoke evidence remains pending</x:v>
+      </x:c>
+      <x:c r="K12" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>SEC-003</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/63</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>codex/sec-003-http-migration-integrity</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>80ef902</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>WOW-MD PR 41 head ef13ff5</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>2 HTTP policy tests; 2 migration verifier tests; 93 files unique; backend typecheck/lint and 794 tests with 9 skipped; upgraded wow_db and fresh 93-migration database passed</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Run migrations before application rollout and verify headers through the Railway ingress</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>Revert application/header changes but retain applied migration history and safe schema additions for roll-forward</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>Historical databases retain old collision rows plus new idempotent reconciliation rows; ingress evidence remains pending</x:v>
+      </x:c>
+      <x:c r="K13" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>codex/ops-001-replicated-jobs</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>57e13d0</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>2bf76a1</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>WOW-MD commit a06067a; PR 42</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>Focused replica tests 7 of 7; backend full suite 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Deploy normally after approval; verify two replicas produce one owner and one skipped invocation for outbox and payout/reminder jobs</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>Revert PR 64 and redeploy; no database or configuration rollback</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>Outbox delivery is at-least-once if a worker dies after an external side effect and before processedAt; downstream Kafka consumers must honor the outbox UUID idempotency key</x:v>
+      </x:c>
+      <x:c r="K14" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>OBS-001</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/69</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>codex/obs-001-backend-observability</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>122ae2d</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>9d34f68</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>WOW-MD PR 43 merged as 2db719b</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Focused observability and replica-lock integration 27 of 27; backend typecheck and lint plus nginx contract passed; protected CI recorded on PR 69</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Set RELEASE; keep QA capture disabled; confirm a live request ID matches response backend and nginx logs</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>Revert PR 69 and redeploy; remove optional observability variables; no database rollback</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>OBS-002 client error intake and OBS-003 Loki Vector host files 30-day retention remain open; live provider correlation smoke remains</x:v>
+      </x:c>
+      <x:c r="K15" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
+      <x:c r="K17"/>
+      <x:c r="L17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
+      <x:c r="K18"/>
+      <x:c r="L18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
+      <x:c r="I19"/>
+      <x:c r="J19"/>
+      <x:c r="K19"/>
+      <x:c r="L19"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5626,7 +6656,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998f60580a2a4686"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re34e5b2e80104411"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record OBS-003 handoff
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R30f34b6cf68a479c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R29c368d037af4a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R518005db4602425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R328df1b9cecb476a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rf59eb498d24d447e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R41c7ecedbd834286"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R18432713b03e431a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rae971aa8878a4382"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R37759bbb55db4b73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R43f2d00d33eb4454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8363d4ab68c0401c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R0483a261dea643fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R619b640a444e489f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R195f9a45aa1c4c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R37d3442a5b6447b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R41d20f48ce894af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R592db801caa846d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rd035b38cbf2b4e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8abca5f0300749fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R75446ace44e7456f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R061f15398a4b4fc4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R241e6607a82f416d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1434,7 +1434,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1442,7 +1442,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1476,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1484,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9e0768e4c7348f9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R934f084633e843b0"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2982b85399ee43db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R068394b04cc4457e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2457,10 +2457,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F13" s="72" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H13" s="26" t="str">
         <x:v>OBS-001</x:v>
@@ -2474,9 +2474,11 @@
       <x:c r="K13" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/13</x:v>
       </x:c>
-      <x:c r="L13" s="26" t="str"/>
+      <x:c r="L13" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/71</x:v>
+      </x:c>
       <x:c r="M13" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
@@ -3950,7 +3952,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d8ce612c81e4551"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a1bd56ba91a45e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4434,7 +4436,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R305eab3893d14d36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8399ddc4b3a4c2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4839,7 +4841,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31e2daa392bf4050"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe72213628b64177"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5276,7 +5278,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20917015e6424849"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70539203b8af49a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5623,7 +5625,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcecc7b4aaf194642"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c8a7adfbaa54120"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5962,7 +5964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdffa93aab41d4c0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54d3f5285878445d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6135,7 +6137,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad07f7e7e16e4838"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf944248192ee48c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6588,18 +6590,42 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16"/>
-      <x:c r="B16"/>
-      <x:c r="C16"/>
-      <x:c r="D16"/>
-      <x:c r="E16"/>
-      <x:c r="F16"/>
-      <x:c r="G16"/>
-      <x:c r="H16"/>
-      <x:c r="I16"/>
-      <x:c r="J16"/>
-      <x:c r="K16"/>
-      <x:c r="L16"/>
+      <x:c r="A16" t="str">
+        <x:v>OBS-003</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/71</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>codex/obs-003-local-log-platform</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>f5d87f0</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>555a1fe</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Collector/Loki config validation; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; 7 provisioned alerts; Loki buffer recovery; frontend-restart persistence all pass</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Set WOW_LOG_DIR and a unique GRAFANA_ADMIN_PASSWORD; start the observability Compose profile; Grafana binds to 127.0.0.1:3300</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>Stop/remove observability containers and revert PR 71; retained host logs are not automatically deleted; application services remain independent</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>Single-host logs are not disaster recovery; Vector outage has only bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>Ready for Review</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17"/>
@@ -6656,7 +6682,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re34e5b2e80104411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a6bedf623164e35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: reconcile merged production tracking (#70)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb1a81da2f2014435"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Ra7461bf4dcfb4305"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R0e96e3e2600e4214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R98da020119b44f1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R8aa33dab71ba45c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R92f26e4c0b364480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R26c31c2a0f784e41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6f685f0304024924"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R1ee073186a0d4a52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7e6fe2172f234a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R30f34b6cf68a479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R29c368d037af4a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R518005db4602425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R328df1b9cecb476a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rf59eb498d24d447e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R41c7ecedbd834286"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R18432713b03e431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rae971aa8878a4382"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R37759bbb55db4b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R43f2d00d33eb4454"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,8 +68,23 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF16794A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF7A4B00"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFB42318"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +94,81 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F6EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE8E8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -124,7 +214,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="76">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -213,6 +303,102 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -830,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8b785583de834eb6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R061f15398a4b4fc4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -840,7 +1026,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -960,7 +1146,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1207,7 +1393,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-05. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-06. Reconciled to canonical registers and final merged PR/issue state.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1235,20 +1421,20 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$37,"P0",'Open Items'!$F$6:$F$37,"&lt;&gt;Done")</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1256,7 +1442,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1290,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1298,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1311,7 +1497,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H9" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1319,7 +1505,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
@@ -1332,7 +1518,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1340,7 +1526,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1439,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44d35715b66648ca"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9e0768e4c7348f9"/>
 </x:worksheet>
 </file>
 
@@ -1899,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d61ae7eeb044cf6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2982b85399ee43db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1982,7 +2168,7 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>Enforce administrator MFA and production provider policy</x:v>
+        <x:v>Align authentication with Zoho SSO and multi-identifier login policy</x:v>
       </x:c>
       <x:c r="C6" s="25" t="str">
         <x:v>Public beta safety</x:v>
@@ -1993,27 +2179,27 @@
       <x:c r="E6" s="25" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F6" s="25" t="str">
-        <x:v>Blocked</x:v>
+      <x:c r="F6" s="70" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str"/>
       <x:c r="I6" s="25" t="str">
-        <x:v>Admin cannot use privileged access without MFA; unsafe production provider combinations fail startup</x:v>
+        <x:v>Administrators use Zoho SSO; existing users may use Zoho SSO or username/email/mobile plus password; OTP is verification/recovery only; unsafe public provider combinations fail startup</x:v>
       </x:c>
       <x:c r="J6" s="25" t="str">
-        <x:v>Production plan Task 1A</x:v>
+        <x:v>Production plan Task 1A and user authentication decision</x:v>
       </x:c>
       <x:c r="K6" s="25" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/6</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
       </x:c>
       <x:c r="M6" s="28" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -2032,11 +2218,11 @@
       <x:c r="E7" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F7" s="26" t="str">
-        <x:v>Open</x:v>
+      <x:c r="F7" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G7" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H7" s="26" t="str">
         <x:v>SEC-001</x:v>
@@ -2050,9 +2236,11 @@
       <x:c r="K7" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/7</x:v>
       </x:c>
-      <x:c r="L7" s="26" t="str"/>
+      <x:c r="L7" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/62</x:v>
+      </x:c>
       <x:c r="M7" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -2071,11 +2259,11 @@
       <x:c r="E8" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F8" s="26" t="str">
-        <x:v>Open</x:v>
+      <x:c r="F8" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str"/>
       <x:c r="I8" s="26" t="str">
@@ -2087,9 +2275,11 @@
       <x:c r="K8" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/8</x:v>
       </x:c>
-      <x:c r="L8" s="26" t="str"/>
+      <x:c r="L8" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+      </x:c>
       <x:c r="M8" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -2108,11 +2298,11 @@
       <x:c r="E9" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F9" s="26" t="str">
-        <x:v>Open</x:v>
+      <x:c r="F9" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G9" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H9" s="26" t="str"/>
       <x:c r="I9" s="26" t="str">
@@ -2124,9 +2314,11 @@
       <x:c r="K9" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/9</x:v>
       </x:c>
-      <x:c r="L9" s="26" t="str"/>
+      <x:c r="L9" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/63</x:v>
+      </x:c>
       <x:c r="M9" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -2145,15 +2337,15 @@
       <x:c r="E10" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F10" s="26" t="str">
-        <x:v>Open</x:v>
+      <x:c r="F10" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str"/>
       <x:c r="I10" s="26" t="str">
-        <x:v>No unaccepted critical/high production advisory; CI blocks regression</x:v>
+        <x:v>No unaccepted critical/high runtime advisory; CI blocks regressions; explicitly documented no-fix build-tool exceptions remain narrow and reviewable</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
         <x:v>Production plan Task 1E</x:v>
@@ -2161,9 +2353,11 @@
       <x:c r="K10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/10</x:v>
       </x:c>
-      <x:c r="L10" s="26" t="str"/>
+      <x:c r="L10" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
+      </x:c>
       <x:c r="M10" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -2182,8 +2376,8 @@
       <x:c r="E11" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F11" s="26" t="str">
-        <x:v>PR Open</x:v>
+      <x:c r="F11" s="71" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
         <x:v>Codex</x:v>
@@ -2201,7 +2395,7 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/11</x:v>
       </x:c>
       <x:c r="L11" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/65</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/69</x:v>
       </x:c>
       <x:c r="M11" s="29" t="str">
         <x:v>2026-10-05</x:v>
@@ -2223,7 +2417,7 @@
       <x:c r="E12" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F12" s="26" t="str">
+      <x:c r="F12" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G12" s="26" t="str">
@@ -2262,7 +2456,7 @@
       <x:c r="E13" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F13" s="26" t="str">
+      <x:c r="F13" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
@@ -2301,7 +2495,7 @@
       <x:c r="E14" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F14" s="26" t="str">
+      <x:c r="F14" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
@@ -2340,7 +2534,7 @@
       <x:c r="E15" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F15" s="26" t="str">
+      <x:c r="F15" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G15" s="26" t="str">
@@ -2379,7 +2573,7 @@
       <x:c r="E16" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F16" s="26" t="str">
+      <x:c r="F16" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G16" s="26" t="str">
@@ -2418,7 +2612,7 @@
       <x:c r="E17" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F17" s="26" t="str">
+      <x:c r="F17" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G17" s="26" t="str">
@@ -2457,7 +2651,7 @@
       <x:c r="E18" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F18" s="26" t="str">
+      <x:c r="F18" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G18" s="26" t="str">
@@ -2496,7 +2690,7 @@
       <x:c r="E19" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F19" s="26" t="str">
+      <x:c r="F19" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G19" s="26" t="str">
@@ -2524,7 +2718,7 @@
         <x:v>AUTH-001</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Add scoped administrator MFA step-up</x:v>
+        <x:v>Add scoped administrator fresh-authentication step-up</x:v>
       </x:c>
       <x:c r="C20" s="26" t="str">
         <x:v>Migration control</x:v>
@@ -2535,7 +2729,7 @@
       <x:c r="E20" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F20" s="26" t="str">
+      <x:c r="F20" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G20" s="26" t="str">
@@ -2545,17 +2739,17 @@
         <x:v>SEC-001,CFG-001</x:v>
       </x:c>
       <x:c r="I20" s="26" t="str">
-        <x:v>Five-minute single-use scoped token protects migration start</x:v>
+        <x:v>Fresh Zoho reauthentication issues a five-minute single-use action-scoped token for migration start; application TOTP is a documented fallback only</x:v>
       </x:c>
       <x:c r="J20" s="26" t="str">
-        <x:v>Production plan Task 9</x:v>
+        <x:v>Production plan Task 9 and user authentication decision</x:v>
       </x:c>
       <x:c r="K20" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/20</x:v>
       </x:c>
       <x:c r="L20" s="26" t="str"/>
       <x:c r="M20" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -2574,7 +2768,7 @@
       <x:c r="E21" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F21" s="26" t="str">
+      <x:c r="F21" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G21" s="26" t="str">
@@ -2613,7 +2807,7 @@
       <x:c r="E22" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F22" s="26" t="str">
+      <x:c r="F22" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G22" s="26" t="str">
@@ -2652,7 +2846,7 @@
       <x:c r="E23" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F23" s="26" t="str">
+      <x:c r="F23" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G23" s="26" t="str">
@@ -2691,7 +2885,7 @@
       <x:c r="E24" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F24" s="26" t="str">
+      <x:c r="F24" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G24" s="26" t="str">
@@ -2730,7 +2924,7 @@
       <x:c r="E25" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F25" s="26" t="str">
+      <x:c r="F25" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G25" s="26" t="str">
@@ -2769,7 +2963,7 @@
       <x:c r="E26" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F26" s="26" t="str">
+      <x:c r="F26" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G26" s="26" t="str">
@@ -2808,7 +3002,7 @@
       <x:c r="E27" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F27" s="26" t="str">
+      <x:c r="F27" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G27" s="26" t="str">
@@ -2847,7 +3041,7 @@
       <x:c r="E28" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F28" s="26" t="str">
+      <x:c r="F28" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G28" s="26" t="str">
@@ -2886,7 +3080,7 @@
       <x:c r="E29" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F29" s="26" t="str">
+      <x:c r="F29" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G29" s="26" t="str">
@@ -2925,7 +3119,7 @@
       <x:c r="E30" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F30" s="26" t="str">
+      <x:c r="F30" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G30" s="26" t="str">
@@ -2964,7 +3158,7 @@
       <x:c r="E31" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F31" s="26" t="str">
+      <x:c r="F31" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G31" s="26" t="str">
@@ -3001,7 +3195,7 @@
       <x:c r="E32" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F32" s="26" t="str">
+      <x:c r="F32" s="73" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G32" s="26" t="str">
@@ -3042,7 +3236,7 @@
       <x:c r="E33" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F33" s="26" t="str">
+      <x:c r="F33" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G33" s="26" t="str">
@@ -3079,7 +3273,7 @@
       <x:c r="E34" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F34" s="26" t="str">
+      <x:c r="F34" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G34" s="26" t="str">
@@ -3118,7 +3312,7 @@
       <x:c r="E35" s="26" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F35" s="26" t="str">
+      <x:c r="F35" s="72" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G35" s="26" t="str">
@@ -3157,7 +3351,7 @@
       <x:c r="E36" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F36" s="26" t="str">
+      <x:c r="F36" s="71" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G36" s="26" t="str">
@@ -3177,7 +3371,7 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/54</x:v>
       </x:c>
       <x:c r="M36" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
@@ -3196,7 +3390,7 @@
       <x:c r="E37" s="27" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F37" s="27" t="str">
+      <x:c r="F37" s="74" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G37" s="27" t="str">
@@ -3216,8 +3410,529 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
       <x:c r="M37" s="30" t="str">
-        <x:v>2026-10-04</x:v>
-      </x:c>
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>GOV-003</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>Reconcile authentication and dependency tracking</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>Governance</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F38" s="75" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>SEC-001,DEP-001</x:v>
+      </x:c>
+      <x:c r="I38" t="str">
+        <x:v>Canonical registers workbook and operating guidance match the implemented authentication policy and dependency evidence</x:v>
+      </x:c>
+      <x:c r="J38" t="str">
+        <x:v>User request</x:v>
+      </x:c>
+      <x:c r="K38" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/60</x:v>
+      </x:c>
+      <x:c r="L38" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
+      </x:c>
+      <x:c r="M38" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39"/>
+      <x:c r="B39"/>
+      <x:c r="C39"/>
+      <x:c r="D39"/>
+      <x:c r="E39"/>
+      <x:c r="F39"/>
+      <x:c r="G39"/>
+      <x:c r="H39"/>
+      <x:c r="I39"/>
+      <x:c r="J39"/>
+      <x:c r="K39"/>
+      <x:c r="L39"/>
+      <x:c r="M39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40"/>
+      <x:c r="B40"/>
+      <x:c r="C40"/>
+      <x:c r="D40"/>
+      <x:c r="E40"/>
+      <x:c r="F40"/>
+      <x:c r="G40"/>
+      <x:c r="H40"/>
+      <x:c r="I40"/>
+      <x:c r="J40"/>
+      <x:c r="K40"/>
+      <x:c r="L40"/>
+      <x:c r="M40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41"/>
+      <x:c r="B41"/>
+      <x:c r="C41"/>
+      <x:c r="D41"/>
+      <x:c r="E41"/>
+      <x:c r="F41"/>
+      <x:c r="G41"/>
+      <x:c r="H41"/>
+      <x:c r="I41"/>
+      <x:c r="J41"/>
+      <x:c r="K41"/>
+      <x:c r="L41"/>
+      <x:c r="M41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42"/>
+      <x:c r="B42"/>
+      <x:c r="C42"/>
+      <x:c r="D42"/>
+      <x:c r="E42"/>
+      <x:c r="F42"/>
+      <x:c r="G42"/>
+      <x:c r="H42"/>
+      <x:c r="I42"/>
+      <x:c r="J42"/>
+      <x:c r="K42"/>
+      <x:c r="L42"/>
+      <x:c r="M42"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43"/>
+      <x:c r="B43"/>
+      <x:c r="C43"/>
+      <x:c r="D43"/>
+      <x:c r="E43"/>
+      <x:c r="F43"/>
+      <x:c r="G43"/>
+      <x:c r="H43"/>
+      <x:c r="I43"/>
+      <x:c r="J43"/>
+      <x:c r="K43"/>
+      <x:c r="L43"/>
+      <x:c r="M43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44"/>
+      <x:c r="B44"/>
+      <x:c r="C44"/>
+      <x:c r="D44"/>
+      <x:c r="E44"/>
+      <x:c r="F44"/>
+      <x:c r="G44"/>
+      <x:c r="H44"/>
+      <x:c r="I44"/>
+      <x:c r="J44"/>
+      <x:c r="K44"/>
+      <x:c r="L44"/>
+      <x:c r="M44"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45"/>
+      <x:c r="B45"/>
+      <x:c r="C45"/>
+      <x:c r="D45"/>
+      <x:c r="E45"/>
+      <x:c r="F45"/>
+      <x:c r="G45"/>
+      <x:c r="H45"/>
+      <x:c r="I45"/>
+      <x:c r="J45"/>
+      <x:c r="K45"/>
+      <x:c r="L45"/>
+      <x:c r="M45"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46"/>
+      <x:c r="B46"/>
+      <x:c r="C46"/>
+      <x:c r="D46"/>
+      <x:c r="E46"/>
+      <x:c r="F46"/>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
+      <x:c r="I46"/>
+      <x:c r="J46"/>
+      <x:c r="K46"/>
+      <x:c r="L46"/>
+      <x:c r="M46"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47"/>
+      <x:c r="B47"/>
+      <x:c r="C47"/>
+      <x:c r="D47"/>
+      <x:c r="E47"/>
+      <x:c r="F47"/>
+      <x:c r="G47"/>
+      <x:c r="H47"/>
+      <x:c r="I47"/>
+      <x:c r="J47"/>
+      <x:c r="K47"/>
+      <x:c r="L47"/>
+      <x:c r="M47"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48"/>
+      <x:c r="B48"/>
+      <x:c r="C48"/>
+      <x:c r="D48"/>
+      <x:c r="E48"/>
+      <x:c r="F48"/>
+      <x:c r="G48"/>
+      <x:c r="H48"/>
+      <x:c r="I48"/>
+      <x:c r="J48"/>
+      <x:c r="K48"/>
+      <x:c r="L48"/>
+      <x:c r="M48"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49"/>
+      <x:c r="B49"/>
+      <x:c r="C49"/>
+      <x:c r="D49"/>
+      <x:c r="E49"/>
+      <x:c r="F49"/>
+      <x:c r="G49"/>
+      <x:c r="H49"/>
+      <x:c r="I49"/>
+      <x:c r="J49"/>
+      <x:c r="K49"/>
+      <x:c r="L49"/>
+      <x:c r="M49"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50"/>
+      <x:c r="B50"/>
+      <x:c r="C50"/>
+      <x:c r="D50"/>
+      <x:c r="E50"/>
+      <x:c r="F50"/>
+      <x:c r="G50"/>
+      <x:c r="H50"/>
+      <x:c r="I50"/>
+      <x:c r="J50"/>
+      <x:c r="K50"/>
+      <x:c r="L50"/>
+      <x:c r="M50"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51"/>
+      <x:c r="B51"/>
+      <x:c r="C51"/>
+      <x:c r="D51"/>
+      <x:c r="E51"/>
+      <x:c r="F51"/>
+      <x:c r="G51"/>
+      <x:c r="H51"/>
+      <x:c r="I51"/>
+      <x:c r="J51"/>
+      <x:c r="K51"/>
+      <x:c r="L51"/>
+      <x:c r="M51"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52"/>
+      <x:c r="B52"/>
+      <x:c r="C52"/>
+      <x:c r="D52"/>
+      <x:c r="E52"/>
+      <x:c r="F52"/>
+      <x:c r="G52"/>
+      <x:c r="H52"/>
+      <x:c r="I52"/>
+      <x:c r="J52"/>
+      <x:c r="K52"/>
+      <x:c r="L52"/>
+      <x:c r="M52"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53"/>
+      <x:c r="B53"/>
+      <x:c r="C53"/>
+      <x:c r="D53"/>
+      <x:c r="E53"/>
+      <x:c r="F53"/>
+      <x:c r="G53"/>
+      <x:c r="H53"/>
+      <x:c r="I53"/>
+      <x:c r="J53"/>
+      <x:c r="K53"/>
+      <x:c r="L53"/>
+      <x:c r="M53"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54"/>
+      <x:c r="B54"/>
+      <x:c r="C54"/>
+      <x:c r="D54"/>
+      <x:c r="E54"/>
+      <x:c r="F54"/>
+      <x:c r="G54"/>
+      <x:c r="H54"/>
+      <x:c r="I54"/>
+      <x:c r="J54"/>
+      <x:c r="K54"/>
+      <x:c r="L54"/>
+      <x:c r="M54"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55"/>
+      <x:c r="B55"/>
+      <x:c r="C55"/>
+      <x:c r="D55"/>
+      <x:c r="E55"/>
+      <x:c r="F55"/>
+      <x:c r="G55"/>
+      <x:c r="H55"/>
+      <x:c r="I55"/>
+      <x:c r="J55"/>
+      <x:c r="K55"/>
+      <x:c r="L55"/>
+      <x:c r="M55"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56"/>
+      <x:c r="B56"/>
+      <x:c r="C56"/>
+      <x:c r="D56"/>
+      <x:c r="E56"/>
+      <x:c r="F56"/>
+      <x:c r="G56"/>
+      <x:c r="H56"/>
+      <x:c r="I56"/>
+      <x:c r="J56"/>
+      <x:c r="K56"/>
+      <x:c r="L56"/>
+      <x:c r="M56"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57"/>
+      <x:c r="B57"/>
+      <x:c r="C57"/>
+      <x:c r="D57"/>
+      <x:c r="E57"/>
+      <x:c r="F57"/>
+      <x:c r="G57"/>
+      <x:c r="H57"/>
+      <x:c r="I57"/>
+      <x:c r="J57"/>
+      <x:c r="K57"/>
+      <x:c r="L57"/>
+      <x:c r="M57"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58"/>
+      <x:c r="B58"/>
+      <x:c r="C58"/>
+      <x:c r="D58"/>
+      <x:c r="E58"/>
+      <x:c r="F58"/>
+      <x:c r="G58"/>
+      <x:c r="H58"/>
+      <x:c r="I58"/>
+      <x:c r="J58"/>
+      <x:c r="K58"/>
+      <x:c r="L58"/>
+      <x:c r="M58"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59"/>
+      <x:c r="B59"/>
+      <x:c r="C59"/>
+      <x:c r="D59"/>
+      <x:c r="E59"/>
+      <x:c r="F59"/>
+      <x:c r="G59"/>
+      <x:c r="H59"/>
+      <x:c r="I59"/>
+      <x:c r="J59"/>
+      <x:c r="K59"/>
+      <x:c r="L59"/>
+      <x:c r="M59"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60"/>
+      <x:c r="B60"/>
+      <x:c r="C60"/>
+      <x:c r="D60"/>
+      <x:c r="E60"/>
+      <x:c r="F60"/>
+      <x:c r="G60"/>
+      <x:c r="H60"/>
+      <x:c r="I60"/>
+      <x:c r="J60"/>
+      <x:c r="K60"/>
+      <x:c r="L60"/>
+      <x:c r="M60"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61"/>
+      <x:c r="B61"/>
+      <x:c r="C61"/>
+      <x:c r="D61"/>
+      <x:c r="E61"/>
+      <x:c r="F61"/>
+      <x:c r="G61"/>
+      <x:c r="H61"/>
+      <x:c r="I61"/>
+      <x:c r="J61"/>
+      <x:c r="K61"/>
+      <x:c r="L61"/>
+      <x:c r="M61"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62"/>
+      <x:c r="B62"/>
+      <x:c r="C62"/>
+      <x:c r="D62"/>
+      <x:c r="E62"/>
+      <x:c r="F62"/>
+      <x:c r="G62"/>
+      <x:c r="H62"/>
+      <x:c r="I62"/>
+      <x:c r="J62"/>
+      <x:c r="K62"/>
+      <x:c r="L62"/>
+      <x:c r="M62"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63"/>
+      <x:c r="B63"/>
+      <x:c r="C63"/>
+      <x:c r="D63"/>
+      <x:c r="E63"/>
+      <x:c r="F63"/>
+      <x:c r="G63"/>
+      <x:c r="H63"/>
+      <x:c r="I63"/>
+      <x:c r="J63"/>
+      <x:c r="K63"/>
+      <x:c r="L63"/>
+      <x:c r="M63"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64"/>
+      <x:c r="B64"/>
+      <x:c r="C64"/>
+      <x:c r="D64"/>
+      <x:c r="E64"/>
+      <x:c r="F64"/>
+      <x:c r="G64"/>
+      <x:c r="H64"/>
+      <x:c r="I64"/>
+      <x:c r="J64"/>
+      <x:c r="K64"/>
+      <x:c r="L64"/>
+      <x:c r="M64"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65"/>
+      <x:c r="B65"/>
+      <x:c r="C65"/>
+      <x:c r="D65"/>
+      <x:c r="E65"/>
+      <x:c r="F65"/>
+      <x:c r="G65"/>
+      <x:c r="H65"/>
+      <x:c r="I65"/>
+      <x:c r="J65"/>
+      <x:c r="K65"/>
+      <x:c r="L65"/>
+      <x:c r="M65"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66"/>
+      <x:c r="B66"/>
+      <x:c r="C66"/>
+      <x:c r="D66"/>
+      <x:c r="E66"/>
+      <x:c r="F66"/>
+      <x:c r="G66"/>
+      <x:c r="H66"/>
+      <x:c r="I66"/>
+      <x:c r="J66"/>
+      <x:c r="K66"/>
+      <x:c r="L66"/>
+      <x:c r="M66"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67"/>
+      <x:c r="B67"/>
+      <x:c r="C67"/>
+      <x:c r="D67"/>
+      <x:c r="E67"/>
+      <x:c r="F67"/>
+      <x:c r="G67"/>
+      <x:c r="H67"/>
+      <x:c r="I67"/>
+      <x:c r="J67"/>
+      <x:c r="K67"/>
+      <x:c r="L67"/>
+      <x:c r="M67"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68"/>
+      <x:c r="B68"/>
+      <x:c r="C68"/>
+      <x:c r="D68"/>
+      <x:c r="E68"/>
+      <x:c r="F68"/>
+      <x:c r="G68"/>
+      <x:c r="H68"/>
+      <x:c r="I68"/>
+      <x:c r="J68"/>
+      <x:c r="K68"/>
+      <x:c r="L68"/>
+      <x:c r="M68"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69"/>
+      <x:c r="B69"/>
+      <x:c r="C69"/>
+      <x:c r="D69"/>
+      <x:c r="E69"/>
+      <x:c r="F69"/>
+      <x:c r="G69"/>
+      <x:c r="H69"/>
+      <x:c r="I69"/>
+      <x:c r="J69"/>
+      <x:c r="K69"/>
+      <x:c r="L69"/>
+      <x:c r="M69"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70"/>
+      <x:c r="B70"/>
+      <x:c r="C70"/>
+      <x:c r="D70"/>
+      <x:c r="E70"/>
+      <x:c r="F70"/>
+      <x:c r="G70"/>
+      <x:c r="H70"/>
+      <x:c r="I70"/>
+      <x:c r="J70"/>
+      <x:c r="K70"/>
+      <x:c r="L70"/>
+      <x:c r="M70"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3235,7 +3950,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13810d1b976a4191"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d8ce612c81e4551"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3719,7 +4434,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R718b81cadaf445d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R305eab3893d14d36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4049,13 +4764,82 @@
         <x:v>OBS-001</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>QA-SEC-002</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>WebSocket origins tokens calls and presence authorization</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>SEC-002 PR 62 and WOW-MD PR 40</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>Focused gateways 11 passed; full backend 800 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Run staged hostile-origin and two-account WebSocket smoke</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>SEC-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>QA-SEC-003</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>HTTP headers private Swagger and migration integrity</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>SEC-003 PR 63 and WOW-MD PR 41</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>HTTP 2 passed; migration verifier 2 passed; 93 migrations verified and clean database upgrade passed; backend 794 passed 9 skipped</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Deploy and verify production headers Swagger denial and migration startup</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>SEC-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>QA-OPS-001</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Replica safety</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8285d63d48484bc4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31e2daa392bf4050"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4492,7 +5276,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94914057e8ce466d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20917015e6424849"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4839,7 +5623,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd40f85e1aac467e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcecc7b4aaf194642"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5178,7 +5962,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf86f2bf9b8614332"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdffa93aab41d4c0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5351,7 +6135,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re46edf7e1d584ba5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad07f7e7e16e4838"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5456,11 +6240,11 @@
       <x:c r="J6" s="25" t="str">
         <x:v>GitHub plan blocks protected private branches native secret scanning and native CodeQL upload; offline SARIF and CI Gitleaks compensate; tracked by GOV-001</x:v>
       </x:c>
-      <x:c r="K6" s="25" t="str">
-        <x:v>Ready to Merge</x:v>
+      <x:c r="K6" s="70" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L6" s="28" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -5492,11 +6276,11 @@
       <x:c r="J7" s="26" t="str">
         <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
       </x:c>
-      <x:c r="K7" s="26" t="str">
-        <x:v>Ready to Merge</x:v>
+      <x:c r="K7" s="71" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L7" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -5504,37 +6288,37 @@
         <x:v>SEC-001</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/56</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/58</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>codex/sec-001-admin-mfa-provider-policy</x:v>
+        <x:v>codex/sec-001-sso-login-policy</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>57e13d0</x:v>
+        <x:v>29537ee</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>fad2ef5</x:v>
+        <x:v>3eaa03c</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>WOW-MD PR 37 merged as b28c334; application mirror commit 1482d83</x:v>
+        <x:v>WOW-MD PR 38 head f685774</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>Config policy 6/6; auth and JWT 49/49; WOW-MD mirror focused suite 55/55; backend typecheck and lint pass; governance and synchronization 19/19; protected production and source CI passed including retained 30-day CodeQL SARIF</x:v>
+        <x:v>Backend typecheck/lint and 71 focused auth/config tests pass; frontend typecheck and 173 tests pass; mobile typecheck passes; CodeQL security gate passes after refresh cookies were sealed and session hashes moved to memory-hard derivation; remaining protected CI jobs are recorded on the PR</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str">
-        <x:v>Configure Zoho SMTP S3 HTTPS and administrator TOTP in staging; select public-beta only after delivery and enrollment evidence</x:v>
+        <x:v>At the final release gate configure exact Zoho OAuth client/callback domain SPF DKIM DMARC sender mailbox and SMTP application password; then run controlled admin/non-admin SSO and email tests</x:v>
       </x:c>
       <x:c r="I8" s="26" t="str">
-        <x:v>Restore previous image/config; do not fall back to log/mock in a public tier; pause email-dependent workflows</x:v>
+        <x:v>Restore the prior image/config and disable Zoho SSO; do not enable passwordless OTP or log-based mail in public tier</x:v>
       </x:c>
       <x:c r="J8" s="26" t="str">
-        <x:v>Zoho owner/DNS/secrets and first delivery are pending; administrators must enrol before public tier; Zoho Mail is low-volume only</x:v>
-      </x:c>
-      <x:c r="K8" s="26" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred to the final release gate</x:v>
+      </x:c>
+      <x:c r="K8" s="71" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -5568,50 +6352,296 @@
       <x:c r="J9" s="27" t="str">
         <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
       </x:c>
-      <x:c r="K9" s="27" t="str">
-        <x:v>Blocked</x:v>
+      <x:c r="K9" s="74" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L9" s="30" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>OBS-001</x:v>
+        <x:v>DEP-001</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/65</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>codex/obs-001-backend-observability</x:v>
+        <x:v>codex/dep-001-dependency-remediation</x:v>
       </x:c>
       <x:c r="D10" t="str">
         <x:v>29537ee</x:v>
       </x:c>
       <x:c r="E10" t="str">
-        <x:v>48c1351</x:v>
+        <x:v>1ecbfdf</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>WOW-MD commit 69c2aea; PR 43</x:v>
+        <x:v>WOW-MD PR 39 head d8ef995</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>Focused observability 20 of 20; backend full suite 812 passed 9 skipped; typecheck lint nginx contract frontend image build and nginx syntax passed</x:v>
+        <x:v>Backend clean install typecheck lint build and 792 tests pass with 9 skipped; frontend clean install typecheck 173 tests build and 10 Playwright flows pass; runtime audits: backend 0 critical/0 high frontend 0; exact-ID mobile gate passes; production and source protected CI pass</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>Merge SEC-003 first then rebase; set RELEASE; keep QA capture disabled; confirm a live request ID matches response backend and nginx logs</x:v>
+        <x:v>No deployment before review and merge; after merge let GitHub rescan manifests and confirm alert counts and audit gates on main</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>Revert PR 65 and redeploy; remove optional observability variables; no database rollback</x:v>
+        <x:v>Revert PR 59; restore prior lockfiles and packages; retain the audit report for comparison</x:v>
       </x:c>
       <x:c r="J10" t="str">
-        <x:v>OBS-002 client error intake and OBS-003 Loki Vector host files 30-day retention remain open; live provider correlation smoke remains</x:v>
-      </x:c>
-      <x:c r="K10" t="str">
-        <x:v>Ready for Review</x:v>
+        <x:v>Backend moderate/low build-tool advisories and four exact no-fix Expo advisory roots remain; forced NestJS 12 and Expo downgrades were tested and rejected as unsafe</x:v>
+      </x:c>
+      <x:c r="K10" s="75" t="str">
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L10" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>GOV-003</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>codex/gov-003-auth-dependency-tracking</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>1235cd3</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>SEC-001 PR 58 and DEP-001 PR 59 evidence only</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Register validator workbook regeneration and formula-error scan pass; dashboard visually reviewed</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Governance and documentation only; no application or hosting deployment</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>Revert PR 61; implementation PRs and their evidence remain unchanged</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>Implementation PRs still require review/merge and GitHub rescan; Zoho live configuration remains a final release gate</x:v>
+      </x:c>
+      <x:c r="K11" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>SEC-002</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/62</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>codex/sec-002-websocket-authorization</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>4c5e7b4</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>WOW-MD PR 40 head 9265a27</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>11 focused chat/admin gateway tests; backend typecheck and lint; complete backend suite 800 passed with 9 skipped</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Set exact CORS_ORIGINS and smoke-test browser/native reconnect on the Railway candidate; no schema migration</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>Revert PR 62; REST chat remains available while socket traffic is paused</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Native clients are allowed without an Origin header and remain protected by bearer-token/account checks; Railway cross-origin smoke evidence remains pending</x:v>
+      </x:c>
+      <x:c r="K12" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>SEC-003</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/63</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>codex/sec-003-http-migration-integrity</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>29537ee</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>80ef902</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>WOW-MD PR 41 head ef13ff5</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>2 HTTP policy tests; 2 migration verifier tests; 93 files unique; backend typecheck/lint and 794 tests with 9 skipped; upgraded wow_db and fresh 93-migration database passed</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Run migrations before application rollout and verify headers through the Railway ingress</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>Revert application/header changes but retain applied migration history and safe schema additions for roll-forward</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>Historical databases retain old collision rows plus new idempotent reconciliation rows; ingress evidence remains pending</x:v>
+      </x:c>
+      <x:c r="K13" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>codex/ops-001-replicated-jobs</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>57e13d0</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>2bf76a1</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>WOW-MD commit a06067a; PR 42</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>Focused replica tests 7 of 7; backend full suite 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Deploy normally after approval; verify two replicas produce one owner and one skipped invocation for outbox and payout/reminder jobs</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>Revert PR 64 and redeploy; no database or configuration rollback</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>Outbox delivery is at-least-once if a worker dies after an external side effect and before processedAt; downstream Kafka consumers must honor the outbox UUID idempotency key</x:v>
+      </x:c>
+      <x:c r="K14" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>OBS-001</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/69</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>codex/obs-001-backend-observability</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>122ae2d</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>9d34f68</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>WOW-MD PR 43 merged as 2db719b</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Focused observability and replica-lock integration 27 of 27; backend typecheck and lint plus nginx contract passed; protected CI recorded on PR 69</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Set RELEASE; keep QA capture disabled; confirm a live request ID matches response backend and nginx logs</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>Revert PR 69 and redeploy; remove optional observability variables; no database rollback</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>OBS-002 client error intake and OBS-003 Loki Vector host files 30-day retention remain open; live provider correlation smoke remains</x:v>
+      </x:c>
+      <x:c r="K15" s="75" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16"/>
+      <x:c r="L16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
+      <x:c r="K17"/>
+      <x:c r="L17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
+      <x:c r="K18"/>
+      <x:c r="L18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
+      <x:c r="I19"/>
+      <x:c r="J19"/>
+      <x:c r="K19"/>
+      <x:c r="L19"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5626,7 +6656,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998f60580a2a4686"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re34e5b2e80104411"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[OBS-003] Add durable local Loki and Grafana logging (#71)
* feat: add durable local log platform

* docs: record OBS-003 handoff

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R30f34b6cf68a479c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R29c368d037af4a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R518005db4602425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R328df1b9cecb476a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rf59eb498d24d447e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R41c7ecedbd834286"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R18432713b03e431a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rae971aa8878a4382"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R37759bbb55db4b73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R43f2d00d33eb4454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8363d4ab68c0401c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R0483a261dea643fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R619b640a444e489f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R195f9a45aa1c4c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R37d3442a5b6447b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R41d20f48ce894af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R592db801caa846d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rd035b38cbf2b4e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8abca5f0300749fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R75446ace44e7456f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R061f15398a4b4fc4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R241e6607a82f416d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1434,7 +1434,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1442,7 +1442,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1476,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1484,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9e0768e4c7348f9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R934f084633e843b0"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2982b85399ee43db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R068394b04cc4457e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2457,10 +2457,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F13" s="72" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H13" s="26" t="str">
         <x:v>OBS-001</x:v>
@@ -2474,9 +2474,11 @@
       <x:c r="K13" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/13</x:v>
       </x:c>
-      <x:c r="L13" s="26" t="str"/>
+      <x:c r="L13" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/71</x:v>
+      </x:c>
       <x:c r="M13" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
@@ -3950,7 +3952,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d8ce612c81e4551"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a1bd56ba91a45e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4434,7 +4436,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R305eab3893d14d36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8399ddc4b3a4c2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4839,7 +4841,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31e2daa392bf4050"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe72213628b64177"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5276,7 +5278,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20917015e6424849"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70539203b8af49a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5623,7 +5625,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcecc7b4aaf194642"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c8a7adfbaa54120"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5962,7 +5964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdffa93aab41d4c0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54d3f5285878445d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6135,7 +6137,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad07f7e7e16e4838"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf944248192ee48c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6588,18 +6590,42 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16"/>
-      <x:c r="B16"/>
-      <x:c r="C16"/>
-      <x:c r="D16"/>
-      <x:c r="E16"/>
-      <x:c r="F16"/>
-      <x:c r="G16"/>
-      <x:c r="H16"/>
-      <x:c r="I16"/>
-      <x:c r="J16"/>
-      <x:c r="K16"/>
-      <x:c r="L16"/>
+      <x:c r="A16" t="str">
+        <x:v>OBS-003</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/71</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>codex/obs-003-local-log-platform</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>f5d87f0</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>555a1fe</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Collector/Loki config validation; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; 7 provisioned alerts; Loki buffer recovery; frontend-restart persistence all pass</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Set WOW_LOG_DIR and a unique GRAFANA_ADMIN_PASSWORD; start the observability Compose profile; Grafana binds to 127.0.0.1:3300</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>Stop/remove observability containers and revert PR 71; retained host logs are not automatically deleted; application services remain independent</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>Single-host logs are not disaster recovery; Vector outage has only bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>Ready for Review</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17"/>
@@ -6656,7 +6682,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re34e5b2e80104411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a6bedf623164e35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record OBS-003 merge and CFG-001 handoff
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8363d4ab68c0401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R0483a261dea643fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R619b640a444e489f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R195f9a45aa1c4c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R37d3442a5b6447b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R41d20f48ce894af7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R592db801caa846d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rd035b38cbf2b4e95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8abca5f0300749fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R75446ace44e7456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R21051e6975494f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rf48bf49924d0415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb3fbb1b7131f4bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R5f50b8ce9eaa428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rab64af5fca934ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R77cf6543731f4a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra7a6693082b240a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rcf46b4fa8a0b4b53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rd2de30d3279c46af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R786316df5f8d4f80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R241e6607a82f416d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8109f43b506541fb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1428,13 +1428,13 @@
       </x:c>
       <x:c r="E6" s="34" t="n">
         <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1442,7 +1442,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1518,7 +1518,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1526,7 +1526,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R934f084633e843b0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8633c727178490a"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R068394b04cc4457e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R148b65fbe21b4822"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2457,7 +2457,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F13" s="72" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
         <x:v>Codex</x:v>
@@ -2498,10 +2498,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F14" s="72" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H14" s="26" t="str">
         <x:v>SEC-001</x:v>
@@ -2515,9 +2515,11 @@
       <x:c r="K14" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/14</x:v>
       </x:c>
-      <x:c r="L14" s="26" t="str"/>
+      <x:c r="L14" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/72</x:v>
+      </x:c>
       <x:c r="M14" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
@@ -3952,7 +3954,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a1bd56ba91a45e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf79a22028df0467c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4436,7 +4438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8399ddc4b3a4c2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R463d03379c8749c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4841,7 +4843,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe72213628b64177"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998280114ed2448d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5278,7 +5280,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70539203b8af49a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1c3084fc9484b48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5625,7 +5627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c8a7adfbaa54120"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb6aae68d5d4768"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5964,7 +5966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54d3f5285878445d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf29101dc1fa34c54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6137,7 +6139,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf944248192ee48c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R678a7a4ffc4a4a2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6600,16 +6602,16 @@
         <x:v>codex/obs-003-local-log-platform</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>f5d87f0</x:v>
+        <x:v>dd39ccc</x:v>
       </x:c>
       <x:c r="E16" t="str">
-        <x:v>555a1fe</x:v>
+        <x:v>0d1e02f</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>None</x:v>
+        <x:v>WOW-MD PR 48 merged as 7384378</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>Collector/Loki config validation; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; 7 provisioned alerts; Loki buffer recovery; frontend-restart persistence all pass</x:v>
+        <x:v>Collector and Loki configuration; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; seven alerts; Loki buffer recovery; frontend restart persistence all pass</x:v>
       </x:c>
       <x:c r="H16" t="str">
         <x:v>Set WOW_LOG_DIR and a unique GRAFANA_ADMIN_PASSWORD; start the observability Compose profile; Grafana binds to 127.0.0.1:3300</x:v>
@@ -6618,28 +6620,52 @@
         <x:v>Stop/remove observability containers and revert PR 71; retained host logs are not automatically deleted; application services remain independent</x:v>
       </x:c>
       <x:c r="J16" t="str">
-        <x:v>Single-host logs are not disaster recovery; Vector outage has only bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
+        <x:v>Single-host logs are not disaster recovery; Vector outage has bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>Ready for Review</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L16" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17"/>
-      <x:c r="B17"/>
-      <x:c r="C17"/>
-      <x:c r="D17"/>
-      <x:c r="E17"/>
-      <x:c r="F17"/>
-      <x:c r="G17"/>
-      <x:c r="H17"/>
-      <x:c r="I17"/>
-      <x:c r="J17"/>
-      <x:c r="K17"/>
-      <x:c r="L17"/>
+      <x:c r="A17" t="str">
+        <x:v>CFG-001</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/72</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>codex/cfg-001-platform-config</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>568b4a8</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>8efb49c</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>WOW-MD PR 46 merged as 9135e2f</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Focused configuration contract 12 of 12; backend full suite 840 passed with 9 skipped; lint typecheck boundary scan Compose validation and production image build passed; production audit has no high or critical findings</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Review and merge after OBS-003 PR 71; retain secrets in environment or secret stores; public tiers must provide S3 bucket secure cookies and disabled Swagger</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>Revert PR 72 and rebuild; all pre-existing environment variables remain compatible and no database rollback is required</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>Public and revenue validation deliberately refuses unsafe provider combinations; existing moderate or low framework-chain dependency findings remain outside this change</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>Ready for Review</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18"/>
@@ -6682,7 +6708,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a6bedf623164e35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23f582faaceb4715"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
CFG-001: centralize typed platform configuration (#72)
* feat: centralize platform configuration

* docs: record OBS-003 merge and CFG-001 handoff

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8363d4ab68c0401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R0483a261dea643fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R619b640a444e489f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R195f9a45aa1c4c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R37d3442a5b6447b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R41d20f48ce894af7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R592db801caa846d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rd035b38cbf2b4e95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8abca5f0300749fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R75446ace44e7456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R21051e6975494f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rf48bf49924d0415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb3fbb1b7131f4bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R5f50b8ce9eaa428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rab64af5fca934ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R77cf6543731f4a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra7a6693082b240a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rcf46b4fa8a0b4b53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rd2de30d3279c46af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R786316df5f8d4f80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R241e6607a82f416d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8109f43b506541fb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1428,13 +1428,13 @@
       </x:c>
       <x:c r="E6" s="34" t="n">
         <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1442,7 +1442,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1518,7 +1518,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1526,7 +1526,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R934f084633e843b0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8633c727178490a"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R068394b04cc4457e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R148b65fbe21b4822"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2457,7 +2457,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F13" s="72" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
         <x:v>Codex</x:v>
@@ -2498,10 +2498,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F14" s="72" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H14" s="26" t="str">
         <x:v>SEC-001</x:v>
@@ -2515,9 +2515,11 @@
       <x:c r="K14" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/14</x:v>
       </x:c>
-      <x:c r="L14" s="26" t="str"/>
+      <x:c r="L14" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/72</x:v>
+      </x:c>
       <x:c r="M14" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
@@ -3952,7 +3954,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a1bd56ba91a45e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf79a22028df0467c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4436,7 +4438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8399ddc4b3a4c2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R463d03379c8749c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4841,7 +4843,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe72213628b64177"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998280114ed2448d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5278,7 +5280,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70539203b8af49a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1c3084fc9484b48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5625,7 +5627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c8a7adfbaa54120"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb6aae68d5d4768"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5964,7 +5966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54d3f5285878445d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf29101dc1fa34c54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6137,7 +6139,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf944248192ee48c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R678a7a4ffc4a4a2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6600,16 +6602,16 @@
         <x:v>codex/obs-003-local-log-platform</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>f5d87f0</x:v>
+        <x:v>dd39ccc</x:v>
       </x:c>
       <x:c r="E16" t="str">
-        <x:v>555a1fe</x:v>
+        <x:v>0d1e02f</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>None</x:v>
+        <x:v>WOW-MD PR 48 merged as 7384378</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>Collector/Loki config validation; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; 7 provisioned alerts; Loki buffer recovery; frontend-restart persistence all pass</x:v>
+        <x:v>Collector and Loki configuration; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; seven alerts; Loki buffer recovery; frontend restart persistence all pass</x:v>
       </x:c>
       <x:c r="H16" t="str">
         <x:v>Set WOW_LOG_DIR and a unique GRAFANA_ADMIN_PASSWORD; start the observability Compose profile; Grafana binds to 127.0.0.1:3300</x:v>
@@ -6618,28 +6620,52 @@
         <x:v>Stop/remove observability containers and revert PR 71; retained host logs are not automatically deleted; application services remain independent</x:v>
       </x:c>
       <x:c r="J16" t="str">
-        <x:v>Single-host logs are not disaster recovery; Vector outage has only bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
+        <x:v>Single-host logs are not disaster recovery; Vector outage has bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>Ready for Review</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L16" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17"/>
-      <x:c r="B17"/>
-      <x:c r="C17"/>
-      <x:c r="D17"/>
-      <x:c r="E17"/>
-      <x:c r="F17"/>
-      <x:c r="G17"/>
-      <x:c r="H17"/>
-      <x:c r="I17"/>
-      <x:c r="J17"/>
-      <x:c r="K17"/>
-      <x:c r="L17"/>
+      <x:c r="A17" t="str">
+        <x:v>CFG-001</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/72</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>codex/cfg-001-platform-config</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>568b4a8</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>8efb49c</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>WOW-MD PR 46 merged as 9135e2f</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Focused configuration contract 12 of 12; backend full suite 840 passed with 9 skipped; lint typecheck boundary scan Compose validation and production image build passed; production audit has no high or critical findings</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Review and merge after OBS-003 PR 71; retain secrets in environment or secret stores; public tiers must provide S3 bucket secure cookies and disabled Swagger</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>Revert PR 72 and rebuild; all pre-existing environment variables remain compatible and no database rollback is required</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>Public and revenue validation deliberately refuses unsafe provider combinations; existing moderate or low framework-chain dependency findings remain outside this change</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>Ready for Review</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18"/>
@@ -6682,7 +6708,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a6bedf623164e35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23f582faaceb4715"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close OBS-003 and CFG-001 tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R21051e6975494f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rf48bf49924d0415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb3fbb1b7131f4bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R5f50b8ce9eaa428d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rab64af5fca934ab5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R77cf6543731f4a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra7a6693082b240a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rcf46b4fa8a0b4b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rd2de30d3279c46af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R786316df5f8d4f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R06bdd98b8e504195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R0314cb2fce054c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R7840a3d36e4349e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R614f37c22c2044e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R2eb5ab7153d047eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd20002fb7c6d4025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rfc64fd97170f458f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R307722b69e2a4a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8a50446223224219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7b58e02b311d41d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8109f43b506541fb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R22278067379f4d04"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1428,7 +1428,7 @@
       </x:c>
       <x:c r="E6" s="34" t="n">
         <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1476,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1484,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1518,7 +1518,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1526,7 +1526,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8633c727178490a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3332e733c449c9"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R148b65fbe21b4822"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3480d53364144423"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2498,7 +2498,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F14" s="72" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
         <x:v>Codex</x:v>
@@ -3954,7 +3954,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf79a22028df0467c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93cd7ee5aae74377"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4438,7 +4438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R463d03379c8749c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref81fec817204068"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4843,7 +4843,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998280114ed2448d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2b0b65139c6464f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5280,7 +5280,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1c3084fc9484b48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb21a8a9ea29344eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5627,7 +5627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb6aae68d5d4768"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67e6017715ed45b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5966,7 +5966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf29101dc1fa34c54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd55c08b656d7427c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6139,7 +6139,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R678a7a4ffc4a4a2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R916cbd6b116241df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6652,7 +6652,7 @@
         <x:v>Focused configuration contract 12 of 12; backend full suite 840 passed with 9 skipped; lint typecheck boundary scan Compose validation and production image build passed; production audit has no high or critical findings</x:v>
       </x:c>
       <x:c r="H17" t="str">
-        <x:v>Review and merge after OBS-003 PR 71; retain secrets in environment or secret stores; public tiers must provide S3 bucket secure cookies and disabled Swagger</x:v>
+        <x:v>Merged after OBS-003 PR 71; retain secrets in environment or secret stores; public tiers must provide S3 bucket secure cookies and disabled Swagger</x:v>
       </x:c>
       <x:c r="I17" t="str">
         <x:v>Revert PR 72 and rebuild; all pre-existing environment variables remain compatible and no database rollback is required</x:v>
@@ -6661,7 +6661,7 @@
         <x:v>Public and revenue validation deliberately refuses unsafe provider combinations; existing moderate or low framework-chain dependency findings remain outside this change</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>Ready for Review</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L17" t="str">
         <x:v>2026-10-06</x:v>
@@ -6708,7 +6708,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23f582faaceb4715"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd921fde77ed74bbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close OBS-003 and CFG-001 tracking (#75)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R21051e6975494f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rf48bf49924d0415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb3fbb1b7131f4bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R5f50b8ce9eaa428d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rab64af5fca934ab5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R77cf6543731f4a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra7a6693082b240a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rcf46b4fa8a0b4b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rd2de30d3279c46af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R786316df5f8d4f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R06bdd98b8e504195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R0314cb2fce054c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R7840a3d36e4349e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R614f37c22c2044e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R2eb5ab7153d047eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd20002fb7c6d4025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rfc64fd97170f458f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R307722b69e2a4a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8a50446223224219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7b58e02b311d41d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8109f43b506541fb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R22278067379f4d04"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1428,7 +1428,7 @@
       </x:c>
       <x:c r="E6" s="34" t="n">
         <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1476,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1484,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1518,7 +1518,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1526,7 +1526,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8633c727178490a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3332e733c449c9"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R148b65fbe21b4822"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3480d53364144423"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2498,7 +2498,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F14" s="72" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
         <x:v>Codex</x:v>
@@ -3954,7 +3954,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf79a22028df0467c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93cd7ee5aae74377"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4438,7 +4438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R463d03379c8749c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref81fec817204068"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4843,7 +4843,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998280114ed2448d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2b0b65139c6464f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5280,7 +5280,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1c3084fc9484b48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb21a8a9ea29344eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5627,7 +5627,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb6aae68d5d4768"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67e6017715ed45b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5966,7 +5966,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf29101dc1fa34c54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd55c08b656d7427c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6139,7 +6139,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R678a7a4ffc4a4a2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R916cbd6b116241df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6652,7 +6652,7 @@
         <x:v>Focused configuration contract 12 of 12; backend full suite 840 passed with 9 skipped; lint typecheck boundary scan Compose validation and production image build passed; production audit has no high or critical findings</x:v>
       </x:c>
       <x:c r="H17" t="str">
-        <x:v>Review and merge after OBS-003 PR 71; retain secrets in environment or secret stores; public tiers must provide S3 bucket secure cookies and disabled Swagger</x:v>
+        <x:v>Merged after OBS-003 PR 71; retain secrets in environment or secret stores; public tiers must provide S3 bucket secure cookies and disabled Swagger</x:v>
       </x:c>
       <x:c r="I17" t="str">
         <x:v>Revert PR 72 and rebuild; all pre-existing environment variables remain compatible and no database rollback is required</x:v>
@@ -6661,7 +6661,7 @@
         <x:v>Public and revenue validation deliberately refuses unsafe provider combinations; existing moderate or low framework-chain dependency findings remain outside this change</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>Ready for Review</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L17" t="str">
         <x:v>2026-10-06</x:v>
@@ -6708,7 +6708,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23f582faaceb4715"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd921fde77ed74bbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record SYNC-003 source intake
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R06bdd98b8e504195"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R0314cb2fce054c28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R7840a3d36e4349e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R614f37c22c2044e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R2eb5ab7153d047eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd20002fb7c6d4025"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rfc64fd97170f458f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R307722b69e2a4a9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8a50446223224219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7b58e02b311d41d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R872375fef45a4c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R74e1c5a6b6054d7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rda48b0bc970f474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R9e9b401f03bf41a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R413b7e69c7f34a8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R5ca11344152442c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rad529d7daee24f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rab67fcd281eb458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R1363de0fec5e4d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R466a400e38ba4e62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R22278067379f4d04"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R459d78fa033343f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1421,7 +1421,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
@@ -1476,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1484,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3332e733c449c9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3a256d09a3f4604"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3480d53364144423"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4590220a4ebb4046"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3459,19 +3459,45 @@
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39"/>
-      <x:c r="B39"/>
-      <x:c r="C39"/>
-      <x:c r="D39"/>
-      <x:c r="E39"/>
-      <x:c r="F39"/>
-      <x:c r="G39"/>
-      <x:c r="H39"/>
-      <x:c r="I39"/>
-      <x:c r="J39"/>
-      <x:c r="K39"/>
-      <x:c r="L39"/>
-      <x:c r="M39"/>
+      <x:c r="A39" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>Integrate committed immersive consumer UI</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>UI/UX synchronization</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F39" s="51" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>SYNC-002</x:v>
+      </x:c>
+      <x:c r="I39" t="str">
+        <x:v>Committed public login registration and consumer portal UI is present in WOW-MD and production without overwriting production hardening</x:v>
+      </x:c>
+      <x:c r="J39" t="str">
+        <x:v>WOW-MD PR 50 and production issue 76</x:v>
+      </x:c>
+      <x:c r="K39" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/76</x:v>
+      </x:c>
+      <x:c r="L39" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40"/>
@@ -3954,7 +3980,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93cd7ee5aae74377"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b7996ecc534f40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4438,7 +4464,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref81fec817204068"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c6cd28a6674496c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4843,7 +4869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2b0b65139c6464f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbd448fc75404e18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5280,7 +5306,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb21a8a9ea29344eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aa44f17600a4d10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5627,7 +5653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67e6017715ed45b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1294d632ba6040b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5966,7 +5992,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd55c08b656d7427c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R355f205229304700"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6133,13 +6159,83 @@
         <x:v>Local main is 21 commits ahead of origin; scheduled GitHub review intentionally sees pushed commits only</x:v>
       </x:c>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="27" t="str">
+        <x:v>CHG-004</x:v>
+      </x:c>
+      <x:c r="B9" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C9" s="27" t="str">
+        <x:v>2ddfaf6b6d55d3e4833f905565d5048f3cd9c010</x:v>
+      </x:c>
+      <x:c r="D9" s="27" t="str">
+        <x:v>frontend/ (40 paths)</x:v>
+      </x:c>
+      <x:c r="E9" s="27" t="str">
+        <x:v>UI/UX and tests</x:v>
+      </x:c>
+      <x:c r="F9" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
+      </x:c>
+      <x:c r="I9" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J9" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K9" s="27" t="str">
+        <x:v>WOW-MD PR 50 published the reviewed 07218b4..8a147a6 UI line; production accepts only the reconciled frontend paths</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="27" t="str">
+        <x:v>CHG-005</x:v>
+      </x:c>
+      <x:c r="B10" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C10" s="27" t="str">
+        <x:v>2ddfaf6b6d55d3e4833f905565d5048f3cd9c010</x:v>
+      </x:c>
+      <x:c r="D10" s="27" t="str">
+        <x:v>docker/docker-compose.preview.yml; docs/wow-consumer-portal-design-preview.html</x:v>
+      </x:c>
+      <x:c r="E10" s="27" t="str">
+        <x:v>Preview-only source artifacts</x:v>
+      </x:c>
+      <x:c r="F10" s="27" t="str">
+        <x:v>Rejected for production</x:v>
+      </x:c>
+      <x:c r="G10" s="27" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="H10" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
+      </x:c>
+      <x:c r="I10" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J10" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K10" s="27" t="str">
+        <x:v>Remain in WOW-MD for design preview use; not part of the production deployment line</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:K3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R916cbd6b116241df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90363bcee4c84e92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6668,18 +6764,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18"/>
-      <x:c r="B18"/>
-      <x:c r="C18"/>
-      <x:c r="D18"/>
-      <x:c r="E18"/>
-      <x:c r="F18"/>
-      <x:c r="G18"/>
-      <x:c r="H18"/>
-      <x:c r="I18"/>
-      <x:c r="J18"/>
-      <x:c r="K18"/>
-      <x:c r="L18"/>
+      <x:c r="A18" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>codex/sync-003-consumer-ui</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>3e05702</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>83c2400</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>WOW-MD PR 50 merged as 2ddfaf6; reviewed local source range 07218b4..8a147a6</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Frontend typecheck; 19 test files and 180 tests; production build; WOW-MD protected build-and-test frontend mobile Docker and CodeQL checks; production protected CI pending</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Rebuild and deploy only the frontend image; smoke public home login registration and bride groom family navigation</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>Revert PR 77 and rebuild the frontend image; no database configuration or infrastructure rollback</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>Live post-deployment visual and role smoke remains; main client bundle is about 1.9 MB raw and 505 KB gzip; source-only preview artifacts were rejected</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>Ready for Review</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19"/>
@@ -6708,7 +6828,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd921fde77ed74bbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8f77c6222d41b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
SYNC-003: synchronize immersive consumer UI (#77)
* feat: synchronize immersive consumer UI

* docs: record SYNC-003 source intake

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R06bdd98b8e504195"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R0314cb2fce054c28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R7840a3d36e4349e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R614f37c22c2044e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R2eb5ab7153d047eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd20002fb7c6d4025"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rfc64fd97170f458f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R307722b69e2a4a9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8a50446223224219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7b58e02b311d41d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R872375fef45a4c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R74e1c5a6b6054d7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rda48b0bc970f474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R9e9b401f03bf41a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R413b7e69c7f34a8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R5ca11344152442c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rad529d7daee24f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rab67fcd281eb458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R1363de0fec5e4d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R466a400e38ba4e62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R22278067379f4d04"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R459d78fa033343f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1421,7 +1421,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
@@ -1476,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1484,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3332e733c449c9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3a256d09a3f4604"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3480d53364144423"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4590220a4ebb4046"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3459,19 +3459,45 @@
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39"/>
-      <x:c r="B39"/>
-      <x:c r="C39"/>
-      <x:c r="D39"/>
-      <x:c r="E39"/>
-      <x:c r="F39"/>
-      <x:c r="G39"/>
-      <x:c r="H39"/>
-      <x:c r="I39"/>
-      <x:c r="J39"/>
-      <x:c r="K39"/>
-      <x:c r="L39"/>
-      <x:c r="M39"/>
+      <x:c r="A39" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>Integrate committed immersive consumer UI</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>UI/UX synchronization</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F39" s="51" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>SYNC-002</x:v>
+      </x:c>
+      <x:c r="I39" t="str">
+        <x:v>Committed public login registration and consumer portal UI is present in WOW-MD and production without overwriting production hardening</x:v>
+      </x:c>
+      <x:c r="J39" t="str">
+        <x:v>WOW-MD PR 50 and production issue 76</x:v>
+      </x:c>
+      <x:c r="K39" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/76</x:v>
+      </x:c>
+      <x:c r="L39" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40"/>
@@ -3954,7 +3980,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93cd7ee5aae74377"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b7996ecc534f40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4438,7 +4464,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref81fec817204068"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c6cd28a6674496c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4843,7 +4869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2b0b65139c6464f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbd448fc75404e18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5280,7 +5306,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb21a8a9ea29344eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aa44f17600a4d10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5627,7 +5653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67e6017715ed45b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1294d632ba6040b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5966,7 +5992,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd55c08b656d7427c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R355f205229304700"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6133,13 +6159,83 @@
         <x:v>Local main is 21 commits ahead of origin; scheduled GitHub review intentionally sees pushed commits only</x:v>
       </x:c>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="27" t="str">
+        <x:v>CHG-004</x:v>
+      </x:c>
+      <x:c r="B9" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C9" s="27" t="str">
+        <x:v>2ddfaf6b6d55d3e4833f905565d5048f3cd9c010</x:v>
+      </x:c>
+      <x:c r="D9" s="27" t="str">
+        <x:v>frontend/ (40 paths)</x:v>
+      </x:c>
+      <x:c r="E9" s="27" t="str">
+        <x:v>UI/UX and tests</x:v>
+      </x:c>
+      <x:c r="F9" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
+      </x:c>
+      <x:c r="I9" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J9" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K9" s="27" t="str">
+        <x:v>WOW-MD PR 50 published the reviewed 07218b4..8a147a6 UI line; production accepts only the reconciled frontend paths</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="27" t="str">
+        <x:v>CHG-005</x:v>
+      </x:c>
+      <x:c r="B10" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C10" s="27" t="str">
+        <x:v>2ddfaf6b6d55d3e4833f905565d5048f3cd9c010</x:v>
+      </x:c>
+      <x:c r="D10" s="27" t="str">
+        <x:v>docker/docker-compose.preview.yml; docs/wow-consumer-portal-design-preview.html</x:v>
+      </x:c>
+      <x:c r="E10" s="27" t="str">
+        <x:v>Preview-only source artifacts</x:v>
+      </x:c>
+      <x:c r="F10" s="27" t="str">
+        <x:v>Rejected for production</x:v>
+      </x:c>
+      <x:c r="G10" s="27" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="H10" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
+      </x:c>
+      <x:c r="I10" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J10" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K10" s="27" t="str">
+        <x:v>Remain in WOW-MD for design preview use; not part of the production deployment line</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:K3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R916cbd6b116241df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90363bcee4c84e92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6668,18 +6764,42 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18"/>
-      <x:c r="B18"/>
-      <x:c r="C18"/>
-      <x:c r="D18"/>
-      <x:c r="E18"/>
-      <x:c r="F18"/>
-      <x:c r="G18"/>
-      <x:c r="H18"/>
-      <x:c r="I18"/>
-      <x:c r="J18"/>
-      <x:c r="K18"/>
-      <x:c r="L18"/>
+      <x:c r="A18" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>codex/sync-003-consumer-ui</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>3e05702</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>83c2400</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>WOW-MD PR 50 merged as 2ddfaf6; reviewed local source range 07218b4..8a147a6</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Frontend typecheck; 19 test files and 180 tests; production build; WOW-MD protected build-and-test frontend mobile Docker and CodeQL checks; production protected CI pending</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Rebuild and deploy only the frontend image; smoke public home login registration and bride groom family navigation</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>Revert PR 77 and rebuild the frontend image; no database configuration or infrastructure rollback</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>Live post-deployment visual and role smoke remains; main client bundle is about 1.9 MB raw and 505 KB gzip; source-only preview artifacts were rejected</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>Ready for Review</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19"/>
@@ -6708,7 +6828,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd921fde77ed74bbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8f77c6222d41b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close SYNC-003 tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R872375fef45a4c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R74e1c5a6b6054d7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rda48b0bc970f474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R9e9b401f03bf41a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R413b7e69c7f34a8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R5ca11344152442c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rad529d7daee24f64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rab67fcd281eb458a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R1363de0fec5e4d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R466a400e38ba4e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3de8f63b82fd420d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rdcd68412a637431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf76ed813c3c24bc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R751a3b7573874a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Red2ac527042549df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1548b4414d134591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R46dbb2d5ef104b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R70db7b490e064955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R4188bb4f27d1483e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R5bcaee5d3b654e90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R459d78fa033343f7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R730326f62e01449f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1476,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1484,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1518,7 +1518,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1526,7 +1526,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3a256d09a3f4604"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae957dcd8c64077"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4590220a4ebb4046"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8da4d947e724249"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3475,7 +3475,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F39" s="51" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G39" t="str">
         <x:v>Codex</x:v>
@@ -3980,7 +3980,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b7996ecc534f40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6f2cb12aa8c4ae3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4464,7 +4464,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c6cd28a6674496c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12f98c5b37834f48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4869,7 +4869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbd448fc75404e18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc00254046549445d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5306,7 +5306,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aa44f17600a4d10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a95c18c1d074114"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5653,7 +5653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1294d632ba6040b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb91ffbe105f74cb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5992,7 +5992,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R355f205229304700"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56bec80054264d49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6235,7 +6235,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90363bcee4c84e92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e363ead270d4cd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6783,10 +6783,10 @@
         <x:v>WOW-MD PR 50 merged as 2ddfaf6; reviewed local source range 07218b4..8a147a6</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>Frontend typecheck; 19 test files and 180 tests; production build; WOW-MD protected build-and-test frontend mobile Docker and CodeQL checks; production protected CI pending</x:v>
+        <x:v>Frontend typecheck; 19 test files and 180 tests; production build; protected backend suite and E2E frontend mobile Docker CodeQL secrets and governance checks passed</x:v>
       </x:c>
       <x:c r="H18" t="str">
-        <x:v>Rebuild and deploy only the frontend image; smoke public home login registration and bride groom family navigation</x:v>
+        <x:v>Merged; rebuild and deploy only the frontend image then smoke public home login registration and bride groom family navigation</x:v>
       </x:c>
       <x:c r="I18" t="str">
         <x:v>Revert PR 77 and rebuild the frontend image; no database configuration or infrastructure rollback</x:v>
@@ -6795,7 +6795,7 @@
         <x:v>Live post-deployment visual and role smoke remains; main client bundle is about 1.9 MB raw and 505 KB gzip; source-only preview artifacts were rejected</x:v>
       </x:c>
       <x:c r="K18" t="str">
-        <x:v>Ready for Review</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L18" t="str">
         <x:v>2026-10-06</x:v>
@@ -6828,7 +6828,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8f77c6222d41b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc946bbe4f82b463a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close SYNC-003 tracking (#78)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R872375fef45a4c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R74e1c5a6b6054d7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rda48b0bc970f474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R9e9b401f03bf41a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R413b7e69c7f34a8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R5ca11344152442c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rad529d7daee24f64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rab67fcd281eb458a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R1363de0fec5e4d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R466a400e38ba4e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3de8f63b82fd420d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rdcd68412a637431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf76ed813c3c24bc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R751a3b7573874a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Red2ac527042549df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1548b4414d134591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R46dbb2d5ef104b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R70db7b490e064955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R4188bb4f27d1483e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R5bcaee5d3b654e90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R459d78fa033343f7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R730326f62e01449f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1476,7 +1476,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1484,7 +1484,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1518,7 +1518,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1526,7 +1526,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3a256d09a3f4604"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae957dcd8c64077"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4590220a4ebb4046"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8da4d947e724249"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3475,7 +3475,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F39" s="51" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G39" t="str">
         <x:v>Codex</x:v>
@@ -3980,7 +3980,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b7996ecc534f40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6f2cb12aa8c4ae3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4464,7 +4464,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c6cd28a6674496c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12f98c5b37834f48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4869,7 +4869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbd448fc75404e18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc00254046549445d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5306,7 +5306,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aa44f17600a4d10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a95c18c1d074114"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5653,7 +5653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1294d632ba6040b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb91ffbe105f74cb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5992,7 +5992,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R355f205229304700"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56bec80054264d49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6235,7 +6235,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90363bcee4c84e92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e363ead270d4cd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6783,10 +6783,10 @@
         <x:v>WOW-MD PR 50 merged as 2ddfaf6; reviewed local source range 07218b4..8a147a6</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>Frontend typecheck; 19 test files and 180 tests; production build; WOW-MD protected build-and-test frontend mobile Docker and CodeQL checks; production protected CI pending</x:v>
+        <x:v>Frontend typecheck; 19 test files and 180 tests; production build; protected backend suite and E2E frontend mobile Docker CodeQL secrets and governance checks passed</x:v>
       </x:c>
       <x:c r="H18" t="str">
-        <x:v>Rebuild and deploy only the frontend image; smoke public home login registration and bride groom family navigation</x:v>
+        <x:v>Merged; rebuild and deploy only the frontend image then smoke public home login registration and bride groom family navigation</x:v>
       </x:c>
       <x:c r="I18" t="str">
         <x:v>Revert PR 77 and rebuild the frontend image; no database configuration or infrastructure rollback</x:v>
@@ -6795,7 +6795,7 @@
         <x:v>Live post-deployment visual and role smoke remains; main client bundle is about 1.9 MB raw and 505 KB gzip; source-only preview artifacts were rejected</x:v>
       </x:c>
       <x:c r="K18" t="str">
-        <x:v>Ready for Review</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L18" t="str">
         <x:v>2026-10-06</x:v>
@@ -6828,7 +6828,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8f77c6222d41b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc946bbe4f82b463a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
deps: finalize exact source lock synchronization
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3de8f63b82fd420d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rdcd68412a637431a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf76ed813c3c24bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R751a3b7573874a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Red2ac527042549df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1548b4414d134591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R46dbb2d5ef104b6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R70db7b490e064955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R4188bb4f27d1483e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R5bcaee5d3b654e90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb66fa110142f4493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R278300a9d37147eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R916ce95896314575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R1dc83eb342434ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R4b56ed2da5e8408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R578d06b1a37b4258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R21b62ecafdd34f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re1101413a5594e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R41024dbb5e2940a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R6b626566f817463d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R730326f62e01449f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d9ee8990eeb43a3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae957dcd8c64077"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4505c1f091224785"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8da4d947e724249"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc4fcdd7c5647e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3980,7 +3980,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6f2cb12aa8c4ae3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2839a1a98d304860"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4464,7 +4464,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12f98c5b37834f48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08c672e326c947c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4869,7 +4869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc00254046549445d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e0a146b3665477e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5306,7 +5306,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a95c18c1d074114"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89e8a5d8aab64c7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5653,7 +5653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb91ffbe105f74cb5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c0531a9184d4e9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5992,7 +5992,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56bec80054264d49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14665dc032fd4736"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6229,13 +6229,48 @@
         <x:v>Remain in WOW-MD for design preview use; not part of the production deployment line</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
+        <x:v>CHG-006</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C11" s="27" t="str">
+        <x:v>51790dfa57126a64e31e5b605ddccca85cd09b85</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="str">
+        <x:v>frontend/package-lock.json</x:v>
+      </x:c>
+      <x:c r="E11" s="27" t="str">
+        <x:v>Dependency lockfile</x:v>
+      </x:c>
+      <x:c r="F11" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="str">
+        <x:v>DEP-001</x:v>
+      </x:c>
+      <x:c r="H11" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/81</x:v>
+      </x:c>
+      <x:c r="I11" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J11" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K11" s="27" t="str">
+        <x:v>WOW-MD PR 49 and production PRs 79 and 81 reconcile source-map-js 1.2.2 and the exact frontend lock graph</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:K3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e363ead270d4cd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e7de65b578c42fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6476,25 +6511,25 @@
         <x:v>1ecbfdf</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>WOW-MD PR 39 head d8ef995</x:v>
+        <x:v>WOW-MD PR 39 head d8ef995; WOW-MD PR 49 merged as 51790df; supplemental production PRs 73, 79, and 81</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>Backend clean install typecheck lint build and 792 tests pass with 9 skipped; frontend clean install typecheck 173 tests build and 10 Playwright flows pass; runtime audits: backend 0 critical/0 high frontend 0; exact-ID mobile gate passes; production and source protected CI pass</x:v>
+        <x:v>Backend and frontend production audits have no high or critical findings; frontend clean install typecheck 180 tests build passed on PR 81; exact frontend trees match</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>No deployment before review and merge; after merge let GitHub rescan manifests and confirm alert counts and audit gates on main</x:v>
+        <x:v>Merged; no runtime deployment is required for the PR 81 development-only lock reconciliation; retain normal rebuild verification</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>Revert PR 59; restore prior lockfiles and packages; retain the audit report for comparison</x:v>
+        <x:v>Revert the affected supplemental PR and restore its paired WOW-MD lockfile if clean install or build regresses</x:v>
       </x:c>
       <x:c r="J10" t="str">
-        <x:v>Backend moderate/low build-tool advisories and four exact no-fix Expo advisory roots remain; forced NestJS 12 and Expo downgrades were tested and rejected as unsafe</x:v>
+        <x:v>Three moderate mammoth-chain findings and four exact no-fix Expo advisory roots remain; forced breaking downgrades remain rejected</x:v>
       </x:c>
       <x:c r="K10" s="75" t="str">
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L10" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6828,7 +6863,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc946bbe4f82b463a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5c780db6fa46b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
DEP: finalize exact source lock synchronization (#81)
* deps: finalize exact source lock synchronization

* ci: refresh mirror gate metadata

* ci: apply traceability template

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3de8f63b82fd420d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rdcd68412a637431a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf76ed813c3c24bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R751a3b7573874a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Red2ac527042549df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1548b4414d134591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R46dbb2d5ef104b6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R70db7b490e064955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R4188bb4f27d1483e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R5bcaee5d3b654e90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb66fa110142f4493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R278300a9d37147eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R916ce95896314575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R1dc83eb342434ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R4b56ed2da5e8408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R578d06b1a37b4258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R21b62ecafdd34f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re1101413a5594e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R41024dbb5e2940a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R6b626566f817463d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1016,7 +1016,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R730326f62e01449f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d9ee8990eeb43a3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1625,7 +1625,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae957dcd8c64077"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4505c1f091224785"/>
 </x:worksheet>
 </file>
 
@@ -2085,7 +2085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8da4d947e724249"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc4fcdd7c5647e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3980,7 +3980,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6f2cb12aa8c4ae3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2839a1a98d304860"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4464,7 +4464,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12f98c5b37834f48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08c672e326c947c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4869,7 +4869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc00254046549445d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e0a146b3665477e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5306,7 +5306,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a95c18c1d074114"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89e8a5d8aab64c7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5653,7 +5653,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb91ffbe105f74cb5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c0531a9184d4e9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5992,7 +5992,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56bec80054264d49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14665dc032fd4736"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6229,13 +6229,48 @@
         <x:v>Remain in WOW-MD for design preview use; not part of the production deployment line</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="27" t="str">
+        <x:v>CHG-006</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C11" s="27" t="str">
+        <x:v>51790dfa57126a64e31e5b605ddccca85cd09b85</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="str">
+        <x:v>frontend/package-lock.json</x:v>
+      </x:c>
+      <x:c r="E11" s="27" t="str">
+        <x:v>Dependency lockfile</x:v>
+      </x:c>
+      <x:c r="F11" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="str">
+        <x:v>DEP-001</x:v>
+      </x:c>
+      <x:c r="H11" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/81</x:v>
+      </x:c>
+      <x:c r="I11" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J11" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K11" s="27" t="str">
+        <x:v>WOW-MD PR 49 and production PRs 79 and 81 reconcile source-map-js 1.2.2 and the exact frontend lock graph</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:K3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e363ead270d4cd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e7de65b578c42fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6476,25 +6511,25 @@
         <x:v>1ecbfdf</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>WOW-MD PR 39 head d8ef995</x:v>
+        <x:v>WOW-MD PR 39 head d8ef995; WOW-MD PR 49 merged as 51790df; supplemental production PRs 73, 79, and 81</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>Backend clean install typecheck lint build and 792 tests pass with 9 skipped; frontend clean install typecheck 173 tests build and 10 Playwright flows pass; runtime audits: backend 0 critical/0 high frontend 0; exact-ID mobile gate passes; production and source protected CI pass</x:v>
+        <x:v>Backend and frontend production audits have no high or critical findings; frontend clean install typecheck 180 tests build passed on PR 81; exact frontend trees match</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>No deployment before review and merge; after merge let GitHub rescan manifests and confirm alert counts and audit gates on main</x:v>
+        <x:v>Merged; no runtime deployment is required for the PR 81 development-only lock reconciliation; retain normal rebuild verification</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>Revert PR 59; restore prior lockfiles and packages; retain the audit report for comparison</x:v>
+        <x:v>Revert the affected supplemental PR and restore its paired WOW-MD lockfile if clean install or build regresses</x:v>
       </x:c>
       <x:c r="J10" t="str">
-        <x:v>Backend moderate/low build-tool advisories and four exact no-fix Expo advisory roots remain; forced NestJS 12 and Expo downgrades were tested and rejected as unsafe</x:v>
+        <x:v>Three moderate mammoth-chain findings and four exact no-fix Expo advisory roots remain; forced breaking downgrades remain rejected</x:v>
       </x:c>
       <x:c r="K10" s="75" t="str">
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L10" t="str">
-        <x:v>2026-10-05</x:v>
+        <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6828,7 +6863,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc946bbe4f82b463a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5c780db6fa46b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize dependency tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb66fa110142f4493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R278300a9d37147eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R916ce95896314575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R1dc83eb342434ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R4b56ed2da5e8408d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R578d06b1a37b4258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R21b62ecafdd34f52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re1101413a5594e5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R41024dbb5e2940a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R6b626566f817463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4dac9e61b8f647e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R726792ba74a444a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rac8d13ad987e4019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Raf4371b23e3349cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R40cff3d2fe8b4e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R259d15eeee2647ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R83ec67f2a1ad4bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rae9434a4a6d442b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rc5bbb6216a3d4213"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rd9227feb95244459"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,23 +68,8 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF16794A"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF7A4B00"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FFB42318"/>
-      <x:name val="Arial"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -96,88 +81,23 @@
         <x:fgColor rgb="FF6E1026"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
   <x:borders count="7">
-    <x:border/>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -186,35 +106,53 @@
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9CDD0"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFD9CDD0"/>
       </x:top>
       <x:bottom style="thin">
         <x:color rgb="FFD9CDD0"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFD9CDD0"/>
       </x:top>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="76">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -303,102 +241,6 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -410,7 +252,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -420,7 +262,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -430,7 +272,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -441,7 +283,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -451,7 +293,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -461,7 +303,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -472,7 +314,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -482,7 +324,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -492,7 +334,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -503,7 +345,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -513,7 +355,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -523,7 +365,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -534,7 +376,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -544,7 +386,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -554,7 +396,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -565,7 +407,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -575,7 +417,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -585,7 +427,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -595,7 +437,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -605,7 +447,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -616,7 +458,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -626,7 +468,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -636,7 +478,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -646,7 +488,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -656,7 +498,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -667,7 +509,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -677,7 +519,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -687,7 +529,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -697,7 +539,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -707,7 +549,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -718,7 +560,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -728,7 +570,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -738,7 +580,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -748,7 +590,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -758,7 +600,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -769,7 +611,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -779,7 +621,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -789,7 +631,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -800,7 +642,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -810,7 +652,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -1016,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d9ee8990eeb43a3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08294142a8e34b91"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1026,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1047,7 +889,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Requirement"/>
@@ -1062,7 +904,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Layer"/>
@@ -1077,7 +919,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -1127,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1146,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1166,7 +1008,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1393,7 +1235,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-06. Reconciled to canonical registers and final merged PR/issue state.</x:v>
+        <x:v>As of 2026-10-06. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1421,19 +1263,21 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>34</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$41)</x:f>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$41,"P0",'Open Items'!$F$6:$F$41,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
+        <x:f>B7</x:f>
         <x:v>21</x:v>
       </x:c>
     </x:row>
@@ -1442,6 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1455,6 +1300,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H7" s="39" t="n">
+        <x:f>B8</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1463,19 +1309,21 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$18,"Open")</x:f>
+        <x:f>COUNTIF(Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
+        <x:f>B9</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1484,19 +1332,21 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$18,"P0",Risks!$H$6:$H$18,"Open")</x:f>
+        <x:f>COUNTIFS(Risks!$E$6:$E$19,"P0",Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H9" s="39" t="n">
+        <x:f>B10</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1505,20 +1355,22 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIF(Requirements!$G$6:$G$23,"Approved")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF(Requirements!$G$6:$G$27,"Approved")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G10" s="39" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>12</x:v>
+        <x:f>B11</x:f>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1526,7 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>12</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Done")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1625,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4505c1f091224785"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903a4fe60ae145b1"/>
 </x:worksheet>
 </file>
 
@@ -2047,36 +1900,62 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="27" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>DOC-015</x:v>
       </x:c>
-      <x:c r="B20" s="27" t="str">
-        <x:v>Zoho Mail SMTP operating guide</x:v>
-      </x:c>
-      <x:c r="C20" s="27" t="str">
+      <x:c r="B20" s="26" t="str">
+        <x:v>Zoho SSO and mail operating guide</x:v>
+      </x:c>
+      <x:c r="C20" s="26" t="str">
         <x:v>docs/operations/zoho-mail.md</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="str">
+      <x:c r="D20" s="26" t="str">
         <x:v>Security and operations</x:v>
       </x:c>
-      <x:c r="E20" s="27" t="str">
+      <x:c r="E20" s="26" t="str">
         <x:v>Approved candidate</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>Quarterly or provider change</x:v>
       </x:c>
-      <x:c r="G20" s="27" t="str">
-        <x:v>2026-10-04</x:v>
-      </x:c>
-      <x:c r="H20" s="27" t="str">
-        <x:v>SEC-001 OPS-003</x:v>
+      <x:c r="G20" s="26" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="H20" s="26" t="str">
+        <x:v>SEC-001 AUTH-001 OPS-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="27" t="str">
+        <x:v>DOC-016</x:v>
+      </x:c>
+      <x:c r="B21" s="27" t="str">
+        <x:v>Dependency remediation record</x:v>
+      </x:c>
+      <x:c r="C21" s="27" t="str">
+        <x:v>docs/security/dependency-remediation-2026-10-04.md</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>Approved candidate</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="str">
+        <x:v>Each dependency change</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="str">
+        <x:v>DEP-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E20">
+  <x:conditionalFormatting sqref="E6:E21">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -2085,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc4fcdd7c5647e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16e3b18f8eff45a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2179,7 +2058,7 @@
       <x:c r="E6" s="25" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F6" s="70" t="str">
+      <x:c r="F6" s="25" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
@@ -2218,7 +2097,7 @@
       <x:c r="E7" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F7" s="71" t="str">
+      <x:c r="F7" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G7" s="26" t="str">
@@ -2259,7 +2138,7 @@
       <x:c r="E8" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F8" s="71" t="str">
+      <x:c r="F8" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
@@ -2298,7 +2177,7 @@
       <x:c r="E9" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F9" s="71" t="str">
+      <x:c r="F9" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G9" s="26" t="str">
@@ -2337,7 +2216,7 @@
       <x:c r="E10" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F10" s="71" t="str">
+      <x:c r="F10" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
@@ -2376,7 +2255,7 @@
       <x:c r="E11" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F11" s="71" t="str">
+      <x:c r="F11" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
@@ -2417,7 +2296,7 @@
       <x:c r="E12" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F12" s="72" t="str">
+      <x:c r="F12" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G12" s="26" t="str">
@@ -2456,7 +2335,7 @@
       <x:c r="E13" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F13" s="72" t="str">
+      <x:c r="F13" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
@@ -2497,7 +2376,7 @@
       <x:c r="E14" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F14" s="72" t="str">
+      <x:c r="F14" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
@@ -2538,7 +2417,7 @@
       <x:c r="E15" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F15" s="72" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G15" s="26" t="str">
@@ -2577,7 +2456,7 @@
       <x:c r="E16" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F16" s="72" t="str">
+      <x:c r="F16" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G16" s="26" t="str">
@@ -2616,7 +2495,7 @@
       <x:c r="E17" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F17" s="72" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G17" s="26" t="str">
@@ -2655,7 +2534,7 @@
       <x:c r="E18" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F18" s="72" t="str">
+      <x:c r="F18" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G18" s="26" t="str">
@@ -2694,7 +2573,7 @@
       <x:c r="E19" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F19" s="72" t="str">
+      <x:c r="F19" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G19" s="26" t="str">
@@ -2733,7 +2612,7 @@
       <x:c r="E20" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F20" s="72" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G20" s="26" t="str">
@@ -2772,7 +2651,7 @@
       <x:c r="E21" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F21" s="72" t="str">
+      <x:c r="F21" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G21" s="26" t="str">
@@ -2811,7 +2690,7 @@
       <x:c r="E22" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F22" s="72" t="str">
+      <x:c r="F22" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G22" s="26" t="str">
@@ -2850,7 +2729,7 @@
       <x:c r="E23" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F23" s="72" t="str">
+      <x:c r="F23" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G23" s="26" t="str">
@@ -2889,7 +2768,7 @@
       <x:c r="E24" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F24" s="72" t="str">
+      <x:c r="F24" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G24" s="26" t="str">
@@ -2928,7 +2807,7 @@
       <x:c r="E25" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F25" s="72" t="str">
+      <x:c r="F25" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G25" s="26" t="str">
@@ -2967,7 +2846,7 @@
       <x:c r="E26" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F26" s="72" t="str">
+      <x:c r="F26" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G26" s="26" t="str">
@@ -3006,7 +2885,7 @@
       <x:c r="E27" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F27" s="72" t="str">
+      <x:c r="F27" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G27" s="26" t="str">
@@ -3045,7 +2924,7 @@
       <x:c r="E28" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F28" s="72" t="str">
+      <x:c r="F28" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G28" s="26" t="str">
@@ -3084,7 +2963,7 @@
       <x:c r="E29" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F29" s="72" t="str">
+      <x:c r="F29" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G29" s="26" t="str">
@@ -3123,7 +3002,7 @@
       <x:c r="E30" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F30" s="72" t="str">
+      <x:c r="F30" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G30" s="26" t="str">
@@ -3162,7 +3041,7 @@
       <x:c r="E31" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F31" s="72" t="str">
+      <x:c r="F31" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G31" s="26" t="str">
@@ -3199,7 +3078,7 @@
       <x:c r="E32" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F32" s="73" t="str">
+      <x:c r="F32" s="26" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G32" s="26" t="str">
@@ -3240,7 +3119,7 @@
       <x:c r="E33" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F33" s="72" t="str">
+      <x:c r="F33" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G33" s="26" t="str">
@@ -3277,7 +3156,7 @@
       <x:c r="E34" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F34" s="72" t="str">
+      <x:c r="F34" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G34" s="26" t="str">
@@ -3316,7 +3195,7 @@
       <x:c r="E35" s="26" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F35" s="72" t="str">
+      <x:c r="F35" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G35" s="26" t="str">
@@ -3355,7 +3234,7 @@
       <x:c r="E36" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F36" s="71" t="str">
+      <x:c r="F36" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G36" s="26" t="str">
@@ -3379,599 +3258,216 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
-      <x:c r="A37" s="27" t="str">
+      <x:c r="A37" s="26" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B37" s="27" t="str">
+      <x:c r="B37" s="26" t="str">
         <x:v>Establish SDLC knowledge and tracking system</x:v>
       </x:c>
-      <x:c r="C37" s="27" t="str">
+      <x:c r="C37" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="D37" s="27" t="str">
+      <x:c r="D37" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="E37" s="27" t="str">
+      <x:c r="E37" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F37" s="74" t="str">
+      <x:c r="F37" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G37" s="27" t="str">
+      <x:c r="G37" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H37" s="27" t="str"/>
-      <x:c r="I37" s="27" t="str">
+      <x:c r="H37" s="26" t="str"/>
+      <x:c r="I37" s="26" t="str">
         <x:v>Markdown CSV Excel issues PR protocol and Obsidian index are linked and verified</x:v>
       </x:c>
-      <x:c r="J37" s="27" t="str">
+      <x:c r="J37" s="26" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K37" s="27" t="str">
+      <x:c r="K37" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/37</x:v>
       </x:c>
-      <x:c r="L37" s="27" t="str">
+      <x:c r="L37" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
-      <x:c r="M37" s="30" t="str">
+      <x:c r="M37" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" t="str">
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="26" t="str">
         <x:v>GOV-003</x:v>
       </x:c>
-      <x:c r="B38" t="str">
+      <x:c r="B38" s="26" t="str">
         <x:v>Reconcile authentication and dependency tracking</x:v>
       </x:c>
-      <x:c r="C38" t="str">
+      <x:c r="C38" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="D38" t="str">
+      <x:c r="D38" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="E38" t="str">
+      <x:c r="E38" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F38" s="75" t="str">
+      <x:c r="F38" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G38" t="str">
+      <x:c r="G38" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H38" t="str">
+      <x:c r="H38" s="26" t="str">
         <x:v>SEC-001,DEP-001</x:v>
       </x:c>
-      <x:c r="I38" t="str">
+      <x:c r="I38" s="26" t="str">
         <x:v>Canonical registers workbook and operating guidance match the implemented authentication policy and dependency evidence</x:v>
       </x:c>
-      <x:c r="J38" t="str">
+      <x:c r="J38" s="26" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K38" t="str">
+      <x:c r="K38" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/60</x:v>
       </x:c>
-      <x:c r="L38" t="str">
+      <x:c r="L38" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
       </x:c>
-      <x:c r="M38" t="str">
+      <x:c r="M38" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" t="str">
+    <x:row r="39" ht="30" customHeight="1">
+      <x:c r="A39" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="B39" t="str">
+      <x:c r="B39" s="26" t="str">
         <x:v>Integrate committed immersive consumer UI</x:v>
       </x:c>
-      <x:c r="C39" t="str">
+      <x:c r="C39" s="26" t="str">
         <x:v>Source intake</x:v>
       </x:c>
-      <x:c r="D39" t="str">
+      <x:c r="D39" s="26" t="str">
         <x:v>UI/UX synchronization</x:v>
       </x:c>
-      <x:c r="E39" t="str">
+      <x:c r="E39" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F39" s="51" t="str">
+      <x:c r="F39" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G39" t="str">
+      <x:c r="G39" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H39" t="str">
+      <x:c r="H39" s="26" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="I39" t="str">
+      <x:c r="I39" s="26" t="str">
         <x:v>Committed public login registration and consumer portal UI is present in WOW-MD and production without overwriting production hardening</x:v>
       </x:c>
-      <x:c r="J39" t="str">
+      <x:c r="J39" s="26" t="str">
         <x:v>WOW-MD PR 50 and production issue 76</x:v>
       </x:c>
-      <x:c r="K39" t="str">
+      <x:c r="K39" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/76</x:v>
       </x:c>
-      <x:c r="L39" t="str">
+      <x:c r="L39" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
       </x:c>
-      <x:c r="M39" t="str">
+      <x:c r="M39" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40"/>
-      <x:c r="B40"/>
-      <x:c r="C40"/>
-      <x:c r="D40"/>
-      <x:c r="E40"/>
-      <x:c r="F40"/>
-      <x:c r="G40"/>
-      <x:c r="H40"/>
-      <x:c r="I40"/>
-      <x:c r="J40"/>
-      <x:c r="K40"/>
-      <x:c r="L40"/>
-      <x:c r="M40"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41"/>
-      <x:c r="B41"/>
-      <x:c r="C41"/>
-      <x:c r="D41"/>
-      <x:c r="E41"/>
-      <x:c r="F41"/>
-      <x:c r="G41"/>
-      <x:c r="H41"/>
-      <x:c r="I41"/>
-      <x:c r="J41"/>
-      <x:c r="K41"/>
-      <x:c r="L41"/>
-      <x:c r="M41"/>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42"/>
-      <x:c r="B42"/>
-      <x:c r="C42"/>
-      <x:c r="D42"/>
-      <x:c r="E42"/>
-      <x:c r="F42"/>
-      <x:c r="G42"/>
-      <x:c r="H42"/>
-      <x:c r="I42"/>
-      <x:c r="J42"/>
-      <x:c r="K42"/>
-      <x:c r="L42"/>
-      <x:c r="M42"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43"/>
-      <x:c r="B43"/>
-      <x:c r="C43"/>
-      <x:c r="D43"/>
-      <x:c r="E43"/>
-      <x:c r="F43"/>
-      <x:c r="G43"/>
-      <x:c r="H43"/>
-      <x:c r="I43"/>
-      <x:c r="J43"/>
-      <x:c r="K43"/>
-      <x:c r="L43"/>
-      <x:c r="M43"/>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44"/>
-      <x:c r="B44"/>
-      <x:c r="C44"/>
-      <x:c r="D44"/>
-      <x:c r="E44"/>
-      <x:c r="F44"/>
-      <x:c r="G44"/>
-      <x:c r="H44"/>
-      <x:c r="I44"/>
-      <x:c r="J44"/>
-      <x:c r="K44"/>
-      <x:c r="L44"/>
-      <x:c r="M44"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45"/>
-      <x:c r="B45"/>
-      <x:c r="C45"/>
-      <x:c r="D45"/>
-      <x:c r="E45"/>
-      <x:c r="F45"/>
-      <x:c r="G45"/>
-      <x:c r="H45"/>
-      <x:c r="I45"/>
-      <x:c r="J45"/>
-      <x:c r="K45"/>
-      <x:c r="L45"/>
-      <x:c r="M45"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46"/>
-      <x:c r="B46"/>
-      <x:c r="C46"/>
-      <x:c r="D46"/>
-      <x:c r="E46"/>
-      <x:c r="F46"/>
-      <x:c r="G46"/>
-      <x:c r="H46"/>
-      <x:c r="I46"/>
-      <x:c r="J46"/>
-      <x:c r="K46"/>
-      <x:c r="L46"/>
-      <x:c r="M46"/>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47"/>
-      <x:c r="B47"/>
-      <x:c r="C47"/>
-      <x:c r="D47"/>
-      <x:c r="E47"/>
-      <x:c r="F47"/>
-      <x:c r="G47"/>
-      <x:c r="H47"/>
-      <x:c r="I47"/>
-      <x:c r="J47"/>
-      <x:c r="K47"/>
-      <x:c r="L47"/>
-      <x:c r="M47"/>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48"/>
-      <x:c r="B48"/>
-      <x:c r="C48"/>
-      <x:c r="D48"/>
-      <x:c r="E48"/>
-      <x:c r="F48"/>
-      <x:c r="G48"/>
-      <x:c r="H48"/>
-      <x:c r="I48"/>
-      <x:c r="J48"/>
-      <x:c r="K48"/>
-      <x:c r="L48"/>
-      <x:c r="M48"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49"/>
-      <x:c r="B49"/>
-      <x:c r="C49"/>
-      <x:c r="D49"/>
-      <x:c r="E49"/>
-      <x:c r="F49"/>
-      <x:c r="G49"/>
-      <x:c r="H49"/>
-      <x:c r="I49"/>
-      <x:c r="J49"/>
-      <x:c r="K49"/>
-      <x:c r="L49"/>
-      <x:c r="M49"/>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50"/>
-      <x:c r="B50"/>
-      <x:c r="C50"/>
-      <x:c r="D50"/>
-      <x:c r="E50"/>
-      <x:c r="F50"/>
-      <x:c r="G50"/>
-      <x:c r="H50"/>
-      <x:c r="I50"/>
-      <x:c r="J50"/>
-      <x:c r="K50"/>
-      <x:c r="L50"/>
-      <x:c r="M50"/>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51"/>
-      <x:c r="B51"/>
-      <x:c r="C51"/>
-      <x:c r="D51"/>
-      <x:c r="E51"/>
-      <x:c r="F51"/>
-      <x:c r="G51"/>
-      <x:c r="H51"/>
-      <x:c r="I51"/>
-      <x:c r="J51"/>
-      <x:c r="K51"/>
-      <x:c r="L51"/>
-      <x:c r="M51"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52"/>
-      <x:c r="B52"/>
-      <x:c r="C52"/>
-      <x:c r="D52"/>
-      <x:c r="E52"/>
-      <x:c r="F52"/>
-      <x:c r="G52"/>
-      <x:c r="H52"/>
-      <x:c r="I52"/>
-      <x:c r="J52"/>
-      <x:c r="K52"/>
-      <x:c r="L52"/>
-      <x:c r="M52"/>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53"/>
-      <x:c r="B53"/>
-      <x:c r="C53"/>
-      <x:c r="D53"/>
-      <x:c r="E53"/>
-      <x:c r="F53"/>
-      <x:c r="G53"/>
-      <x:c r="H53"/>
-      <x:c r="I53"/>
-      <x:c r="J53"/>
-      <x:c r="K53"/>
-      <x:c r="L53"/>
-      <x:c r="M53"/>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54"/>
-      <x:c r="B54"/>
-      <x:c r="C54"/>
-      <x:c r="D54"/>
-      <x:c r="E54"/>
-      <x:c r="F54"/>
-      <x:c r="G54"/>
-      <x:c r="H54"/>
-      <x:c r="I54"/>
-      <x:c r="J54"/>
-      <x:c r="K54"/>
-      <x:c r="L54"/>
-      <x:c r="M54"/>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55"/>
-      <x:c r="B55"/>
-      <x:c r="C55"/>
-      <x:c r="D55"/>
-      <x:c r="E55"/>
-      <x:c r="F55"/>
-      <x:c r="G55"/>
-      <x:c r="H55"/>
-      <x:c r="I55"/>
-      <x:c r="J55"/>
-      <x:c r="K55"/>
-      <x:c r="L55"/>
-      <x:c r="M55"/>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56"/>
-      <x:c r="B56"/>
-      <x:c r="C56"/>
-      <x:c r="D56"/>
-      <x:c r="E56"/>
-      <x:c r="F56"/>
-      <x:c r="G56"/>
-      <x:c r="H56"/>
-      <x:c r="I56"/>
-      <x:c r="J56"/>
-      <x:c r="K56"/>
-      <x:c r="L56"/>
-      <x:c r="M56"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57"/>
-      <x:c r="B57"/>
-      <x:c r="C57"/>
-      <x:c r="D57"/>
-      <x:c r="E57"/>
-      <x:c r="F57"/>
-      <x:c r="G57"/>
-      <x:c r="H57"/>
-      <x:c r="I57"/>
-      <x:c r="J57"/>
-      <x:c r="K57"/>
-      <x:c r="L57"/>
-      <x:c r="M57"/>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58"/>
-      <x:c r="B58"/>
-      <x:c r="C58"/>
-      <x:c r="D58"/>
-      <x:c r="E58"/>
-      <x:c r="F58"/>
-      <x:c r="G58"/>
-      <x:c r="H58"/>
-      <x:c r="I58"/>
-      <x:c r="J58"/>
-      <x:c r="K58"/>
-      <x:c r="L58"/>
-      <x:c r="M58"/>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59"/>
-      <x:c r="B59"/>
-      <x:c r="C59"/>
-      <x:c r="D59"/>
-      <x:c r="E59"/>
-      <x:c r="F59"/>
-      <x:c r="G59"/>
-      <x:c r="H59"/>
-      <x:c r="I59"/>
-      <x:c r="J59"/>
-      <x:c r="K59"/>
-      <x:c r="L59"/>
-      <x:c r="M59"/>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60"/>
-      <x:c r="B60"/>
-      <x:c r="C60"/>
-      <x:c r="D60"/>
-      <x:c r="E60"/>
-      <x:c r="F60"/>
-      <x:c r="G60"/>
-      <x:c r="H60"/>
-      <x:c r="I60"/>
-      <x:c r="J60"/>
-      <x:c r="K60"/>
-      <x:c r="L60"/>
-      <x:c r="M60"/>
-    </x:row>
-    <x:row r="61">
-      <x:c r="A61"/>
-      <x:c r="B61"/>
-      <x:c r="C61"/>
-      <x:c r="D61"/>
-      <x:c r="E61"/>
-      <x:c r="F61"/>
-      <x:c r="G61"/>
-      <x:c r="H61"/>
-      <x:c r="I61"/>
-      <x:c r="J61"/>
-      <x:c r="K61"/>
-      <x:c r="L61"/>
-      <x:c r="M61"/>
-    </x:row>
-    <x:row r="62">
-      <x:c r="A62"/>
-      <x:c r="B62"/>
-      <x:c r="C62"/>
-      <x:c r="D62"/>
-      <x:c r="E62"/>
-      <x:c r="F62"/>
-      <x:c r="G62"/>
-      <x:c r="H62"/>
-      <x:c r="I62"/>
-      <x:c r="J62"/>
-      <x:c r="K62"/>
-      <x:c r="L62"/>
-      <x:c r="M62"/>
-    </x:row>
-    <x:row r="63">
-      <x:c r="A63"/>
-      <x:c r="B63"/>
-      <x:c r="C63"/>
-      <x:c r="D63"/>
-      <x:c r="E63"/>
-      <x:c r="F63"/>
-      <x:c r="G63"/>
-      <x:c r="H63"/>
-      <x:c r="I63"/>
-      <x:c r="J63"/>
-      <x:c r="K63"/>
-      <x:c r="L63"/>
-      <x:c r="M63"/>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64"/>
-      <x:c r="B64"/>
-      <x:c r="C64"/>
-      <x:c r="D64"/>
-      <x:c r="E64"/>
-      <x:c r="F64"/>
-      <x:c r="G64"/>
-      <x:c r="H64"/>
-      <x:c r="I64"/>
-      <x:c r="J64"/>
-      <x:c r="K64"/>
-      <x:c r="L64"/>
-      <x:c r="M64"/>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65"/>
-      <x:c r="B65"/>
-      <x:c r="C65"/>
-      <x:c r="D65"/>
-      <x:c r="E65"/>
-      <x:c r="F65"/>
-      <x:c r="G65"/>
-      <x:c r="H65"/>
-      <x:c r="I65"/>
-      <x:c r="J65"/>
-      <x:c r="K65"/>
-      <x:c r="L65"/>
-      <x:c r="M65"/>
-    </x:row>
-    <x:row r="66">
-      <x:c r="A66"/>
-      <x:c r="B66"/>
-      <x:c r="C66"/>
-      <x:c r="D66"/>
-      <x:c r="E66"/>
-      <x:c r="F66"/>
-      <x:c r="G66"/>
-      <x:c r="H66"/>
-      <x:c r="I66"/>
-      <x:c r="J66"/>
-      <x:c r="K66"/>
-      <x:c r="L66"/>
-      <x:c r="M66"/>
-    </x:row>
-    <x:row r="67">
-      <x:c r="A67"/>
-      <x:c r="B67"/>
-      <x:c r="C67"/>
-      <x:c r="D67"/>
-      <x:c r="E67"/>
-      <x:c r="F67"/>
-      <x:c r="G67"/>
-      <x:c r="H67"/>
-      <x:c r="I67"/>
-      <x:c r="J67"/>
-      <x:c r="K67"/>
-      <x:c r="L67"/>
-      <x:c r="M67"/>
-    </x:row>
-    <x:row r="68">
-      <x:c r="A68"/>
-      <x:c r="B68"/>
-      <x:c r="C68"/>
-      <x:c r="D68"/>
-      <x:c r="E68"/>
-      <x:c r="F68"/>
-      <x:c r="G68"/>
-      <x:c r="H68"/>
-      <x:c r="I68"/>
-      <x:c r="J68"/>
-      <x:c r="K68"/>
-      <x:c r="L68"/>
-      <x:c r="M68"/>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69"/>
-      <x:c r="B69"/>
-      <x:c r="C69"/>
-      <x:c r="D69"/>
-      <x:c r="E69"/>
-      <x:c r="F69"/>
-      <x:c r="G69"/>
-      <x:c r="H69"/>
-      <x:c r="I69"/>
-      <x:c r="J69"/>
-      <x:c r="K69"/>
-      <x:c r="L69"/>
-      <x:c r="M69"/>
-    </x:row>
-    <x:row r="70">
-      <x:c r="A70"/>
-      <x:c r="B70"/>
-      <x:c r="C70"/>
-      <x:c r="D70"/>
-      <x:c r="E70"/>
-      <x:c r="F70"/>
-      <x:c r="G70"/>
-      <x:c r="H70"/>
-      <x:c r="I70"/>
-      <x:c r="J70"/>
-      <x:c r="K70"/>
-      <x:c r="L70"/>
-      <x:c r="M70"/>
+    <x:row r="40" ht="30" customHeight="1">
+      <x:c r="A40" s="26" t="str">
+        <x:v>DEP-002</x:v>
+      </x:c>
+      <x:c r="B40" s="26" t="str">
+        <x:v>Reconcile compatible dependency upgrade set</x:v>
+      </x:c>
+      <x:c r="C40" s="26" t="str">
+        <x:v>Public beta safety</x:v>
+      </x:c>
+      <x:c r="D40" s="26" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E40" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F40" s="26" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G40" s="26" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H40" s="26" t="str">
+        <x:v>DEP-001</x:v>
+      </x:c>
+      <x:c r="I40" s="26" t="str">
+        <x:v>Compatible React, Nest, test, CI and Terraform upgrades pass all mandatory suites; incompatible ioredis 6 and Expo Router 58 upgrades remain explicitly constrained</x:v>
+      </x:c>
+      <x:c r="J40" s="26" t="str">
+        <x:v>WOW-MD PR 52</x:v>
+      </x:c>
+      <x:c r="K40" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/82</x:v>
+      </x:c>
+      <x:c r="L40" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/83</x:v>
+      </x:c>
+      <x:c r="M40" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="A41" s="27" t="str">
+        <x:v>DEP-003</x:v>
+      </x:c>
+      <x:c r="B41" s="27" t="str">
+        <x:v>Complete remaining dependency source mirrors</x:v>
+      </x:c>
+      <x:c r="C41" s="27" t="str">
+        <x:v>Public beta safety</x:v>
+      </x:c>
+      <x:c r="D41" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E41" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F41" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G41" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H41" s="27" t="str">
+        <x:v>DEP-002</x:v>
+      </x:c>
+      <x:c r="I41" s="27" t="str">
+        <x:v>Production carries the reviewed glob lockfile, Node and nginx images, AWS modules and GitHub Actions versions from WOW-MD with production-only workflows upgraded consistently</x:v>
+      </x:c>
+      <x:c r="J41" s="27" t="str">
+        <x:v>WOW-MD PRs 18 20 21 22 27 53</x:v>
+      </x:c>
+      <x:c r="K41" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/85</x:v>
+      </x:c>
+      <x:c r="L41" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
+      </x:c>
+      <x:c r="M41" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E37">
+  <x:conditionalFormatting sqref="E6:E41">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F37">
+  <x:conditionalFormatting sqref="F6:F41">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3980,7 +3476,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2839a1a98d304860"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R774f5477c69b4acb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4426,25 +3922,117 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="27" t="str">
+      <x:c r="A23" s="26" t="str">
         <x:v>REQ-REV-001</x:v>
       </x:c>
-      <x:c r="B23" s="27" t="str">
+      <x:c r="B23" s="26" t="str">
         <x:v>AWS migration readiness reports INR 1.2M target and INR 1.5M preferred monthly net revenue</x:v>
       </x:c>
-      <x:c r="C23" s="27" t="str">
+      <x:c r="C23" s="26" t="str">
         <x:v>Migration design</x:v>
       </x:c>
-      <x:c r="D23" s="27" t="str">
+      <x:c r="D23" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="E23" s="27" t="str">
+      <x:c r="E23" s="26" t="str">
         <x:v>Admin readiness UI test</x:v>
       </x:c>
-      <x:c r="F23" s="27" t="str">
+      <x:c r="F23" s="26" t="str">
         <x:v>UI-001</x:v>
       </x:c>
-      <x:c r="G23" s="27" t="str">
+      <x:c r="G23" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="26" t="str">
+        <x:v>REQ-AUTH-001</x:v>
+      </x:c>
+      <x:c r="B24" s="26" t="str">
+        <x:v>Administrators authenticate through Zoho SSO and do not require routine application TOTP</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E24" s="26" t="str">
+        <x:v>Authentication integration tests and controlled Zoho sign-in evidence</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G24" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="26" t="str">
+        <x:v>REQ-AUTH-002</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="str">
+        <x:v>Existing users may sign in with Zoho SSO or username email or mobile plus password and any valid email provider is accepted</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>Backend frontend mobile and Playwright authentication tests</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="A26" s="26" t="str">
+        <x:v>REQ-AUTH-003</x:v>
+      </x:c>
+      <x:c r="B26" s="26" t="str">
+        <x:v>OTP is used only for signup/contact verification and password recovery and never as passwordless login</x:v>
+      </x:c>
+      <x:c r="C26" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="str">
+        <x:v>Route inventory and authentication tests</x:v>
+      </x:c>
+      <x:c r="F26" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G26" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="27" t="str">
+        <x:v>REQ-AUTH-004</x:v>
+      </x:c>
+      <x:c r="B27" s="27" t="str">
+        <x:v>Zoho domain DNS sender mailbox SMTP application password and production OAuth callback are configured only at the final deployment gate</x:v>
+      </x:c>
+      <x:c r="C27" s="27" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D27" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E27" s="27" t="str">
+        <x:v>Final release checklist and controlled delivery/SSO evidence</x:v>
+      </x:c>
+      <x:c r="F27" s="27" t="str">
+        <x:v>SEC-001,REL-001</x:v>
+      </x:c>
+      <x:c r="G27" s="27" t="str">
         <x:v>Approved</x:v>
       </x:c>
     </x:row>
@@ -4452,10 +4040,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D23">
+  <x:conditionalFormatting sqref="D6:D27">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G6:G23">
+  <x:conditionalFormatting sqref="G6:G27">
     <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Blocked"/>
@@ -4464,7 +4052,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08c672e326c947c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d83ca7b8304ed7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4749,118 +4337,118 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="27" t="str">
+      <x:c r="A16" s="26" t="str">
         <x:v>QA-GOV-001</x:v>
       </x:c>
-      <x:c r="B16" s="27" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>Source synchronization</x:v>
       </x:c>
-      <x:c r="C16" s="27" t="str">
+      <x:c r="C16" s="26" t="str">
         <x:v>Private-source report and shared-code mirror gate</x:v>
       </x:c>
-      <x:c r="D16" s="27" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>PR 55 local evidence</x:v>
       </x:c>
-      <x:c r="E16" s="27" t="str">
+      <x:c r="E16" s="26" t="str">
         <x:v>19 of 19 governance and synchronization tests passed</x:v>
       </x:c>
-      <x:c r="F16" s="27" t="str">
+      <x:c r="F16" s="26" t="str">
         <x:v>Configure WOW_SYNC_TOKEN and capture first scheduled artifact</x:v>
       </x:c>
-      <x:c r="G16" s="27" t="str">
+      <x:c r="G16" s="26" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="26" t="str">
+        <x:v>QA-SEC-002</x:v>
+      </x:c>
+      <x:c r="B17" s="26" t="str">
+        <x:v>WebSocket authorization</x:v>
+      </x:c>
+      <x:c r="C17" s="26" t="str">
+        <x:v>Origin token-version forced-reset call relay and presence audience</x:v>
+      </x:c>
+      <x:c r="D17" s="26" t="str">
+        <x:v>SEC-002 PR 62</x:v>
+      </x:c>
+      <x:c r="E17" s="26" t="str">
+        <x:v>11 focused gateway tests and complete backend suite 800 passed with 9 skipped</x:v>
+      </x:c>
+      <x:c r="F17" s="26" t="str">
+        <x:v>Repeat browser and native reconnect smoke tests on Railway candidate</x:v>
+      </x:c>
+      <x:c r="G17" s="26" t="str">
+        <x:v>SEC-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="26" t="str">
+        <x:v>QA-SEC-003</x:v>
+      </x:c>
+      <x:c r="B18" s="26" t="str">
+        <x:v>HTTP and migration integrity</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>Production Swagger headers migration uniqueness fresh and upgrade paths</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="str">
+        <x:v>SEC-003 PR 63</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="str">
+        <x:v>2 HTTP tests; 2 verifier tests; 93-file verification; 794 backend tests passed with 9 skipped; fresh and upgraded databases passed</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="str">
+        <x:v>Repeat ingress header checks on Railway candidate</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
+        <x:v>SEC-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="26" t="str">
+        <x:v>QA-OPS-001</x:v>
+      </x:c>
+      <x:c r="B19" s="26" t="str">
+        <x:v>Replica safety</x:v>
+      </x:c>
+      <x:c r="C19" s="26" t="str">
+        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="str">
+        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="str">
+        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="F19" s="26" t="str">
+        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
+      </x:c>
+      <x:c r="G19" s="26" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="27" t="str">
         <x:v>QA-OBS-001</x:v>
       </x:c>
-      <x:c r="B17" t="str">
+      <x:c r="B20" s="27" t="str">
         <x:v>Observability</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C20" s="27" t="str">
         <x:v>Request correlation redaction provider logs QA capture audit failures payout sweep and nginx JSON</x:v>
       </x:c>
-      <x:c r="D17" t="str">
-        <x:v>OBS-001 PR 65 and WOW-MD PR 43</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>Focused 20 of 20; full backend 812 passed 9 skipped; typecheck lint nginx contract image build and syntax passed</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>Deploy after SEC-003 and verify live response/log correlation with capture disabled</x:v>
-      </x:c>
-      <x:c r="G17" t="str">
+      <x:c r="D20" s="27" t="str">
+        <x:v>OBS-001 PR 69 and merged WOW-MD PR 43</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>Focused observability and replica-lock integration 27 of 27; typecheck lint and nginx contract passed; protected CI recorded on PR 69</x:v>
+      </x:c>
+      <x:c r="F20" s="27" t="str">
+        <x:v>Verify live response/log correlation with capture disabled</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="str">
         <x:v>OBS-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>QA-SEC-002</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>WebSocket origins tokens calls and presence authorization</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>SEC-002 PR 62 and WOW-MD PR 40</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
-        <x:v>Focused gateways 11 passed; full backend 800 passed 9 skipped; typecheck and lint passed</x:v>
-      </x:c>
-      <x:c r="F18" t="str">
-        <x:v>Run staged hostile-origin and two-account WebSocket smoke</x:v>
-      </x:c>
-      <x:c r="G18" t="str">
-        <x:v>SEC-002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>QA-SEC-003</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="C19" t="str">
-        <x:v>HTTP headers private Swagger and migration integrity</x:v>
-      </x:c>
-      <x:c r="D19" t="str">
-        <x:v>SEC-003 PR 63 and WOW-MD PR 41</x:v>
-      </x:c>
-      <x:c r="E19" t="str">
-        <x:v>HTTP 2 passed; migration verifier 2 passed; 93 migrations verified and clean database upgrade passed; backend 794 passed 9 skipped</x:v>
-      </x:c>
-      <x:c r="F19" t="str">
-        <x:v>Deploy and verify production headers Swagger denial and migration startup</x:v>
-      </x:c>
-      <x:c r="G19" t="str">
-        <x:v>SEC-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>QA-OPS-001</x:v>
-      </x:c>
-      <x:c r="B20" t="str">
-        <x:v>Replica safety</x:v>
-      </x:c>
-      <x:c r="C20" t="str">
-        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
-      </x:c>
-      <x:c r="E20" t="str">
-        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
-      </x:c>
-      <x:c r="F20" t="str">
-        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
-      </x:c>
-      <x:c r="G20" t="str">
-        <x:v>OPS-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4869,7 +4457,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e0a146b3665477e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R880cfabdb5234d85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5262,42 +4850,71 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="27" t="str">
+      <x:c r="A18" s="26" t="str">
         <x:v>RISK-013</x:v>
       </x:c>
-      <x:c r="B18" s="27" t="str">
-        <x:v>Public deployment tier is enabled before every administrator enrols MFA</x:v>
-      </x:c>
-      <x:c r="C18" s="27" t="str">
+      <x:c r="B18" s="26" t="str">
+        <x:v>Public deployment tier is enabled before Zoho SSO and administrator recovery are proven</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D18" s="27" t="str">
+      <x:c r="D18" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E18" s="27" t="str">
+      <x:c r="E18" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F18" s="27" t="str">
-        <x:v>Enrol and verify each administrator in restricted staging before selecting public-beta; keep a documented recovery owner</x:v>
-      </x:c>
-      <x:c r="G18" s="27" t="str">
+      <x:c r="F18" s="26" t="str">
+        <x:v>Verify exact OAuth client callback administrator matching-email login Zoho-account MFA and a documented recovery owner in restricted staging before public-beta</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H18" s="27" t="str">
+      <x:c r="H18" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="I18" s="27" t="str">
-        <x:v>SEC-001 PR 56 rejects unenrolled login and existing sessions; staged enrollment evidence still required</x:v>
+      <x:c r="I18" s="26" t="str">
+        <x:v>SEC-001 PR 58 implements Zoho-only administrator login; production Zoho configuration is intentionally deferred to the final gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="27" t="str">
+        <x:v>RISK-014</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="str">
+        <x:v>Framework and mobile build-tool dependency advisories remain after runtime remediation</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="str">
+        <x:v>Block new critical/high runtime advisories; allow only four exact no-fix Expo advisory IDs; schedule Nest major migration and review exceptions each release</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="H19" s="27" t="str">
+        <x:v>Mitigated</x:v>
+      </x:c>
+      <x:c r="I19" s="27" t="str">
+        <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E18">
+  <x:conditionalFormatting sqref="E6:E19">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H18">
+  <x:conditionalFormatting sqref="H6:H19">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -5306,7 +4923,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89e8a5d8aab64c7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6374f0038df94186"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5537,16 +5154,16 @@
         <x:v>ACC-007</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>Operational email</x:v>
+        <x:v>Zoho identity and operational email</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>Zoho domain mailbox DNS authentication reports and app-password rotation</x:v>
+        <x:v>OAuth application exact callback domain mailbox DNS authentication reports and SMTP app-password rotation</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>Zoho SMTP identity</x:v>
+        <x:v>Zoho OAuth and SMTP identities</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
         <x:v>GitHub Railway or Kubernetes secrets</x:v>
@@ -5556,7 +5173,7 @@
       </x:c>
       <x:c r="H12" s="29" t="str"/>
       <x:c r="I12" s="26" t="str">
-        <x:v>Low-volume beta only; owner must configure domain MFA app password and first delivery evidence</x:v>
+        <x:v>Configure only at final deployment; protect the Zoho owner with Zoho MFA and retain controlled SSO/mail evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -5621,7 +5238,7 @@
         <x:v>WOW-MD source review</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
-        <x:v>Private repository contents read for scheduled change reports</x:v>
+        <x:v>Repository contents read for scheduled change reports</x:v>
       </x:c>
       <x:c r="D15" s="27" t="str">
         <x:v>RohithTadiparti</x:v>
@@ -5633,11 +5250,11 @@
         <x:v>Production GitHub Actions secret</x:v>
       </x:c>
       <x:c r="G15" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="H15" s="30" t="str"/>
       <x:c r="I15" s="27" t="str">
-        <x:v>Scope only to WOW-MD Contents read; rotate within 90 days</x:v>
+        <x:v>Not technically required while WOW-MD is public; create before returning it private so the private-ready workflow keeps working; scope only to WOW-MD Contents read and rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5653,7 +5270,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c0531a9184d4e9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cdd09bc2d384d86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5992,7 +5609,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14665dc032fd4736"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91ae813e008c4ad1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6125,143 +5742,213 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="A8" s="26" t="str">
         <x:v>CHG-003</x:v>
       </x:c>
-      <x:c r="B8" s="27" t="str">
+      <x:c r="B8" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C8" s="27" t="str">
+      <x:c r="C8" s="26" t="str">
         <x:v>07218b4..de7d8dd (LOCAL ONLY)</x:v>
       </x:c>
-      <x:c r="D8" s="27" t="str">
+      <x:c r="D8" s="26" t="str">
         <x:v>37 committed paths</x:v>
       </x:c>
-      <x:c r="E8" s="27" t="str">
+      <x:c r="E8" s="26" t="str">
         <x:v>Functional UI candidates</x:v>
       </x:c>
-      <x:c r="F8" s="27" t="str">
+      <x:c r="F8" s="26" t="str">
         <x:v>Await source publication and per-commit review</x:v>
       </x:c>
-      <x:c r="G8" s="27" t="str">
+      <x:c r="G8" s="26" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="H8" s="27" t="str">
+      <x:c r="H8" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
       </x:c>
-      <x:c r="I8" s="27" t="str">
+      <x:c r="I8" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J8" s="30" t="str">
+      <x:c r="J8" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
-      <x:c r="K8" s="27" t="str">
+      <x:c r="K8" s="26" t="str">
         <x:v>Local main is 21 commits ahead of origin; scheduled GitHub review intentionally sees pushed commits only</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="26" t="str">
         <x:v>CHG-004</x:v>
       </x:c>
-      <x:c r="B9" s="27" t="str">
+      <x:c r="B9" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C9" s="27" t="str">
+      <x:c r="C9" s="26" t="str">
         <x:v>2ddfaf6b6d55d3e4833f905565d5048f3cd9c010</x:v>
       </x:c>
-      <x:c r="D9" s="27" t="str">
+      <x:c r="D9" s="26" t="str">
         <x:v>frontend/ (40 paths)</x:v>
       </x:c>
-      <x:c r="E9" s="27" t="str">
+      <x:c r="E9" s="26" t="str">
         <x:v>UI/UX and tests</x:v>
       </x:c>
-      <x:c r="F9" s="27" t="str">
+      <x:c r="F9" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G9" s="27" t="str">
+      <x:c r="G9" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="H9" s="27" t="str">
+      <x:c r="H9" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
       </x:c>
-      <x:c r="I9" s="27" t="str">
+      <x:c r="I9" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J9" s="30" t="str">
+      <x:c r="J9" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K9" s="27" t="str">
+      <x:c r="K9" s="26" t="str">
         <x:v>WOW-MD PR 50 published the reviewed 07218b4..8a147a6 UI line; production accepts only the reconciled frontend paths</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="26" t="str">
         <x:v>CHG-005</x:v>
       </x:c>
-      <x:c r="B10" s="27" t="str">
+      <x:c r="B10" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C10" s="27" t="str">
+      <x:c r="C10" s="26" t="str">
         <x:v>2ddfaf6b6d55d3e4833f905565d5048f3cd9c010</x:v>
       </x:c>
-      <x:c r="D10" s="27" t="str">
+      <x:c r="D10" s="26" t="str">
         <x:v>docker/docker-compose.preview.yml; docs/wow-consumer-portal-design-preview.html</x:v>
       </x:c>
-      <x:c r="E10" s="27" t="str">
+      <x:c r="E10" s="26" t="str">
         <x:v>Preview-only source artifacts</x:v>
       </x:c>
-      <x:c r="F10" s="27" t="str">
+      <x:c r="F10" s="26" t="str">
         <x:v>Rejected for production</x:v>
       </x:c>
-      <x:c r="G10" s="27" t="str">
+      <x:c r="G10" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="H10" s="27" t="str">
+      <x:c r="H10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
       </x:c>
-      <x:c r="I10" s="27" t="str">
+      <x:c r="I10" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J10" s="30" t="str">
+      <x:c r="J10" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K10" s="27" t="str">
+      <x:c r="K10" s="26" t="str">
         <x:v>Remain in WOW-MD for design preview use; not part of the production deployment line</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="26" t="str">
         <x:v>CHG-006</x:v>
       </x:c>
-      <x:c r="B11" s="27" t="str">
+      <x:c r="B11" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C11" s="27" t="str">
+      <x:c r="C11" s="26" t="str">
         <x:v>51790dfa57126a64e31e5b605ddccca85cd09b85</x:v>
       </x:c>
-      <x:c r="D11" s="27" t="str">
+      <x:c r="D11" s="26" t="str">
         <x:v>frontend/package-lock.json</x:v>
       </x:c>
-      <x:c r="E11" s="27" t="str">
+      <x:c r="E11" s="26" t="str">
         <x:v>Dependency lockfile</x:v>
       </x:c>
-      <x:c r="F11" s="27" t="str">
+      <x:c r="F11" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G11" s="27" t="str">
+      <x:c r="G11" s="26" t="str">
         <x:v>DEP-001</x:v>
       </x:c>
-      <x:c r="H11" s="27" t="str">
+      <x:c r="H11" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/81</x:v>
       </x:c>
-      <x:c r="I11" s="27" t="str">
+      <x:c r="I11" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J11" s="30" t="str">
+      <x:c r="J11" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K11" s="27" t="str">
+      <x:c r="K11" s="26" t="str">
         <x:v>WOW-MD PR 49 and production PRs 79 and 81 reconcile source-map-js 1.2.2 and the exact frontend lock graph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="26" t="str">
+        <x:v>CHG-007</x:v>
+      </x:c>
+      <x:c r="B12" s="26" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C12" s="26" t="str">
+        <x:v>d3d66eae45ddefc262121f356b36ddfa94516baf</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="str">
+        <x:v>backend/; frontend/; mobile/; docker/; terraform/; .github/workflows/</x:v>
+      </x:c>
+      <x:c r="E12" s="26" t="str">
+        <x:v>Dependency and compatibility rollup</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G12" s="26" t="str">
+        <x:v>DEP-002</x:v>
+      </x:c>
+      <x:c r="H12" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/83</x:v>
+      </x:c>
+      <x:c r="I12" s="26" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J12" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K12" s="26" t="str">
+        <x:v>WOW-MD PR 52; accepted compatible React Nest Vitest Node Terraform and security updates; retained ioredis 5 and Expo Router 57 because proposed majors violate current peer contracts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="27" t="str">
+        <x:v>CHG-008</x:v>
+      </x:c>
+      <x:c r="B13" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C13" s="27" t="str">
+        <x:v>b373bb48e389a3456a98db12e1c880b901b75e49</x:v>
+      </x:c>
+      <x:c r="D13" s="27" t="str">
+        <x:v>backend/package-lock.json; docker/Dockerfile; docker/Dockerfile.frontend; terraform/eks.tf; terraform/rds.tf; .github/workflows/</x:v>
+      </x:c>
+      <x:c r="E13" s="27" t="str">
+        <x:v>Dependency and infrastructure mirrors</x:v>
+      </x:c>
+      <x:c r="F13" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G13" s="27" t="str">
+        <x:v>DEP-003</x:v>
+      </x:c>
+      <x:c r="H13" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
+      </x:c>
+      <x:c r="I13" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J13" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K13" s="27" t="str">
+        <x:v>WOW-MD PRs 18 20 21 22 27 and 53; production-only governance and source-review workflows receive the same reviewed action majors</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6270,7 +5957,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e7de65b578c42fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R919a65b175624e9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6375,7 +6062,7 @@
       <x:c r="J6" s="25" t="str">
         <x:v>GitHub plan blocks protected private branches native secret scanning and native CodeQL upload; offline SARIF and CI Gitleaks compensate; tracked by GOV-001</x:v>
       </x:c>
-      <x:c r="K6" s="70" t="str">
+      <x:c r="K6" s="25" t="str">
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L6" s="28" t="str">
@@ -6411,7 +6098,7 @@
       <x:c r="J7" s="26" t="str">
         <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
       </x:c>
-      <x:c r="K7" s="71" t="str">
+      <x:c r="K7" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L7" s="29" t="str">
@@ -6449,7 +6136,7 @@
       <x:c r="J8" s="26" t="str">
         <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred to the final release gate</x:v>
       </x:c>
-      <x:c r="K8" s="71" t="str">
+      <x:c r="K8" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
@@ -6457,404 +6144,466 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="27" t="str">
+      <x:c r="A9" s="26" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="B9" s="27" t="str">
+      <x:c r="B9" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
       </x:c>
-      <x:c r="C9" s="27" t="str">
+      <x:c r="C9" s="26" t="str">
         <x:v>codex/sync-002-gated-source-review</x:v>
       </x:c>
-      <x:c r="D9" s="27" t="str">
+      <x:c r="D9" s="26" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E9" s="27" t="str">
+      <x:c r="E9" s="26" t="str">
         <x:v>422cbc4</x:v>
       </x:c>
-      <x:c r="F9" s="27" t="str">
+      <x:c r="F9" s="26" t="str">
         <x:v>07218b4..de7d8dd local review only</x:v>
       </x:c>
-      <x:c r="G9" s="27" t="str">
+      <x:c r="G9" s="26" t="str">
         <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
       </x:c>
-      <x:c r="H9" s="27" t="str">
+      <x:c r="H9" s="26" t="str">
         <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
       </x:c>
-      <x:c r="I9" s="27" t="str">
+      <x:c r="I9" s="26" t="str">
         <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
       </x:c>
-      <x:c r="J9" s="27" t="str">
+      <x:c r="J9" s="26" t="str">
         <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
       </x:c>
-      <x:c r="K9" s="74" t="str">
+      <x:c r="K9" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L9" s="30" t="str">
+      <x:c r="L9" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="26" t="str">
         <x:v>DEP-001</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="B10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
       </x:c>
-      <x:c r="C10" t="str">
+      <x:c r="C10" s="26" t="str">
         <x:v>codex/dep-001-dependency-remediation</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="D10" s="26" t="str">
         <x:v>29537ee</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="E10" s="26" t="str">
         <x:v>1ecbfdf</x:v>
       </x:c>
-      <x:c r="F10" t="str">
+      <x:c r="F10" s="26" t="str">
         <x:v>WOW-MD PR 39 head d8ef995; WOW-MD PR 49 merged as 51790df; supplemental production PRs 73, 79, and 81</x:v>
       </x:c>
-      <x:c r="G10" t="str">
+      <x:c r="G10" s="26" t="str">
         <x:v>Backend and frontend production audits have no high or critical findings; frontend clean install typecheck 180 tests build passed on PR 81; exact frontend trees match</x:v>
       </x:c>
-      <x:c r="H10" t="str">
+      <x:c r="H10" s="26" t="str">
         <x:v>Merged; no runtime deployment is required for the PR 81 development-only lock reconciliation; retain normal rebuild verification</x:v>
       </x:c>
-      <x:c r="I10" t="str">
+      <x:c r="I10" s="26" t="str">
         <x:v>Revert the affected supplemental PR and restore its paired WOW-MD lockfile if clean install or build regresses</x:v>
       </x:c>
-      <x:c r="J10" t="str">
+      <x:c r="J10" s="26" t="str">
         <x:v>Three moderate mammoth-chain findings and four exact no-fix Expo advisory roots remain; forced breaking downgrades remain rejected</x:v>
       </x:c>
-      <x:c r="K10" s="75" t="str">
+      <x:c r="K10" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L10" t="str">
+      <x:c r="L10" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="26" t="str">
         <x:v>GOV-003</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="B11" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
       </x:c>
-      <x:c r="C11" t="str">
+      <x:c r="C11" s="26" t="str">
         <x:v>codex/gov-003-auth-dependency-tracking</x:v>
       </x:c>
-      <x:c r="D11" t="str">
+      <x:c r="D11" s="26" t="str">
         <x:v>29537ee</x:v>
       </x:c>
-      <x:c r="E11" t="str">
+      <x:c r="E11" s="26" t="str">
         <x:v>1235cd3</x:v>
       </x:c>
-      <x:c r="F11" t="str">
+      <x:c r="F11" s="26" t="str">
         <x:v>SEC-001 PR 58 and DEP-001 PR 59 evidence only</x:v>
       </x:c>
-      <x:c r="G11" t="str">
+      <x:c r="G11" s="26" t="str">
         <x:v>Register validator workbook regeneration and formula-error scan pass; dashboard visually reviewed</x:v>
       </x:c>
-      <x:c r="H11" t="str">
+      <x:c r="H11" s="26" t="str">
         <x:v>Governance and documentation only; no application or hosting deployment</x:v>
       </x:c>
-      <x:c r="I11" t="str">
+      <x:c r="I11" s="26" t="str">
         <x:v>Revert PR 61; implementation PRs and their evidence remain unchanged</x:v>
       </x:c>
-      <x:c r="J11" t="str">
+      <x:c r="J11" s="26" t="str">
         <x:v>Implementation PRs still require review/merge and GitHub rescan; Zoho live configuration remains a final release gate</x:v>
       </x:c>
-      <x:c r="K11" s="75" t="str">
+      <x:c r="K11" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L11" t="str">
+      <x:c r="L11" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="26" t="str">
         <x:v>SEC-002</x:v>
       </x:c>
-      <x:c r="B12" t="str">
+      <x:c r="B12" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/62</x:v>
       </x:c>
-      <x:c r="C12" t="str">
+      <x:c r="C12" s="26" t="str">
         <x:v>codex/sec-002-websocket-authorization</x:v>
       </x:c>
-      <x:c r="D12" t="str">
+      <x:c r="D12" s="26" t="str">
         <x:v>29537ee</x:v>
       </x:c>
-      <x:c r="E12" t="str">
+      <x:c r="E12" s="26" t="str">
         <x:v>4c5e7b4</x:v>
       </x:c>
-      <x:c r="F12" t="str">
+      <x:c r="F12" s="26" t="str">
         <x:v>WOW-MD PR 40 head 9265a27</x:v>
       </x:c>
-      <x:c r="G12" t="str">
+      <x:c r="G12" s="26" t="str">
         <x:v>11 focused chat/admin gateway tests; backend typecheck and lint; complete backend suite 800 passed with 9 skipped</x:v>
       </x:c>
-      <x:c r="H12" t="str">
+      <x:c r="H12" s="26" t="str">
         <x:v>Set exact CORS_ORIGINS and smoke-test browser/native reconnect on the Railway candidate; no schema migration</x:v>
       </x:c>
-      <x:c r="I12" t="str">
+      <x:c r="I12" s="26" t="str">
         <x:v>Revert PR 62; REST chat remains available while socket traffic is paused</x:v>
       </x:c>
-      <x:c r="J12" t="str">
+      <x:c r="J12" s="26" t="str">
         <x:v>Native clients are allowed without an Origin header and remain protected by bearer-token/account checks; Railway cross-origin smoke evidence remains pending</x:v>
       </x:c>
-      <x:c r="K12" s="75" t="str">
+      <x:c r="K12" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L12" t="str">
+      <x:c r="L12" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="26" t="str">
         <x:v>SEC-003</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B13" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/63</x:v>
       </x:c>
-      <x:c r="C13" t="str">
+      <x:c r="C13" s="26" t="str">
         <x:v>codex/sec-003-http-migration-integrity</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D13" s="26" t="str">
         <x:v>29537ee</x:v>
       </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="E13" s="26" t="str">
         <x:v>80ef902</x:v>
       </x:c>
-      <x:c r="F13" t="str">
+      <x:c r="F13" s="26" t="str">
         <x:v>WOW-MD PR 41 head ef13ff5</x:v>
       </x:c>
-      <x:c r="G13" t="str">
+      <x:c r="G13" s="26" t="str">
         <x:v>2 HTTP policy tests; 2 migration verifier tests; 93 files unique; backend typecheck/lint and 794 tests with 9 skipped; upgraded wow_db and fresh 93-migration database passed</x:v>
       </x:c>
-      <x:c r="H13" t="str">
+      <x:c r="H13" s="26" t="str">
         <x:v>Run migrations before application rollout and verify headers through the Railway ingress</x:v>
       </x:c>
-      <x:c r="I13" t="str">
+      <x:c r="I13" s="26" t="str">
         <x:v>Revert application/header changes but retain applied migration history and safe schema additions for roll-forward</x:v>
       </x:c>
-      <x:c r="J13" t="str">
+      <x:c r="J13" s="26" t="str">
         <x:v>Historical databases retain old collision rows plus new idempotent reconciliation rows; ingress evidence remains pending</x:v>
       </x:c>
-      <x:c r="K13" s="75" t="str">
+      <x:c r="K13" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L13" t="str">
+      <x:c r="L13" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="26" t="str">
         <x:v>OPS-001</x:v>
       </x:c>
-      <x:c r="B14" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
       </x:c>
-      <x:c r="C14" t="str">
+      <x:c r="C14" s="26" t="str">
         <x:v>codex/ops-001-replicated-jobs</x:v>
       </x:c>
-      <x:c r="D14" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E14" t="str">
+      <x:c r="E14" s="26" t="str">
         <x:v>2bf76a1</x:v>
       </x:c>
-      <x:c r="F14" t="str">
+      <x:c r="F14" s="26" t="str">
         <x:v>WOW-MD commit a06067a; PR 42</x:v>
       </x:c>
-      <x:c r="G14" t="str">
+      <x:c r="G14" s="26" t="str">
         <x:v>Focused replica tests 7 of 7; backend full suite 797 passed 9 skipped; typecheck and lint passed</x:v>
       </x:c>
-      <x:c r="H14" t="str">
+      <x:c r="H14" s="26" t="str">
         <x:v>Deploy normally after approval; verify two replicas produce one owner and one skipped invocation for outbox and payout/reminder jobs</x:v>
       </x:c>
-      <x:c r="I14" t="str">
+      <x:c r="I14" s="26" t="str">
         <x:v>Revert PR 64 and redeploy; no database or configuration rollback</x:v>
       </x:c>
-      <x:c r="J14" t="str">
+      <x:c r="J14" s="26" t="str">
         <x:v>Outbox delivery is at-least-once if a worker dies after an external side effect and before processedAt; downstream Kafka consumers must honor the outbox UUID idempotency key</x:v>
       </x:c>
-      <x:c r="K14" s="75" t="str">
+      <x:c r="K14" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L14" t="str">
+      <x:c r="L14" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="26" t="str">
         <x:v>OBS-001</x:v>
       </x:c>
-      <x:c r="B15" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/69</x:v>
       </x:c>
-      <x:c r="C15" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>codex/obs-001-backend-observability</x:v>
       </x:c>
-      <x:c r="D15" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>122ae2d</x:v>
       </x:c>
-      <x:c r="E15" t="str">
+      <x:c r="E15" s="26" t="str">
         <x:v>9d34f68</x:v>
       </x:c>
-      <x:c r="F15" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>WOW-MD PR 43 merged as 2db719b</x:v>
       </x:c>
-      <x:c r="G15" t="str">
+      <x:c r="G15" s="26" t="str">
         <x:v>Focused observability and replica-lock integration 27 of 27; backend typecheck and lint plus nginx contract passed; protected CI recorded on PR 69</x:v>
       </x:c>
-      <x:c r="H15" t="str">
+      <x:c r="H15" s="26" t="str">
         <x:v>Set RELEASE; keep QA capture disabled; confirm a live request ID matches response backend and nginx logs</x:v>
       </x:c>
-      <x:c r="I15" t="str">
+      <x:c r="I15" s="26" t="str">
         <x:v>Revert PR 69 and redeploy; remove optional observability variables; no database rollback</x:v>
       </x:c>
-      <x:c r="J15" t="str">
+      <x:c r="J15" s="26" t="str">
         <x:v>OBS-002 client error intake and OBS-003 Loki Vector host files 30-day retention remain open; live provider correlation smoke remains</x:v>
       </x:c>
-      <x:c r="K15" s="75" t="str">
+      <x:c r="K15" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L15" t="str">
+      <x:c r="L15" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="26" t="str">
         <x:v>OBS-003</x:v>
       </x:c>
-      <x:c r="B16" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/71</x:v>
       </x:c>
-      <x:c r="C16" t="str">
+      <x:c r="C16" s="26" t="str">
         <x:v>codex/obs-003-local-log-platform</x:v>
       </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>dd39ccc</x:v>
       </x:c>
-      <x:c r="E16" t="str">
+      <x:c r="E16" s="26" t="str">
         <x:v>0d1e02f</x:v>
       </x:c>
-      <x:c r="F16" t="str">
+      <x:c r="F16" s="26" t="str">
         <x:v>WOW-MD PR 48 merged as 7384378</x:v>
       </x:c>
-      <x:c r="G16" t="str">
-        <x:v>Collector and Loki configuration; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; seven alerts; Loki buffer recovery; frontend restart persistence all pass</x:v>
-      </x:c>
-      <x:c r="H16" t="str">
+      <x:c r="G16" s="26" t="str">
+        <x:v>Collector/Loki config validation; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; 7 provisioned alerts; Loki buffer recovery; frontend-restart persistence all pass</x:v>
+      </x:c>
+      <x:c r="H16" s="26" t="str">
         <x:v>Set WOW_LOG_DIR and a unique GRAFANA_ADMIN_PASSWORD; start the observability Compose profile; Grafana binds to 127.0.0.1:3300</x:v>
       </x:c>
-      <x:c r="I16" t="str">
+      <x:c r="I16" s="26" t="str">
         <x:v>Stop/remove observability containers and revert PR 71; retained host logs are not automatically deleted; application services remain independent</x:v>
       </x:c>
-      <x:c r="J16" t="str">
-        <x:v>Single-host logs are not disaster recovery; Vector outage has bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
-      </x:c>
-      <x:c r="K16" t="str">
+      <x:c r="J16" s="26" t="str">
+        <x:v>Single-host logs are not disaster recovery; Vector outage has only bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
+      </x:c>
+      <x:c r="K16" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L16" t="str">
+      <x:c r="L16" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="26" t="str">
         <x:v>CFG-001</x:v>
       </x:c>
-      <x:c r="B17" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/72</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>codex/cfg-001-platform-config</x:v>
       </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>568b4a8</x:v>
       </x:c>
-      <x:c r="E17" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>8efb49c</x:v>
       </x:c>
-      <x:c r="F17" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>WOW-MD PR 46 merged as 9135e2f</x:v>
       </x:c>
-      <x:c r="G17" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>Focused configuration contract 12 of 12; backend full suite 840 passed with 9 skipped; lint typecheck boundary scan Compose validation and production image build passed; production audit has no high or critical findings</x:v>
       </x:c>
-      <x:c r="H17" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>Merged after OBS-003 PR 71; retain secrets in environment or secret stores; public tiers must provide S3 bucket secure cookies and disabled Swagger</x:v>
       </x:c>
-      <x:c r="I17" t="str">
+      <x:c r="I17" s="26" t="str">
         <x:v>Revert PR 72 and rebuild; all pre-existing environment variables remain compatible and no database rollback is required</x:v>
       </x:c>
-      <x:c r="J17" t="str">
+      <x:c r="J17" s="26" t="str">
         <x:v>Public and revenue validation deliberately refuses unsafe provider combinations; existing moderate or low framework-chain dependency findings remain outside this change</x:v>
       </x:c>
-      <x:c r="K17" t="str">
+      <x:c r="K17" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L17" t="str">
+      <x:c r="L17" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="B18" t="str">
+      <x:c r="B18" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
       </x:c>
-      <x:c r="C18" t="str">
+      <x:c r="C18" s="26" t="str">
         <x:v>codex/sync-003-consumer-ui</x:v>
       </x:c>
-      <x:c r="D18" t="str">
+      <x:c r="D18" s="26" t="str">
         <x:v>3e05702</x:v>
       </x:c>
-      <x:c r="E18" t="str">
+      <x:c r="E18" s="26" t="str">
         <x:v>83c2400</x:v>
       </x:c>
-      <x:c r="F18" t="str">
+      <x:c r="F18" s="26" t="str">
         <x:v>WOW-MD PR 50 merged as 2ddfaf6; reviewed local source range 07218b4..8a147a6</x:v>
       </x:c>
-      <x:c r="G18" t="str">
+      <x:c r="G18" s="26" t="str">
         <x:v>Frontend typecheck; 19 test files and 180 tests; production build; protected backend suite and E2E frontend mobile Docker CodeQL secrets and governance checks passed</x:v>
       </x:c>
-      <x:c r="H18" t="str">
+      <x:c r="H18" s="26" t="str">
         <x:v>Merged; rebuild and deploy only the frontend image then smoke public home login registration and bride groom family navigation</x:v>
       </x:c>
-      <x:c r="I18" t="str">
+      <x:c r="I18" s="26" t="str">
         <x:v>Revert PR 77 and rebuild the frontend image; no database configuration or infrastructure rollback</x:v>
       </x:c>
-      <x:c r="J18" t="str">
+      <x:c r="J18" s="26" t="str">
         <x:v>Live post-deployment visual and role smoke remains; main client bundle is about 1.9 MB raw and 505 KB gzip; source-only preview artifacts were rejected</x:v>
       </x:c>
-      <x:c r="K18" t="str">
+      <x:c r="K18" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L18" t="str">
+      <x:c r="L18" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19"/>
-      <x:c r="B19"/>
-      <x:c r="C19"/>
-      <x:c r="D19"/>
-      <x:c r="E19"/>
-      <x:c r="F19"/>
-      <x:c r="G19"/>
-      <x:c r="H19"/>
-      <x:c r="I19"/>
-      <x:c r="J19"/>
-      <x:c r="K19"/>
-      <x:c r="L19"/>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="26" t="str">
+        <x:v>DEP-002</x:v>
+      </x:c>
+      <x:c r="B19" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/83</x:v>
+      </x:c>
+      <x:c r="C19" s="26" t="str">
+        <x:v>codex/dep-002-dependency-rollup</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="str">
+        <x:v>9e8aac5</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="str">
+        <x:v>8c2ebf8</x:v>
+      </x:c>
+      <x:c r="F19" s="26" t="str">
+        <x:v>WOW-MD PR 52 merged as d3d66ea; source heads 882a904 05b92a7 896cebf 752a340 f0b0237</x:v>
+      </x:c>
+      <x:c r="G19" s="26" t="str">
+        <x:v>Backend typecheck lint 837 tests build and clean production audit; E2E 51 of 51 including real Chrome; frontend typecheck 180 tests build; mobile audit typecheck Android export; source Docker and CodeQL green</x:v>
+      </x:c>
+      <x:c r="H19" s="26" t="str">
+        <x:v>Build backend and frontend images; run migrations before rollout; smoke health public entry sign-in biodata upload and an authenticated role page</x:v>
+      </x:c>
+      <x:c r="I19" s="26" t="str">
+        <x:v>Revert PR 83 and rebuild previous Node 20 Nest 10 React 18 images; no database rollback</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="str">
+        <x:v>ioredis 6 and Expo Router 58 remain rejected until their TypeORM and Expo SDK peer lines move; Terraform CLI unavailable locally</x:v>
+      </x:c>
+      <x:c r="K19" s="26" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L19" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="27" t="str">
+        <x:v>DEP-003</x:v>
+      </x:c>
+      <x:c r="B20" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
+        <x:v>dependabot/npm_and_yarn/backend/glob-10.5.0</x:v>
+      </x:c>
+      <x:c r="D20" s="27" t="str">
+        <x:v>0935ede</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>8b5a62b</x:v>
+      </x:c>
+      <x:c r="F20" s="27" t="str">
+        <x:v>WOW-MD PRs 18 20 21 22 27 and 53; reviewed through b373bb4</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="str">
+        <x:v>Production backend E2E frontend mobile Docker CodeQL secrets and governance passed on the final head; local governance 10 of 10 and Node 26 backend plus nginx 1.31 frontend image builds passed</x:v>
+      </x:c>
+      <x:c r="H20" s="27" t="str">
+        <x:v>Rebuild backend and frontend images with Node 26 and nginx 1.31; no application schema change</x:v>
+      </x:c>
+      <x:c r="I20" s="27" t="str">
+        <x:v>Revert PR 84 and rebuild previous images; no database rollback</x:v>
+      </x:c>
+      <x:c r="J20" s="27" t="str">
+        <x:v>Terraform provider and module constraints still require plan evidence before AWS apply</x:v>
+      </x:c>
+      <x:c r="K20" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L20" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K9">
+  <x:conditionalFormatting sqref="K6:K20">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6863,7 +6612,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5c780db6fa46b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aaf73c040d340a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize dependency tracking (#86)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb66fa110142f4493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R278300a9d37147eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R916ce95896314575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R1dc83eb342434ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R4b56ed2da5e8408d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R578d06b1a37b4258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R21b62ecafdd34f52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re1101413a5594e5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R41024dbb5e2940a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R6b626566f817463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4dac9e61b8f647e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R726792ba74a444a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rac8d13ad987e4019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Raf4371b23e3349cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R40cff3d2fe8b4e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R259d15eeee2647ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R83ec67f2a1ad4bef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rae9434a4a6d442b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rc5bbb6216a3d4213"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rd9227feb95244459"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,23 +68,8 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF16794A"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF7A4B00"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FFB42318"/>
-      <x:name val="Arial"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -96,88 +81,23 @@
         <x:fgColor rgb="FF6E1026"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7F6EC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF4CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDE8E8"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
   <x:borders count="7">
-    <x:border/>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -186,35 +106,53 @@
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFD9CDD0"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFD9CDD0"/>
       </x:top>
       <x:bottom style="thin">
         <x:color rgb="FFD9CDD0"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFD9CDD0"/>
       </x:top>
+      <x:bottom/>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="76">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -303,102 +241,6 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="16" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="17" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -410,7 +252,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -420,7 +262,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -430,7 +272,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -441,7 +283,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -451,7 +293,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -461,7 +303,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -472,7 +314,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -482,7 +324,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -492,7 +334,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -503,7 +345,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -513,7 +355,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -523,7 +365,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -534,7 +376,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -544,7 +386,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -554,7 +396,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -565,7 +407,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -575,7 +417,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -585,7 +427,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -595,7 +437,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -605,7 +447,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -616,7 +458,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -626,7 +468,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -636,7 +478,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -646,7 +488,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -656,7 +498,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -667,7 +509,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -677,7 +519,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -687,7 +529,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -697,7 +539,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -707,7 +549,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -718,7 +560,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -728,7 +570,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -738,7 +580,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -748,7 +590,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -758,7 +600,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -769,7 +611,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -779,7 +621,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -789,7 +631,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -800,7 +642,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -810,7 +652,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -1016,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d9ee8990eeb43a3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08294142a8e34b91"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1026,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1047,7 +889,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Requirement"/>
@@ -1062,7 +904,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Layer"/>
@@ -1077,7 +919,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -1127,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1146,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1166,7 +1008,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1393,7 +1235,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-06. Reconciled to canonical registers and final merged PR/issue state.</x:v>
+        <x:v>As of 2026-10-06. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1421,19 +1263,21 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>34</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$41)</x:f>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$38,"P0",'Open Items'!$F$6:$F$38,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$41,"P0",'Open Items'!$F$6:$F$41,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H6" s="39" t="n">
+        <x:f>B7</x:f>
         <x:v>21</x:v>
       </x:c>
     </x:row>
@@ -1442,6 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1455,6 +1300,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H7" s="39" t="n">
+        <x:f>B8</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1463,19 +1309,21 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$18,"Open")</x:f>
+        <x:f>COUNTIF(Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="H8" s="39" t="n">
+        <x:f>B9</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1484,19 +1332,21 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$18,"P0",Risks!$H$6:$H$18,"Open")</x:f>
+        <x:f>COUNTIFS(Risks!$E$6:$E$19,"P0",Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H9" s="39" t="n">
+        <x:f>B10</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1505,20 +1355,22 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIF(Requirements!$G$6:$G$23,"Approved")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF(Requirements!$G$6:$G$27,"Approved")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G10" s="39" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="H10" s="39" t="n">
-        <x:v>12</x:v>
+        <x:f>B11</x:f>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1526,7 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>12</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Done")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1625,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4505c1f091224785"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903a4fe60ae145b1"/>
 </x:worksheet>
 </file>
 
@@ -2047,36 +1900,62 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="27" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>DOC-015</x:v>
       </x:c>
-      <x:c r="B20" s="27" t="str">
-        <x:v>Zoho Mail SMTP operating guide</x:v>
-      </x:c>
-      <x:c r="C20" s="27" t="str">
+      <x:c r="B20" s="26" t="str">
+        <x:v>Zoho SSO and mail operating guide</x:v>
+      </x:c>
+      <x:c r="C20" s="26" t="str">
         <x:v>docs/operations/zoho-mail.md</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="str">
+      <x:c r="D20" s="26" t="str">
         <x:v>Security and operations</x:v>
       </x:c>
-      <x:c r="E20" s="27" t="str">
+      <x:c r="E20" s="26" t="str">
         <x:v>Approved candidate</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>Quarterly or provider change</x:v>
       </x:c>
-      <x:c r="G20" s="27" t="str">
-        <x:v>2026-10-04</x:v>
-      </x:c>
-      <x:c r="H20" s="27" t="str">
-        <x:v>SEC-001 OPS-003</x:v>
+      <x:c r="G20" s="26" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="H20" s="26" t="str">
+        <x:v>SEC-001 AUTH-001 OPS-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="27" t="str">
+        <x:v>DOC-016</x:v>
+      </x:c>
+      <x:c r="B21" s="27" t="str">
+        <x:v>Dependency remediation record</x:v>
+      </x:c>
+      <x:c r="C21" s="27" t="str">
+        <x:v>docs/security/dependency-remediation-2026-10-04.md</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>Approved candidate</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="str">
+        <x:v>Each dependency change</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="str">
+        <x:v>2026-10-05</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="str">
+        <x:v>DEP-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E20">
+  <x:conditionalFormatting sqref="E6:E21">
     <x:cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="35" priority="3" operator="containsText" text="Blocked"/>
@@ -2085,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc4fcdd7c5647e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16e3b18f8eff45a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2179,7 +2058,7 @@
       <x:c r="E6" s="25" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F6" s="70" t="str">
+      <x:c r="F6" s="25" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G6" s="25" t="str">
@@ -2218,7 +2097,7 @@
       <x:c r="E7" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F7" s="71" t="str">
+      <x:c r="F7" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G7" s="26" t="str">
@@ -2259,7 +2138,7 @@
       <x:c r="E8" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F8" s="71" t="str">
+      <x:c r="F8" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
@@ -2298,7 +2177,7 @@
       <x:c r="E9" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F9" s="71" t="str">
+      <x:c r="F9" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G9" s="26" t="str">
@@ -2337,7 +2216,7 @@
       <x:c r="E10" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F10" s="71" t="str">
+      <x:c r="F10" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
@@ -2376,7 +2255,7 @@
       <x:c r="E11" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F11" s="71" t="str">
+      <x:c r="F11" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G11" s="26" t="str">
@@ -2417,7 +2296,7 @@
       <x:c r="E12" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F12" s="72" t="str">
+      <x:c r="F12" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G12" s="26" t="str">
@@ -2456,7 +2335,7 @@
       <x:c r="E13" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F13" s="72" t="str">
+      <x:c r="F13" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
@@ -2497,7 +2376,7 @@
       <x:c r="E14" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F14" s="72" t="str">
+      <x:c r="F14" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G14" s="26" t="str">
@@ -2538,7 +2417,7 @@
       <x:c r="E15" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F15" s="72" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G15" s="26" t="str">
@@ -2577,7 +2456,7 @@
       <x:c r="E16" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F16" s="72" t="str">
+      <x:c r="F16" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G16" s="26" t="str">
@@ -2616,7 +2495,7 @@
       <x:c r="E17" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F17" s="72" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G17" s="26" t="str">
@@ -2655,7 +2534,7 @@
       <x:c r="E18" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F18" s="72" t="str">
+      <x:c r="F18" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G18" s="26" t="str">
@@ -2694,7 +2573,7 @@
       <x:c r="E19" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F19" s="72" t="str">
+      <x:c r="F19" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G19" s="26" t="str">
@@ -2733,7 +2612,7 @@
       <x:c r="E20" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F20" s="72" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G20" s="26" t="str">
@@ -2772,7 +2651,7 @@
       <x:c r="E21" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F21" s="72" t="str">
+      <x:c r="F21" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G21" s="26" t="str">
@@ -2811,7 +2690,7 @@
       <x:c r="E22" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F22" s="72" t="str">
+      <x:c r="F22" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G22" s="26" t="str">
@@ -2850,7 +2729,7 @@
       <x:c r="E23" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F23" s="72" t="str">
+      <x:c r="F23" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G23" s="26" t="str">
@@ -2889,7 +2768,7 @@
       <x:c r="E24" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F24" s="72" t="str">
+      <x:c r="F24" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G24" s="26" t="str">
@@ -2928,7 +2807,7 @@
       <x:c r="E25" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F25" s="72" t="str">
+      <x:c r="F25" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G25" s="26" t="str">
@@ -2967,7 +2846,7 @@
       <x:c r="E26" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F26" s="72" t="str">
+      <x:c r="F26" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G26" s="26" t="str">
@@ -3006,7 +2885,7 @@
       <x:c r="E27" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F27" s="72" t="str">
+      <x:c r="F27" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G27" s="26" t="str">
@@ -3045,7 +2924,7 @@
       <x:c r="E28" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F28" s="72" t="str">
+      <x:c r="F28" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G28" s="26" t="str">
@@ -3084,7 +2963,7 @@
       <x:c r="E29" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F29" s="72" t="str">
+      <x:c r="F29" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G29" s="26" t="str">
@@ -3123,7 +3002,7 @@
       <x:c r="E30" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F30" s="72" t="str">
+      <x:c r="F30" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G30" s="26" t="str">
@@ -3162,7 +3041,7 @@
       <x:c r="E31" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F31" s="72" t="str">
+      <x:c r="F31" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G31" s="26" t="str">
@@ -3199,7 +3078,7 @@
       <x:c r="E32" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F32" s="73" t="str">
+      <x:c r="F32" s="26" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G32" s="26" t="str">
@@ -3240,7 +3119,7 @@
       <x:c r="E33" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="F33" s="72" t="str">
+      <x:c r="F33" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G33" s="26" t="str">
@@ -3277,7 +3156,7 @@
       <x:c r="E34" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F34" s="72" t="str">
+      <x:c r="F34" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G34" s="26" t="str">
@@ -3316,7 +3195,7 @@
       <x:c r="E35" s="26" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="F35" s="72" t="str">
+      <x:c r="F35" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="G35" s="26" t="str">
@@ -3355,7 +3234,7 @@
       <x:c r="E36" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F36" s="71" t="str">
+      <x:c r="F36" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G36" s="26" t="str">
@@ -3379,599 +3258,216 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="30" customHeight="1">
-      <x:c r="A37" s="27" t="str">
+      <x:c r="A37" s="26" t="str">
         <x:v>GOV-002</x:v>
       </x:c>
-      <x:c r="B37" s="27" t="str">
+      <x:c r="B37" s="26" t="str">
         <x:v>Establish SDLC knowledge and tracking system</x:v>
       </x:c>
-      <x:c r="C37" s="27" t="str">
+      <x:c r="C37" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="D37" s="27" t="str">
+      <x:c r="D37" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="E37" s="27" t="str">
+      <x:c r="E37" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F37" s="74" t="str">
+      <x:c r="F37" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G37" s="27" t="str">
+      <x:c r="G37" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H37" s="27" t="str"/>
-      <x:c r="I37" s="27" t="str">
+      <x:c r="H37" s="26" t="str"/>
+      <x:c r="I37" s="26" t="str">
         <x:v>Markdown CSV Excel issues PR protocol and Obsidian index are linked and verified</x:v>
       </x:c>
-      <x:c r="J37" s="27" t="str">
+      <x:c r="J37" s="26" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K37" s="27" t="str">
+      <x:c r="K37" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/37</x:v>
       </x:c>
-      <x:c r="L37" s="27" t="str">
+      <x:c r="L37" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/49</x:v>
       </x:c>
-      <x:c r="M37" s="30" t="str">
+      <x:c r="M37" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" t="str">
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="26" t="str">
         <x:v>GOV-003</x:v>
       </x:c>
-      <x:c r="B38" t="str">
+      <x:c r="B38" s="26" t="str">
         <x:v>Reconcile authentication and dependency tracking</x:v>
       </x:c>
-      <x:c r="C38" t="str">
+      <x:c r="C38" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="D38" t="str">
+      <x:c r="D38" s="26" t="str">
         <x:v>Governance</x:v>
       </x:c>
-      <x:c r="E38" t="str">
+      <x:c r="E38" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F38" s="75" t="str">
+      <x:c r="F38" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G38" t="str">
+      <x:c r="G38" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H38" t="str">
+      <x:c r="H38" s="26" t="str">
         <x:v>SEC-001,DEP-001</x:v>
       </x:c>
-      <x:c r="I38" t="str">
+      <x:c r="I38" s="26" t="str">
         <x:v>Canonical registers workbook and operating guidance match the implemented authentication policy and dependency evidence</x:v>
       </x:c>
-      <x:c r="J38" t="str">
+      <x:c r="J38" s="26" t="str">
         <x:v>User request</x:v>
       </x:c>
-      <x:c r="K38" t="str">
+      <x:c r="K38" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/60</x:v>
       </x:c>
-      <x:c r="L38" t="str">
+      <x:c r="L38" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
       </x:c>
-      <x:c r="M38" t="str">
+      <x:c r="M38" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" t="str">
+    <x:row r="39" ht="30" customHeight="1">
+      <x:c r="A39" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="B39" t="str">
+      <x:c r="B39" s="26" t="str">
         <x:v>Integrate committed immersive consumer UI</x:v>
       </x:c>
-      <x:c r="C39" t="str">
+      <x:c r="C39" s="26" t="str">
         <x:v>Source intake</x:v>
       </x:c>
-      <x:c r="D39" t="str">
+      <x:c r="D39" s="26" t="str">
         <x:v>UI/UX synchronization</x:v>
       </x:c>
-      <x:c r="E39" t="str">
+      <x:c r="E39" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F39" s="51" t="str">
+      <x:c r="F39" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G39" t="str">
+      <x:c r="G39" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H39" t="str">
+      <x:c r="H39" s="26" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="I39" t="str">
+      <x:c r="I39" s="26" t="str">
         <x:v>Committed public login registration and consumer portal UI is present in WOW-MD and production without overwriting production hardening</x:v>
       </x:c>
-      <x:c r="J39" t="str">
+      <x:c r="J39" s="26" t="str">
         <x:v>WOW-MD PR 50 and production issue 76</x:v>
       </x:c>
-      <x:c r="K39" t="str">
+      <x:c r="K39" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/76</x:v>
       </x:c>
-      <x:c r="L39" t="str">
+      <x:c r="L39" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
       </x:c>
-      <x:c r="M39" t="str">
+      <x:c r="M39" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40"/>
-      <x:c r="B40"/>
-      <x:c r="C40"/>
-      <x:c r="D40"/>
-      <x:c r="E40"/>
-      <x:c r="F40"/>
-      <x:c r="G40"/>
-      <x:c r="H40"/>
-      <x:c r="I40"/>
-      <x:c r="J40"/>
-      <x:c r="K40"/>
-      <x:c r="L40"/>
-      <x:c r="M40"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41"/>
-      <x:c r="B41"/>
-      <x:c r="C41"/>
-      <x:c r="D41"/>
-      <x:c r="E41"/>
-      <x:c r="F41"/>
-      <x:c r="G41"/>
-      <x:c r="H41"/>
-      <x:c r="I41"/>
-      <x:c r="J41"/>
-      <x:c r="K41"/>
-      <x:c r="L41"/>
-      <x:c r="M41"/>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42"/>
-      <x:c r="B42"/>
-      <x:c r="C42"/>
-      <x:c r="D42"/>
-      <x:c r="E42"/>
-      <x:c r="F42"/>
-      <x:c r="G42"/>
-      <x:c r="H42"/>
-      <x:c r="I42"/>
-      <x:c r="J42"/>
-      <x:c r="K42"/>
-      <x:c r="L42"/>
-      <x:c r="M42"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43"/>
-      <x:c r="B43"/>
-      <x:c r="C43"/>
-      <x:c r="D43"/>
-      <x:c r="E43"/>
-      <x:c r="F43"/>
-      <x:c r="G43"/>
-      <x:c r="H43"/>
-      <x:c r="I43"/>
-      <x:c r="J43"/>
-      <x:c r="K43"/>
-      <x:c r="L43"/>
-      <x:c r="M43"/>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44"/>
-      <x:c r="B44"/>
-      <x:c r="C44"/>
-      <x:c r="D44"/>
-      <x:c r="E44"/>
-      <x:c r="F44"/>
-      <x:c r="G44"/>
-      <x:c r="H44"/>
-      <x:c r="I44"/>
-      <x:c r="J44"/>
-      <x:c r="K44"/>
-      <x:c r="L44"/>
-      <x:c r="M44"/>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45"/>
-      <x:c r="B45"/>
-      <x:c r="C45"/>
-      <x:c r="D45"/>
-      <x:c r="E45"/>
-      <x:c r="F45"/>
-      <x:c r="G45"/>
-      <x:c r="H45"/>
-      <x:c r="I45"/>
-      <x:c r="J45"/>
-      <x:c r="K45"/>
-      <x:c r="L45"/>
-      <x:c r="M45"/>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46"/>
-      <x:c r="B46"/>
-      <x:c r="C46"/>
-      <x:c r="D46"/>
-      <x:c r="E46"/>
-      <x:c r="F46"/>
-      <x:c r="G46"/>
-      <x:c r="H46"/>
-      <x:c r="I46"/>
-      <x:c r="J46"/>
-      <x:c r="K46"/>
-      <x:c r="L46"/>
-      <x:c r="M46"/>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47"/>
-      <x:c r="B47"/>
-      <x:c r="C47"/>
-      <x:c r="D47"/>
-      <x:c r="E47"/>
-      <x:c r="F47"/>
-      <x:c r="G47"/>
-      <x:c r="H47"/>
-      <x:c r="I47"/>
-      <x:c r="J47"/>
-      <x:c r="K47"/>
-      <x:c r="L47"/>
-      <x:c r="M47"/>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48"/>
-      <x:c r="B48"/>
-      <x:c r="C48"/>
-      <x:c r="D48"/>
-      <x:c r="E48"/>
-      <x:c r="F48"/>
-      <x:c r="G48"/>
-      <x:c r="H48"/>
-      <x:c r="I48"/>
-      <x:c r="J48"/>
-      <x:c r="K48"/>
-      <x:c r="L48"/>
-      <x:c r="M48"/>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49"/>
-      <x:c r="B49"/>
-      <x:c r="C49"/>
-      <x:c r="D49"/>
-      <x:c r="E49"/>
-      <x:c r="F49"/>
-      <x:c r="G49"/>
-      <x:c r="H49"/>
-      <x:c r="I49"/>
-      <x:c r="J49"/>
-      <x:c r="K49"/>
-      <x:c r="L49"/>
-      <x:c r="M49"/>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50"/>
-      <x:c r="B50"/>
-      <x:c r="C50"/>
-      <x:c r="D50"/>
-      <x:c r="E50"/>
-      <x:c r="F50"/>
-      <x:c r="G50"/>
-      <x:c r="H50"/>
-      <x:c r="I50"/>
-      <x:c r="J50"/>
-      <x:c r="K50"/>
-      <x:c r="L50"/>
-      <x:c r="M50"/>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51"/>
-      <x:c r="B51"/>
-      <x:c r="C51"/>
-      <x:c r="D51"/>
-      <x:c r="E51"/>
-      <x:c r="F51"/>
-      <x:c r="G51"/>
-      <x:c r="H51"/>
-      <x:c r="I51"/>
-      <x:c r="J51"/>
-      <x:c r="K51"/>
-      <x:c r="L51"/>
-      <x:c r="M51"/>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52"/>
-      <x:c r="B52"/>
-      <x:c r="C52"/>
-      <x:c r="D52"/>
-      <x:c r="E52"/>
-      <x:c r="F52"/>
-      <x:c r="G52"/>
-      <x:c r="H52"/>
-      <x:c r="I52"/>
-      <x:c r="J52"/>
-      <x:c r="K52"/>
-      <x:c r="L52"/>
-      <x:c r="M52"/>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53"/>
-      <x:c r="B53"/>
-      <x:c r="C53"/>
-      <x:c r="D53"/>
-      <x:c r="E53"/>
-      <x:c r="F53"/>
-      <x:c r="G53"/>
-      <x:c r="H53"/>
-      <x:c r="I53"/>
-      <x:c r="J53"/>
-      <x:c r="K53"/>
-      <x:c r="L53"/>
-      <x:c r="M53"/>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54"/>
-      <x:c r="B54"/>
-      <x:c r="C54"/>
-      <x:c r="D54"/>
-      <x:c r="E54"/>
-      <x:c r="F54"/>
-      <x:c r="G54"/>
-      <x:c r="H54"/>
-      <x:c r="I54"/>
-      <x:c r="J54"/>
-      <x:c r="K54"/>
-      <x:c r="L54"/>
-      <x:c r="M54"/>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55"/>
-      <x:c r="B55"/>
-      <x:c r="C55"/>
-      <x:c r="D55"/>
-      <x:c r="E55"/>
-      <x:c r="F55"/>
-      <x:c r="G55"/>
-      <x:c r="H55"/>
-      <x:c r="I55"/>
-      <x:c r="J55"/>
-      <x:c r="K55"/>
-      <x:c r="L55"/>
-      <x:c r="M55"/>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56"/>
-      <x:c r="B56"/>
-      <x:c r="C56"/>
-      <x:c r="D56"/>
-      <x:c r="E56"/>
-      <x:c r="F56"/>
-      <x:c r="G56"/>
-      <x:c r="H56"/>
-      <x:c r="I56"/>
-      <x:c r="J56"/>
-      <x:c r="K56"/>
-      <x:c r="L56"/>
-      <x:c r="M56"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57"/>
-      <x:c r="B57"/>
-      <x:c r="C57"/>
-      <x:c r="D57"/>
-      <x:c r="E57"/>
-      <x:c r="F57"/>
-      <x:c r="G57"/>
-      <x:c r="H57"/>
-      <x:c r="I57"/>
-      <x:c r="J57"/>
-      <x:c r="K57"/>
-      <x:c r="L57"/>
-      <x:c r="M57"/>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58"/>
-      <x:c r="B58"/>
-      <x:c r="C58"/>
-      <x:c r="D58"/>
-      <x:c r="E58"/>
-      <x:c r="F58"/>
-      <x:c r="G58"/>
-      <x:c r="H58"/>
-      <x:c r="I58"/>
-      <x:c r="J58"/>
-      <x:c r="K58"/>
-      <x:c r="L58"/>
-      <x:c r="M58"/>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59"/>
-      <x:c r="B59"/>
-      <x:c r="C59"/>
-      <x:c r="D59"/>
-      <x:c r="E59"/>
-      <x:c r="F59"/>
-      <x:c r="G59"/>
-      <x:c r="H59"/>
-      <x:c r="I59"/>
-      <x:c r="J59"/>
-      <x:c r="K59"/>
-      <x:c r="L59"/>
-      <x:c r="M59"/>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60"/>
-      <x:c r="B60"/>
-      <x:c r="C60"/>
-      <x:c r="D60"/>
-      <x:c r="E60"/>
-      <x:c r="F60"/>
-      <x:c r="G60"/>
-      <x:c r="H60"/>
-      <x:c r="I60"/>
-      <x:c r="J60"/>
-      <x:c r="K60"/>
-      <x:c r="L60"/>
-      <x:c r="M60"/>
-    </x:row>
-    <x:row r="61">
-      <x:c r="A61"/>
-      <x:c r="B61"/>
-      <x:c r="C61"/>
-      <x:c r="D61"/>
-      <x:c r="E61"/>
-      <x:c r="F61"/>
-      <x:c r="G61"/>
-      <x:c r="H61"/>
-      <x:c r="I61"/>
-      <x:c r="J61"/>
-      <x:c r="K61"/>
-      <x:c r="L61"/>
-      <x:c r="M61"/>
-    </x:row>
-    <x:row r="62">
-      <x:c r="A62"/>
-      <x:c r="B62"/>
-      <x:c r="C62"/>
-      <x:c r="D62"/>
-      <x:c r="E62"/>
-      <x:c r="F62"/>
-      <x:c r="G62"/>
-      <x:c r="H62"/>
-      <x:c r="I62"/>
-      <x:c r="J62"/>
-      <x:c r="K62"/>
-      <x:c r="L62"/>
-      <x:c r="M62"/>
-    </x:row>
-    <x:row r="63">
-      <x:c r="A63"/>
-      <x:c r="B63"/>
-      <x:c r="C63"/>
-      <x:c r="D63"/>
-      <x:c r="E63"/>
-      <x:c r="F63"/>
-      <x:c r="G63"/>
-      <x:c r="H63"/>
-      <x:c r="I63"/>
-      <x:c r="J63"/>
-      <x:c r="K63"/>
-      <x:c r="L63"/>
-      <x:c r="M63"/>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64"/>
-      <x:c r="B64"/>
-      <x:c r="C64"/>
-      <x:c r="D64"/>
-      <x:c r="E64"/>
-      <x:c r="F64"/>
-      <x:c r="G64"/>
-      <x:c r="H64"/>
-      <x:c r="I64"/>
-      <x:c r="J64"/>
-      <x:c r="K64"/>
-      <x:c r="L64"/>
-      <x:c r="M64"/>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65"/>
-      <x:c r="B65"/>
-      <x:c r="C65"/>
-      <x:c r="D65"/>
-      <x:c r="E65"/>
-      <x:c r="F65"/>
-      <x:c r="G65"/>
-      <x:c r="H65"/>
-      <x:c r="I65"/>
-      <x:c r="J65"/>
-      <x:c r="K65"/>
-      <x:c r="L65"/>
-      <x:c r="M65"/>
-    </x:row>
-    <x:row r="66">
-      <x:c r="A66"/>
-      <x:c r="B66"/>
-      <x:c r="C66"/>
-      <x:c r="D66"/>
-      <x:c r="E66"/>
-      <x:c r="F66"/>
-      <x:c r="G66"/>
-      <x:c r="H66"/>
-      <x:c r="I66"/>
-      <x:c r="J66"/>
-      <x:c r="K66"/>
-      <x:c r="L66"/>
-      <x:c r="M66"/>
-    </x:row>
-    <x:row r="67">
-      <x:c r="A67"/>
-      <x:c r="B67"/>
-      <x:c r="C67"/>
-      <x:c r="D67"/>
-      <x:c r="E67"/>
-      <x:c r="F67"/>
-      <x:c r="G67"/>
-      <x:c r="H67"/>
-      <x:c r="I67"/>
-      <x:c r="J67"/>
-      <x:c r="K67"/>
-      <x:c r="L67"/>
-      <x:c r="M67"/>
-    </x:row>
-    <x:row r="68">
-      <x:c r="A68"/>
-      <x:c r="B68"/>
-      <x:c r="C68"/>
-      <x:c r="D68"/>
-      <x:c r="E68"/>
-      <x:c r="F68"/>
-      <x:c r="G68"/>
-      <x:c r="H68"/>
-      <x:c r="I68"/>
-      <x:c r="J68"/>
-      <x:c r="K68"/>
-      <x:c r="L68"/>
-      <x:c r="M68"/>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69"/>
-      <x:c r="B69"/>
-      <x:c r="C69"/>
-      <x:c r="D69"/>
-      <x:c r="E69"/>
-      <x:c r="F69"/>
-      <x:c r="G69"/>
-      <x:c r="H69"/>
-      <x:c r="I69"/>
-      <x:c r="J69"/>
-      <x:c r="K69"/>
-      <x:c r="L69"/>
-      <x:c r="M69"/>
-    </x:row>
-    <x:row r="70">
-      <x:c r="A70"/>
-      <x:c r="B70"/>
-      <x:c r="C70"/>
-      <x:c r="D70"/>
-      <x:c r="E70"/>
-      <x:c r="F70"/>
-      <x:c r="G70"/>
-      <x:c r="H70"/>
-      <x:c r="I70"/>
-      <x:c r="J70"/>
-      <x:c r="K70"/>
-      <x:c r="L70"/>
-      <x:c r="M70"/>
+    <x:row r="40" ht="30" customHeight="1">
+      <x:c r="A40" s="26" t="str">
+        <x:v>DEP-002</x:v>
+      </x:c>
+      <x:c r="B40" s="26" t="str">
+        <x:v>Reconcile compatible dependency upgrade set</x:v>
+      </x:c>
+      <x:c r="C40" s="26" t="str">
+        <x:v>Public beta safety</x:v>
+      </x:c>
+      <x:c r="D40" s="26" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E40" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F40" s="26" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G40" s="26" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H40" s="26" t="str">
+        <x:v>DEP-001</x:v>
+      </x:c>
+      <x:c r="I40" s="26" t="str">
+        <x:v>Compatible React, Nest, test, CI and Terraform upgrades pass all mandatory suites; incompatible ioredis 6 and Expo Router 58 upgrades remain explicitly constrained</x:v>
+      </x:c>
+      <x:c r="J40" s="26" t="str">
+        <x:v>WOW-MD PR 52</x:v>
+      </x:c>
+      <x:c r="K40" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/82</x:v>
+      </x:c>
+      <x:c r="L40" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/83</x:v>
+      </x:c>
+      <x:c r="M40" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="A41" s="27" t="str">
+        <x:v>DEP-003</x:v>
+      </x:c>
+      <x:c r="B41" s="27" t="str">
+        <x:v>Complete remaining dependency source mirrors</x:v>
+      </x:c>
+      <x:c r="C41" s="27" t="str">
+        <x:v>Public beta safety</x:v>
+      </x:c>
+      <x:c r="D41" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E41" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F41" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G41" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H41" s="27" t="str">
+        <x:v>DEP-002</x:v>
+      </x:c>
+      <x:c r="I41" s="27" t="str">
+        <x:v>Production carries the reviewed glob lockfile, Node and nginx images, AWS modules and GitHub Actions versions from WOW-MD with production-only workflows upgraded consistently</x:v>
+      </x:c>
+      <x:c r="J41" s="27" t="str">
+        <x:v>WOW-MD PRs 18 20 21 22 27 53</x:v>
+      </x:c>
+      <x:c r="K41" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/85</x:v>
+      </x:c>
+      <x:c r="L41" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
+      </x:c>
+      <x:c r="M41" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E37">
+  <x:conditionalFormatting sqref="E6:E41">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F37">
+  <x:conditionalFormatting sqref="F6:F41">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3980,7 +3476,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2839a1a98d304860"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R774f5477c69b4acb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4426,25 +3922,117 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="27" t="str">
+      <x:c r="A23" s="26" t="str">
         <x:v>REQ-REV-001</x:v>
       </x:c>
-      <x:c r="B23" s="27" t="str">
+      <x:c r="B23" s="26" t="str">
         <x:v>AWS migration readiness reports INR 1.2M target and INR 1.5M preferred monthly net revenue</x:v>
       </x:c>
-      <x:c r="C23" s="27" t="str">
+      <x:c r="C23" s="26" t="str">
         <x:v>Migration design</x:v>
       </x:c>
-      <x:c r="D23" s="27" t="str">
+      <x:c r="D23" s="26" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="E23" s="27" t="str">
+      <x:c r="E23" s="26" t="str">
         <x:v>Admin readiness UI test</x:v>
       </x:c>
-      <x:c r="F23" s="27" t="str">
+      <x:c r="F23" s="26" t="str">
         <x:v>UI-001</x:v>
       </x:c>
-      <x:c r="G23" s="27" t="str">
+      <x:c r="G23" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="26" t="str">
+        <x:v>REQ-AUTH-001</x:v>
+      </x:c>
+      <x:c r="B24" s="26" t="str">
+        <x:v>Administrators authenticate through Zoho SSO and do not require routine application TOTP</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E24" s="26" t="str">
+        <x:v>Authentication integration tests and controlled Zoho sign-in evidence</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G24" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="26" t="str">
+        <x:v>REQ-AUTH-002</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="str">
+        <x:v>Existing users may sign in with Zoho SSO or username email or mobile plus password and any valid email provider is accepted</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>Backend frontend mobile and Playwright authentication tests</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="A26" s="26" t="str">
+        <x:v>REQ-AUTH-003</x:v>
+      </x:c>
+      <x:c r="B26" s="26" t="str">
+        <x:v>OTP is used only for signup/contact verification and password recovery and never as passwordless login</x:v>
+      </x:c>
+      <x:c r="C26" s="26" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="str">
+        <x:v>Route inventory and authentication tests</x:v>
+      </x:c>
+      <x:c r="F26" s="26" t="str">
+        <x:v>SEC-001</x:v>
+      </x:c>
+      <x:c r="G26" s="26" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="27" t="str">
+        <x:v>REQ-AUTH-004</x:v>
+      </x:c>
+      <x:c r="B27" s="27" t="str">
+        <x:v>Zoho domain DNS sender mailbox SMTP application password and production OAuth callback are configured only at the final deployment gate</x:v>
+      </x:c>
+      <x:c r="C27" s="27" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="D27" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="E27" s="27" t="str">
+        <x:v>Final release checklist and controlled delivery/SSO evidence</x:v>
+      </x:c>
+      <x:c r="F27" s="27" t="str">
+        <x:v>SEC-001,REL-001</x:v>
+      </x:c>
+      <x:c r="G27" s="27" t="str">
         <x:v>Approved</x:v>
       </x:c>
     </x:row>
@@ -4452,10 +4040,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D6:D23">
+  <x:conditionalFormatting sqref="D6:D27">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="G6:G23">
+  <x:conditionalFormatting sqref="G6:G27">
     <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Blocked"/>
@@ -4464,7 +4052,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08c672e326c947c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d83ca7b8304ed7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4749,118 +4337,118 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="27" t="str">
+      <x:c r="A16" s="26" t="str">
         <x:v>QA-GOV-001</x:v>
       </x:c>
-      <x:c r="B16" s="27" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>Source synchronization</x:v>
       </x:c>
-      <x:c r="C16" s="27" t="str">
+      <x:c r="C16" s="26" t="str">
         <x:v>Private-source report and shared-code mirror gate</x:v>
       </x:c>
-      <x:c r="D16" s="27" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>PR 55 local evidence</x:v>
       </x:c>
-      <x:c r="E16" s="27" t="str">
+      <x:c r="E16" s="26" t="str">
         <x:v>19 of 19 governance and synchronization tests passed</x:v>
       </x:c>
-      <x:c r="F16" s="27" t="str">
+      <x:c r="F16" s="26" t="str">
         <x:v>Configure WOW_SYNC_TOKEN and capture first scheduled artifact</x:v>
       </x:c>
-      <x:c r="G16" s="27" t="str">
+      <x:c r="G16" s="26" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="26" t="str">
+        <x:v>QA-SEC-002</x:v>
+      </x:c>
+      <x:c r="B17" s="26" t="str">
+        <x:v>WebSocket authorization</x:v>
+      </x:c>
+      <x:c r="C17" s="26" t="str">
+        <x:v>Origin token-version forced-reset call relay and presence audience</x:v>
+      </x:c>
+      <x:c r="D17" s="26" t="str">
+        <x:v>SEC-002 PR 62</x:v>
+      </x:c>
+      <x:c r="E17" s="26" t="str">
+        <x:v>11 focused gateway tests and complete backend suite 800 passed with 9 skipped</x:v>
+      </x:c>
+      <x:c r="F17" s="26" t="str">
+        <x:v>Repeat browser and native reconnect smoke tests on Railway candidate</x:v>
+      </x:c>
+      <x:c r="G17" s="26" t="str">
+        <x:v>SEC-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="26" t="str">
+        <x:v>QA-SEC-003</x:v>
+      </x:c>
+      <x:c r="B18" s="26" t="str">
+        <x:v>HTTP and migration integrity</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>Production Swagger headers migration uniqueness fresh and upgrade paths</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="str">
+        <x:v>SEC-003 PR 63</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="str">
+        <x:v>2 HTTP tests; 2 verifier tests; 93-file verification; 794 backend tests passed with 9 skipped; fresh and upgraded databases passed</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="str">
+        <x:v>Repeat ingress header checks on Railway candidate</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
+        <x:v>SEC-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="26" t="str">
+        <x:v>QA-OPS-001</x:v>
+      </x:c>
+      <x:c r="B19" s="26" t="str">
+        <x:v>Replica safety</x:v>
+      </x:c>
+      <x:c r="C19" s="26" t="str">
+        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="str">
+        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="str">
+        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
+      </x:c>
+      <x:c r="F19" s="26" t="str">
+        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
+      </x:c>
+      <x:c r="G19" s="26" t="str">
+        <x:v>OPS-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="27" t="str">
         <x:v>QA-OBS-001</x:v>
       </x:c>
-      <x:c r="B17" t="str">
+      <x:c r="B20" s="27" t="str">
         <x:v>Observability</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C20" s="27" t="str">
         <x:v>Request correlation redaction provider logs QA capture audit failures payout sweep and nginx JSON</x:v>
       </x:c>
-      <x:c r="D17" t="str">
-        <x:v>OBS-001 PR 65 and WOW-MD PR 43</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>Focused 20 of 20; full backend 812 passed 9 skipped; typecheck lint nginx contract image build and syntax passed</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>Deploy after SEC-003 and verify live response/log correlation with capture disabled</x:v>
-      </x:c>
-      <x:c r="G17" t="str">
+      <x:c r="D20" s="27" t="str">
+        <x:v>OBS-001 PR 69 and merged WOW-MD PR 43</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>Focused observability and replica-lock integration 27 of 27; typecheck lint and nginx contract passed; protected CI recorded on PR 69</x:v>
+      </x:c>
+      <x:c r="F20" s="27" t="str">
+        <x:v>Verify live response/log correlation with capture disabled</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="str">
         <x:v>OBS-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>QA-SEC-002</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>WebSocket origins tokens calls and presence authorization</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>SEC-002 PR 62 and WOW-MD PR 40</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
-        <x:v>Focused gateways 11 passed; full backend 800 passed 9 skipped; typecheck and lint passed</x:v>
-      </x:c>
-      <x:c r="F18" t="str">
-        <x:v>Run staged hostile-origin and two-account WebSocket smoke</x:v>
-      </x:c>
-      <x:c r="G18" t="str">
-        <x:v>SEC-002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>QA-SEC-003</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="C19" t="str">
-        <x:v>HTTP headers private Swagger and migration integrity</x:v>
-      </x:c>
-      <x:c r="D19" t="str">
-        <x:v>SEC-003 PR 63 and WOW-MD PR 41</x:v>
-      </x:c>
-      <x:c r="E19" t="str">
-        <x:v>HTTP 2 passed; migration verifier 2 passed; 93 migrations verified and clean database upgrade passed; backend 794 passed 9 skipped</x:v>
-      </x:c>
-      <x:c r="F19" t="str">
-        <x:v>Deploy and verify production headers Swagger denial and migration startup</x:v>
-      </x:c>
-      <x:c r="G19" t="str">
-        <x:v>SEC-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>QA-OPS-001</x:v>
-      </x:c>
-      <x:c r="B20" t="str">
-        <x:v>Replica safety</x:v>
-      </x:c>
-      <x:c r="C20" t="str">
-        <x:v>Outbox dispatcher and all scheduled notification payment and maintenance jobs</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>OPS-001 PR 64 and WOW-MD PR 42</x:v>
-      </x:c>
-      <x:c r="E20" t="str">
-        <x:v>Focused two-worker tests 7 of 7; full backend 797 passed 9 skipped; typecheck and lint passed</x:v>
-      </x:c>
-      <x:c r="F20" t="str">
-        <x:v>Run two Railway replicas and confirm one owner and one skipped invocation in correlated logs</x:v>
-      </x:c>
-      <x:c r="G20" t="str">
-        <x:v>OPS-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4869,7 +4457,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e0a146b3665477e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R880cfabdb5234d85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5262,42 +4850,71 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="27" t="str">
+      <x:c r="A18" s="26" t="str">
         <x:v>RISK-013</x:v>
       </x:c>
-      <x:c r="B18" s="27" t="str">
-        <x:v>Public deployment tier is enabled before every administrator enrols MFA</x:v>
-      </x:c>
-      <x:c r="C18" s="27" t="str">
+      <x:c r="B18" s="26" t="str">
+        <x:v>Public deployment tier is enabled before Zoho SSO and administrator recovery are proven</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D18" s="27" t="str">
+      <x:c r="D18" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E18" s="27" t="str">
+      <x:c r="E18" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F18" s="27" t="str">
-        <x:v>Enrol and verify each administrator in restricted staging before selecting public-beta; keep a documented recovery owner</x:v>
-      </x:c>
-      <x:c r="G18" s="27" t="str">
+      <x:c r="F18" s="26" t="str">
+        <x:v>Verify exact OAuth client callback administrator matching-email login Zoho-account MFA and a documented recovery owner in restricted staging before public-beta</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H18" s="27" t="str">
+      <x:c r="H18" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="I18" s="27" t="str">
-        <x:v>SEC-001 PR 56 rejects unenrolled login and existing sessions; staged enrollment evidence still required</x:v>
+      <x:c r="I18" s="26" t="str">
+        <x:v>SEC-001 PR 58 implements Zoho-only administrator login; production Zoho configuration is intentionally deferred to the final gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="27" t="str">
+        <x:v>RISK-014</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="str">
+        <x:v>Framework and mobile build-tool dependency advisories remain after runtime remediation</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="str">
+        <x:v>Block new critical/high runtime advisories; allow only four exact no-fix Expo advisory IDs; schedule Nest major migration and review exceptions each release</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="H19" s="27" t="str">
+        <x:v>Mitigated</x:v>
+      </x:c>
+      <x:c r="I19" s="27" t="str">
+        <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E18">
+  <x:conditionalFormatting sqref="E6:E19">
     <x:cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="H6:H18">
+  <x:conditionalFormatting sqref="H6:H19">
     <x:cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="15" priority="4" operator="containsText" text="Blocked"/>
@@ -5306,7 +4923,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89e8a5d8aab64c7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6374f0038df94186"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5537,16 +5154,16 @@
         <x:v>ACC-007</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>Operational email</x:v>
+        <x:v>Zoho identity and operational email</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>Zoho domain mailbox DNS authentication reports and app-password rotation</x:v>
+        <x:v>OAuth application exact callback domain mailbox DNS authentication reports and SMTP app-password rotation</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
         <x:v>To be confirmed</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
-        <x:v>Zoho SMTP identity</x:v>
+        <x:v>Zoho OAuth and SMTP identities</x:v>
       </x:c>
       <x:c r="F12" s="26" t="str">
         <x:v>GitHub Railway or Kubernetes secrets</x:v>
@@ -5556,7 +5173,7 @@
       </x:c>
       <x:c r="H12" s="29" t="str"/>
       <x:c r="I12" s="26" t="str">
-        <x:v>Low-volume beta only; owner must configure domain MFA app password and first delivery evidence</x:v>
+        <x:v>Configure only at final deployment; protect the Zoho owner with Zoho MFA and retain controlled SSO/mail evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -5621,7 +5238,7 @@
         <x:v>WOW-MD source review</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
-        <x:v>Private repository contents read for scheduled change reports</x:v>
+        <x:v>Repository contents read for scheduled change reports</x:v>
       </x:c>
       <x:c r="D15" s="27" t="str">
         <x:v>RohithTadiparti</x:v>
@@ -5633,11 +5250,11 @@
         <x:v>Production GitHub Actions secret</x:v>
       </x:c>
       <x:c r="G15" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="H15" s="30" t="str"/>
       <x:c r="I15" s="27" t="str">
-        <x:v>Scope only to WOW-MD Contents read; rotate within 90 days</x:v>
+        <x:v>Not technically required while WOW-MD is public; create before returning it private so the private-ready workflow keeps working; scope only to WOW-MD Contents read and rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5653,7 +5270,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c0531a9184d4e9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cdd09bc2d384d86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5992,7 +5609,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14665dc032fd4736"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91ae813e008c4ad1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6125,143 +5742,213 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="27" t="str">
+      <x:c r="A8" s="26" t="str">
         <x:v>CHG-003</x:v>
       </x:c>
-      <x:c r="B8" s="27" t="str">
+      <x:c r="B8" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C8" s="27" t="str">
+      <x:c r="C8" s="26" t="str">
         <x:v>07218b4..de7d8dd (LOCAL ONLY)</x:v>
       </x:c>
-      <x:c r="D8" s="27" t="str">
+      <x:c r="D8" s="26" t="str">
         <x:v>37 committed paths</x:v>
       </x:c>
-      <x:c r="E8" s="27" t="str">
+      <x:c r="E8" s="26" t="str">
         <x:v>Functional UI candidates</x:v>
       </x:c>
-      <x:c r="F8" s="27" t="str">
+      <x:c r="F8" s="26" t="str">
         <x:v>Await source publication and per-commit review</x:v>
       </x:c>
-      <x:c r="G8" s="27" t="str">
+      <x:c r="G8" s="26" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="H8" s="27" t="str">
+      <x:c r="H8" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
       </x:c>
-      <x:c r="I8" s="27" t="str">
+      <x:c r="I8" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J8" s="30" t="str">
+      <x:c r="J8" s="29" t="str">
         <x:v>2026-10-04</x:v>
       </x:c>
-      <x:c r="K8" s="27" t="str">
+      <x:c r="K8" s="26" t="str">
         <x:v>Local main is 21 commits ahead of origin; scheduled GitHub review intentionally sees pushed commits only</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="26" t="str">
         <x:v>CHG-004</x:v>
       </x:c>
-      <x:c r="B9" s="27" t="str">
+      <x:c r="B9" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C9" s="27" t="str">
+      <x:c r="C9" s="26" t="str">
         <x:v>2ddfaf6b6d55d3e4833f905565d5048f3cd9c010</x:v>
       </x:c>
-      <x:c r="D9" s="27" t="str">
+      <x:c r="D9" s="26" t="str">
         <x:v>frontend/ (40 paths)</x:v>
       </x:c>
-      <x:c r="E9" s="27" t="str">
+      <x:c r="E9" s="26" t="str">
         <x:v>UI/UX and tests</x:v>
       </x:c>
-      <x:c r="F9" s="27" t="str">
+      <x:c r="F9" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G9" s="27" t="str">
+      <x:c r="G9" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="H9" s="27" t="str">
+      <x:c r="H9" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
       </x:c>
-      <x:c r="I9" s="27" t="str">
+      <x:c r="I9" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J9" s="30" t="str">
+      <x:c r="J9" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K9" s="27" t="str">
+      <x:c r="K9" s="26" t="str">
         <x:v>WOW-MD PR 50 published the reviewed 07218b4..8a147a6 UI line; production accepts only the reconciled frontend paths</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="27" t="str">
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="26" t="str">
         <x:v>CHG-005</x:v>
       </x:c>
-      <x:c r="B10" s="27" t="str">
+      <x:c r="B10" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C10" s="27" t="str">
+      <x:c r="C10" s="26" t="str">
         <x:v>2ddfaf6b6d55d3e4833f905565d5048f3cd9c010</x:v>
       </x:c>
-      <x:c r="D10" s="27" t="str">
+      <x:c r="D10" s="26" t="str">
         <x:v>docker/docker-compose.preview.yml; docs/wow-consumer-portal-design-preview.html</x:v>
       </x:c>
-      <x:c r="E10" s="27" t="str">
+      <x:c r="E10" s="26" t="str">
         <x:v>Preview-only source artifacts</x:v>
       </x:c>
-      <x:c r="F10" s="27" t="str">
+      <x:c r="F10" s="26" t="str">
         <x:v>Rejected for production</x:v>
       </x:c>
-      <x:c r="G10" s="27" t="str">
+      <x:c r="G10" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="H10" s="27" t="str">
+      <x:c r="H10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
       </x:c>
-      <x:c r="I10" s="27" t="str">
+      <x:c r="I10" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J10" s="30" t="str">
+      <x:c r="J10" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K10" s="27" t="str">
+      <x:c r="K10" s="26" t="str">
         <x:v>Remain in WOW-MD for design preview use; not part of the production deployment line</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="27" t="str">
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="26" t="str">
         <x:v>CHG-006</x:v>
       </x:c>
-      <x:c r="B11" s="27" t="str">
+      <x:c r="B11" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C11" s="27" t="str">
+      <x:c r="C11" s="26" t="str">
         <x:v>51790dfa57126a64e31e5b605ddccca85cd09b85</x:v>
       </x:c>
-      <x:c r="D11" s="27" t="str">
+      <x:c r="D11" s="26" t="str">
         <x:v>frontend/package-lock.json</x:v>
       </x:c>
-      <x:c r="E11" s="27" t="str">
+      <x:c r="E11" s="26" t="str">
         <x:v>Dependency lockfile</x:v>
       </x:c>
-      <x:c r="F11" s="27" t="str">
+      <x:c r="F11" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G11" s="27" t="str">
+      <x:c r="G11" s="26" t="str">
         <x:v>DEP-001</x:v>
       </x:c>
-      <x:c r="H11" s="27" t="str">
+      <x:c r="H11" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/81</x:v>
       </x:c>
-      <x:c r="I11" s="27" t="str">
+      <x:c r="I11" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J11" s="30" t="str">
+      <x:c r="J11" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K11" s="27" t="str">
+      <x:c r="K11" s="26" t="str">
         <x:v>WOW-MD PR 49 and production PRs 79 and 81 reconcile source-map-js 1.2.2 and the exact frontend lock graph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="26" t="str">
+        <x:v>CHG-007</x:v>
+      </x:c>
+      <x:c r="B12" s="26" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C12" s="26" t="str">
+        <x:v>d3d66eae45ddefc262121f356b36ddfa94516baf</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="str">
+        <x:v>backend/; frontend/; mobile/; docker/; terraform/; .github/workflows/</x:v>
+      </x:c>
+      <x:c r="E12" s="26" t="str">
+        <x:v>Dependency and compatibility rollup</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G12" s="26" t="str">
+        <x:v>DEP-002</x:v>
+      </x:c>
+      <x:c r="H12" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/83</x:v>
+      </x:c>
+      <x:c r="I12" s="26" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J12" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K12" s="26" t="str">
+        <x:v>WOW-MD PR 52; accepted compatible React Nest Vitest Node Terraform and security updates; retained ioredis 5 and Expo Router 57 because proposed majors violate current peer contracts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="27" t="str">
+        <x:v>CHG-008</x:v>
+      </x:c>
+      <x:c r="B13" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C13" s="27" t="str">
+        <x:v>b373bb48e389a3456a98db12e1c880b901b75e49</x:v>
+      </x:c>
+      <x:c r="D13" s="27" t="str">
+        <x:v>backend/package-lock.json; docker/Dockerfile; docker/Dockerfile.frontend; terraform/eks.tf; terraform/rds.tf; .github/workflows/</x:v>
+      </x:c>
+      <x:c r="E13" s="27" t="str">
+        <x:v>Dependency and infrastructure mirrors</x:v>
+      </x:c>
+      <x:c r="F13" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G13" s="27" t="str">
+        <x:v>DEP-003</x:v>
+      </x:c>
+      <x:c r="H13" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
+      </x:c>
+      <x:c r="I13" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J13" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K13" s="27" t="str">
+        <x:v>WOW-MD PRs 18 20 21 22 27 and 53; production-only governance and source-review workflows receive the same reviewed action majors</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6270,7 +5957,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e7de65b578c42fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R919a65b175624e9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6375,7 +6062,7 @@
       <x:c r="J6" s="25" t="str">
         <x:v>GitHub plan blocks protected private branches native secret scanning and native CodeQL upload; offline SARIF and CI Gitleaks compensate; tracked by GOV-001</x:v>
       </x:c>
-      <x:c r="K6" s="70" t="str">
+      <x:c r="K6" s="25" t="str">
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L6" s="28" t="str">
@@ -6411,7 +6098,7 @@
       <x:c r="J7" s="26" t="str">
         <x:v>Public source and historical development credential; 83 dependency alerts</x:v>
       </x:c>
-      <x:c r="K7" s="71" t="str">
+      <x:c r="K7" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L7" s="29" t="str">
@@ -6449,7 +6136,7 @@
       <x:c r="J8" s="26" t="str">
         <x:v>Production Zoho credentials/DNS and live-provider evidence are intentionally deferred to the final release gate</x:v>
       </x:c>
-      <x:c r="K8" s="71" t="str">
+      <x:c r="K8" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L8" s="29" t="str">
@@ -6457,404 +6144,466 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="27" t="str">
+      <x:c r="A9" s="26" t="str">
         <x:v>SYNC-002</x:v>
       </x:c>
-      <x:c r="B9" s="27" t="str">
+      <x:c r="B9" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/55</x:v>
       </x:c>
-      <x:c r="C9" s="27" t="str">
+      <x:c r="C9" s="26" t="str">
         <x:v>codex/sync-002-gated-source-review</x:v>
       </x:c>
-      <x:c r="D9" s="27" t="str">
+      <x:c r="D9" s="26" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E9" s="27" t="str">
+      <x:c r="E9" s="26" t="str">
         <x:v>422cbc4</x:v>
       </x:c>
-      <x:c r="F9" s="27" t="str">
+      <x:c r="F9" s="26" t="str">
         <x:v>07218b4..de7d8dd local review only</x:v>
       </x:c>
-      <x:c r="G9" s="27" t="str">
+      <x:c r="G9" s="26" t="str">
         <x:v>Protected PR checks passed: build-and-test frontend mobile docker-build registers secrets CodeQL JavaScript/TypeScript and Actions; local source report found 21 commits and 37 paths with zero dependency or unsafe paths</x:v>
       </x:c>
-      <x:c r="H9" s="27" t="str">
+      <x:c r="H9" s="26" t="str">
         <x:v>Add read-only WOW_SYNC_TOKEN then run the scheduled workflow once; no application or hosting deployment</x:v>
       </x:c>
-      <x:c r="I9" s="27" t="str">
+      <x:c r="I9" s="26" t="str">
         <x:v>Revert PR 55 and remove WOW_SYNC_TOKEN; source and production histories remain unchanged</x:v>
       </x:c>
-      <x:c r="J9" s="27" t="str">
+      <x:c r="J9" s="26" t="str">
         <x:v>Private-source token is not configured; local/unpushed source commits remain intentionally invisible to GitHub Actions</x:v>
       </x:c>
-      <x:c r="K9" s="74" t="str">
+      <x:c r="K9" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L9" s="30" t="str">
+      <x:c r="L9" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="26" t="str">
         <x:v>DEP-001</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="B10" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/59</x:v>
       </x:c>
-      <x:c r="C10" t="str">
+      <x:c r="C10" s="26" t="str">
         <x:v>codex/dep-001-dependency-remediation</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="D10" s="26" t="str">
         <x:v>29537ee</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="E10" s="26" t="str">
         <x:v>1ecbfdf</x:v>
       </x:c>
-      <x:c r="F10" t="str">
+      <x:c r="F10" s="26" t="str">
         <x:v>WOW-MD PR 39 head d8ef995; WOW-MD PR 49 merged as 51790df; supplemental production PRs 73, 79, and 81</x:v>
       </x:c>
-      <x:c r="G10" t="str">
+      <x:c r="G10" s="26" t="str">
         <x:v>Backend and frontend production audits have no high or critical findings; frontend clean install typecheck 180 tests build passed on PR 81; exact frontend trees match</x:v>
       </x:c>
-      <x:c r="H10" t="str">
+      <x:c r="H10" s="26" t="str">
         <x:v>Merged; no runtime deployment is required for the PR 81 development-only lock reconciliation; retain normal rebuild verification</x:v>
       </x:c>
-      <x:c r="I10" t="str">
+      <x:c r="I10" s="26" t="str">
         <x:v>Revert the affected supplemental PR and restore its paired WOW-MD lockfile if clean install or build regresses</x:v>
       </x:c>
-      <x:c r="J10" t="str">
+      <x:c r="J10" s="26" t="str">
         <x:v>Three moderate mammoth-chain findings and four exact no-fix Expo advisory roots remain; forced breaking downgrades remain rejected</x:v>
       </x:c>
-      <x:c r="K10" s="75" t="str">
+      <x:c r="K10" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L10" t="str">
+      <x:c r="L10" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="26" t="str">
         <x:v>GOV-003</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="B11" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/61</x:v>
       </x:c>
-      <x:c r="C11" t="str">
+      <x:c r="C11" s="26" t="str">
         <x:v>codex/gov-003-auth-dependency-tracking</x:v>
       </x:c>
-      <x:c r="D11" t="str">
+      <x:c r="D11" s="26" t="str">
         <x:v>29537ee</x:v>
       </x:c>
-      <x:c r="E11" t="str">
+      <x:c r="E11" s="26" t="str">
         <x:v>1235cd3</x:v>
       </x:c>
-      <x:c r="F11" t="str">
+      <x:c r="F11" s="26" t="str">
         <x:v>SEC-001 PR 58 and DEP-001 PR 59 evidence only</x:v>
       </x:c>
-      <x:c r="G11" t="str">
+      <x:c r="G11" s="26" t="str">
         <x:v>Register validator workbook regeneration and formula-error scan pass; dashboard visually reviewed</x:v>
       </x:c>
-      <x:c r="H11" t="str">
+      <x:c r="H11" s="26" t="str">
         <x:v>Governance and documentation only; no application or hosting deployment</x:v>
       </x:c>
-      <x:c r="I11" t="str">
+      <x:c r="I11" s="26" t="str">
         <x:v>Revert PR 61; implementation PRs and their evidence remain unchanged</x:v>
       </x:c>
-      <x:c r="J11" t="str">
+      <x:c r="J11" s="26" t="str">
         <x:v>Implementation PRs still require review/merge and GitHub rescan; Zoho live configuration remains a final release gate</x:v>
       </x:c>
-      <x:c r="K11" s="75" t="str">
+      <x:c r="K11" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L11" t="str">
+      <x:c r="L11" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="26" t="str">
         <x:v>SEC-002</x:v>
       </x:c>
-      <x:c r="B12" t="str">
+      <x:c r="B12" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/62</x:v>
       </x:c>
-      <x:c r="C12" t="str">
+      <x:c r="C12" s="26" t="str">
         <x:v>codex/sec-002-websocket-authorization</x:v>
       </x:c>
-      <x:c r="D12" t="str">
+      <x:c r="D12" s="26" t="str">
         <x:v>29537ee</x:v>
       </x:c>
-      <x:c r="E12" t="str">
+      <x:c r="E12" s="26" t="str">
         <x:v>4c5e7b4</x:v>
       </x:c>
-      <x:c r="F12" t="str">
+      <x:c r="F12" s="26" t="str">
         <x:v>WOW-MD PR 40 head 9265a27</x:v>
       </x:c>
-      <x:c r="G12" t="str">
+      <x:c r="G12" s="26" t="str">
         <x:v>11 focused chat/admin gateway tests; backend typecheck and lint; complete backend suite 800 passed with 9 skipped</x:v>
       </x:c>
-      <x:c r="H12" t="str">
+      <x:c r="H12" s="26" t="str">
         <x:v>Set exact CORS_ORIGINS and smoke-test browser/native reconnect on the Railway candidate; no schema migration</x:v>
       </x:c>
-      <x:c r="I12" t="str">
+      <x:c r="I12" s="26" t="str">
         <x:v>Revert PR 62; REST chat remains available while socket traffic is paused</x:v>
       </x:c>
-      <x:c r="J12" t="str">
+      <x:c r="J12" s="26" t="str">
         <x:v>Native clients are allowed without an Origin header and remain protected by bearer-token/account checks; Railway cross-origin smoke evidence remains pending</x:v>
       </x:c>
-      <x:c r="K12" s="75" t="str">
+      <x:c r="K12" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L12" t="str">
+      <x:c r="L12" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="26" t="str">
         <x:v>SEC-003</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B13" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/63</x:v>
       </x:c>
-      <x:c r="C13" t="str">
+      <x:c r="C13" s="26" t="str">
         <x:v>codex/sec-003-http-migration-integrity</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D13" s="26" t="str">
         <x:v>29537ee</x:v>
       </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="E13" s="26" t="str">
         <x:v>80ef902</x:v>
       </x:c>
-      <x:c r="F13" t="str">
+      <x:c r="F13" s="26" t="str">
         <x:v>WOW-MD PR 41 head ef13ff5</x:v>
       </x:c>
-      <x:c r="G13" t="str">
+      <x:c r="G13" s="26" t="str">
         <x:v>2 HTTP policy tests; 2 migration verifier tests; 93 files unique; backend typecheck/lint and 794 tests with 9 skipped; upgraded wow_db and fresh 93-migration database passed</x:v>
       </x:c>
-      <x:c r="H13" t="str">
+      <x:c r="H13" s="26" t="str">
         <x:v>Run migrations before application rollout and verify headers through the Railway ingress</x:v>
       </x:c>
-      <x:c r="I13" t="str">
+      <x:c r="I13" s="26" t="str">
         <x:v>Revert application/header changes but retain applied migration history and safe schema additions for roll-forward</x:v>
       </x:c>
-      <x:c r="J13" t="str">
+      <x:c r="J13" s="26" t="str">
         <x:v>Historical databases retain old collision rows plus new idempotent reconciliation rows; ingress evidence remains pending</x:v>
       </x:c>
-      <x:c r="K13" s="75" t="str">
+      <x:c r="K13" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L13" t="str">
+      <x:c r="L13" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="26" t="str">
         <x:v>OPS-001</x:v>
       </x:c>
-      <x:c r="B14" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/64</x:v>
       </x:c>
-      <x:c r="C14" t="str">
+      <x:c r="C14" s="26" t="str">
         <x:v>codex/ops-001-replicated-jobs</x:v>
       </x:c>
-      <x:c r="D14" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>57e13d0</x:v>
       </x:c>
-      <x:c r="E14" t="str">
+      <x:c r="E14" s="26" t="str">
         <x:v>2bf76a1</x:v>
       </x:c>
-      <x:c r="F14" t="str">
+      <x:c r="F14" s="26" t="str">
         <x:v>WOW-MD commit a06067a; PR 42</x:v>
       </x:c>
-      <x:c r="G14" t="str">
+      <x:c r="G14" s="26" t="str">
         <x:v>Focused replica tests 7 of 7; backend full suite 797 passed 9 skipped; typecheck and lint passed</x:v>
       </x:c>
-      <x:c r="H14" t="str">
+      <x:c r="H14" s="26" t="str">
         <x:v>Deploy normally after approval; verify two replicas produce one owner and one skipped invocation for outbox and payout/reminder jobs</x:v>
       </x:c>
-      <x:c r="I14" t="str">
+      <x:c r="I14" s="26" t="str">
         <x:v>Revert PR 64 and redeploy; no database or configuration rollback</x:v>
       </x:c>
-      <x:c r="J14" t="str">
+      <x:c r="J14" s="26" t="str">
         <x:v>Outbox delivery is at-least-once if a worker dies after an external side effect and before processedAt; downstream Kafka consumers must honor the outbox UUID idempotency key</x:v>
       </x:c>
-      <x:c r="K14" s="75" t="str">
+      <x:c r="K14" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L14" t="str">
+      <x:c r="L14" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="26" t="str">
         <x:v>OBS-001</x:v>
       </x:c>
-      <x:c r="B15" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/69</x:v>
       </x:c>
-      <x:c r="C15" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>codex/obs-001-backend-observability</x:v>
       </x:c>
-      <x:c r="D15" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>122ae2d</x:v>
       </x:c>
-      <x:c r="E15" t="str">
+      <x:c r="E15" s="26" t="str">
         <x:v>9d34f68</x:v>
       </x:c>
-      <x:c r="F15" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>WOW-MD PR 43 merged as 2db719b</x:v>
       </x:c>
-      <x:c r="G15" t="str">
+      <x:c r="G15" s="26" t="str">
         <x:v>Focused observability and replica-lock integration 27 of 27; backend typecheck and lint plus nginx contract passed; protected CI recorded on PR 69</x:v>
       </x:c>
-      <x:c r="H15" t="str">
+      <x:c r="H15" s="26" t="str">
         <x:v>Set RELEASE; keep QA capture disabled; confirm a live request ID matches response backend and nginx logs</x:v>
       </x:c>
-      <x:c r="I15" t="str">
+      <x:c r="I15" s="26" t="str">
         <x:v>Revert PR 69 and redeploy; remove optional observability variables; no database rollback</x:v>
       </x:c>
-      <x:c r="J15" t="str">
+      <x:c r="J15" s="26" t="str">
         <x:v>OBS-002 client error intake and OBS-003 Loki Vector host files 30-day retention remain open; live provider correlation smoke remains</x:v>
       </x:c>
-      <x:c r="K15" s="75" t="str">
+      <x:c r="K15" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L15" t="str">
+      <x:c r="L15" s="29" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="26" t="str">
         <x:v>OBS-003</x:v>
       </x:c>
-      <x:c r="B16" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/71</x:v>
       </x:c>
-      <x:c r="C16" t="str">
+      <x:c r="C16" s="26" t="str">
         <x:v>codex/obs-003-local-log-platform</x:v>
       </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>dd39ccc</x:v>
       </x:c>
-      <x:c r="E16" t="str">
+      <x:c r="E16" s="26" t="str">
         <x:v>0d1e02f</x:v>
       </x:c>
-      <x:c r="F16" t="str">
+      <x:c r="F16" s="26" t="str">
         <x:v>WOW-MD PR 48 merged as 7384378</x:v>
       </x:c>
-      <x:c r="G16" t="str">
-        <x:v>Collector and Loki configuration; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; seven alerts; Loki buffer recovery; frontend restart persistence all pass</x:v>
-      </x:c>
-      <x:c r="H16" t="str">
+      <x:c r="G16" s="26" t="str">
+        <x:v>Collector/Loki config validation; Grafana provisioning; retention sandbox; Compose validation; live JSONL and Loki lookup; secret canaries; exact labels; 7 provisioned alerts; Loki buffer recovery; frontend-restart persistence all pass</x:v>
+      </x:c>
+      <x:c r="H16" s="26" t="str">
         <x:v>Set WOW_LOG_DIR and a unique GRAFANA_ADMIN_PASSWORD; start the observability Compose profile; Grafana binds to 127.0.0.1:3300</x:v>
       </x:c>
-      <x:c r="I16" t="str">
+      <x:c r="I16" s="26" t="str">
         <x:v>Stop/remove observability containers and revert PR 71; retained host logs are not automatically deleted; application services remain independent</x:v>
       </x:c>
-      <x:c r="J16" t="str">
-        <x:v>Single-host logs are not disaster recovery; Vector outage has bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
-      </x:c>
-      <x:c r="K16" t="str">
+      <x:c r="J16" s="26" t="str">
+        <x:v>Single-host logs are not disaster recovery; Vector outage has only bounded Docker fallback and no guaranteed backfill; remote Loki and external alert recipients remain operator configuration</x:v>
+      </x:c>
+      <x:c r="K16" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L16" t="str">
+      <x:c r="L16" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="26" t="str">
         <x:v>CFG-001</x:v>
       </x:c>
-      <x:c r="B17" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/72</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>codex/cfg-001-platform-config</x:v>
       </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>568b4a8</x:v>
       </x:c>
-      <x:c r="E17" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>8efb49c</x:v>
       </x:c>
-      <x:c r="F17" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>WOW-MD PR 46 merged as 9135e2f</x:v>
       </x:c>
-      <x:c r="G17" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>Focused configuration contract 12 of 12; backend full suite 840 passed with 9 skipped; lint typecheck boundary scan Compose validation and production image build passed; production audit has no high or critical findings</x:v>
       </x:c>
-      <x:c r="H17" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>Merged after OBS-003 PR 71; retain secrets in environment or secret stores; public tiers must provide S3 bucket secure cookies and disabled Swagger</x:v>
       </x:c>
-      <x:c r="I17" t="str">
+      <x:c r="I17" s="26" t="str">
         <x:v>Revert PR 72 and rebuild; all pre-existing environment variables remain compatible and no database rollback is required</x:v>
       </x:c>
-      <x:c r="J17" t="str">
+      <x:c r="J17" s="26" t="str">
         <x:v>Public and revenue validation deliberately refuses unsafe provider combinations; existing moderate or low framework-chain dependency findings remain outside this change</x:v>
       </x:c>
-      <x:c r="K17" t="str">
+      <x:c r="K17" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L17" t="str">
+      <x:c r="L17" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="B18" t="str">
+      <x:c r="B18" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/77</x:v>
       </x:c>
-      <x:c r="C18" t="str">
+      <x:c r="C18" s="26" t="str">
         <x:v>codex/sync-003-consumer-ui</x:v>
       </x:c>
-      <x:c r="D18" t="str">
+      <x:c r="D18" s="26" t="str">
         <x:v>3e05702</x:v>
       </x:c>
-      <x:c r="E18" t="str">
+      <x:c r="E18" s="26" t="str">
         <x:v>83c2400</x:v>
       </x:c>
-      <x:c r="F18" t="str">
+      <x:c r="F18" s="26" t="str">
         <x:v>WOW-MD PR 50 merged as 2ddfaf6; reviewed local source range 07218b4..8a147a6</x:v>
       </x:c>
-      <x:c r="G18" t="str">
+      <x:c r="G18" s="26" t="str">
         <x:v>Frontend typecheck; 19 test files and 180 tests; production build; protected backend suite and E2E frontend mobile Docker CodeQL secrets and governance checks passed</x:v>
       </x:c>
-      <x:c r="H18" t="str">
+      <x:c r="H18" s="26" t="str">
         <x:v>Merged; rebuild and deploy only the frontend image then smoke public home login registration and bride groom family navigation</x:v>
       </x:c>
-      <x:c r="I18" t="str">
+      <x:c r="I18" s="26" t="str">
         <x:v>Revert PR 77 and rebuild the frontend image; no database configuration or infrastructure rollback</x:v>
       </x:c>
-      <x:c r="J18" t="str">
+      <x:c r="J18" s="26" t="str">
         <x:v>Live post-deployment visual and role smoke remains; main client bundle is about 1.9 MB raw and 505 KB gzip; source-only preview artifacts were rejected</x:v>
       </x:c>
-      <x:c r="K18" t="str">
+      <x:c r="K18" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L18" t="str">
+      <x:c r="L18" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19"/>
-      <x:c r="B19"/>
-      <x:c r="C19"/>
-      <x:c r="D19"/>
-      <x:c r="E19"/>
-      <x:c r="F19"/>
-      <x:c r="G19"/>
-      <x:c r="H19"/>
-      <x:c r="I19"/>
-      <x:c r="J19"/>
-      <x:c r="K19"/>
-      <x:c r="L19"/>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="26" t="str">
+        <x:v>DEP-002</x:v>
+      </x:c>
+      <x:c r="B19" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/83</x:v>
+      </x:c>
+      <x:c r="C19" s="26" t="str">
+        <x:v>codex/dep-002-dependency-rollup</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="str">
+        <x:v>9e8aac5</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="str">
+        <x:v>8c2ebf8</x:v>
+      </x:c>
+      <x:c r="F19" s="26" t="str">
+        <x:v>WOW-MD PR 52 merged as d3d66ea; source heads 882a904 05b92a7 896cebf 752a340 f0b0237</x:v>
+      </x:c>
+      <x:c r="G19" s="26" t="str">
+        <x:v>Backend typecheck lint 837 tests build and clean production audit; E2E 51 of 51 including real Chrome; frontend typecheck 180 tests build; mobile audit typecheck Android export; source Docker and CodeQL green</x:v>
+      </x:c>
+      <x:c r="H19" s="26" t="str">
+        <x:v>Build backend and frontend images; run migrations before rollout; smoke health public entry sign-in biodata upload and an authenticated role page</x:v>
+      </x:c>
+      <x:c r="I19" s="26" t="str">
+        <x:v>Revert PR 83 and rebuild previous Node 20 Nest 10 React 18 images; no database rollback</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="str">
+        <x:v>ioredis 6 and Expo Router 58 remain rejected until their TypeORM and Expo SDK peer lines move; Terraform CLI unavailable locally</x:v>
+      </x:c>
+      <x:c r="K19" s="26" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L19" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="27" t="str">
+        <x:v>DEP-003</x:v>
+      </x:c>
+      <x:c r="B20" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
+        <x:v>dependabot/npm_and_yarn/backend/glob-10.5.0</x:v>
+      </x:c>
+      <x:c r="D20" s="27" t="str">
+        <x:v>0935ede</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>8b5a62b</x:v>
+      </x:c>
+      <x:c r="F20" s="27" t="str">
+        <x:v>WOW-MD PRs 18 20 21 22 27 and 53; reviewed through b373bb4</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="str">
+        <x:v>Production backend E2E frontend mobile Docker CodeQL secrets and governance passed on the final head; local governance 10 of 10 and Node 26 backend plus nginx 1.31 frontend image builds passed</x:v>
+      </x:c>
+      <x:c r="H20" s="27" t="str">
+        <x:v>Rebuild backend and frontend images with Node 26 and nginx 1.31; no application schema change</x:v>
+      </x:c>
+      <x:c r="I20" s="27" t="str">
+        <x:v>Revert PR 84 and rebuild previous images; no database rollback</x:v>
+      </x:c>
+      <x:c r="J20" s="27" t="str">
+        <x:v>Terraform provider and module constraints still require plan evidence before AWS apply</x:v>
+      </x:c>
+      <x:c r="K20" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L20" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K9">
+  <x:conditionalFormatting sqref="K6:K20">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6863,7 +6612,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5c780db6fa46b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aaf73c040d340a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize DEP-004 tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4dac9e61b8f647e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R726792ba74a444a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rac8d13ad987e4019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Raf4371b23e3349cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R40cff3d2fe8b4e15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R259d15eeee2647ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R83ec67f2a1ad4bef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rae9434a4a6d442b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rc5bbb6216a3d4213"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rd9227feb95244459"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3096213e9a264624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rc8281c02ce4d4508"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Ra9e0692ea21b467c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rcb8547c5892740ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R049e88ba5b3e49fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rdca6959475464098"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf747b20b6f534d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R8dd1bfabb3cf474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0980d065be694651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R20594c3ba7184f97"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08294142a8e34b91"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6dae80578dd643e8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -868,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1263,14 +1263,14 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$41)</x:f>
-        <x:v>36</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$42)</x:f>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$41,"P0",'Open Items'!$F$6:$F$41,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$42,"P0",'Open Items'!$F$6:$F$42,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1286,7 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1309,7 +1309,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"PR Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
@@ -1355,7 +1355,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Blocked")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Done")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Done")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903a4fe60ae145b1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e0c6f4ace294adf"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16e3b18f8eff45a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9eb44f698a94ffe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3420,43 +3420,84 @@
       </x:c>
     </x:row>
     <x:row r="41" ht="30" customHeight="1">
-      <x:c r="A41" s="27" t="str">
+      <x:c r="A41" s="26" t="str">
         <x:v>DEP-003</x:v>
       </x:c>
-      <x:c r="B41" s="27" t="str">
+      <x:c r="B41" s="26" t="str">
         <x:v>Complete remaining dependency source mirrors</x:v>
       </x:c>
-      <x:c r="C41" s="27" t="str">
+      <x:c r="C41" s="26" t="str">
         <x:v>Public beta safety</x:v>
       </x:c>
-      <x:c r="D41" s="27" t="str">
+      <x:c r="D41" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="E41" s="27" t="str">
+      <x:c r="E41" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F41" s="27" t="str">
+      <x:c r="F41" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G41" s="27" t="str">
+      <x:c r="G41" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H41" s="27" t="str">
+      <x:c r="H41" s="26" t="str">
         <x:v>DEP-002</x:v>
       </x:c>
-      <x:c r="I41" s="27" t="str">
+      <x:c r="I41" s="26" t="str">
         <x:v>Production carries the reviewed glob lockfile, Node and nginx images, AWS modules and GitHub Actions versions from WOW-MD with production-only workflows upgraded consistently</x:v>
       </x:c>
-      <x:c r="J41" s="27" t="str">
+      <x:c r="J41" s="26" t="str">
         <x:v>WOW-MD PRs 18 20 21 22 27 53</x:v>
       </x:c>
-      <x:c r="K41" s="27" t="str">
+      <x:c r="K41" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/85</x:v>
       </x:c>
-      <x:c r="L41" s="27" t="str">
+      <x:c r="L41" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
       </x:c>
-      <x:c r="M41" s="30" t="str">
+      <x:c r="M41" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="30" customHeight="1">
+      <x:c r="A42" s="27" t="str">
+        <x:v>DEP-004</x:v>
+      </x:c>
+      <x:c r="B42" s="27" t="str">
+        <x:v>Restore Express runtime dependency</x:v>
+      </x:c>
+      <x:c r="C42" s="27" t="str">
+        <x:v>Public beta safety</x:v>
+      </x:c>
+      <x:c r="D42" s="27" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="E42" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F42" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G42" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H42" s="27" t="str">
+        <x:v>DEP-003</x:v>
+      </x:c>
+      <x:c r="I42" s="27" t="str">
+        <x:v>The final backend production image contains the explicit Express 4 compatibility package imported by dist/main.js and starts successfully</x:v>
+      </x:c>
+      <x:c r="J42" s="27" t="str">
+        <x:v>WOW-MD PRs 54 and 55</x:v>
+      </x:c>
+      <x:c r="K42" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/87</x:v>
+      </x:c>
+      <x:c r="L42" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
+      </x:c>
+      <x:c r="M42" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -3464,10 +3505,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E41">
+  <x:conditionalFormatting sqref="E6:E42">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F41">
+  <x:conditionalFormatting sqref="F6:F42">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3476,7 +3517,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R774f5477c69b4acb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4054179318af4c19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4052,7 +4093,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d83ca7b8304ed7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378a32c8f4f74f7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4457,7 +4498,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R880cfabdb5234d85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ceaa730524b4624"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4923,7 +4964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6374f0038df94186"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d9c6ebef2c14242"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5270,7 +5311,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cdd09bc2d384d86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365bd295a35441e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5609,7 +5650,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91ae813e008c4ad1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58c0b6825fbc4b15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5917,38 +5958,73 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="27" t="str">
+      <x:c r="A13" s="26" t="str">
         <x:v>CHG-008</x:v>
       </x:c>
-      <x:c r="B13" s="27" t="str">
+      <x:c r="B13" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C13" s="27" t="str">
+      <x:c r="C13" s="26" t="str">
         <x:v>b373bb48e389a3456a98db12e1c880b901b75e49</x:v>
       </x:c>
-      <x:c r="D13" s="27" t="str">
+      <x:c r="D13" s="26" t="str">
         <x:v>backend/package-lock.json; docker/Dockerfile; docker/Dockerfile.frontend; terraform/eks.tf; terraform/rds.tf; .github/workflows/</x:v>
       </x:c>
-      <x:c r="E13" s="27" t="str">
+      <x:c r="E13" s="26" t="str">
         <x:v>Dependency and infrastructure mirrors</x:v>
       </x:c>
-      <x:c r="F13" s="27" t="str">
+      <x:c r="F13" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G13" s="27" t="str">
+      <x:c r="G13" s="26" t="str">
         <x:v>DEP-003</x:v>
       </x:c>
-      <x:c r="H13" s="27" t="str">
+      <x:c r="H13" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
       </x:c>
-      <x:c r="I13" s="27" t="str">
+      <x:c r="I13" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J13" s="30" t="str">
+      <x:c r="J13" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K13" s="27" t="str">
+      <x:c r="K13" s="26" t="str">
         <x:v>WOW-MD PRs 18 20 21 22 27 and 53; production-only governance and source-review workflows receive the same reviewed action majors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="27" t="str">
+        <x:v>CHG-009</x:v>
+      </x:c>
+      <x:c r="B14" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C14" s="27" t="str">
+        <x:v>4b58009d505a162520cf21a4518f636df293f6e2</x:v>
+      </x:c>
+      <x:c r="D14" s="27" t="str">
+        <x:v>backend/package.json; backend/package-lock.json; .github/workflows/ci.yml</x:v>
+      </x:c>
+      <x:c r="E14" s="27" t="str">
+        <x:v>Runtime dependency correction</x:v>
+      </x:c>
+      <x:c r="F14" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G14" s="27" t="str">
+        <x:v>DEP-004</x:v>
+      </x:c>
+      <x:c r="H14" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
+      </x:c>
+      <x:c r="I14" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J14" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K14" s="27" t="str">
+        <x:v>WOW-MD PRs 54 and 55; Express 4.22.1 is a production dependency because dist/main.js imports it directly and the built runtime image verifies it can resolve the package</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5957,7 +6033,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R919a65b175624e9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39aa16639acf40d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6562,40 +6638,78 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="27" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>DEP-003</x:v>
       </x:c>
-      <x:c r="B20" s="27" t="str">
+      <x:c r="B20" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
       </x:c>
-      <x:c r="C20" s="27" t="str">
+      <x:c r="C20" s="26" t="str">
         <x:v>dependabot/npm_and_yarn/backend/glob-10.5.0</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="str">
+      <x:c r="D20" s="26" t="str">
         <x:v>0935ede</x:v>
       </x:c>
-      <x:c r="E20" s="27" t="str">
+      <x:c r="E20" s="26" t="str">
         <x:v>8b5a62b</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>WOW-MD PRs 18 20 21 22 27 and 53; reviewed through b373bb4</x:v>
       </x:c>
-      <x:c r="G20" s="27" t="str">
+      <x:c r="G20" s="26" t="str">
         <x:v>Production backend E2E frontend mobile Docker CodeQL secrets and governance passed on the final head; local governance 10 of 10 and Node 26 backend plus nginx 1.31 frontend image builds passed</x:v>
       </x:c>
-      <x:c r="H20" s="27" t="str">
+      <x:c r="H20" s="26" t="str">
         <x:v>Rebuild backend and frontend images with Node 26 and nginx 1.31; no application schema change</x:v>
       </x:c>
-      <x:c r="I20" s="27" t="str">
+      <x:c r="I20" s="26" t="str">
         <x:v>Revert PR 84 and rebuild previous images; no database rollback</x:v>
       </x:c>
-      <x:c r="J20" s="27" t="str">
+      <x:c r="J20" s="26" t="str">
         <x:v>Terraform provider and module constraints still require plan evidence before AWS apply</x:v>
       </x:c>
-      <x:c r="K20" s="27" t="str">
+      <x:c r="K20" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L20" s="30" t="str">
+      <x:c r="L20" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="27" t="str">
+        <x:v>DEP-004</x:v>
+      </x:c>
+      <x:c r="B21" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
+      </x:c>
+      <x:c r="C21" s="27" t="str">
+        <x:v>codex/dep-003-express-runtime</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="str">
+        <x:v>5a8d62a</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>5a0a402</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="str">
+        <x:v>WOW-MD PR 54 merged as 68f6ecb; runtime regression gate PR 55 merged as 4b58009</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="str">
+        <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; the final runtime image resolves Express; repaired local and tunneled health returned 200</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="str">
+        <x:v>Rebuild the backend image and verify local plus tunneled health before rollout</x:v>
+      </x:c>
+      <x:c r="I21" s="27" t="str">
+        <x:v>Revert PR 88 and rebuild the prior image; no database rollback</x:v>
+      </x:c>
+      <x:c r="J21" s="27" t="str">
+        <x:v>The targeted image check covers the discovered dependency; a full startup smoke still requires PostgreSQL Redis and provider configuration</x:v>
+      </x:c>
+      <x:c r="K21" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L21" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -6603,7 +6717,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K20">
+  <x:conditionalFormatting sqref="K6:K21">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6612,7 +6726,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aaf73c040d340a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R677e4d2ca39d4efc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize DEP-004 tracking (#89)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4dac9e61b8f647e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R726792ba74a444a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rac8d13ad987e4019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Raf4371b23e3349cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R40cff3d2fe8b4e15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R259d15eeee2647ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R83ec67f2a1ad4bef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rae9434a4a6d442b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rc5bbb6216a3d4213"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rd9227feb95244459"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3096213e9a264624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rc8281c02ce4d4508"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Ra9e0692ea21b467c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rcb8547c5892740ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R049e88ba5b3e49fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rdca6959475464098"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf747b20b6f534d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R8dd1bfabb3cf474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0980d065be694651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R20594c3ba7184f97"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08294142a8e34b91"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6dae80578dd643e8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -868,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1263,14 +1263,14 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$41)</x:f>
-        <x:v>36</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$42)</x:f>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$41,"P0",'Open Items'!$F$6:$F$41,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$42,"P0",'Open Items'!$F$6:$F$42,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1286,7 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1309,7 +1309,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"PR Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
@@ -1355,7 +1355,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Blocked")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$41,"Done")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Done")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903a4fe60ae145b1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e0c6f4ace294adf"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16e3b18f8eff45a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9eb44f698a94ffe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3420,43 +3420,84 @@
       </x:c>
     </x:row>
     <x:row r="41" ht="30" customHeight="1">
-      <x:c r="A41" s="27" t="str">
+      <x:c r="A41" s="26" t="str">
         <x:v>DEP-003</x:v>
       </x:c>
-      <x:c r="B41" s="27" t="str">
+      <x:c r="B41" s="26" t="str">
         <x:v>Complete remaining dependency source mirrors</x:v>
       </x:c>
-      <x:c r="C41" s="27" t="str">
+      <x:c r="C41" s="26" t="str">
         <x:v>Public beta safety</x:v>
       </x:c>
-      <x:c r="D41" s="27" t="str">
+      <x:c r="D41" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="E41" s="27" t="str">
+      <x:c r="E41" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F41" s="27" t="str">
+      <x:c r="F41" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G41" s="27" t="str">
+      <x:c r="G41" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H41" s="27" t="str">
+      <x:c r="H41" s="26" t="str">
         <x:v>DEP-002</x:v>
       </x:c>
-      <x:c r="I41" s="27" t="str">
+      <x:c r="I41" s="26" t="str">
         <x:v>Production carries the reviewed glob lockfile, Node and nginx images, AWS modules and GitHub Actions versions from WOW-MD with production-only workflows upgraded consistently</x:v>
       </x:c>
-      <x:c r="J41" s="27" t="str">
+      <x:c r="J41" s="26" t="str">
         <x:v>WOW-MD PRs 18 20 21 22 27 53</x:v>
       </x:c>
-      <x:c r="K41" s="27" t="str">
+      <x:c r="K41" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/85</x:v>
       </x:c>
-      <x:c r="L41" s="27" t="str">
+      <x:c r="L41" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
       </x:c>
-      <x:c r="M41" s="30" t="str">
+      <x:c r="M41" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="30" customHeight="1">
+      <x:c r="A42" s="27" t="str">
+        <x:v>DEP-004</x:v>
+      </x:c>
+      <x:c r="B42" s="27" t="str">
+        <x:v>Restore Express runtime dependency</x:v>
+      </x:c>
+      <x:c r="C42" s="27" t="str">
+        <x:v>Public beta safety</x:v>
+      </x:c>
+      <x:c r="D42" s="27" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="E42" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F42" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G42" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H42" s="27" t="str">
+        <x:v>DEP-003</x:v>
+      </x:c>
+      <x:c r="I42" s="27" t="str">
+        <x:v>The final backend production image contains the explicit Express 4 compatibility package imported by dist/main.js and starts successfully</x:v>
+      </x:c>
+      <x:c r="J42" s="27" t="str">
+        <x:v>WOW-MD PRs 54 and 55</x:v>
+      </x:c>
+      <x:c r="K42" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/87</x:v>
+      </x:c>
+      <x:c r="L42" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
+      </x:c>
+      <x:c r="M42" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -3464,10 +3505,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E41">
+  <x:conditionalFormatting sqref="E6:E42">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F41">
+  <x:conditionalFormatting sqref="F6:F42">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3476,7 +3517,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R774f5477c69b4acb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4054179318af4c19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4052,7 +4093,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d83ca7b8304ed7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378a32c8f4f74f7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4457,7 +4498,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R880cfabdb5234d85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ceaa730524b4624"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4923,7 +4964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6374f0038df94186"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d9c6ebef2c14242"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5270,7 +5311,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cdd09bc2d384d86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365bd295a35441e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5609,7 +5650,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91ae813e008c4ad1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58c0b6825fbc4b15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5917,38 +5958,73 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="27" t="str">
+      <x:c r="A13" s="26" t="str">
         <x:v>CHG-008</x:v>
       </x:c>
-      <x:c r="B13" s="27" t="str">
+      <x:c r="B13" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C13" s="27" t="str">
+      <x:c r="C13" s="26" t="str">
         <x:v>b373bb48e389a3456a98db12e1c880b901b75e49</x:v>
       </x:c>
-      <x:c r="D13" s="27" t="str">
+      <x:c r="D13" s="26" t="str">
         <x:v>backend/package-lock.json; docker/Dockerfile; docker/Dockerfile.frontend; terraform/eks.tf; terraform/rds.tf; .github/workflows/</x:v>
       </x:c>
-      <x:c r="E13" s="27" t="str">
+      <x:c r="E13" s="26" t="str">
         <x:v>Dependency and infrastructure mirrors</x:v>
       </x:c>
-      <x:c r="F13" s="27" t="str">
+      <x:c r="F13" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G13" s="27" t="str">
+      <x:c r="G13" s="26" t="str">
         <x:v>DEP-003</x:v>
       </x:c>
-      <x:c r="H13" s="27" t="str">
+      <x:c r="H13" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
       </x:c>
-      <x:c r="I13" s="27" t="str">
+      <x:c r="I13" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J13" s="30" t="str">
+      <x:c r="J13" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K13" s="27" t="str">
+      <x:c r="K13" s="26" t="str">
         <x:v>WOW-MD PRs 18 20 21 22 27 and 53; production-only governance and source-review workflows receive the same reviewed action majors</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="27" t="str">
+        <x:v>CHG-009</x:v>
+      </x:c>
+      <x:c r="B14" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C14" s="27" t="str">
+        <x:v>4b58009d505a162520cf21a4518f636df293f6e2</x:v>
+      </x:c>
+      <x:c r="D14" s="27" t="str">
+        <x:v>backend/package.json; backend/package-lock.json; .github/workflows/ci.yml</x:v>
+      </x:c>
+      <x:c r="E14" s="27" t="str">
+        <x:v>Runtime dependency correction</x:v>
+      </x:c>
+      <x:c r="F14" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G14" s="27" t="str">
+        <x:v>DEP-004</x:v>
+      </x:c>
+      <x:c r="H14" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
+      </x:c>
+      <x:c r="I14" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J14" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K14" s="27" t="str">
+        <x:v>WOW-MD PRs 54 and 55; Express 4.22.1 is a production dependency because dist/main.js imports it directly and the built runtime image verifies it can resolve the package</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5957,7 +6033,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R919a65b175624e9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39aa16639acf40d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6562,40 +6638,78 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="27" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>DEP-003</x:v>
       </x:c>
-      <x:c r="B20" s="27" t="str">
+      <x:c r="B20" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/84</x:v>
       </x:c>
-      <x:c r="C20" s="27" t="str">
+      <x:c r="C20" s="26" t="str">
         <x:v>dependabot/npm_and_yarn/backend/glob-10.5.0</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="str">
+      <x:c r="D20" s="26" t="str">
         <x:v>0935ede</x:v>
       </x:c>
-      <x:c r="E20" s="27" t="str">
+      <x:c r="E20" s="26" t="str">
         <x:v>8b5a62b</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>WOW-MD PRs 18 20 21 22 27 and 53; reviewed through b373bb4</x:v>
       </x:c>
-      <x:c r="G20" s="27" t="str">
+      <x:c r="G20" s="26" t="str">
         <x:v>Production backend E2E frontend mobile Docker CodeQL secrets and governance passed on the final head; local governance 10 of 10 and Node 26 backend plus nginx 1.31 frontend image builds passed</x:v>
       </x:c>
-      <x:c r="H20" s="27" t="str">
+      <x:c r="H20" s="26" t="str">
         <x:v>Rebuild backend and frontend images with Node 26 and nginx 1.31; no application schema change</x:v>
       </x:c>
-      <x:c r="I20" s="27" t="str">
+      <x:c r="I20" s="26" t="str">
         <x:v>Revert PR 84 and rebuild previous images; no database rollback</x:v>
       </x:c>
-      <x:c r="J20" s="27" t="str">
+      <x:c r="J20" s="26" t="str">
         <x:v>Terraform provider and module constraints still require plan evidence before AWS apply</x:v>
       </x:c>
-      <x:c r="K20" s="27" t="str">
+      <x:c r="K20" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L20" s="30" t="str">
+      <x:c r="L20" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="27" t="str">
+        <x:v>DEP-004</x:v>
+      </x:c>
+      <x:c r="B21" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
+      </x:c>
+      <x:c r="C21" s="27" t="str">
+        <x:v>codex/dep-003-express-runtime</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="str">
+        <x:v>5a8d62a</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>5a0a402</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="str">
+        <x:v>WOW-MD PR 54 merged as 68f6ecb; runtime regression gate PR 55 merged as 4b58009</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="str">
+        <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; the final runtime image resolves Express; repaired local and tunneled health returned 200</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="str">
+        <x:v>Rebuild the backend image and verify local plus tunneled health before rollout</x:v>
+      </x:c>
+      <x:c r="I21" s="27" t="str">
+        <x:v>Revert PR 88 and rebuild the prior image; no database rollback</x:v>
+      </x:c>
+      <x:c r="J21" s="27" t="str">
+        <x:v>The targeted image check covers the discovered dependency; a full startup smoke still requires PostgreSQL Redis and provider configuration</x:v>
+      </x:c>
+      <x:c r="K21" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L21" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -6603,7 +6717,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K20">
+  <x:conditionalFormatting sqref="K6:K21">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6612,7 +6726,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aaf73c040d340a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R677e4d2ca39d4efc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize SYNC-004 tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3096213e9a264624"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rc8281c02ce4d4508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Ra9e0692ea21b467c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rcb8547c5892740ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R049e88ba5b3e49fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rdca6959475464098"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf747b20b6f534d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R8dd1bfabb3cf474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0980d065be694651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R20594c3ba7184f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re64dd9545264410b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R4c03b21d525c4725"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R64381f3351a54c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R7a7fbd0e6585416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rf0fd24f27d9d48a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R4a1dc7979ec246b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R84a316c47b334015"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R00aa60daf4744e11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0695a94581284111"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R875e39c45727442a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6dae80578dd643e8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ea69d5f72ab4d86"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -868,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1263,14 +1263,14 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$42)</x:f>
-        <x:v>37</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$43)</x:f>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$42,"P0",'Open Items'!$F$6:$F$42,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$43,"P0",'Open Items'!$F$6:$F$43,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1286,7 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1309,7 +1309,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"PR Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
@@ -1355,7 +1355,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Blocked")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Done")</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Done")</x:f>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e0c6f4ace294adf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f429cef35a04ad9"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9eb44f698a94ffe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R139cb3d991bc4327"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3461,43 +3461,84 @@
       </x:c>
     </x:row>
     <x:row r="42" ht="30" customHeight="1">
-      <x:c r="A42" s="27" t="str">
+      <x:c r="A42" s="26" t="str">
         <x:v>DEP-004</x:v>
       </x:c>
-      <x:c r="B42" s="27" t="str">
+      <x:c r="B42" s="26" t="str">
         <x:v>Restore Express runtime dependency</x:v>
       </x:c>
-      <x:c r="C42" s="27" t="str">
+      <x:c r="C42" s="26" t="str">
         <x:v>Public beta safety</x:v>
       </x:c>
-      <x:c r="D42" s="27" t="str">
+      <x:c r="D42" s="26" t="str">
         <x:v>Reliability</x:v>
       </x:c>
-      <x:c r="E42" s="27" t="str">
+      <x:c r="E42" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F42" s="27" t="str">
+      <x:c r="F42" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G42" s="27" t="str">
+      <x:c r="G42" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H42" s="27" t="str">
+      <x:c r="H42" s="26" t="str">
         <x:v>DEP-003</x:v>
       </x:c>
-      <x:c r="I42" s="27" t="str">
+      <x:c r="I42" s="26" t="str">
         <x:v>The final backend production image contains the explicit Express 4 compatibility package imported by dist/main.js and starts successfully</x:v>
       </x:c>
-      <x:c r="J42" s="27" t="str">
+      <x:c r="J42" s="26" t="str">
         <x:v>WOW-MD PRs 54 and 55</x:v>
       </x:c>
-      <x:c r="K42" s="27" t="str">
+      <x:c r="K42" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/87</x:v>
       </x:c>
-      <x:c r="L42" s="27" t="str">
+      <x:c r="L42" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
       </x:c>
-      <x:c r="M42" s="30" t="str">
+      <x:c r="M42" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="A43" s="27" t="str">
+        <x:v>SYNC-004</x:v>
+      </x:c>
+      <x:c r="B43" s="27" t="str">
+        <x:v>Mirror latest committed local functional fixes</x:v>
+      </x:c>
+      <x:c r="C43" s="27" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D43" s="27" t="str">
+        <x:v>Change intake</x:v>
+      </x:c>
+      <x:c r="E43" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F43" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G43" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H43" s="27" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="I43" s="27" t="str">
+        <x:v>The production repository exactly mirrors the reviewed profile validation biodata progression and mock-storage proxy fixes without unrelated dirty files</x:v>
+      </x:c>
+      <x:c r="J43" s="27" t="str">
+        <x:v>WOW-MD PR 56</x:v>
+      </x:c>
+      <x:c r="K43" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/90</x:v>
+      </x:c>
+      <x:c r="L43" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
+      </x:c>
+      <x:c r="M43" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -3505,10 +3546,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E42">
+  <x:conditionalFormatting sqref="E6:E43">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F42">
+  <x:conditionalFormatting sqref="F6:F43">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3517,7 +3558,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4054179318af4c19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb6a1a9e57c84be3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4093,7 +4134,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378a32c8f4f74f7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R202d69b56da14ded"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4498,7 +4539,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ceaa730524b4624"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89aa45a801b94497"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4964,7 +5005,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d9c6ebef2c14242"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra78aa86d24d04b12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5311,7 +5352,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365bd295a35441e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f6da32b9f914f27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5650,7 +5691,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58c0b6825fbc4b15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R876a7877cc4c4da0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5993,38 +6034,73 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="27" t="str">
+      <x:c r="A14" s="26" t="str">
         <x:v>CHG-009</x:v>
       </x:c>
-      <x:c r="B14" s="27" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C14" s="27" t="str">
+      <x:c r="C14" s="26" t="str">
         <x:v>4b58009d505a162520cf21a4518f636df293f6e2</x:v>
       </x:c>
-      <x:c r="D14" s="27" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>backend/package.json; backend/package-lock.json; .github/workflows/ci.yml</x:v>
       </x:c>
-      <x:c r="E14" s="27" t="str">
+      <x:c r="E14" s="26" t="str">
         <x:v>Runtime dependency correction</x:v>
       </x:c>
-      <x:c r="F14" s="27" t="str">
+      <x:c r="F14" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G14" s="27" t="str">
+      <x:c r="G14" s="26" t="str">
         <x:v>DEP-004</x:v>
       </x:c>
-      <x:c r="H14" s="27" t="str">
+      <x:c r="H14" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
       </x:c>
-      <x:c r="I14" s="27" t="str">
+      <x:c r="I14" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J14" s="30" t="str">
+      <x:c r="J14" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K14" s="27" t="str">
+      <x:c r="K14" s="26" t="str">
         <x:v>WOW-MD PRs 54 and 55; Express 4.22.1 is a production dependency because dist/main.js imports it directly and the built runtime image verifies it can resolve the package</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="27" t="str">
+        <x:v>CHG-010</x:v>
+      </x:c>
+      <x:c r="B15" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C15" s="27" t="str">
+        <x:v>3a5321272a857ef6cd2aac96d956924c7cc1f36b</x:v>
+      </x:c>
+      <x:c r="D15" s="27" t="str">
+        <x:v>backend/src/common/decorators/; backend/src/modules/agents/dto/managed-profile.dto.ts; backend/src/modules/profile-details/dto/profile-details.dto.ts; backend/src/modules/users/; frontend/nginx.conf; frontend/src/pages/Biodata.tsx</x:v>
+      </x:c>
+      <x:c r="E15" s="27" t="str">
+        <x:v>Committed local functional fixes</x:v>
+      </x:c>
+      <x:c r="F15" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G15" s="27" t="str">
+        <x:v>SYNC-004</x:v>
+      </x:c>
+      <x:c r="H15" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
+      </x:c>
+      <x:c r="I15" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J15" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K15" s="27" t="str">
+        <x:v>WOW-MD PR 56; mirror duplicate-mobile and adult-age validation, biodata save progression and mock-storage media proxying without unrelated dirty working-tree files</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6033,7 +6109,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39aa16639acf40d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree1baa173fb0433f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6676,40 +6752,78 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="27" t="str">
+      <x:c r="A21" s="26" t="str">
         <x:v>DEP-004</x:v>
       </x:c>
-      <x:c r="B21" s="27" t="str">
+      <x:c r="B21" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
       </x:c>
-      <x:c r="C21" s="27" t="str">
+      <x:c r="C21" s="26" t="str">
         <x:v>codex/dep-003-express-runtime</x:v>
       </x:c>
-      <x:c r="D21" s="27" t="str">
+      <x:c r="D21" s="26" t="str">
         <x:v>5a8d62a</x:v>
       </x:c>
-      <x:c r="E21" s="27" t="str">
+      <x:c r="E21" s="26" t="str">
         <x:v>5a0a402</x:v>
       </x:c>
-      <x:c r="F21" s="27" t="str">
+      <x:c r="F21" s="26" t="str">
         <x:v>WOW-MD PR 54 merged as 68f6ecb; runtime regression gate PR 55 merged as 4b58009</x:v>
       </x:c>
-      <x:c r="G21" s="27" t="str">
+      <x:c r="G21" s="26" t="str">
         <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; the final runtime image resolves Express; repaired local and tunneled health returned 200</x:v>
       </x:c>
-      <x:c r="H21" s="27" t="str">
+      <x:c r="H21" s="26" t="str">
         <x:v>Rebuild the backend image and verify local plus tunneled health before rollout</x:v>
       </x:c>
-      <x:c r="I21" s="27" t="str">
+      <x:c r="I21" s="26" t="str">
         <x:v>Revert PR 88 and rebuild the prior image; no database rollback</x:v>
       </x:c>
-      <x:c r="J21" s="27" t="str">
+      <x:c r="J21" s="26" t="str">
         <x:v>The targeted image check covers the discovered dependency; a full startup smoke still requires PostgreSQL Redis and provider configuration</x:v>
       </x:c>
-      <x:c r="K21" s="27" t="str">
+      <x:c r="K21" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L21" s="30" t="str">
+      <x:c r="L21" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="27" t="str">
+        <x:v>SYNC-004</x:v>
+      </x:c>
+      <x:c r="B22" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
+      </x:c>
+      <x:c r="C22" s="27" t="str">
+        <x:v>codex/sync-004-local-functional</x:v>
+      </x:c>
+      <x:c r="D22" s="27" t="str">
+        <x:v>b4ec092</x:v>
+      </x:c>
+      <x:c r="E22" s="27" t="str">
+        <x:v>ca5118c</x:v>
+      </x:c>
+      <x:c r="F22" s="27" t="str">
+        <x:v>WOW-MD PR 56 merged as 3a53212</x:v>
+      </x:c>
+      <x:c r="G22" s="27" t="str">
+        <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; the exact combined source tree was deployed locally and local plus tunneled health returned 200</x:v>
+      </x:c>
+      <x:c r="H22" s="27" t="str">
+        <x:v>Rebuild backend and frontend images and smoke profile save biodata continuation media rendering and health</x:v>
+      </x:c>
+      <x:c r="I22" s="27" t="str">
+        <x:v>Revert PR 91 and rebuild the prior images; no schema rollback</x:v>
+      </x:c>
+      <x:c r="J22" s="27" t="str">
+        <x:v>The dirty primary checkout remains outside this reviewed mirror and continues under SYNC-001 and SYNC-002</x:v>
+      </x:c>
+      <x:c r="K22" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L22" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -6717,7 +6831,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K21">
+  <x:conditionalFormatting sqref="K6:K22">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6726,7 +6840,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R677e4d2ca39d4efc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe8898aa42349e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize SYNC-004 tracking (#92)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3096213e9a264624"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rc8281c02ce4d4508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Ra9e0692ea21b467c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rcb8547c5892740ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R049e88ba5b3e49fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rdca6959475464098"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf747b20b6f534d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R8dd1bfabb3cf474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0980d065be694651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R20594c3ba7184f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re64dd9545264410b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R4c03b21d525c4725"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R64381f3351a54c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R7a7fbd0e6585416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rf0fd24f27d9d48a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R4a1dc7979ec246b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R84a316c47b334015"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R00aa60daf4744e11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0695a94581284111"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R875e39c45727442a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6dae80578dd643e8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ea69d5f72ab4d86"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -868,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1263,14 +1263,14 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$42)</x:f>
-        <x:v>37</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$43)</x:f>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$42,"P0",'Open Items'!$F$6:$F$42,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$43,"P0",'Open Items'!$F$6:$F$43,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1286,7 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1309,7 +1309,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"PR Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
@@ -1355,7 +1355,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Blocked")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$42,"Done")</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Done")</x:f>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e0c6f4ace294adf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f429cef35a04ad9"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9eb44f698a94ffe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R139cb3d991bc4327"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3461,43 +3461,84 @@
       </x:c>
     </x:row>
     <x:row r="42" ht="30" customHeight="1">
-      <x:c r="A42" s="27" t="str">
+      <x:c r="A42" s="26" t="str">
         <x:v>DEP-004</x:v>
       </x:c>
-      <x:c r="B42" s="27" t="str">
+      <x:c r="B42" s="26" t="str">
         <x:v>Restore Express runtime dependency</x:v>
       </x:c>
-      <x:c r="C42" s="27" t="str">
+      <x:c r="C42" s="26" t="str">
         <x:v>Public beta safety</x:v>
       </x:c>
-      <x:c r="D42" s="27" t="str">
+      <x:c r="D42" s="26" t="str">
         <x:v>Reliability</x:v>
       </x:c>
-      <x:c r="E42" s="27" t="str">
+      <x:c r="E42" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F42" s="27" t="str">
+      <x:c r="F42" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G42" s="27" t="str">
+      <x:c r="G42" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H42" s="27" t="str">
+      <x:c r="H42" s="26" t="str">
         <x:v>DEP-003</x:v>
       </x:c>
-      <x:c r="I42" s="27" t="str">
+      <x:c r="I42" s="26" t="str">
         <x:v>The final backend production image contains the explicit Express 4 compatibility package imported by dist/main.js and starts successfully</x:v>
       </x:c>
-      <x:c r="J42" s="27" t="str">
+      <x:c r="J42" s="26" t="str">
         <x:v>WOW-MD PRs 54 and 55</x:v>
       </x:c>
-      <x:c r="K42" s="27" t="str">
+      <x:c r="K42" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/87</x:v>
       </x:c>
-      <x:c r="L42" s="27" t="str">
+      <x:c r="L42" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
       </x:c>
-      <x:c r="M42" s="30" t="str">
+      <x:c r="M42" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="A43" s="27" t="str">
+        <x:v>SYNC-004</x:v>
+      </x:c>
+      <x:c r="B43" s="27" t="str">
+        <x:v>Mirror latest committed local functional fixes</x:v>
+      </x:c>
+      <x:c r="C43" s="27" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D43" s="27" t="str">
+        <x:v>Change intake</x:v>
+      </x:c>
+      <x:c r="E43" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F43" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G43" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H43" s="27" t="str">
+        <x:v>SYNC-003</x:v>
+      </x:c>
+      <x:c r="I43" s="27" t="str">
+        <x:v>The production repository exactly mirrors the reviewed profile validation biodata progression and mock-storage proxy fixes without unrelated dirty files</x:v>
+      </x:c>
+      <x:c r="J43" s="27" t="str">
+        <x:v>WOW-MD PR 56</x:v>
+      </x:c>
+      <x:c r="K43" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/90</x:v>
+      </x:c>
+      <x:c r="L43" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
+      </x:c>
+      <x:c r="M43" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -3505,10 +3546,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E42">
+  <x:conditionalFormatting sqref="E6:E43">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F42">
+  <x:conditionalFormatting sqref="F6:F43">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3517,7 +3558,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4054179318af4c19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb6a1a9e57c84be3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4093,7 +4134,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378a32c8f4f74f7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R202d69b56da14ded"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4498,7 +4539,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ceaa730524b4624"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89aa45a801b94497"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4964,7 +5005,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d9c6ebef2c14242"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra78aa86d24d04b12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5311,7 +5352,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365bd295a35441e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f6da32b9f914f27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5650,7 +5691,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58c0b6825fbc4b15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R876a7877cc4c4da0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5993,38 +6034,73 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="27" t="str">
+      <x:c r="A14" s="26" t="str">
         <x:v>CHG-009</x:v>
       </x:c>
-      <x:c r="B14" s="27" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C14" s="27" t="str">
+      <x:c r="C14" s="26" t="str">
         <x:v>4b58009d505a162520cf21a4518f636df293f6e2</x:v>
       </x:c>
-      <x:c r="D14" s="27" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>backend/package.json; backend/package-lock.json; .github/workflows/ci.yml</x:v>
       </x:c>
-      <x:c r="E14" s="27" t="str">
+      <x:c r="E14" s="26" t="str">
         <x:v>Runtime dependency correction</x:v>
       </x:c>
-      <x:c r="F14" s="27" t="str">
+      <x:c r="F14" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G14" s="27" t="str">
+      <x:c r="G14" s="26" t="str">
         <x:v>DEP-004</x:v>
       </x:c>
-      <x:c r="H14" s="27" t="str">
+      <x:c r="H14" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
       </x:c>
-      <x:c r="I14" s="27" t="str">
+      <x:c r="I14" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J14" s="30" t="str">
+      <x:c r="J14" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K14" s="27" t="str">
+      <x:c r="K14" s="26" t="str">
         <x:v>WOW-MD PRs 54 and 55; Express 4.22.1 is a production dependency because dist/main.js imports it directly and the built runtime image verifies it can resolve the package</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="27" t="str">
+        <x:v>CHG-010</x:v>
+      </x:c>
+      <x:c r="B15" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C15" s="27" t="str">
+        <x:v>3a5321272a857ef6cd2aac96d956924c7cc1f36b</x:v>
+      </x:c>
+      <x:c r="D15" s="27" t="str">
+        <x:v>backend/src/common/decorators/; backend/src/modules/agents/dto/managed-profile.dto.ts; backend/src/modules/profile-details/dto/profile-details.dto.ts; backend/src/modules/users/; frontend/nginx.conf; frontend/src/pages/Biodata.tsx</x:v>
+      </x:c>
+      <x:c r="E15" s="27" t="str">
+        <x:v>Committed local functional fixes</x:v>
+      </x:c>
+      <x:c r="F15" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G15" s="27" t="str">
+        <x:v>SYNC-004</x:v>
+      </x:c>
+      <x:c r="H15" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
+      </x:c>
+      <x:c r="I15" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J15" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K15" s="27" t="str">
+        <x:v>WOW-MD PR 56; mirror duplicate-mobile and adult-age validation, biodata save progression and mock-storage media proxying without unrelated dirty working-tree files</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6033,7 +6109,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39aa16639acf40d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree1baa173fb0433f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6676,40 +6752,78 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="27" t="str">
+      <x:c r="A21" s="26" t="str">
         <x:v>DEP-004</x:v>
       </x:c>
-      <x:c r="B21" s="27" t="str">
+      <x:c r="B21" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/88</x:v>
       </x:c>
-      <x:c r="C21" s="27" t="str">
+      <x:c r="C21" s="26" t="str">
         <x:v>codex/dep-003-express-runtime</x:v>
       </x:c>
-      <x:c r="D21" s="27" t="str">
+      <x:c r="D21" s="26" t="str">
         <x:v>5a8d62a</x:v>
       </x:c>
-      <x:c r="E21" s="27" t="str">
+      <x:c r="E21" s="26" t="str">
         <x:v>5a0a402</x:v>
       </x:c>
-      <x:c r="F21" s="27" t="str">
+      <x:c r="F21" s="26" t="str">
         <x:v>WOW-MD PR 54 merged as 68f6ecb; runtime regression gate PR 55 merged as 4b58009</x:v>
       </x:c>
-      <x:c r="G21" s="27" t="str">
+      <x:c r="G21" s="26" t="str">
         <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; the final runtime image resolves Express; repaired local and tunneled health returned 200</x:v>
       </x:c>
-      <x:c r="H21" s="27" t="str">
+      <x:c r="H21" s="26" t="str">
         <x:v>Rebuild the backend image and verify local plus tunneled health before rollout</x:v>
       </x:c>
-      <x:c r="I21" s="27" t="str">
+      <x:c r="I21" s="26" t="str">
         <x:v>Revert PR 88 and rebuild the prior image; no database rollback</x:v>
       </x:c>
-      <x:c r="J21" s="27" t="str">
+      <x:c r="J21" s="26" t="str">
         <x:v>The targeted image check covers the discovered dependency; a full startup smoke still requires PostgreSQL Redis and provider configuration</x:v>
       </x:c>
-      <x:c r="K21" s="27" t="str">
+      <x:c r="K21" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L21" s="30" t="str">
+      <x:c r="L21" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="27" t="str">
+        <x:v>SYNC-004</x:v>
+      </x:c>
+      <x:c r="B22" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
+      </x:c>
+      <x:c r="C22" s="27" t="str">
+        <x:v>codex/sync-004-local-functional</x:v>
+      </x:c>
+      <x:c r="D22" s="27" t="str">
+        <x:v>b4ec092</x:v>
+      </x:c>
+      <x:c r="E22" s="27" t="str">
+        <x:v>ca5118c</x:v>
+      </x:c>
+      <x:c r="F22" s="27" t="str">
+        <x:v>WOW-MD PR 56 merged as 3a53212</x:v>
+      </x:c>
+      <x:c r="G22" s="27" t="str">
+        <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; the exact combined source tree was deployed locally and local plus tunneled health returned 200</x:v>
+      </x:c>
+      <x:c r="H22" s="27" t="str">
+        <x:v>Rebuild backend and frontend images and smoke profile save biodata continuation media rendering and health</x:v>
+      </x:c>
+      <x:c r="I22" s="27" t="str">
+        <x:v>Revert PR 91 and rebuild the prior images; no schema rollback</x:v>
+      </x:c>
+      <x:c r="J22" s="27" t="str">
+        <x:v>The dirty primary checkout remains outside this reviewed mirror and continues under SYNC-001 and SYNC-002</x:v>
+      </x:c>
+      <x:c r="K22" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L22" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -6717,7 +6831,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K21">
+  <x:conditionalFormatting sqref="K6:K22">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6726,7 +6840,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R677e4d2ca39d4efc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe8898aa42349e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize OBS-004 tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re64dd9545264410b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R4c03b21d525c4725"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R64381f3351a54c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R7a7fbd0e6585416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rf0fd24f27d9d48a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R4a1dc7979ec246b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R84a316c47b334015"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R00aa60daf4744e11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0695a94581284111"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R875e39c45727442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R942ffbbb2e1f4fb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R3151609748134ed1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rfbfdf3ebec47436c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R781fa2502de54f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R47e03c3edb2a4065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R3c56a117638c44ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf0bdac3a92184c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R9e04aef798284bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R9f6723b2e54045db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rbbf4a62bda8549cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ea69d5f72ab4d86"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5a7092c124b7419c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -868,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1263,14 +1263,14 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$43)</x:f>
-        <x:v>38</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$44)</x:f>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$43,"P0",'Open Items'!$F$6:$F$43,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$44,"P0",'Open Items'!$F$6:$F$44,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1286,7 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1309,7 +1309,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"PR Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
@@ -1355,7 +1355,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Blocked")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Done")</x:f>
-        <x:v>16</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Done")</x:f>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f429cef35a04ad9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f82b2d541384dac"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R139cb3d991bc4327"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R374e9ed5240d44e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3502,43 +3502,84 @@
       </x:c>
     </x:row>
     <x:row r="43" ht="30" customHeight="1">
-      <x:c r="A43" s="27" t="str">
+      <x:c r="A43" s="26" t="str">
         <x:v>SYNC-004</x:v>
       </x:c>
-      <x:c r="B43" s="27" t="str">
+      <x:c r="B43" s="26" t="str">
         <x:v>Mirror latest committed local functional fixes</x:v>
       </x:c>
-      <x:c r="C43" s="27" t="str">
+      <x:c r="C43" s="26" t="str">
         <x:v>Source intake</x:v>
       </x:c>
-      <x:c r="D43" s="27" t="str">
+      <x:c r="D43" s="26" t="str">
         <x:v>Change intake</x:v>
       </x:c>
-      <x:c r="E43" s="27" t="str">
+      <x:c r="E43" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F43" s="27" t="str">
+      <x:c r="F43" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G43" s="27" t="str">
+      <x:c r="G43" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H43" s="27" t="str">
+      <x:c r="H43" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="I43" s="27" t="str">
+      <x:c r="I43" s="26" t="str">
         <x:v>The production repository exactly mirrors the reviewed profile validation biodata progression and mock-storage proxy fixes without unrelated dirty files</x:v>
       </x:c>
-      <x:c r="J43" s="27" t="str">
+      <x:c r="J43" s="26" t="str">
         <x:v>WOW-MD PR 56</x:v>
       </x:c>
-      <x:c r="K43" s="27" t="str">
+      <x:c r="K43" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/90</x:v>
       </x:c>
-      <x:c r="L43" s="27" t="str">
+      <x:c r="L43" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
       </x:c>
-      <x:c r="M43" s="30" t="str">
+      <x:c r="M43" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="30" customHeight="1">
+      <x:c r="A44" s="27" t="str">
+        <x:v>OBS-004</x:v>
+      </x:c>
+      <x:c r="B44" s="27" t="str">
+        <x:v>Stabilize Vector disk buffer on Windows hosts</x:v>
+      </x:c>
+      <x:c r="C44" s="27" t="str">
+        <x:v>Observability</x:v>
+      </x:c>
+      <x:c r="D44" s="27" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="E44" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F44" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G44" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H44" s="27" t="str">
+        <x:v>OBS-003</x:v>
+      </x:c>
+      <x:c r="I44" s="27" t="str">
+        <x:v>Vector retains its delivery buffer across recreation without NTFS reader panics while operator-readable JSONL logs remain on the host</x:v>
+      </x:c>
+      <x:c r="J44" s="27" t="str">
+        <x:v>WOW-MD PR 57</x:v>
+      </x:c>
+      <x:c r="K44" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/93</x:v>
+      </x:c>
+      <x:c r="L44" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
+      </x:c>
+      <x:c r="M44" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -3546,10 +3587,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E43">
+  <x:conditionalFormatting sqref="E6:E44">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F43">
+  <x:conditionalFormatting sqref="F6:F44">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3558,7 +3599,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb6a1a9e57c84be3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f8aaadacbdf4bbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4134,7 +4175,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R202d69b56da14ded"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff913bde120a46af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4539,7 +4580,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89aa45a801b94497"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R177734aafc8b4f78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5005,7 +5046,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra78aa86d24d04b12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R414b23321a114492"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5352,7 +5393,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f6da32b9f914f27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7853b004e9aa4cc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5691,7 +5732,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R876a7877cc4c4da0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6276587996bf4317"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6069,38 +6110,73 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="27" t="str">
+      <x:c r="A15" s="26" t="str">
         <x:v>CHG-010</x:v>
       </x:c>
-      <x:c r="B15" s="27" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C15" s="27" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>3a5321272a857ef6cd2aac96d956924c7cc1f36b</x:v>
       </x:c>
-      <x:c r="D15" s="27" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>backend/src/common/decorators/; backend/src/modules/agents/dto/managed-profile.dto.ts; backend/src/modules/profile-details/dto/profile-details.dto.ts; backend/src/modules/users/; frontend/nginx.conf; frontend/src/pages/Biodata.tsx</x:v>
       </x:c>
-      <x:c r="E15" s="27" t="str">
+      <x:c r="E15" s="26" t="str">
         <x:v>Committed local functional fixes</x:v>
       </x:c>
-      <x:c r="F15" s="27" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G15" s="27" t="str">
+      <x:c r="G15" s="26" t="str">
         <x:v>SYNC-004</x:v>
       </x:c>
-      <x:c r="H15" s="27" t="str">
+      <x:c r="H15" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
       </x:c>
-      <x:c r="I15" s="27" t="str">
+      <x:c r="I15" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J15" s="30" t="str">
+      <x:c r="J15" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K15" s="27" t="str">
+      <x:c r="K15" s="26" t="str">
         <x:v>WOW-MD PR 56; mirror duplicate-mobile and adult-age validation, biodata save progression and mock-storage media proxying without unrelated dirty working-tree files</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="27" t="str">
+        <x:v>CHG-011</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C16" s="27" t="str">
+        <x:v>1a92ef11008645c8986b81b17c1ff3de177a669f</x:v>
+      </x:c>
+      <x:c r="D16" s="27" t="str">
+        <x:v>docker/docker-compose.yml</x:v>
+      </x:c>
+      <x:c r="E16" s="27" t="str">
+        <x:v>Vector buffer storage correction</x:v>
+      </x:c>
+      <x:c r="F16" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="str">
+        <x:v>OBS-004</x:v>
+      </x:c>
+      <x:c r="H16" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
+      </x:c>
+      <x:c r="I16" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J16" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K16" s="27" t="str">
+        <x:v>WOW-MD PR 57; Docker-managed Vector disk buffer avoids Windows bind-mount reader panics while JSONL service logs remain host-readable</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6109,7 +6185,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree1baa173fb0433f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R672ab9362c594dc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6790,40 +6866,78 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="27" t="str">
+      <x:c r="A22" s="26" t="str">
         <x:v>SYNC-004</x:v>
       </x:c>
-      <x:c r="B22" s="27" t="str">
+      <x:c r="B22" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
       </x:c>
-      <x:c r="C22" s="27" t="str">
+      <x:c r="C22" s="26" t="str">
         <x:v>codex/sync-004-local-functional</x:v>
       </x:c>
-      <x:c r="D22" s="27" t="str">
+      <x:c r="D22" s="26" t="str">
         <x:v>b4ec092</x:v>
       </x:c>
-      <x:c r="E22" s="27" t="str">
+      <x:c r="E22" s="26" t="str">
         <x:v>ca5118c</x:v>
       </x:c>
-      <x:c r="F22" s="27" t="str">
+      <x:c r="F22" s="26" t="str">
         <x:v>WOW-MD PR 56 merged as 3a53212</x:v>
       </x:c>
-      <x:c r="G22" s="27" t="str">
+      <x:c r="G22" s="26" t="str">
         <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; the exact combined source tree was deployed locally and local plus tunneled health returned 200</x:v>
       </x:c>
-      <x:c r="H22" s="27" t="str">
+      <x:c r="H22" s="26" t="str">
         <x:v>Rebuild backend and frontend images and smoke profile save biodata continuation media rendering and health</x:v>
       </x:c>
-      <x:c r="I22" s="27" t="str">
+      <x:c r="I22" s="26" t="str">
         <x:v>Revert PR 91 and rebuild the prior images; no schema rollback</x:v>
       </x:c>
-      <x:c r="J22" s="27" t="str">
+      <x:c r="J22" s="26" t="str">
         <x:v>The dirty primary checkout remains outside this reviewed mirror and continues under SYNC-001 and SYNC-002</x:v>
       </x:c>
-      <x:c r="K22" s="27" t="str">
+      <x:c r="K22" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L22" s="30" t="str">
+      <x:c r="L22" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="27" t="str">
+        <x:v>OBS-004</x:v>
+      </x:c>
+      <x:c r="B23" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
+      </x:c>
+      <x:c r="C23" s="27" t="str">
+        <x:v>codex/obs-004-vector-buffer</x:v>
+      </x:c>
+      <x:c r="D23" s="27" t="str">
+        <x:v>4e49f72</x:v>
+      </x:c>
+      <x:c r="E23" s="27" t="str">
+        <x:v>eca96ba</x:v>
+      </x:c>
+      <x:c r="F23" s="27" t="str">
+        <x:v>WOW-MD PR 57 merged as 1a92ef1</x:v>
+      </x:c>
+      <x:c r="G23" s="27" t="str">
+        <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; local Vector recreated on obs003_vector_data; three wow-prefixed churn probes completed with zero restarts or errors; Loki remained ready</x:v>
+      </x:c>
+      <x:c r="H23" s="27" t="str">
+        <x:v>Recreate Vector with the observability profile and preserve the configured host JSONL log directory</x:v>
+      </x:c>
+      <x:c r="I23" s="27" t="str">
+        <x:v>Revert PR 94 and recreate Vector with the prior bind mount; preserve host JSONL logs</x:v>
+      </x:c>
+      <x:c r="J23" s="27" t="str">
+        <x:v>The obsolete corrupted host buffer remains outside the active named volume and can be archived or removed separately</x:v>
+      </x:c>
+      <x:c r="K23" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L23" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -6831,7 +6945,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K22">
+  <x:conditionalFormatting sqref="K6:K23">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6840,7 +6954,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe8898aa42349e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a48fb98b72e4b62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize OBS-004 tracking (#95)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re64dd9545264410b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R4c03b21d525c4725"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R64381f3351a54c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R7a7fbd0e6585416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rf0fd24f27d9d48a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R4a1dc7979ec246b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R84a316c47b334015"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R00aa60daf4744e11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R0695a94581284111"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R875e39c45727442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R942ffbbb2e1f4fb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R3151609748134ed1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rfbfdf3ebec47436c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R781fa2502de54f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R47e03c3edb2a4065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R3c56a117638c44ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf0bdac3a92184c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R9e04aef798284bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R9f6723b2e54045db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rbbf4a62bda8549cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ea69d5f72ab4d86"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5a7092c124b7419c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -868,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1263,14 +1263,14 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$43)</x:f>
-        <x:v>38</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$44)</x:f>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$43,"P0",'Open Items'!$F$6:$F$43,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$44,"P0",'Open Items'!$F$6:$F$44,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1286,7 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1309,7 +1309,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"PR Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
@@ -1355,7 +1355,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Blocked")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$43,"Done")</x:f>
-        <x:v>16</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Done")</x:f>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f429cef35a04ad9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f82b2d541384dac"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R139cb3d991bc4327"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R374e9ed5240d44e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3502,43 +3502,84 @@
       </x:c>
     </x:row>
     <x:row r="43" ht="30" customHeight="1">
-      <x:c r="A43" s="27" t="str">
+      <x:c r="A43" s="26" t="str">
         <x:v>SYNC-004</x:v>
       </x:c>
-      <x:c r="B43" s="27" t="str">
+      <x:c r="B43" s="26" t="str">
         <x:v>Mirror latest committed local functional fixes</x:v>
       </x:c>
-      <x:c r="C43" s="27" t="str">
+      <x:c r="C43" s="26" t="str">
         <x:v>Source intake</x:v>
       </x:c>
-      <x:c r="D43" s="27" t="str">
+      <x:c r="D43" s="26" t="str">
         <x:v>Change intake</x:v>
       </x:c>
-      <x:c r="E43" s="27" t="str">
+      <x:c r="E43" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F43" s="27" t="str">
+      <x:c r="F43" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G43" s="27" t="str">
+      <x:c r="G43" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H43" s="27" t="str">
+      <x:c r="H43" s="26" t="str">
         <x:v>SYNC-003</x:v>
       </x:c>
-      <x:c r="I43" s="27" t="str">
+      <x:c r="I43" s="26" t="str">
         <x:v>The production repository exactly mirrors the reviewed profile validation biodata progression and mock-storage proxy fixes without unrelated dirty files</x:v>
       </x:c>
-      <x:c r="J43" s="27" t="str">
+      <x:c r="J43" s="26" t="str">
         <x:v>WOW-MD PR 56</x:v>
       </x:c>
-      <x:c r="K43" s="27" t="str">
+      <x:c r="K43" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/90</x:v>
       </x:c>
-      <x:c r="L43" s="27" t="str">
+      <x:c r="L43" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
       </x:c>
-      <x:c r="M43" s="30" t="str">
+      <x:c r="M43" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="30" customHeight="1">
+      <x:c r="A44" s="27" t="str">
+        <x:v>OBS-004</x:v>
+      </x:c>
+      <x:c r="B44" s="27" t="str">
+        <x:v>Stabilize Vector disk buffer on Windows hosts</x:v>
+      </x:c>
+      <x:c r="C44" s="27" t="str">
+        <x:v>Observability</x:v>
+      </x:c>
+      <x:c r="D44" s="27" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="E44" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F44" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G44" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H44" s="27" t="str">
+        <x:v>OBS-003</x:v>
+      </x:c>
+      <x:c r="I44" s="27" t="str">
+        <x:v>Vector retains its delivery buffer across recreation without NTFS reader panics while operator-readable JSONL logs remain on the host</x:v>
+      </x:c>
+      <x:c r="J44" s="27" t="str">
+        <x:v>WOW-MD PR 57</x:v>
+      </x:c>
+      <x:c r="K44" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/93</x:v>
+      </x:c>
+      <x:c r="L44" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
+      </x:c>
+      <x:c r="M44" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -3546,10 +3587,10 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E43">
+  <x:conditionalFormatting sqref="E6:E44">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F43">
+  <x:conditionalFormatting sqref="F6:F44">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3558,7 +3599,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb6a1a9e57c84be3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f8aaadacbdf4bbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4134,7 +4175,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R202d69b56da14ded"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff913bde120a46af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4539,7 +4580,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89aa45a801b94497"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R177734aafc8b4f78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5005,7 +5046,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra78aa86d24d04b12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R414b23321a114492"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5352,7 +5393,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f6da32b9f914f27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7853b004e9aa4cc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5691,7 +5732,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R876a7877cc4c4da0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6276587996bf4317"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6069,38 +6110,73 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="27" t="str">
+      <x:c r="A15" s="26" t="str">
         <x:v>CHG-010</x:v>
       </x:c>
-      <x:c r="B15" s="27" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C15" s="27" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>3a5321272a857ef6cd2aac96d956924c7cc1f36b</x:v>
       </x:c>
-      <x:c r="D15" s="27" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>backend/src/common/decorators/; backend/src/modules/agents/dto/managed-profile.dto.ts; backend/src/modules/profile-details/dto/profile-details.dto.ts; backend/src/modules/users/; frontend/nginx.conf; frontend/src/pages/Biodata.tsx</x:v>
       </x:c>
-      <x:c r="E15" s="27" t="str">
+      <x:c r="E15" s="26" t="str">
         <x:v>Committed local functional fixes</x:v>
       </x:c>
-      <x:c r="F15" s="27" t="str">
+      <x:c r="F15" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G15" s="27" t="str">
+      <x:c r="G15" s="26" t="str">
         <x:v>SYNC-004</x:v>
       </x:c>
-      <x:c r="H15" s="27" t="str">
+      <x:c r="H15" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
       </x:c>
-      <x:c r="I15" s="27" t="str">
+      <x:c r="I15" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J15" s="30" t="str">
+      <x:c r="J15" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K15" s="27" t="str">
+      <x:c r="K15" s="26" t="str">
         <x:v>WOW-MD PR 56; mirror duplicate-mobile and adult-age validation, biodata save progression and mock-storage media proxying without unrelated dirty working-tree files</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="27" t="str">
+        <x:v>CHG-011</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C16" s="27" t="str">
+        <x:v>1a92ef11008645c8986b81b17c1ff3de177a669f</x:v>
+      </x:c>
+      <x:c r="D16" s="27" t="str">
+        <x:v>docker/docker-compose.yml</x:v>
+      </x:c>
+      <x:c r="E16" s="27" t="str">
+        <x:v>Vector buffer storage correction</x:v>
+      </x:c>
+      <x:c r="F16" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="str">
+        <x:v>OBS-004</x:v>
+      </x:c>
+      <x:c r="H16" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
+      </x:c>
+      <x:c r="I16" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J16" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K16" s="27" t="str">
+        <x:v>WOW-MD PR 57; Docker-managed Vector disk buffer avoids Windows bind-mount reader panics while JSONL service logs remain host-readable</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6109,7 +6185,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree1baa173fb0433f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R672ab9362c594dc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6790,40 +6866,78 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="27" t="str">
+      <x:c r="A22" s="26" t="str">
         <x:v>SYNC-004</x:v>
       </x:c>
-      <x:c r="B22" s="27" t="str">
+      <x:c r="B22" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/91</x:v>
       </x:c>
-      <x:c r="C22" s="27" t="str">
+      <x:c r="C22" s="26" t="str">
         <x:v>codex/sync-004-local-functional</x:v>
       </x:c>
-      <x:c r="D22" s="27" t="str">
+      <x:c r="D22" s="26" t="str">
         <x:v>b4ec092</x:v>
       </x:c>
-      <x:c r="E22" s="27" t="str">
+      <x:c r="E22" s="26" t="str">
         <x:v>ca5118c</x:v>
       </x:c>
-      <x:c r="F22" s="27" t="str">
+      <x:c r="F22" s="26" t="str">
         <x:v>WOW-MD PR 56 merged as 3a53212</x:v>
       </x:c>
-      <x:c r="G22" s="27" t="str">
+      <x:c r="G22" s="26" t="str">
         <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; the exact combined source tree was deployed locally and local plus tunneled health returned 200</x:v>
       </x:c>
-      <x:c r="H22" s="27" t="str">
+      <x:c r="H22" s="26" t="str">
         <x:v>Rebuild backend and frontend images and smoke profile save biodata continuation media rendering and health</x:v>
       </x:c>
-      <x:c r="I22" s="27" t="str">
+      <x:c r="I22" s="26" t="str">
         <x:v>Revert PR 91 and rebuild the prior images; no schema rollback</x:v>
       </x:c>
-      <x:c r="J22" s="27" t="str">
+      <x:c r="J22" s="26" t="str">
         <x:v>The dirty primary checkout remains outside this reviewed mirror and continues under SYNC-001 and SYNC-002</x:v>
       </x:c>
-      <x:c r="K22" s="27" t="str">
+      <x:c r="K22" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L22" s="30" t="str">
+      <x:c r="L22" s="29" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="27" t="str">
+        <x:v>OBS-004</x:v>
+      </x:c>
+      <x:c r="B23" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
+      </x:c>
+      <x:c r="C23" s="27" t="str">
+        <x:v>codex/obs-004-vector-buffer</x:v>
+      </x:c>
+      <x:c r="D23" s="27" t="str">
+        <x:v>4e49f72</x:v>
+      </x:c>
+      <x:c r="E23" s="27" t="str">
+        <x:v>eca96ba</x:v>
+      </x:c>
+      <x:c r="F23" s="27" t="str">
+        <x:v>WOW-MD PR 57 merged as 1a92ef1</x:v>
+      </x:c>
+      <x:c r="G23" s="27" t="str">
+        <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; local Vector recreated on obs003_vector_data; three wow-prefixed churn probes completed with zero restarts or errors; Loki remained ready</x:v>
+      </x:c>
+      <x:c r="H23" s="27" t="str">
+        <x:v>Recreate Vector with the observability profile and preserve the configured host JSONL log directory</x:v>
+      </x:c>
+      <x:c r="I23" s="27" t="str">
+        <x:v>Revert PR 94 and recreate Vector with the prior bind mount; preserve host JSONL logs</x:v>
+      </x:c>
+      <x:c r="J23" s="27" t="str">
+        <x:v>The obsolete corrupted host buffer remains outside the active named volume and can be archived or removed separately</x:v>
+      </x:c>
+      <x:c r="K23" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L23" s="30" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
     </x:row>
@@ -6831,7 +6945,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K22">
+  <x:conditionalFormatting sqref="K6:K23">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6840,7 +6954,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbe8898aa42349e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a48fb98b72e4b62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize SYNC-005 tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R942ffbbb2e1f4fb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R3151609748134ed1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rfbfdf3ebec47436c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R781fa2502de54f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R47e03c3edb2a4065"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R3c56a117638c44ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf0bdac3a92184c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R9e04aef798284bfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R9f6723b2e54045db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rbbf4a62bda8549cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R89dd66252f3b4ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R9b7fabd5f9e24877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R5835f604902647f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R89eb7090138c44fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R72b2fa754e014e03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R286b7cc48b234af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R55eeeda03e944737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Ra0093d491f4b45da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra3bbf7ea989c4e57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R142a008446a64906"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5a7092c124b7419c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6b408392b7f4f03"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -868,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1235,7 +1235,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-06. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-07. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1263,14 +1263,14 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$44)</x:f>
-        <x:v>39</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$45)</x:f>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$44,"P0",'Open Items'!$F$6:$F$44,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$45,"P0",'Open Items'!$F$6:$F$45,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1286,7 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1309,7 +1309,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"PR Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
@@ -1355,7 +1355,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Blocked")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Done")</x:f>
-        <x:v>17</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Done")</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f82b2d541384dac"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R166b4b840f3a40db"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R374e9ed5240d44e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0513c2cd3546436e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3543,54 +3543,95 @@
       </x:c>
     </x:row>
     <x:row r="44" ht="30" customHeight="1">
-      <x:c r="A44" s="27" t="str">
+      <x:c r="A44" s="26" t="str">
         <x:v>OBS-004</x:v>
       </x:c>
-      <x:c r="B44" s="27" t="str">
+      <x:c r="B44" s="26" t="str">
         <x:v>Stabilize Vector disk buffer on Windows hosts</x:v>
       </x:c>
-      <x:c r="C44" s="27" t="str">
+      <x:c r="C44" s="26" t="str">
         <x:v>Observability</x:v>
       </x:c>
-      <x:c r="D44" s="27" t="str">
+      <x:c r="D44" s="26" t="str">
         <x:v>Reliability</x:v>
       </x:c>
-      <x:c r="E44" s="27" t="str">
+      <x:c r="E44" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F44" s="27" t="str">
+      <x:c r="F44" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G44" s="27" t="str">
+      <x:c r="G44" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H44" s="27" t="str">
+      <x:c r="H44" s="26" t="str">
         <x:v>OBS-003</x:v>
       </x:c>
-      <x:c r="I44" s="27" t="str">
+      <x:c r="I44" s="26" t="str">
         <x:v>Vector retains its delivery buffer across recreation without NTFS reader panics while operator-readable JSONL logs remain on the host</x:v>
       </x:c>
-      <x:c r="J44" s="27" t="str">
+      <x:c r="J44" s="26" t="str">
         <x:v>WOW-MD PR 57</x:v>
       </x:c>
-      <x:c r="K44" s="27" t="str">
+      <x:c r="K44" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/93</x:v>
       </x:c>
-      <x:c r="L44" s="27" t="str">
+      <x:c r="L44" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
       </x:c>
-      <x:c r="M44" s="30" t="str">
+      <x:c r="M44" s="29" t="str">
         <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="A45" s="27" t="str">
+        <x:v>SYNC-005</x:v>
+      </x:c>
+      <x:c r="B45" s="27" t="str">
+        <x:v>Mirror reviewed biodata caste family and income changes</x:v>
+      </x:c>
+      <x:c r="C45" s="27" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D45" s="27" t="str">
+        <x:v>Change intake</x:v>
+      </x:c>
+      <x:c r="E45" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F45" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G45" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H45" s="27" t="str">
+        <x:v>SYNC-004</x:v>
+      </x:c>
+      <x:c r="I45" s="27" t="str">
+        <x:v>Production exactly mirrors WOW-MD PR 58 with green protected checks and updated source baseline</x:v>
+      </x:c>
+      <x:c r="J45" s="27" t="str">
+        <x:v>WOW-MD PR 58</x:v>
+      </x:c>
+      <x:c r="K45" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/96</x:v>
+      </x:c>
+      <x:c r="L45" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
+      </x:c>
+      <x:c r="M45" s="30" t="str">
+        <x:v>2026-10-07</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E44">
+  <x:conditionalFormatting sqref="E6:E45">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F44">
+  <x:conditionalFormatting sqref="F6:F45">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3599,7 +3640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f8aaadacbdf4bbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f3e6fdf777a46bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4175,7 +4216,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff913bde120a46af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab8536c3820746fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4580,7 +4621,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R177734aafc8b4f78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d32c82550c94c0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5046,7 +5087,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R414b23321a114492"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra463f7274f494934"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5393,7 +5434,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7853b004e9aa4cc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3164d69313c44951"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5732,7 +5773,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6276587996bf4317"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R246b9993dde94e97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6145,38 +6186,73 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="27" t="str">
+      <x:c r="A16" s="26" t="str">
         <x:v>CHG-011</x:v>
       </x:c>
-      <x:c r="B16" s="27" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C16" s="27" t="str">
+      <x:c r="C16" s="26" t="str">
         <x:v>1a92ef11008645c8986b81b17c1ff3de177a669f</x:v>
       </x:c>
-      <x:c r="D16" s="27" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>docker/docker-compose.yml</x:v>
       </x:c>
-      <x:c r="E16" s="27" t="str">
+      <x:c r="E16" s="26" t="str">
         <x:v>Vector buffer storage correction</x:v>
       </x:c>
-      <x:c r="F16" s="27" t="str">
+      <x:c r="F16" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G16" s="27" t="str">
+      <x:c r="G16" s="26" t="str">
         <x:v>OBS-004</x:v>
       </x:c>
-      <x:c r="H16" s="27" t="str">
+      <x:c r="H16" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
       </x:c>
-      <x:c r="I16" s="27" t="str">
+      <x:c r="I16" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J16" s="30" t="str">
+      <x:c r="J16" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K16" s="27" t="str">
+      <x:c r="K16" s="26" t="str">
         <x:v>WOW-MD PR 57; Docker-managed Vector disk buffer avoids Windows bind-mount reader panics while JSONL service logs remain host-readable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="27" t="str">
+        <x:v>CHG-012</x:v>
+      </x:c>
+      <x:c r="B17" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C17" s="27" t="str">
+        <x:v>442111a36f5e93703b27fbd7859c89a1f34b1547</x:v>
+      </x:c>
+      <x:c r="D17" s="27" t="str">
+        <x:v>backend/src/modules/profile-details/; backend/test/business-entries.e2e-spec.ts; frontend/src/components/; frontend/src/pages/Biodata.tsx</x:v>
+      </x:c>
+      <x:c r="E17" s="27" t="str">
+        <x:v>Biodata and profile flow improvements</x:v>
+      </x:c>
+      <x:c r="F17" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="str">
+        <x:v>SYNC-005</x:v>
+      </x:c>
+      <x:c r="H17" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
+      </x:c>
+      <x:c r="I17" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J17" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K17" s="27" t="str">
+        <x:v>WOW-MD PR 58; expanded caste handling, parent courtesy titles, positive income validation, saved-biodata behavior and aligned unit/API regression coverage</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6185,7 +6261,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R672ab9362c594dc5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93704cdc8b514f18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6904,48 +6980,86 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="27" t="str">
+      <x:c r="A23" s="26" t="str">
         <x:v>OBS-004</x:v>
       </x:c>
-      <x:c r="B23" s="27" t="str">
+      <x:c r="B23" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
       </x:c>
-      <x:c r="C23" s="27" t="str">
+      <x:c r="C23" s="26" t="str">
         <x:v>codex/obs-004-vector-buffer</x:v>
       </x:c>
-      <x:c r="D23" s="27" t="str">
+      <x:c r="D23" s="26" t="str">
         <x:v>4e49f72</x:v>
       </x:c>
-      <x:c r="E23" s="27" t="str">
+      <x:c r="E23" s="26" t="str">
         <x:v>eca96ba</x:v>
       </x:c>
-      <x:c r="F23" s="27" t="str">
+      <x:c r="F23" s="26" t="str">
         <x:v>WOW-MD PR 57 merged as 1a92ef1</x:v>
       </x:c>
-      <x:c r="G23" s="27" t="str">
+      <x:c r="G23" s="26" t="str">
         <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; local Vector recreated on obs003_vector_data; three wow-prefixed churn probes completed with zero restarts or errors; Loki remained ready</x:v>
       </x:c>
-      <x:c r="H23" s="27" t="str">
+      <x:c r="H23" s="26" t="str">
         <x:v>Recreate Vector with the observability profile and preserve the configured host JSONL log directory</x:v>
       </x:c>
-      <x:c r="I23" s="27" t="str">
+      <x:c r="I23" s="26" t="str">
         <x:v>Revert PR 94 and recreate Vector with the prior bind mount; preserve host JSONL logs</x:v>
       </x:c>
-      <x:c r="J23" s="27" t="str">
+      <x:c r="J23" s="26" t="str">
         <x:v>The obsolete corrupted host buffer remains outside the active named volume and can be archived or removed separately</x:v>
       </x:c>
-      <x:c r="K23" s="27" t="str">
+      <x:c r="K23" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L23" s="30" t="str">
+      <x:c r="L23" s="29" t="str">
         <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="27" t="str">
+        <x:v>SYNC-005</x:v>
+      </x:c>
+      <x:c r="B24" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
+      </x:c>
+      <x:c r="C24" s="27" t="str">
+        <x:v>codex/sync-005-biodata-flows</x:v>
+      </x:c>
+      <x:c r="D24" s="27" t="str">
+        <x:v>7423193</x:v>
+      </x:c>
+      <x:c r="E24" s="27" t="str">
+        <x:v>c87221f</x:v>
+      </x:c>
+      <x:c r="F24" s="27" t="str">
+        <x:v>WOW-MD PR 58 merged as 442111a</x:v>
+      </x:c>
+      <x:c r="G24" s="27" t="str">
+        <x:v>Source and production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; local backend lint typecheck 839 tests and build plus frontend typecheck 180 tests and build passed</x:v>
+      </x:c>
+      <x:c r="H24" s="27" t="str">
+        <x:v>Rebuild backend and frontend images then smoke health and biodata/profile entry points</x:v>
+      </x:c>
+      <x:c r="I24" s="27" t="str">
+        <x:v>Revert PR 97 and rebuild the prior images; no schema migration or dependency rollback</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="str">
+        <x:v>Legacy zero-valued stored business income remains readable but new submissions require a positive whole-rupee amount</x:v>
+      </x:c>
+      <x:c r="K24" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L24" s="30" t="str">
+        <x:v>2026-10-07</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K23">
+  <x:conditionalFormatting sqref="K6:K24">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6954,7 +7068,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a48fb98b72e4b62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb39cc6ddc21642c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize SYNC-005 tracking (#98)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R942ffbbb2e1f4fb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R3151609748134ed1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rfbfdf3ebec47436c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R781fa2502de54f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R47e03c3edb2a4065"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R3c56a117638c44ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf0bdac3a92184c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R9e04aef798284bfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R9f6723b2e54045db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rbbf4a62bda8549cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R89dd66252f3b4ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R9b7fabd5f9e24877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R5835f604902647f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R89eb7090138c44fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R72b2fa754e014e03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R286b7cc48b234af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R55eeeda03e944737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Ra0093d491f4b45da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra3bbf7ea989c4e57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R142a008446a64906"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5a7092c124b7419c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6b408392b7f4f03"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -868,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -969,7 +969,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1235,7 +1235,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-06. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-07. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1263,14 +1263,14 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$44)</x:f>
-        <x:v>39</x:v>
+        <x:f>COUNTA('Open Items'!$A$6:$A$45)</x:f>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$44,"P0",'Open Items'!$F$6:$F$44,"&lt;&gt;Done")</x:f>
+        <x:f>COUNTIFS('Open Items'!$E$6:$E$45,"P0",'Open Items'!$F$6:$F$45,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1286,7 +1286,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Open")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
@@ -1309,7 +1309,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"In Progress")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"PR Open")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
@@ -1355,7 +1355,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Blocked")</x:f>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1378,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$44,"Done")</x:f>
-        <x:v>17</x:v>
+        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Done")</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1478,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f82b2d541384dac"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R166b4b840f3a40db"/>
 </x:worksheet>
 </file>
 
@@ -1964,7 +1964,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R374e9ed5240d44e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0513c2cd3546436e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3543,54 +3543,95 @@
       </x:c>
     </x:row>
     <x:row r="44" ht="30" customHeight="1">
-      <x:c r="A44" s="27" t="str">
+      <x:c r="A44" s="26" t="str">
         <x:v>OBS-004</x:v>
       </x:c>
-      <x:c r="B44" s="27" t="str">
+      <x:c r="B44" s="26" t="str">
         <x:v>Stabilize Vector disk buffer on Windows hosts</x:v>
       </x:c>
-      <x:c r="C44" s="27" t="str">
+      <x:c r="C44" s="26" t="str">
         <x:v>Observability</x:v>
       </x:c>
-      <x:c r="D44" s="27" t="str">
+      <x:c r="D44" s="26" t="str">
         <x:v>Reliability</x:v>
       </x:c>
-      <x:c r="E44" s="27" t="str">
+      <x:c r="E44" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F44" s="27" t="str">
+      <x:c r="F44" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G44" s="27" t="str">
+      <x:c r="G44" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H44" s="27" t="str">
+      <x:c r="H44" s="26" t="str">
         <x:v>OBS-003</x:v>
       </x:c>
-      <x:c r="I44" s="27" t="str">
+      <x:c r="I44" s="26" t="str">
         <x:v>Vector retains its delivery buffer across recreation without NTFS reader panics while operator-readable JSONL logs remain on the host</x:v>
       </x:c>
-      <x:c r="J44" s="27" t="str">
+      <x:c r="J44" s="26" t="str">
         <x:v>WOW-MD PR 57</x:v>
       </x:c>
-      <x:c r="K44" s="27" t="str">
+      <x:c r="K44" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/93</x:v>
       </x:c>
-      <x:c r="L44" s="27" t="str">
+      <x:c r="L44" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
       </x:c>
-      <x:c r="M44" s="30" t="str">
+      <x:c r="M44" s="29" t="str">
         <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="A45" s="27" t="str">
+        <x:v>SYNC-005</x:v>
+      </x:c>
+      <x:c r="B45" s="27" t="str">
+        <x:v>Mirror reviewed biodata caste family and income changes</x:v>
+      </x:c>
+      <x:c r="C45" s="27" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D45" s="27" t="str">
+        <x:v>Change intake</x:v>
+      </x:c>
+      <x:c r="E45" s="27" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F45" s="27" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G45" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H45" s="27" t="str">
+        <x:v>SYNC-004</x:v>
+      </x:c>
+      <x:c r="I45" s="27" t="str">
+        <x:v>Production exactly mirrors WOW-MD PR 58 with green protected checks and updated source baseline</x:v>
+      </x:c>
+      <x:c r="J45" s="27" t="str">
+        <x:v>WOW-MD PR 58</x:v>
+      </x:c>
+      <x:c r="K45" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/96</x:v>
+      </x:c>
+      <x:c r="L45" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
+      </x:c>
+      <x:c r="M45" s="30" t="str">
+        <x:v>2026-10-07</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:M3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="E6:E44">
+  <x:conditionalFormatting sqref="E6:E45">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="P0"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F6:F44">
+  <x:conditionalFormatting sqref="F6:F45">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
@@ -3599,7 +3640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f8aaadacbdf4bbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f3e6fdf777a46bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4175,7 +4216,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff913bde120a46af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab8536c3820746fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4580,7 +4621,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R177734aafc8b4f78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d32c82550c94c0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5046,7 +5087,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R414b23321a114492"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra463f7274f494934"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5393,7 +5434,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7853b004e9aa4cc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3164d69313c44951"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5732,7 +5773,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6276587996bf4317"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R246b9993dde94e97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6145,38 +6186,73 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="27" t="str">
+      <x:c r="A16" s="26" t="str">
         <x:v>CHG-011</x:v>
       </x:c>
-      <x:c r="B16" s="27" t="str">
+      <x:c r="B16" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C16" s="27" t="str">
+      <x:c r="C16" s="26" t="str">
         <x:v>1a92ef11008645c8986b81b17c1ff3de177a669f</x:v>
       </x:c>
-      <x:c r="D16" s="27" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>docker/docker-compose.yml</x:v>
       </x:c>
-      <x:c r="E16" s="27" t="str">
+      <x:c r="E16" s="26" t="str">
         <x:v>Vector buffer storage correction</x:v>
       </x:c>
-      <x:c r="F16" s="27" t="str">
+      <x:c r="F16" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G16" s="27" t="str">
+      <x:c r="G16" s="26" t="str">
         <x:v>OBS-004</x:v>
       </x:c>
-      <x:c r="H16" s="27" t="str">
+      <x:c r="H16" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
       </x:c>
-      <x:c r="I16" s="27" t="str">
+      <x:c r="I16" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J16" s="30" t="str">
+      <x:c r="J16" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K16" s="27" t="str">
+      <x:c r="K16" s="26" t="str">
         <x:v>WOW-MD PR 57; Docker-managed Vector disk buffer avoids Windows bind-mount reader panics while JSONL service logs remain host-readable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="27" t="str">
+        <x:v>CHG-012</x:v>
+      </x:c>
+      <x:c r="B17" s="27" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C17" s="27" t="str">
+        <x:v>442111a36f5e93703b27fbd7859c89a1f34b1547</x:v>
+      </x:c>
+      <x:c r="D17" s="27" t="str">
+        <x:v>backend/src/modules/profile-details/; backend/test/business-entries.e2e-spec.ts; frontend/src/components/; frontend/src/pages/Biodata.tsx</x:v>
+      </x:c>
+      <x:c r="E17" s="27" t="str">
+        <x:v>Biodata and profile flow improvements</x:v>
+      </x:c>
+      <x:c r="F17" s="27" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="str">
+        <x:v>SYNC-005</x:v>
+      </x:c>
+      <x:c r="H17" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
+      </x:c>
+      <x:c r="I17" s="27" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J17" s="30" t="str">
+        <x:v>2026-10-06</x:v>
+      </x:c>
+      <x:c r="K17" s="27" t="str">
+        <x:v>WOW-MD PR 58; expanded caste handling, parent courtesy titles, positive income validation, saved-biodata behavior and aligned unit/API regression coverage</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6185,7 +6261,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R672ab9362c594dc5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93704cdc8b514f18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6904,48 +6980,86 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="27" t="str">
+      <x:c r="A23" s="26" t="str">
         <x:v>OBS-004</x:v>
       </x:c>
-      <x:c r="B23" s="27" t="str">
+      <x:c r="B23" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/94</x:v>
       </x:c>
-      <x:c r="C23" s="27" t="str">
+      <x:c r="C23" s="26" t="str">
         <x:v>codex/obs-004-vector-buffer</x:v>
       </x:c>
-      <x:c r="D23" s="27" t="str">
+      <x:c r="D23" s="26" t="str">
         <x:v>4e49f72</x:v>
       </x:c>
-      <x:c r="E23" s="27" t="str">
+      <x:c r="E23" s="26" t="str">
         <x:v>eca96ba</x:v>
       </x:c>
-      <x:c r="F23" s="27" t="str">
+      <x:c r="F23" s="26" t="str">
         <x:v>WOW-MD PR 57 merged as 1a92ef1</x:v>
       </x:c>
-      <x:c r="G23" s="27" t="str">
+      <x:c r="G23" s="26" t="str">
         <x:v>Production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; local Vector recreated on obs003_vector_data; three wow-prefixed churn probes completed with zero restarts or errors; Loki remained ready</x:v>
       </x:c>
-      <x:c r="H23" s="27" t="str">
+      <x:c r="H23" s="26" t="str">
         <x:v>Recreate Vector with the observability profile and preserve the configured host JSONL log directory</x:v>
       </x:c>
-      <x:c r="I23" s="27" t="str">
+      <x:c r="I23" s="26" t="str">
         <x:v>Revert PR 94 and recreate Vector with the prior bind mount; preserve host JSONL logs</x:v>
       </x:c>
-      <x:c r="J23" s="27" t="str">
+      <x:c r="J23" s="26" t="str">
         <x:v>The obsolete corrupted host buffer remains outside the active named volume and can be archived or removed separately</x:v>
       </x:c>
-      <x:c r="K23" s="27" t="str">
+      <x:c r="K23" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L23" s="30" t="str">
+      <x:c r="L23" s="29" t="str">
         <x:v>2026-10-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="27" t="str">
+        <x:v>SYNC-005</x:v>
+      </x:c>
+      <x:c r="B24" s="27" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
+      </x:c>
+      <x:c r="C24" s="27" t="str">
+        <x:v>codex/sync-005-biodata-flows</x:v>
+      </x:c>
+      <x:c r="D24" s="27" t="str">
+        <x:v>7423193</x:v>
+      </x:c>
+      <x:c r="E24" s="27" t="str">
+        <x:v>c87221f</x:v>
+      </x:c>
+      <x:c r="F24" s="27" t="str">
+        <x:v>WOW-MD PR 58 merged as 442111a</x:v>
+      </x:c>
+      <x:c r="G24" s="27" t="str">
+        <x:v>Source and production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; local backend lint typecheck 839 tests and build plus frontend typecheck 180 tests and build passed</x:v>
+      </x:c>
+      <x:c r="H24" s="27" t="str">
+        <x:v>Rebuild backend and frontend images then smoke health and biodata/profile entry points</x:v>
+      </x:c>
+      <x:c r="I24" s="27" t="str">
+        <x:v>Revert PR 97 and rebuild the prior images; no schema migration or dependency rollback</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="str">
+        <x:v>Legacy zero-valued stored business income remains readable but new submissions require a positive whole-rupee amount</x:v>
+      </x:c>
+      <x:c r="K24" s="27" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L24" s="30" t="str">
+        <x:v>2026-10-07</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K6:K23">
+  <x:conditionalFormatting sqref="K6:K24">
     <x:cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="29" priority="2" operator="containsText" text="In Progress"/>
     <x:cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="Blocked"/>
@@ -6954,7 +7068,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a48fb98b72e4b62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb39cc6ddc21642c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize QA-004 workflow evidence
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R89dd66252f3b4ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R9b7fabd5f9e24877"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R5835f604902647f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R89eb7090138c44fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R72b2fa754e014e03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R286b7cc48b234af7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R55eeeda03e944737"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Ra0093d491f4b45da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra3bbf7ea989c4e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R142a008446a64906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R94e4317a09984da0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R2f668fd39b2443be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rbdf62a447fe84d91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R0e0218d77b954816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R18ac0789dc614630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R58cf2dbd62054d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra0a1fc87a679474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R18f1628d35f24bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rcbe1e1ff13ac4bb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Re7087bbe36fe4ef5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -252,7 +252,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -262,7 +262,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -272,7 +272,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -283,7 +283,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -293,7 +293,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -303,7 +303,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -314,7 +314,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -324,7 +324,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -334,7 +334,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -345,7 +345,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -355,7 +355,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -365,7 +365,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -376,7 +376,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -386,7 +386,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -396,7 +396,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -407,7 +407,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -417,7 +417,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -427,7 +427,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -437,7 +437,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -447,7 +447,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -458,7 +458,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -468,7 +468,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -478,7 +478,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -488,7 +488,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -498,7 +498,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -509,7 +509,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -519,7 +519,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -529,7 +529,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -539,7 +539,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -549,7 +549,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -560,7 +560,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -570,7 +570,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -580,7 +580,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -590,7 +590,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -600,7 +600,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -611,7 +611,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -621,7 +621,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -631,7 +631,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -642,7 +642,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -652,7 +652,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6b408392b7f4f03"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R35186cf222af4b63"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1235,7 +1235,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-07. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-08. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1263,14 +1263,12 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$45)</x:f>
         <x:v>40</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$45,"P0",'Open Items'!$F$6:$F$45,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1278,7 +1276,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1286,14 +1284,12 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Open")</x:f>
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
       </x:c>
       <x:c r="E7" s="34" t="n">
-        <x:f>COUNTIF('Release Gates'!$E$6:$E$17,"Open")</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="G7" s="39" t="str">
@@ -1309,14 +1305,12 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
@@ -1332,14 +1326,12 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$19,"P0",Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
@@ -1355,14 +1347,12 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIF(Requirements!$G$6:$G$27,"Approved")</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="G10" s="39" t="str">
@@ -1370,7 +1360,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1368,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Done")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1467,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R166b4b840f3a40db"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b1915236554385"/>
 </x:worksheet>
 </file>
 
@@ -1926,28 +1915,28 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="27" t="str">
+      <x:c r="A21" s="26" t="str">
         <x:v>DOC-016</x:v>
       </x:c>
-      <x:c r="B21" s="27" t="str">
+      <x:c r="B21" s="26" t="str">
         <x:v>Dependency remediation record</x:v>
       </x:c>
-      <x:c r="C21" s="27" t="str">
+      <x:c r="C21" s="26" t="str">
         <x:v>docs/security/dependency-remediation-2026-10-04.md</x:v>
       </x:c>
-      <x:c r="D21" s="27" t="str">
+      <x:c r="D21" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="E21" s="27" t="str">
+      <x:c r="E21" s="26" t="str">
         <x:v>Approved candidate</x:v>
       </x:c>
-      <x:c r="F21" s="27" t="str">
+      <x:c r="F21" s="26" t="str">
         <x:v>Each dependency change</x:v>
       </x:c>
-      <x:c r="G21" s="27" t="str">
+      <x:c r="G21" s="26" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
-      <x:c r="H21" s="27" t="str">
+      <x:c r="H21" s="26" t="str">
         <x:v>DEP-001</x:v>
       </x:c>
     </x:row>
@@ -1964,7 +1953,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0513c2cd3546436e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3366dffb46c34d8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3120,24 +3109,26 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F33" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G33" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H33" s="26" t="str"/>
       <x:c r="I33" s="26" t="str">
-        <x:v>Legacy two failures are updated to current accessible contracts and pass</x:v>
+        <x:v>Live registration supplies every required field; visual audit ignores captionless accessible wrappers; matching exposes its accessible journey region; protected and live suites pass</x:v>
       </x:c>
       <x:c r="J33" s="26" t="str">
-        <x:v>QA findings F-002 F-003</x:v>
+        <x:v>QA findings F-002 F-003; WOW-MD PR 59</x:v>
       </x:c>
       <x:c r="K33" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/33</x:v>
       </x:c>
-      <x:c r="L33" s="26" t="str"/>
+      <x:c r="L33" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/99</x:v>
+      </x:c>
       <x:c r="M33" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-08</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="30" customHeight="1">
@@ -3584,43 +3575,43 @@
       </x:c>
     </x:row>
     <x:row r="45" ht="30" customHeight="1">
-      <x:c r="A45" s="27" t="str">
+      <x:c r="A45" s="26" t="str">
         <x:v>SYNC-005</x:v>
       </x:c>
-      <x:c r="B45" s="27" t="str">
+      <x:c r="B45" s="26" t="str">
         <x:v>Mirror reviewed biodata caste family and income changes</x:v>
       </x:c>
-      <x:c r="C45" s="27" t="str">
+      <x:c r="C45" s="26" t="str">
         <x:v>Source intake</x:v>
       </x:c>
-      <x:c r="D45" s="27" t="str">
+      <x:c r="D45" s="26" t="str">
         <x:v>Change intake</x:v>
       </x:c>
-      <x:c r="E45" s="27" t="str">
+      <x:c r="E45" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F45" s="27" t="str">
+      <x:c r="F45" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G45" s="27" t="str">
+      <x:c r="G45" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H45" s="27" t="str">
+      <x:c r="H45" s="26" t="str">
         <x:v>SYNC-004</x:v>
       </x:c>
-      <x:c r="I45" s="27" t="str">
+      <x:c r="I45" s="26" t="str">
         <x:v>Production exactly mirrors WOW-MD PR 58 with green protected checks and updated source baseline</x:v>
       </x:c>
-      <x:c r="J45" s="27" t="str">
+      <x:c r="J45" s="26" t="str">
         <x:v>WOW-MD PR 58</x:v>
       </x:c>
-      <x:c r="K45" s="27" t="str">
+      <x:c r="K45" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/96</x:v>
       </x:c>
-      <x:c r="L45" s="27" t="str">
+      <x:c r="L45" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
       </x:c>
-      <x:c r="M45" s="30" t="str">
+      <x:c r="M45" s="29" t="str">
         <x:v>2026-10-07</x:v>
       </x:c>
     </x:row>
@@ -3640,7 +3631,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f3e6fdf777a46bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R702be71bddd74cc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4178,25 +4169,25 @@
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="27" t="str">
+      <x:c r="A27" s="26" t="str">
         <x:v>REQ-AUTH-004</x:v>
       </x:c>
-      <x:c r="B27" s="27" t="str">
+      <x:c r="B27" s="26" t="str">
         <x:v>Zoho domain DNS sender mailbox SMTP application password and production OAuth callback are configured only at the final deployment gate</x:v>
       </x:c>
-      <x:c r="C27" s="27" t="str">
+      <x:c r="C27" s="26" t="str">
         <x:v>User direction</x:v>
       </x:c>
-      <x:c r="D27" s="27" t="str">
+      <x:c r="D27" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="E27" s="27" t="str">
+      <x:c r="E27" s="26" t="str">
         <x:v>Final release checklist and controlled delivery/SSO evidence</x:v>
       </x:c>
-      <x:c r="F27" s="27" t="str">
+      <x:c r="F27" s="26" t="str">
         <x:v>SEC-001,REL-001</x:v>
       </x:c>
-      <x:c r="G27" s="27" t="str">
+      <x:c r="G27" s="26" t="str">
         <x:v>Approved</x:v>
       </x:c>
     </x:row>
@@ -4216,7 +4207,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab8536c3820746fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c3cf93a1846426e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4324,19 +4315,19 @@
         <x:v>Live UI role navigation</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>105 authenticated screens across 8 roles</x:v>
+        <x:v>Public pages fresh registration and authenticated role journeys across 8 roles</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>QA workbook 2026-10-04</x:v>
+        <x:v>Source live run 37687163848 and production live run 37687169181</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>16 of 18 legacy tests plus replacement flows</x:v>
+        <x:v>25 of 25 passed in both repositories</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>Current locator suite green</x:v>
+        <x:v>Repeat on Railway candidate</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>QA-004</x:v>
+        <x:v>QA-004 REL-001</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -4511,13 +4502,13 @@
         <x:v>Private-source report and shared-code mirror gate</x:v>
       </x:c>
       <x:c r="D16" s="26" t="str">
-        <x:v>PR 55 local evidence</x:v>
+        <x:v>Production source-sync run 37687173815</x:v>
       </x:c>
       <x:c r="E16" s="26" t="str">
-        <x:v>19 of 19 governance and synchronization tests passed</x:v>
+        <x:v>19 of 19 governance tests passed and scheduled review reported zero unreviewed commits or paths</x:v>
       </x:c>
       <x:c r="F16" s="26" t="str">
-        <x:v>Configure WOW_SYNC_TOKEN and capture first scheduled artifact</x:v>
+        <x:v>Replace the temporary broad token with a fine-grained WOW-MD Contents read-only token before private visibility</x:v>
       </x:c>
       <x:c r="G16" s="26" t="str">
         <x:v>SYNC-002</x:v>
@@ -4593,25 +4584,25 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="27" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>QA-OBS-001</x:v>
       </x:c>
-      <x:c r="B20" s="27" t="str">
+      <x:c r="B20" s="26" t="str">
         <x:v>Observability</x:v>
       </x:c>
-      <x:c r="C20" s="27" t="str">
+      <x:c r="C20" s="26" t="str">
         <x:v>Request correlation redaction provider logs QA capture audit failures payout sweep and nginx JSON</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="str">
+      <x:c r="D20" s="26" t="str">
         <x:v>OBS-001 PR 69 and merged WOW-MD PR 43</x:v>
       </x:c>
-      <x:c r="E20" s="27" t="str">
+      <x:c r="E20" s="26" t="str">
         <x:v>Focused observability and replica-lock integration 27 of 27; typecheck lint and nginx contract passed; protected CI recorded on PR 69</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>Verify live response/log correlation with capture disabled</x:v>
       </x:c>
-      <x:c r="G20" s="27" t="str">
+      <x:c r="G20" s="26" t="str">
         <x:v>OBS-001</x:v>
       </x:c>
     </x:row>
@@ -4621,7 +4612,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d32c82550c94c0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39cc8316a26a49a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5043,31 +5034,31 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="27" t="str">
+      <x:c r="A19" s="26" t="str">
         <x:v>RISK-014</x:v>
       </x:c>
-      <x:c r="B19" s="27" t="str">
+      <x:c r="B19" s="26" t="str">
         <x:v>Framework and mobile build-tool dependency advisories remain after runtime remediation</x:v>
       </x:c>
-      <x:c r="C19" s="27" t="str">
+      <x:c r="C19" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D19" s="27" t="str">
+      <x:c r="D19" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E19" s="27" t="str">
+      <x:c r="E19" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F19" s="27" t="str">
+      <x:c r="F19" s="26" t="str">
         <x:v>Block new critical/high runtime advisories; allow only four exact no-fix Expo advisory IDs; schedule Nest major migration and review exceptions each release</x:v>
       </x:c>
-      <x:c r="G19" s="27" t="str">
+      <x:c r="G19" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H19" s="27" t="str">
+      <x:c r="H19" s="26" t="str">
         <x:v>Mitigated</x:v>
       </x:c>
-      <x:c r="I19" s="27" t="str">
+      <x:c r="I19" s="26" t="str">
         <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
       </x:c>
     </x:row>
@@ -5087,7 +5078,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra463f7274f494934"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd50c21949af14669"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5395,30 +5386,32 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="27" t="str">
+      <x:c r="A15" s="26" t="str">
         <x:v>ACC-010</x:v>
       </x:c>
-      <x:c r="B15" s="27" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>WOW-MD source review</x:v>
       </x:c>
-      <x:c r="C15" s="27" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>Repository contents read for scheduled change reports</x:v>
       </x:c>
-      <x:c r="D15" s="27" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>RohithTadiparti</x:v>
       </x:c>
-      <x:c r="E15" s="27" t="str">
-        <x:v>Fine-grained WOW_SYNC_TOKEN</x:v>
-      </x:c>
-      <x:c r="F15" s="27" t="str">
+      <x:c r="E15" s="26" t="str">
+        <x:v>Temporary classic token in WOW_SYNC_TOKEN; replace with fine-grained token</x:v>
+      </x:c>
+      <x:c r="F15" s="26" t="str">
         <x:v>Production GitHub Actions secret</x:v>
       </x:c>
-      <x:c r="G15" s="27" t="str">
-        <x:v>Deferred</x:v>
-      </x:c>
-      <x:c r="H15" s="30" t="str"/>
-      <x:c r="I15" s="27" t="str">
-        <x:v>Not technically required while WOW-MD is public; create before returning it private so the private-ready workflow keeps working; scope only to WOW-MD Contents read and rotate within 90 days</x:v>
+      <x:c r="G15" s="26" t="str">
+        <x:v>Available - replacement required</x:v>
+      </x:c>
+      <x:c r="H15" s="29" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="I15" s="26" t="str">
+        <x:v>Scheduled run 37687173815 passed. Replace the current broad repo/workflow token before private visibility with a token scoped only to WOW-MD Contents read; rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5434,7 +5427,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3164d69313c44951"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc29fd53ae2814446"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5739,26 +5732,26 @@
       <x:c r="H16" s="29" t="str"/>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>GATE-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>Railway decommission</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>Production</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>72-hour stable AWS operation and separate approval</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Product owner</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str"/>
-      <x:c r="H17" s="30" t="str"/>
+      <x:c r="G17" s="26" t="str"/>
+      <x:c r="H17" s="29" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5773,7 +5766,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R246b9993dde94e97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc13916f88b4f429b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6221,38 +6214,73 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>CHG-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>442111a36f5e93703b27fbd7859c89a1f34b1547</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>backend/src/modules/profile-details/; backend/test/business-entries.e2e-spec.ts; frontend/src/components/; frontend/src/pages/Biodata.tsx</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>Biodata and profile flow improvements</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>SYNC-005</x:v>
       </x:c>
-      <x:c r="H17" s="27" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
       </x:c>
-      <x:c r="I17" s="27" t="str">
+      <x:c r="I17" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J17" s="30" t="str">
+      <x:c r="J17" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K17" s="27" t="str">
+      <x:c r="K17" s="26" t="str">
         <x:v>WOW-MD PR 58; expanded caste handling, parent courtesy titles, positive income validation, saved-biodata behavior and aligned unit/API regression coverage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="26" t="str">
+        <x:v>CHG-013</x:v>
+      </x:c>
+      <x:c r="B18" s="26" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>9f063fd678e88f73768f7a665d02293386180e3e</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="str">
+        <x:v>frontend/e2e/register.e2e.ts; frontend/e2e/template.ts; frontend/src/pages/Matches.tsx</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="str">
+        <x:v>Live browser journey contract repairs</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
+        <x:v>QA-004</x:v>
+      </x:c>
+      <x:c r="H18" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/99</x:v>
+      </x:c>
+      <x:c r="I18" s="26" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J18" s="29" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K18" s="26" t="str">
+        <x:v>WOW-MD PR 59; supplies the required registration username, bounds response waiting, excludes captionless accessible wrappers from typography checks and restores the accessible matching journey region</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6261,7 +6289,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93704cdc8b514f18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R574846fae2a9486e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7018,41 +7046,79 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="27" t="str">
+      <x:c r="A24" s="26" t="str">
         <x:v>SYNC-005</x:v>
       </x:c>
-      <x:c r="B24" s="27" t="str">
+      <x:c r="B24" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
       </x:c>
-      <x:c r="C24" s="27" t="str">
+      <x:c r="C24" s="26" t="str">
         <x:v>codex/sync-005-biodata-flows</x:v>
       </x:c>
-      <x:c r="D24" s="27" t="str">
+      <x:c r="D24" s="26" t="str">
         <x:v>7423193</x:v>
       </x:c>
-      <x:c r="E24" s="27" t="str">
+      <x:c r="E24" s="26" t="str">
         <x:v>c87221f</x:v>
       </x:c>
-      <x:c r="F24" s="27" t="str">
+      <x:c r="F24" s="26" t="str">
         <x:v>WOW-MD PR 58 merged as 442111a</x:v>
       </x:c>
-      <x:c r="G24" s="27" t="str">
+      <x:c r="G24" s="26" t="str">
         <x:v>Source and production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; local backend lint typecheck 839 tests and build plus frontend typecheck 180 tests and build passed</x:v>
       </x:c>
-      <x:c r="H24" s="27" t="str">
+      <x:c r="H24" s="26" t="str">
         <x:v>Rebuild backend and frontend images then smoke health and biodata/profile entry points</x:v>
       </x:c>
-      <x:c r="I24" s="27" t="str">
+      <x:c r="I24" s="26" t="str">
         <x:v>Revert PR 97 and rebuild the prior images; no schema migration or dependency rollback</x:v>
       </x:c>
-      <x:c r="J24" s="27" t="str">
+      <x:c r="J24" s="26" t="str">
         <x:v>Legacy zero-valued stored business income remains readable but new submissions require a positive whole-rupee amount</x:v>
       </x:c>
-      <x:c r="K24" s="27" t="str">
+      <x:c r="K24" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L24" s="30" t="str">
+      <x:c r="L24" s="29" t="str">
         <x:v>2026-10-07</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="26" t="str">
+        <x:v>QA-004</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/99</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>codex/qa-004-live-e2e-contracts</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>ff075ae</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>721ebb8</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>WOW-MD PR 59 merged as 9f063fd</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="str">
+        <x:v>Source and production protected frontend backend E2E mobile Docker CodeQL secrets and governance checks passed; local frontend typecheck 180 tests and production build passed; source live E2E run 37687163848 and production live E2E run 37687169181 each passed all 25 cases; source-sync review 37687173815 passed with zero unreviewed commits or paths</x:v>
+      </x:c>
+      <x:c r="H25" s="26" t="str">
+        <x:v>Frontend image rebuilt from 9f063fd; container healthy; local and tunneled health returned 200</x:v>
+      </x:c>
+      <x:c r="I25" s="26" t="str">
+        <x:v>Revert PR 99 and rebuild the prior frontend image; no schema migration or dependency rollback</x:v>
+      </x:c>
+      <x:c r="J25" s="26" t="str">
+        <x:v>The live registration test intentionally creates one test account per run; replace the broad temporary WOW_SYNC_TOKEN with a fine-grained read-only token</x:v>
+      </x:c>
+      <x:c r="K25" s="26" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L25" s="29" t="str">
+        <x:v>2026-10-08</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7068,7 +7134,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb39cc6ddc21642c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e095a8681314739"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finalize QA-004 workflow evidence (#100)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R89dd66252f3b4ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R9b7fabd5f9e24877"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R5835f604902647f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R89eb7090138c44fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R72b2fa754e014e03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R286b7cc48b234af7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R55eeeda03e944737"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Ra0093d491f4b45da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra3bbf7ea989c4e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R142a008446a64906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R94e4317a09984da0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R2f668fd39b2443be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rbdf62a447fe84d91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R0e0218d77b954816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R18ac0789dc614630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R58cf2dbd62054d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra0a1fc87a679474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R18f1628d35f24bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rcbe1e1ff13ac4bb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Re7087bbe36fe4ef5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -252,7 +252,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -262,7 +262,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -272,7 +272,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -283,7 +283,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -293,7 +293,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -303,7 +303,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -314,7 +314,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -324,7 +324,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -334,7 +334,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -345,7 +345,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -355,7 +355,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -365,7 +365,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -376,7 +376,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -386,7 +386,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -396,7 +396,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -407,7 +407,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -417,7 +417,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -427,7 +427,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -437,7 +437,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -447,7 +447,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -458,7 +458,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -468,7 +468,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -478,7 +478,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -488,7 +488,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -498,7 +498,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -509,7 +509,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -519,7 +519,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -529,7 +529,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -539,7 +539,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -549,7 +549,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -560,7 +560,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -570,7 +570,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -580,7 +580,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -590,7 +590,7 @@
         <x:color rgb="FF7A4B00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -600,7 +600,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -611,7 +611,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -621,7 +621,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -631,7 +631,7 @@
         <x:color rgb="FF18733A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5EC"/>
         </x:patternFill>
       </x:fill>
@@ -642,7 +642,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E8"/>
         </x:patternFill>
       </x:fill>
@@ -652,7 +652,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF1FB"/>
         </x:patternFill>
       </x:fill>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6b408392b7f4f03"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R35186cf222af4b63"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1235,7 +1235,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-07. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-08. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1263,14 +1263,12 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:f>COUNTA('Open Items'!$A$6:$A$45)</x:f>
         <x:v>40</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:f>COUNTIFS('Open Items'!$E$6:$E$45,"P0",'Open Items'!$F$6:$F$45,"&lt;&gt;Done")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
@@ -1278,7 +1276,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1286,14 +1284,12 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Open")</x:f>
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
       </x:c>
       <x:c r="E7" s="34" t="n">
-        <x:f>COUNTIF('Release Gates'!$E$6:$E$17,"Open")</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="G7" s="39" t="str">
@@ -1309,14 +1305,12 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:f>COUNTIF(Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
@@ -1332,14 +1326,12 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"PR Open")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
       </x:c>
       <x:c r="E9" s="34" t="n">
-        <x:f>COUNTIFS(Risks!$E$6:$E$19,"P0",Risks!$H$6:$H$19,"Open")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="G9" s="39" t="str">
@@ -1355,14 +1347,12 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Blocked")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
       </x:c>
       <x:c r="E10" s="34" t="n">
-        <x:f>COUNTIF(Requirements!$G$6:$G$27,"Approved")</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="G10" s="39" t="str">
@@ -1370,7 +1360,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1378,8 +1368,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:f>COUNTIF('Open Items'!$F$6:$F$45,"Done")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1478,7 +1467,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R166b4b840f3a40db"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46b1915236554385"/>
 </x:worksheet>
 </file>
 
@@ -1926,28 +1915,28 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="27" t="str">
+      <x:c r="A21" s="26" t="str">
         <x:v>DOC-016</x:v>
       </x:c>
-      <x:c r="B21" s="27" t="str">
+      <x:c r="B21" s="26" t="str">
         <x:v>Dependency remediation record</x:v>
       </x:c>
-      <x:c r="C21" s="27" t="str">
+      <x:c r="C21" s="26" t="str">
         <x:v>docs/security/dependency-remediation-2026-10-04.md</x:v>
       </x:c>
-      <x:c r="D21" s="27" t="str">
+      <x:c r="D21" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="E21" s="27" t="str">
+      <x:c r="E21" s="26" t="str">
         <x:v>Approved candidate</x:v>
       </x:c>
-      <x:c r="F21" s="27" t="str">
+      <x:c r="F21" s="26" t="str">
         <x:v>Each dependency change</x:v>
       </x:c>
-      <x:c r="G21" s="27" t="str">
+      <x:c r="G21" s="26" t="str">
         <x:v>2026-10-05</x:v>
       </x:c>
-      <x:c r="H21" s="27" t="str">
+      <x:c r="H21" s="26" t="str">
         <x:v>DEP-001</x:v>
       </x:c>
     </x:row>
@@ -1964,7 +1953,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0513c2cd3546436e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3366dffb46c34d8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3120,24 +3109,26 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F33" s="26" t="str">
-        <x:v>Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G33" s="26" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H33" s="26" t="str"/>
       <x:c r="I33" s="26" t="str">
-        <x:v>Legacy two failures are updated to current accessible contracts and pass</x:v>
+        <x:v>Live registration supplies every required field; visual audit ignores captionless accessible wrappers; matching exposes its accessible journey region; protected and live suites pass</x:v>
       </x:c>
       <x:c r="J33" s="26" t="str">
-        <x:v>QA findings F-002 F-003</x:v>
+        <x:v>QA findings F-002 F-003; WOW-MD PR 59</x:v>
       </x:c>
       <x:c r="K33" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/33</x:v>
       </x:c>
-      <x:c r="L33" s="26" t="str"/>
+      <x:c r="L33" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/99</x:v>
+      </x:c>
       <x:c r="M33" s="29" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-08</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="30" customHeight="1">
@@ -3584,43 +3575,43 @@
       </x:c>
     </x:row>
     <x:row r="45" ht="30" customHeight="1">
-      <x:c r="A45" s="27" t="str">
+      <x:c r="A45" s="26" t="str">
         <x:v>SYNC-005</x:v>
       </x:c>
-      <x:c r="B45" s="27" t="str">
+      <x:c r="B45" s="26" t="str">
         <x:v>Mirror reviewed biodata caste family and income changes</x:v>
       </x:c>
-      <x:c r="C45" s="27" t="str">
+      <x:c r="C45" s="26" t="str">
         <x:v>Source intake</x:v>
       </x:c>
-      <x:c r="D45" s="27" t="str">
+      <x:c r="D45" s="26" t="str">
         <x:v>Change intake</x:v>
       </x:c>
-      <x:c r="E45" s="27" t="str">
+      <x:c r="E45" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F45" s="27" t="str">
+      <x:c r="F45" s="26" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G45" s="27" t="str">
+      <x:c r="G45" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="H45" s="27" t="str">
+      <x:c r="H45" s="26" t="str">
         <x:v>SYNC-004</x:v>
       </x:c>
-      <x:c r="I45" s="27" t="str">
+      <x:c r="I45" s="26" t="str">
         <x:v>Production exactly mirrors WOW-MD PR 58 with green protected checks and updated source baseline</x:v>
       </x:c>
-      <x:c r="J45" s="27" t="str">
+      <x:c r="J45" s="26" t="str">
         <x:v>WOW-MD PR 58</x:v>
       </x:c>
-      <x:c r="K45" s="27" t="str">
+      <x:c r="K45" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/96</x:v>
       </x:c>
-      <x:c r="L45" s="27" t="str">
+      <x:c r="L45" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
       </x:c>
-      <x:c r="M45" s="30" t="str">
+      <x:c r="M45" s="29" t="str">
         <x:v>2026-10-07</x:v>
       </x:c>
     </x:row>
@@ -3640,7 +3631,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f3e6fdf777a46bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R702be71bddd74cc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4178,25 +4169,25 @@
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
-      <x:c r="A27" s="27" t="str">
+      <x:c r="A27" s="26" t="str">
         <x:v>REQ-AUTH-004</x:v>
       </x:c>
-      <x:c r="B27" s="27" t="str">
+      <x:c r="B27" s="26" t="str">
         <x:v>Zoho domain DNS sender mailbox SMTP application password and production OAuth callback are configured only at the final deployment gate</x:v>
       </x:c>
-      <x:c r="C27" s="27" t="str">
+      <x:c r="C27" s="26" t="str">
         <x:v>User direction</x:v>
       </x:c>
-      <x:c r="D27" s="27" t="str">
+      <x:c r="D27" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="E27" s="27" t="str">
+      <x:c r="E27" s="26" t="str">
         <x:v>Final release checklist and controlled delivery/SSO evidence</x:v>
       </x:c>
-      <x:c r="F27" s="27" t="str">
+      <x:c r="F27" s="26" t="str">
         <x:v>SEC-001,REL-001</x:v>
       </x:c>
-      <x:c r="G27" s="27" t="str">
+      <x:c r="G27" s="26" t="str">
         <x:v>Approved</x:v>
       </x:c>
     </x:row>
@@ -4216,7 +4207,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab8536c3820746fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c3cf93a1846426e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4324,19 +4315,19 @@
         <x:v>Live UI role navigation</x:v>
       </x:c>
       <x:c r="C8" s="26" t="str">
-        <x:v>105 authenticated screens across 8 roles</x:v>
+        <x:v>Public pages fresh registration and authenticated role journeys across 8 roles</x:v>
       </x:c>
       <x:c r="D8" s="26" t="str">
-        <x:v>QA workbook 2026-10-04</x:v>
+        <x:v>Source live run 37687163848 and production live run 37687169181</x:v>
       </x:c>
       <x:c r="E8" s="26" t="str">
-        <x:v>16 of 18 legacy tests plus replacement flows</x:v>
+        <x:v>25 of 25 passed in both repositories</x:v>
       </x:c>
       <x:c r="F8" s="26" t="str">
-        <x:v>Current locator suite green</x:v>
+        <x:v>Repeat on Railway candidate</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>QA-004</x:v>
+        <x:v>QA-004 REL-001</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -4511,13 +4502,13 @@
         <x:v>Private-source report and shared-code mirror gate</x:v>
       </x:c>
       <x:c r="D16" s="26" t="str">
-        <x:v>PR 55 local evidence</x:v>
+        <x:v>Production source-sync run 37687173815</x:v>
       </x:c>
       <x:c r="E16" s="26" t="str">
-        <x:v>19 of 19 governance and synchronization tests passed</x:v>
+        <x:v>19 of 19 governance tests passed and scheduled review reported zero unreviewed commits or paths</x:v>
       </x:c>
       <x:c r="F16" s="26" t="str">
-        <x:v>Configure WOW_SYNC_TOKEN and capture first scheduled artifact</x:v>
+        <x:v>Replace the temporary broad token with a fine-grained WOW-MD Contents read-only token before private visibility</x:v>
       </x:c>
       <x:c r="G16" s="26" t="str">
         <x:v>SYNC-002</x:v>
@@ -4593,25 +4584,25 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
-      <x:c r="A20" s="27" t="str">
+      <x:c r="A20" s="26" t="str">
         <x:v>QA-OBS-001</x:v>
       </x:c>
-      <x:c r="B20" s="27" t="str">
+      <x:c r="B20" s="26" t="str">
         <x:v>Observability</x:v>
       </x:c>
-      <x:c r="C20" s="27" t="str">
+      <x:c r="C20" s="26" t="str">
         <x:v>Request correlation redaction provider logs QA capture audit failures payout sweep and nginx JSON</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="str">
+      <x:c r="D20" s="26" t="str">
         <x:v>OBS-001 PR 69 and merged WOW-MD PR 43</x:v>
       </x:c>
-      <x:c r="E20" s="27" t="str">
+      <x:c r="E20" s="26" t="str">
         <x:v>Focused observability and replica-lock integration 27 of 27; typecheck lint and nginx contract passed; protected CI recorded on PR 69</x:v>
       </x:c>
-      <x:c r="F20" s="27" t="str">
+      <x:c r="F20" s="26" t="str">
         <x:v>Verify live response/log correlation with capture disabled</x:v>
       </x:c>
-      <x:c r="G20" s="27" t="str">
+      <x:c r="G20" s="26" t="str">
         <x:v>OBS-001</x:v>
       </x:c>
     </x:row>
@@ -4621,7 +4612,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d32c82550c94c0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39cc8316a26a49a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5043,31 +5034,31 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="27" t="str">
+      <x:c r="A19" s="26" t="str">
         <x:v>RISK-014</x:v>
       </x:c>
-      <x:c r="B19" s="27" t="str">
+      <x:c r="B19" s="26" t="str">
         <x:v>Framework and mobile build-tool dependency advisories remain after runtime remediation</x:v>
       </x:c>
-      <x:c r="C19" s="27" t="str">
+      <x:c r="C19" s="26" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="D19" s="27" t="str">
+      <x:c r="D19" s="26" t="str">
         <x:v>Possible</x:v>
       </x:c>
-      <x:c r="E19" s="27" t="str">
+      <x:c r="E19" s="26" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="F19" s="27" t="str">
+      <x:c r="F19" s="26" t="str">
         <x:v>Block new critical/high runtime advisories; allow only four exact no-fix Expo advisory IDs; schedule Nest major migration and review exceptions each release</x:v>
       </x:c>
-      <x:c r="G19" s="27" t="str">
+      <x:c r="G19" s="26" t="str">
         <x:v>Security</x:v>
       </x:c>
-      <x:c r="H19" s="27" t="str">
+      <x:c r="H19" s="26" t="str">
         <x:v>Mitigated</x:v>
       </x:c>
-      <x:c r="I19" s="27" t="str">
+      <x:c r="I19" s="26" t="str">
         <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
       </x:c>
     </x:row>
@@ -5087,7 +5078,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra463f7274f494934"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd50c21949af14669"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5395,30 +5386,32 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="27" t="str">
+      <x:c r="A15" s="26" t="str">
         <x:v>ACC-010</x:v>
       </x:c>
-      <x:c r="B15" s="27" t="str">
+      <x:c r="B15" s="26" t="str">
         <x:v>WOW-MD source review</x:v>
       </x:c>
-      <x:c r="C15" s="27" t="str">
+      <x:c r="C15" s="26" t="str">
         <x:v>Repository contents read for scheduled change reports</x:v>
       </x:c>
-      <x:c r="D15" s="27" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>RohithTadiparti</x:v>
       </x:c>
-      <x:c r="E15" s="27" t="str">
-        <x:v>Fine-grained WOW_SYNC_TOKEN</x:v>
-      </x:c>
-      <x:c r="F15" s="27" t="str">
+      <x:c r="E15" s="26" t="str">
+        <x:v>Temporary classic token in WOW_SYNC_TOKEN; replace with fine-grained token</x:v>
+      </x:c>
+      <x:c r="F15" s="26" t="str">
         <x:v>Production GitHub Actions secret</x:v>
       </x:c>
-      <x:c r="G15" s="27" t="str">
-        <x:v>Deferred</x:v>
-      </x:c>
-      <x:c r="H15" s="30" t="str"/>
-      <x:c r="I15" s="27" t="str">
-        <x:v>Not technically required while WOW-MD is public; create before returning it private so the private-ready workflow keeps working; scope only to WOW-MD Contents read and rotate within 90 days</x:v>
+      <x:c r="G15" s="26" t="str">
+        <x:v>Available - replacement required</x:v>
+      </x:c>
+      <x:c r="H15" s="29" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="I15" s="26" t="str">
+        <x:v>Scheduled run 37687173815 passed. Replace the current broad repo/workflow token before private visibility with a token scoped only to WOW-MD Contents read; rotate within 90 days</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5434,7 +5427,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3164d69313c44951"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc29fd53ae2814446"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5739,26 +5732,26 @@
       <x:c r="H16" s="29" t="str"/>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>GATE-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>Railway decommission</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>Production</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>72-hour stable AWS operation and separate approval</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Product owner</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str"/>
-      <x:c r="H17" s="30" t="str"/>
+      <x:c r="G17" s="26" t="str"/>
+      <x:c r="H17" s="29" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5773,7 +5766,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R246b9993dde94e97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc13916f88b4f429b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6221,38 +6214,73 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="A17" s="27" t="str">
+      <x:c r="A17" s="26" t="str">
         <x:v>CHG-012</x:v>
       </x:c>
-      <x:c r="B17" s="27" t="str">
+      <x:c r="B17" s="26" t="str">
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
-      <x:c r="C17" s="27" t="str">
+      <x:c r="C17" s="26" t="str">
         <x:v>442111a36f5e93703b27fbd7859c89a1f34b1547</x:v>
       </x:c>
-      <x:c r="D17" s="27" t="str">
+      <x:c r="D17" s="26" t="str">
         <x:v>backend/src/modules/profile-details/; backend/test/business-entries.e2e-spec.ts; frontend/src/components/; frontend/src/pages/Biodata.tsx</x:v>
       </x:c>
-      <x:c r="E17" s="27" t="str">
+      <x:c r="E17" s="26" t="str">
         <x:v>Biodata and profile flow improvements</x:v>
       </x:c>
-      <x:c r="F17" s="27" t="str">
+      <x:c r="F17" s="26" t="str">
         <x:v>Accepted</x:v>
       </x:c>
-      <x:c r="G17" s="27" t="str">
+      <x:c r="G17" s="26" t="str">
         <x:v>SYNC-005</x:v>
       </x:c>
-      <x:c r="H17" s="27" t="str">
+      <x:c r="H17" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
       </x:c>
-      <x:c r="I17" s="27" t="str">
+      <x:c r="I17" s="26" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="J17" s="30" t="str">
+      <x:c r="J17" s="29" t="str">
         <x:v>2026-10-06</x:v>
       </x:c>
-      <x:c r="K17" s="27" t="str">
+      <x:c r="K17" s="26" t="str">
         <x:v>WOW-MD PR 58; expanded caste handling, parent courtesy titles, positive income validation, saved-biodata behavior and aligned unit/API regression coverage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="26" t="str">
+        <x:v>CHG-013</x:v>
+      </x:c>
+      <x:c r="B18" s="26" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>9f063fd678e88f73768f7a665d02293386180e3e</x:v>
+      </x:c>
+      <x:c r="D18" s="26" t="str">
+        <x:v>frontend/e2e/register.e2e.ts; frontend/e2e/template.ts; frontend/src/pages/Matches.tsx</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="str">
+        <x:v>Live browser journey contract repairs</x:v>
+      </x:c>
+      <x:c r="F18" s="26" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G18" s="26" t="str">
+        <x:v>QA-004</x:v>
+      </x:c>
+      <x:c r="H18" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/99</x:v>
+      </x:c>
+      <x:c r="I18" s="26" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J18" s="29" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K18" s="26" t="str">
+        <x:v>WOW-MD PR 59; supplies the required registration username, bounds response waiting, excludes captionless accessible wrappers from typography checks and restores the accessible matching journey region</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6261,7 +6289,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93704cdc8b514f18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R574846fae2a9486e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7018,41 +7046,79 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="27" t="str">
+      <x:c r="A24" s="26" t="str">
         <x:v>SYNC-005</x:v>
       </x:c>
-      <x:c r="B24" s="27" t="str">
+      <x:c r="B24" s="26" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/97</x:v>
       </x:c>
-      <x:c r="C24" s="27" t="str">
+      <x:c r="C24" s="26" t="str">
         <x:v>codex/sync-005-biodata-flows</x:v>
       </x:c>
-      <x:c r="D24" s="27" t="str">
+      <x:c r="D24" s="26" t="str">
         <x:v>7423193</x:v>
       </x:c>
-      <x:c r="E24" s="27" t="str">
+      <x:c r="E24" s="26" t="str">
         <x:v>c87221f</x:v>
       </x:c>
-      <x:c r="F24" s="27" t="str">
+      <x:c r="F24" s="26" t="str">
         <x:v>WOW-MD PR 58 merged as 442111a</x:v>
       </x:c>
-      <x:c r="G24" s="27" t="str">
+      <x:c r="G24" s="26" t="str">
         <x:v>Source and production protected backend E2E frontend mobile Docker CodeQL secrets and governance checks passed; local backend lint typecheck 839 tests and build plus frontend typecheck 180 tests and build passed</x:v>
       </x:c>
-      <x:c r="H24" s="27" t="str">
+      <x:c r="H24" s="26" t="str">
         <x:v>Rebuild backend and frontend images then smoke health and biodata/profile entry points</x:v>
       </x:c>
-      <x:c r="I24" s="27" t="str">
+      <x:c r="I24" s="26" t="str">
         <x:v>Revert PR 97 and rebuild the prior images; no schema migration or dependency rollback</x:v>
       </x:c>
-      <x:c r="J24" s="27" t="str">
+      <x:c r="J24" s="26" t="str">
         <x:v>Legacy zero-valued stored business income remains readable but new submissions require a positive whole-rupee amount</x:v>
       </x:c>
-      <x:c r="K24" s="27" t="str">
+      <x:c r="K24" s="26" t="str">
         <x:v>Merged</x:v>
       </x:c>
-      <x:c r="L24" s="30" t="str">
+      <x:c r="L24" s="29" t="str">
         <x:v>2026-10-07</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="26" t="str">
+        <x:v>QA-004</x:v>
+      </x:c>
+      <x:c r="B25" s="26" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/99</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>codex/qa-004-live-e2e-contracts</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>ff075ae</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>721ebb8</x:v>
+      </x:c>
+      <x:c r="F25" s="26" t="str">
+        <x:v>WOW-MD PR 59 merged as 9f063fd</x:v>
+      </x:c>
+      <x:c r="G25" s="26" t="str">
+        <x:v>Source and production protected frontend backend E2E mobile Docker CodeQL secrets and governance checks passed; local frontend typecheck 180 tests and production build passed; source live E2E run 37687163848 and production live E2E run 37687169181 each passed all 25 cases; source-sync review 37687173815 passed with zero unreviewed commits or paths</x:v>
+      </x:c>
+      <x:c r="H25" s="26" t="str">
+        <x:v>Frontend image rebuilt from 9f063fd; container healthy; local and tunneled health returned 200</x:v>
+      </x:c>
+      <x:c r="I25" s="26" t="str">
+        <x:v>Revert PR 99 and rebuild the prior frontend image; no schema migration or dependency rollback</x:v>
+      </x:c>
+      <x:c r="J25" s="26" t="str">
+        <x:v>The live registration test intentionally creates one test account per run; replace the broad temporary WOW_SYNC_TOKEN with a fine-grained read-only token</x:v>
+      </x:c>
+      <x:c r="K25" s="26" t="str">
+        <x:v>Merged</x:v>
+      </x:c>
+      <x:c r="L25" s="29" t="str">
+        <x:v>2026-10-08</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7068,7 +7134,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb39cc6ddc21642c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e095a8681314739"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: register SYNC-007 review handoff
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd9c4e5c35c494e42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rb5d9cc3a35924480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R64913b7d72724915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rb19f3e1db94e49d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R2d1c3d9047af40bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd9f3d2d04bf24ebb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rbc11b291fd1b49cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Ra81b0c9c98aa4b3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rf45c542ff593493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R34168879727c4395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf887eae7825843d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rde0479be8d6e47d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R2606ac3a17bb4bdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R644b80ac41cf4f56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb14878795be2432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1a162cc7a71d4273"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf9db761820d14274"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R29238f9dc2b3437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra2844844b52e415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R0e7caa7a59204695"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -157,7 +162,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="46">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -262,6 +267,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -881,7 +898,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raa726b10897c4a86"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2865f41f068944ee"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -891,8 +908,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:M46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:M47"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -913,7 +930,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -929,7 +946,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -945,7 +962,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -963,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -981,7 +998,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -998,8 +1015,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K23"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1018,8 +1035,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L29"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L30"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1039,7 +1056,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1295,13 +1312,13 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1350,7 +1367,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1358,7 +1375,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1499,7 +1516,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dceb6e148a24d7e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21f5cee6ea7e4fad"/>
 </x:worksheet>
 </file>
 
@@ -1531,28 +1548,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2037,7 +2054,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d51db7c620b47c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d84625d62fd4cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2075,43 +2092,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="45" t="str">
+      <x:c r="J5" s="49" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="45" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="45" t="str">
+      <x:c r="L5" s="49" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="45" t="str">
+      <x:c r="M5" s="49" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3743,6 +3760,47 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/102</x:v>
       </x:c>
       <x:c r="M46" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="41" t="str">
+        <x:v>SYNC-007</x:v>
+      </x:c>
+      <x:c r="B47" s="41" t="str">
+        <x:v>Mirror reviewed live E2E defect remediation</x:v>
+      </x:c>
+      <x:c r="C47" s="41" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D47" s="41" t="str">
+        <x:v>Change intake</x:v>
+      </x:c>
+      <x:c r="E47" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F47" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G47" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H47" s="41" t="str">
+        <x:v>SYNC-006</x:v>
+      </x:c>
+      <x:c r="I47" s="41" t="str">
+        <x:v>Production mirrors WOW-MD PR 63 without replacing production-only hardening; protected checks and migration validation pass</x:v>
+      </x:c>
+      <x:c r="J47" s="41" t="str">
+        <x:v>WOW-MD PR 63 merged as 2bd8eaa; irreversible family-interest cleanup is documented</x:v>
+      </x:c>
+      <x:c r="K47" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/108</x:v>
+      </x:c>
+      <x:c r="L47" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/109</x:v>
+      </x:c>
+      <x:c r="M47" s="41" t="str">
         <x:v>2026-10-08</x:v>
       </x:c>
     </x:row>
@@ -3762,7 +3820,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5c264fa805742d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbfb7944a5ba4226"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3794,25 +3852,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4338,7 +4396,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0269733e584457a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb04ae9c602bf4c0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4370,25 +4428,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4789,7 +4847,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7686d8d300f3492f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2040d7bbdd704d46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4823,31 +4881,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5257,7 +5315,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0142f19f19e413c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07e5ba2fa09b4cd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5291,31 +5349,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5606,7 +5664,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b77204f7d94e74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb077a0dfd7ca42c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5639,28 +5697,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -5947,7 +6005,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04602aeb9f4349fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39926d9352054253"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5983,37 +6041,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="45" t="str">
+      <x:c r="J5" s="49" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="45" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6497,6 +6555,146 @@
       </x:c>
       <x:c r="K19" s="41" t="str">
         <x:v>WOW-MD PR 60; reconciles navigation, upload error handling, global call signaling, biodata progression, location formatting and family-account stewardship boundaries</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="41" t="str">
+        <x:v>CHG-015</x:v>
+      </x:c>
+      <x:c r="B20" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C20" s="41" t="str">
+        <x:v>d96e0657424d7cf5b03bc9be00cf1b6a178c578a</x:v>
+      </x:c>
+      <x:c r="D20" s="41" t="str">
+        <x:v>railway/; .github/workflows/railway-deploy.yml; docker/Dockerfile.frontend; frontend/nginx.conf; frontend/e2e/railway-smoke.e2e.ts</x:v>
+      </x:c>
+      <x:c r="E20" s="41" t="str">
+        <x:v>Railway deployment contract</x:v>
+      </x:c>
+      <x:c r="F20" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G20" s="41" t="str">
+        <x:v>RLY-001</x:v>
+      </x:c>
+      <x:c r="H20" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/103</x:v>
+      </x:c>
+      <x:c r="I20" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J20" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K20" s="41" t="str">
+        <x:v>WOW-MD PR 61; accepted four-service Railway Hobby deployment contract and smoke workflow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="41" t="str">
+        <x:v>CHG-016</x:v>
+      </x:c>
+      <x:c r="B21" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C21" s="41" t="str">
+        <x:v>dd2e05c964a2eee337f37b614cd5ad6f485796c7</x:v>
+      </x:c>
+      <x:c r="D21" s="41" t="str">
+        <x:v>backend storage ceiling; terraform/bootstrap/; scripts/storage/; docs/runbooks/s3-media.md</x:v>
+      </x:c>
+      <x:c r="E21" s="41" t="str">
+        <x:v>Private media bootstrap and guardrails</x:v>
+      </x:c>
+      <x:c r="F21" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G21" s="41" t="str">
+        <x:v>S3-001</x:v>
+      </x:c>
+      <x:c r="H21" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/104</x:v>
+      </x:c>
+      <x:c r="I21" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J21" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K21" s="41" t="str">
+        <x:v>WOW-MD PR 62; accepted 10 MiB ceiling, encrypted versioned private S3 bootstrap and reconciliation tooling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="41" t="str">
+        <x:v>CHG-017</x:v>
+      </x:c>
+      <x:c r="B22" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C22" s="41" t="str">
+        <x:v>c9fc8adcf614c89599be43a742a71ee1374d1554</x:v>
+      </x:c>
+      <x:c r="D22" s="41" t="str">
+        <x:v>backend/test/k6/; docs/reports/railway-capacity-baseline.md; scripts/governance/railway-capacity-contract.test.mjs</x:v>
+      </x:c>
+      <x:c r="E22" s="41" t="str">
+        <x:v>Railway capacity test harness</x:v>
+      </x:c>
+      <x:c r="F22" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G22" s="41" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="H22" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/105</x:v>
+      </x:c>
+      <x:c r="I22" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J22" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K22" s="41" t="str">
+        <x:v>WOW-MD PR 64; accepted ramp spike soak and recovery profiles without claiming an unexecuted live capacity result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="41" t="str">
+        <x:v>CHG-018</x:v>
+      </x:c>
+      <x:c r="B23" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C23" s="41" t="str">
+        <x:v>2bd8eaa40013eb694ef44aa103e1b7b89c4d59b3</x:v>
+      </x:c>
+      <x:c r="D23" s="41" t="str">
+        <x:v>backend/; frontend/; mobile/; scripts/; config/platform.yaml; docker/; shared operations and RBAC docs</x:v>
+      </x:c>
+      <x:c r="E23" s="41" t="str">
+        <x:v>Live E2E defect remediation</x:v>
+      </x:c>
+      <x:c r="F23" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G23" s="41" t="str">
+        <x:v>SYNC-007</x:v>
+      </x:c>
+      <x:c r="H23" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/109</x:v>
+      </x:c>
+      <x:c r="I23" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J23" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K23" s="41" t="str">
+        <x:v>WOW-MD PR 63; reviewed session rotation PII masking media-origin gates matchmaking readiness admin verification boundaries maintenance tools and two migrations</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6505,7 +6703,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00c67d608dff4822"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35d7d22a7c1a4fef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6542,40 +6740,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="45" t="str">
+      <x:c r="J5" s="49" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="45" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="45" t="str">
+      <x:c r="L5" s="49" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7486,6 +7684,44 @@
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L29" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="41" t="str">
+        <x:v>SYNC-007</x:v>
+      </x:c>
+      <x:c r="B30" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/109</x:v>
+      </x:c>
+      <x:c r="C30" s="41" t="str">
+        <x:v>codex/sync-007-live-e2e-fixes</x:v>
+      </x:c>
+      <x:c r="D30" s="41" t="str">
+        <x:v>123cefa</x:v>
+      </x:c>
+      <x:c r="E30" s="41" t="str">
+        <x:v>213e0a9</x:v>
+      </x:c>
+      <x:c r="F30" s="41" t="str">
+        <x:v>WOW-MD PR 63 merged as 2bd8eaa</x:v>
+      </x:c>
+      <x:c r="G30" s="41" t="str">
+        <x:v>Source protected checks passed; production backend lint typecheck 1087 tests frontend typecheck 263 tests build mobile audit typecheck governance 19 of 19 registers 9 of 9 migration order 96 files and configuration boundary 514 files passed</x:v>
+      </x:c>
+      <x:c r="H30" s="41" t="str">
+        <x:v>Back up PostgreSQL; run both maintenance commands dry-run first; deploy backend and migrations before frontend and mobile; rerun live all-role smoke</x:v>
+      </x:c>
+      <x:c r="I30" s="41" t="str">
+        <x:v>Revert application images; the profile-code index is reversible but the family-interest cleanup is intentionally irreversible and must not reopen historical interests</x:v>
+      </x:c>
+      <x:c r="J30" s="41" t="str">
+        <x:v>Live E2E matrix remains to be rerun; external media cleanup requires operator review; confirmed fixed matches involving family-own profiles require support review</x:v>
+      </x:c>
+      <x:c r="K30" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L30" s="41" t="str">
         <x:v>2026-10-08</x:v>
       </x:c>
     </x:row>
@@ -7502,7 +7738,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c137c56676e4a4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcddc5247f25c4019"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
SYNC-007: mirror reviewed live E2E fixes (#109)
* fix: mirror reviewed live e2e remediation

* docs: register SYNC-007 review handoff

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd9c4e5c35c494e42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rb5d9cc3a35924480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R64913b7d72724915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rb19f3e1db94e49d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R2d1c3d9047af40bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rd9f3d2d04bf24ebb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rbc11b291fd1b49cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Ra81b0c9c98aa4b3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rf45c542ff593493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R34168879727c4395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf887eae7825843d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rde0479be8d6e47d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R2606ac3a17bb4bdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R644b80ac41cf4f56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb14878795be2432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1a162cc7a71d4273"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf9db761820d14274"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R29238f9dc2b3437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra2844844b52e415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R0e7caa7a59204695"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -157,7 +162,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="46">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -262,6 +267,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -881,7 +898,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raa726b10897c4a86"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2865f41f068944ee"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -891,8 +908,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:M46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:M47"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -913,7 +930,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -929,7 +946,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -945,7 +962,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -963,7 +980,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -981,7 +998,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -998,8 +1015,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K23"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1018,8 +1035,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L29"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L30"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1039,7 +1056,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1295,13 +1312,13 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1350,7 +1367,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1358,7 +1375,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1499,7 +1516,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dceb6e148a24d7e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21f5cee6ea7e4fad"/>
 </x:worksheet>
 </file>
 
@@ -1531,28 +1548,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2037,7 +2054,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d51db7c620b47c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d84625d62fd4cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2075,43 +2092,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="45" t="str">
+      <x:c r="J5" s="49" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="45" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="45" t="str">
+      <x:c r="L5" s="49" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="45" t="str">
+      <x:c r="M5" s="49" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3743,6 +3760,47 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/102</x:v>
       </x:c>
       <x:c r="M46" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="41" t="str">
+        <x:v>SYNC-007</x:v>
+      </x:c>
+      <x:c r="B47" s="41" t="str">
+        <x:v>Mirror reviewed live E2E defect remediation</x:v>
+      </x:c>
+      <x:c r="C47" s="41" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D47" s="41" t="str">
+        <x:v>Change intake</x:v>
+      </x:c>
+      <x:c r="E47" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F47" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G47" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H47" s="41" t="str">
+        <x:v>SYNC-006</x:v>
+      </x:c>
+      <x:c r="I47" s="41" t="str">
+        <x:v>Production mirrors WOW-MD PR 63 without replacing production-only hardening; protected checks and migration validation pass</x:v>
+      </x:c>
+      <x:c r="J47" s="41" t="str">
+        <x:v>WOW-MD PR 63 merged as 2bd8eaa; irreversible family-interest cleanup is documented</x:v>
+      </x:c>
+      <x:c r="K47" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/108</x:v>
+      </x:c>
+      <x:c r="L47" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/109</x:v>
+      </x:c>
+      <x:c r="M47" s="41" t="str">
         <x:v>2026-10-08</x:v>
       </x:c>
     </x:row>
@@ -3762,7 +3820,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5c264fa805742d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbfb7944a5ba4226"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3794,25 +3852,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4338,7 +4396,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0269733e584457a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb04ae9c602bf4c0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4370,25 +4428,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4789,7 +4847,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7686d8d300f3492f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2040d7bbdd704d46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4823,31 +4881,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5257,7 +5315,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0142f19f19e413c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07e5ba2fa09b4cd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5291,31 +5349,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5606,7 +5664,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b77204f7d94e74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb077a0dfd7ca42c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5639,28 +5697,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -5947,7 +6005,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04602aeb9f4349fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39926d9352054253"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5983,37 +6041,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="45" t="str">
+      <x:c r="J5" s="49" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="45" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6497,6 +6555,146 @@
       </x:c>
       <x:c r="K19" s="41" t="str">
         <x:v>WOW-MD PR 60; reconciles navigation, upload error handling, global call signaling, biodata progression, location formatting and family-account stewardship boundaries</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="41" t="str">
+        <x:v>CHG-015</x:v>
+      </x:c>
+      <x:c r="B20" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C20" s="41" t="str">
+        <x:v>d96e0657424d7cf5b03bc9be00cf1b6a178c578a</x:v>
+      </x:c>
+      <x:c r="D20" s="41" t="str">
+        <x:v>railway/; .github/workflows/railway-deploy.yml; docker/Dockerfile.frontend; frontend/nginx.conf; frontend/e2e/railway-smoke.e2e.ts</x:v>
+      </x:c>
+      <x:c r="E20" s="41" t="str">
+        <x:v>Railway deployment contract</x:v>
+      </x:c>
+      <x:c r="F20" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G20" s="41" t="str">
+        <x:v>RLY-001</x:v>
+      </x:c>
+      <x:c r="H20" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/103</x:v>
+      </x:c>
+      <x:c r="I20" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J20" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K20" s="41" t="str">
+        <x:v>WOW-MD PR 61; accepted four-service Railway Hobby deployment contract and smoke workflow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="41" t="str">
+        <x:v>CHG-016</x:v>
+      </x:c>
+      <x:c r="B21" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C21" s="41" t="str">
+        <x:v>dd2e05c964a2eee337f37b614cd5ad6f485796c7</x:v>
+      </x:c>
+      <x:c r="D21" s="41" t="str">
+        <x:v>backend storage ceiling; terraform/bootstrap/; scripts/storage/; docs/runbooks/s3-media.md</x:v>
+      </x:c>
+      <x:c r="E21" s="41" t="str">
+        <x:v>Private media bootstrap and guardrails</x:v>
+      </x:c>
+      <x:c r="F21" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G21" s="41" t="str">
+        <x:v>S3-001</x:v>
+      </x:c>
+      <x:c r="H21" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/104</x:v>
+      </x:c>
+      <x:c r="I21" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J21" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K21" s="41" t="str">
+        <x:v>WOW-MD PR 62; accepted 10 MiB ceiling, encrypted versioned private S3 bootstrap and reconciliation tooling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="41" t="str">
+        <x:v>CHG-017</x:v>
+      </x:c>
+      <x:c r="B22" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C22" s="41" t="str">
+        <x:v>c9fc8adcf614c89599be43a742a71ee1374d1554</x:v>
+      </x:c>
+      <x:c r="D22" s="41" t="str">
+        <x:v>backend/test/k6/; docs/reports/railway-capacity-baseline.md; scripts/governance/railway-capacity-contract.test.mjs</x:v>
+      </x:c>
+      <x:c r="E22" s="41" t="str">
+        <x:v>Railway capacity test harness</x:v>
+      </x:c>
+      <x:c r="F22" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G22" s="41" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="H22" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/105</x:v>
+      </x:c>
+      <x:c r="I22" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J22" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K22" s="41" t="str">
+        <x:v>WOW-MD PR 64; accepted ramp spike soak and recovery profiles without claiming an unexecuted live capacity result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="41" t="str">
+        <x:v>CHG-018</x:v>
+      </x:c>
+      <x:c r="B23" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C23" s="41" t="str">
+        <x:v>2bd8eaa40013eb694ef44aa103e1b7b89c4d59b3</x:v>
+      </x:c>
+      <x:c r="D23" s="41" t="str">
+        <x:v>backend/; frontend/; mobile/; scripts/; config/platform.yaml; docker/; shared operations and RBAC docs</x:v>
+      </x:c>
+      <x:c r="E23" s="41" t="str">
+        <x:v>Live E2E defect remediation</x:v>
+      </x:c>
+      <x:c r="F23" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G23" s="41" t="str">
+        <x:v>SYNC-007</x:v>
+      </x:c>
+      <x:c r="H23" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/109</x:v>
+      </x:c>
+      <x:c r="I23" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J23" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+      <x:c r="K23" s="41" t="str">
+        <x:v>WOW-MD PR 63; reviewed session rotation PII masking media-origin gates matchmaking readiness admin verification boundaries maintenance tools and two migrations</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6505,7 +6703,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00c67d608dff4822"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35d7d22a7c1a4fef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6542,40 +6740,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="49" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="49" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="49" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="49" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="49" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="49" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="45" t="str">
+      <x:c r="J5" s="49" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="45" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="45" t="str">
+      <x:c r="L5" s="49" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7486,6 +7684,44 @@
         <x:v>Merged</x:v>
       </x:c>
       <x:c r="L29" s="41" t="str">
+        <x:v>2026-10-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="41" t="str">
+        <x:v>SYNC-007</x:v>
+      </x:c>
+      <x:c r="B30" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/109</x:v>
+      </x:c>
+      <x:c r="C30" s="41" t="str">
+        <x:v>codex/sync-007-live-e2e-fixes</x:v>
+      </x:c>
+      <x:c r="D30" s="41" t="str">
+        <x:v>123cefa</x:v>
+      </x:c>
+      <x:c r="E30" s="41" t="str">
+        <x:v>213e0a9</x:v>
+      </x:c>
+      <x:c r="F30" s="41" t="str">
+        <x:v>WOW-MD PR 63 merged as 2bd8eaa</x:v>
+      </x:c>
+      <x:c r="G30" s="41" t="str">
+        <x:v>Source protected checks passed; production backend lint typecheck 1087 tests frontend typecheck 263 tests build mobile audit typecheck governance 19 of 19 registers 9 of 9 migration order 96 files and configuration boundary 514 files passed</x:v>
+      </x:c>
+      <x:c r="H30" s="41" t="str">
+        <x:v>Back up PostgreSQL; run both maintenance commands dry-run first; deploy backend and migrations before frontend and mobile; rerun live all-role smoke</x:v>
+      </x:c>
+      <x:c r="I30" s="41" t="str">
+        <x:v>Revert application images; the profile-code index is reversible but the family-interest cleanup is intentionally irreversible and must not reopen historical interests</x:v>
+      </x:c>
+      <x:c r="J30" s="41" t="str">
+        <x:v>Live E2E matrix remains to be rerun; external media cleanup requires operator review; confirmed fixed matches involving family-own profiles require support review</x:v>
+      </x:c>
+      <x:c r="K30" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L30" s="41" t="str">
         <x:v>2026-10-08</x:v>
       </x:c>
     </x:row>
@@ -7502,7 +7738,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c137c56676e4a4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcddc5247f25c4019"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close SYNC-007 tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf887eae7825843d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rde0479be8d6e47d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R2606ac3a17bb4bdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R644b80ac41cf4f56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb14878795be2432d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1a162cc7a71d4273"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf9db761820d14274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R29238f9dc2b3437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra2844844b52e415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R0e7caa7a59204695"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6e56b5f07d8d4a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R98bfb4ac07f64004"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb97312d6f75c464f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R040e79bcff6148dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Re8150c62f4784f28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R57ae3e8362e24e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rfd992a56a0314ec6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6c744d63506b461c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rdaa38fecef194fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb10cc6f2ee954f4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -162,7 +167,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -279,6 +284,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -898,7 +915,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2865f41f068944ee"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33f7ed370fe048f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -908,7 +925,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M47"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -930,7 +947,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -946,7 +963,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -962,7 +979,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -980,7 +997,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -998,7 +1015,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1015,7 +1032,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:K23"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
@@ -1035,7 +1052,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:L30"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
@@ -1056,7 +1073,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1318,7 +1335,7 @@
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1367,7 +1384,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1375,7 +1392,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1409,7 +1426,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1417,7 +1434,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1516,7 +1533,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21f5cee6ea7e4fad"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re750c8b8437c4db7"/>
 </x:worksheet>
 </file>
 
@@ -1548,28 +1565,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2054,7 +2071,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d84625d62fd4cd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32bcd9a369054268"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2092,43 +2109,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="49" t="str">
+      <x:c r="J5" s="53" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="49" t="str">
+      <x:c r="K5" s="53" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="49" t="str">
+      <x:c r="L5" s="53" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="49" t="str">
+      <x:c r="M5" s="53" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3780,7 +3797,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F47" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G47" s="41" t="str">
         <x:v>Codex</x:v>
@@ -3792,7 +3809,7 @@
         <x:v>Production mirrors WOW-MD PR 63 without replacing production-only hardening; protected checks and migration validation pass</x:v>
       </x:c>
       <x:c r="J47" s="41" t="str">
-        <x:v>WOW-MD PR 63 merged as 2bd8eaa; irreversible family-interest cleanup is documented</x:v>
+        <x:v>WOW-MD PR 63 merged as 2bd8eaa; production PR 109 merged as fdf3f3e after all protected checks passed; irreversible family-interest cleanup is documented</x:v>
       </x:c>
       <x:c r="K47" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/108</x:v>
@@ -3820,7 +3837,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbfb7944a5ba4226"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebe211c52d154a6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3852,25 +3869,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4396,7 +4413,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb04ae9c602bf4c0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R270cdbb4c7824feb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4428,25 +4445,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4847,7 +4864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2040d7bbdd704d46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra91d5514fc0b4611"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4881,31 +4898,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5315,7 +5332,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07e5ba2fa09b4cd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57685158522b41e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5349,31 +5366,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5664,7 +5681,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb077a0dfd7ca42c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79dc3050deee40ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5697,28 +5714,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6005,7 +6022,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39926d9352054253"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c57c6d2ee264a11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6041,37 +6058,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="49" t="str">
+      <x:c r="J5" s="53" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="49" t="str">
+      <x:c r="K5" s="53" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6703,7 +6720,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35d7d22a7c1a4fef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6318755a7df64f89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6740,40 +6757,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="49" t="str">
+      <x:c r="J5" s="53" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="49" t="str">
+      <x:c r="K5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="49" t="str">
+      <x:c r="L5" s="53" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7701,13 +7718,13 @@
         <x:v>123cefa</x:v>
       </x:c>
       <x:c r="E30" s="41" t="str">
-        <x:v>213e0a9</x:v>
+        <x:v>2505651</x:v>
       </x:c>
       <x:c r="F30" s="41" t="str">
         <x:v>WOW-MD PR 63 merged as 2bd8eaa</x:v>
       </x:c>
       <x:c r="G30" s="41" t="str">
-        <x:v>Source protected checks passed; production backend lint typecheck 1087 tests frontend typecheck 263 tests build mobile audit typecheck governance 19 of 19 registers 9 of 9 migration order 96 files and configuration boundary 514 files passed</x:v>
+        <x:v>Source protected checks passed; production backend lint typecheck 1087 tests frontend typecheck 263 tests build mobile audit typecheck governance 19 of 19 registers 9 of 9 migration order 96 files and configuration boundary 514 files passed; PR 109 protected CI and Docker image build passed</x:v>
       </x:c>
       <x:c r="H30" s="41" t="str">
         <x:v>Back up PostgreSQL; run both maintenance commands dry-run first; deploy backend and migrations before frontend and mobile; rerun live all-role smoke</x:v>
@@ -7719,7 +7736,7 @@
         <x:v>Live E2E matrix remains to be rerun; external media cleanup requires operator review; confirmed fixed matches involving family-own profiles require support review</x:v>
       </x:c>
       <x:c r="K30" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L30" s="41" t="str">
         <x:v>2026-10-08</x:v>
@@ -7738,7 +7755,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcddc5247f25c4019"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc22975456d554272"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close SYNC-007 tracking (#111)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf887eae7825843d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Rde0479be8d6e47d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R2606ac3a17bb4bdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R644b80ac41cf4f56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb14878795be2432d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R1a162cc7a71d4273"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf9db761820d14274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R29238f9dc2b3437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra2844844b52e415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R0e7caa7a59204695"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6e56b5f07d8d4a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R98bfb4ac07f64004"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb97312d6f75c464f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R040e79bcff6148dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Re8150c62f4784f28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R57ae3e8362e24e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rfd992a56a0314ec6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6c744d63506b461c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rdaa38fecef194fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb10cc6f2ee954f4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -162,7 +167,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -279,6 +284,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -898,7 +915,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2865f41f068944ee"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33f7ed370fe048f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -908,7 +925,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M47"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -930,7 +947,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -946,7 +963,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -962,7 +979,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -980,7 +997,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="32" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -998,7 +1015,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1015,7 +1032,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:K23"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
@@ -1035,7 +1052,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:L30"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
@@ -1056,7 +1073,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1318,7 +1335,7 @@
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1367,7 +1384,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1375,7 +1392,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1409,7 +1426,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1417,7 +1434,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1516,7 +1533,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21f5cee6ea7e4fad"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re750c8b8437c4db7"/>
 </x:worksheet>
 </file>
 
@@ -1548,28 +1565,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2054,7 +2071,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d84625d62fd4cd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32bcd9a369054268"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2092,43 +2109,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="49" t="str">
+      <x:c r="J5" s="53" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="49" t="str">
+      <x:c r="K5" s="53" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="49" t="str">
+      <x:c r="L5" s="53" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="49" t="str">
+      <x:c r="M5" s="53" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3780,7 +3797,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F47" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G47" s="41" t="str">
         <x:v>Codex</x:v>
@@ -3792,7 +3809,7 @@
         <x:v>Production mirrors WOW-MD PR 63 without replacing production-only hardening; protected checks and migration validation pass</x:v>
       </x:c>
       <x:c r="J47" s="41" t="str">
-        <x:v>WOW-MD PR 63 merged as 2bd8eaa; irreversible family-interest cleanup is documented</x:v>
+        <x:v>WOW-MD PR 63 merged as 2bd8eaa; production PR 109 merged as fdf3f3e after all protected checks passed; irreversible family-interest cleanup is documented</x:v>
       </x:c>
       <x:c r="K47" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/108</x:v>
@@ -3820,7 +3837,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbfb7944a5ba4226"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebe211c52d154a6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3852,25 +3869,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4396,7 +4413,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb04ae9c602bf4c0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R270cdbb4c7824feb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4428,25 +4445,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4847,7 +4864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2040d7bbdd704d46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra91d5514fc0b4611"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4881,31 +4898,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5315,7 +5332,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07e5ba2fa09b4cd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57685158522b41e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5349,31 +5366,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5664,7 +5681,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb077a0dfd7ca42c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79dc3050deee40ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5697,28 +5714,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6005,7 +6022,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39926d9352054253"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c57c6d2ee264a11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6041,37 +6058,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="49" t="str">
+      <x:c r="J5" s="53" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="49" t="str">
+      <x:c r="K5" s="53" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6703,7 +6720,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35d7d22a7c1a4fef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6318755a7df64f89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6740,40 +6757,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="53" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="53" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="53" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="53" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="53" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="53" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="53" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="49" t="str">
+      <x:c r="H5" s="53" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="49" t="str">
+      <x:c r="I5" s="53" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="49" t="str">
+      <x:c r="J5" s="53" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="49" t="str">
+      <x:c r="K5" s="53" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="49" t="str">
+      <x:c r="L5" s="53" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7701,13 +7718,13 @@
         <x:v>123cefa</x:v>
       </x:c>
       <x:c r="E30" s="41" t="str">
-        <x:v>213e0a9</x:v>
+        <x:v>2505651</x:v>
       </x:c>
       <x:c r="F30" s="41" t="str">
         <x:v>WOW-MD PR 63 merged as 2bd8eaa</x:v>
       </x:c>
       <x:c r="G30" s="41" t="str">
-        <x:v>Source protected checks passed; production backend lint typecheck 1087 tests frontend typecheck 263 tests build mobile audit typecheck governance 19 of 19 registers 9 of 9 migration order 96 files and configuration boundary 514 files passed</x:v>
+        <x:v>Source protected checks passed; production backend lint typecheck 1087 tests frontend typecheck 263 tests build mobile audit typecheck governance 19 of 19 registers 9 of 9 migration order 96 files and configuration boundary 514 files passed; PR 109 protected CI and Docker image build passed</x:v>
       </x:c>
       <x:c r="H30" s="41" t="str">
         <x:v>Back up PostgreSQL; run both maintenance commands dry-run first; deploy backend and migrations before frontend and mobile; rerun live all-role smoke</x:v>
@@ -7719,7 +7736,7 @@
         <x:v>Live E2E matrix remains to be rerun; external media cleanup requires operator review; confirmed fixed matches involving family-own profiles require support review</x:v>
       </x:c>
       <x:c r="K30" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L30" s="41" t="str">
         <x:v>2026-10-08</x:v>
@@ -7738,7 +7755,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcddc5247f25c4019"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc22975456d554272"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: register OBS-002 pull request
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6e56b5f07d8d4a7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R98bfb4ac07f64004"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb97312d6f75c464f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R040e79bcff6148dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Re8150c62f4784f28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R57ae3e8362e24e52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rfd992a56a0314ec6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6c744d63506b461c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rdaa38fecef194fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb10cc6f2ee954f4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4b63f089cf524947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R26ced0bf5739405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rca7126e8845546b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Racf4f5d051914a3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Ra37c02e643fa4ce0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R240a39bfabd54e49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R9b1516ee4c804224"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R981246c147d74b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rf50d7c4ec23e4d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Re06fb954d6fc4010"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -167,7 +177,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="62">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -296,6 +306,30 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -915,7 +949,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33f7ed370fe048f7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R98ad0f7cfd0647f6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -925,7 +959,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M47"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -947,7 +981,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -963,7 +997,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -979,7 +1013,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -997,7 +1031,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1015,7 +1049,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1032,8 +1066,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K24"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1052,8 +1086,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L31"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1073,7 +1107,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1301,7 +1335,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-08. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-09. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1342,7 +1376,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1350,7 +1384,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1384,7 +1418,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1392,7 +1426,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1533,7 +1567,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re750c8b8437c4db7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c81c0e3942941e0"/>
 </x:worksheet>
 </file>
 
@@ -1565,28 +1599,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="61" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2071,7 +2105,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32bcd9a369054268"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb79d70f459224f34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2109,43 +2143,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="61" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="61" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="53" t="str">
+      <x:c r="J5" s="61" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="53" t="str">
+      <x:c r="K5" s="61" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="53" t="str">
+      <x:c r="L5" s="61" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="53" t="str">
+      <x:c r="M5" s="61" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2404,10 +2438,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F12" s="41" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G12" s="41" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H12" s="41" t="str">
         <x:v>OBS-001</x:v>
@@ -2416,14 +2450,16 @@
         <x:v>Sanitized browser/mobile failures correlate with backend requests</x:v>
       </x:c>
       <x:c r="J12" s="41" t="str">
-        <x:v>client-error-observability plan</x:v>
+        <x:v>client-error-observability plan; WOW-MD PR 65 merged as c3ce5e5</x:v>
       </x:c>
       <x:c r="K12" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/12</x:v>
       </x:c>
-      <x:c r="L12" s="41" t="str"/>
+      <x:c r="L12" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/112</x:v>
+      </x:c>
       <x:c r="M12" s="41" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -3837,7 +3873,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebe211c52d154a6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4700ec39734e492e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3869,25 +3905,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4413,7 +4449,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R270cdbb4c7824feb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc51254b049d8442e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4445,25 +4481,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4864,7 +4900,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra91d5514fc0b4611"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raef5210916e042a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4898,31 +4934,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="61" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="61" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5332,7 +5368,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57685158522b41e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2de6bd9834e24194"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5366,31 +5402,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="61" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="61" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5681,7 +5717,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79dc3050deee40ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7b34230bb0047a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5714,28 +5750,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="61" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6022,7 +6058,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c57c6d2ee264a11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d5fe34652c44ca9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6058,37 +6094,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="61" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="61" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="53" t="str">
+      <x:c r="J5" s="61" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="53" t="str">
+      <x:c r="K5" s="61" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6712,6 +6748,41 @@
       </x:c>
       <x:c r="K23" s="41" t="str">
         <x:v>WOW-MD PR 63; reviewed session rotation PII masking media-origin gates matchmaking readiness admin verification boundaries maintenance tools and two migrations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="41" t="str">
+        <x:v>CHG-019</x:v>
+      </x:c>
+      <x:c r="B24" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C24" s="41" t="str">
+        <x:v>c3ce5e554a5357a042a8187df5547b006afe5c69</x:v>
+      </x:c>
+      <x:c r="D24" s="41" t="str">
+        <x:v>backend client error intake; frontend and mobile error instrumentation</x:v>
+      </x:c>
+      <x:c r="E24" s="41" t="str">
+        <x:v>Sanitized client error observability</x:v>
+      </x:c>
+      <x:c r="F24" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G24" s="41" t="str">
+        <x:v>OBS-002</x:v>
+      </x:c>
+      <x:c r="H24" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/112</x:v>
+      </x:c>
+      <x:c r="I24" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J24" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K24" s="41" t="str">
+        <x:v>WOW-MD PR 65; protected backend frontend mobile Docker and CodeQL checks passed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6720,7 +6791,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6318755a7df64f89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8007ed52cc694b0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6757,40 +6828,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="61" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="61" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="61" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="61" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="61" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="61" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="61" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="61" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="61" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="53" t="str">
+      <x:c r="J5" s="61" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="53" t="str">
+      <x:c r="K5" s="61" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="53" t="str">
+      <x:c r="L5" s="61" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7740,6 +7811,44 @@
       </x:c>
       <x:c r="L30" s="41" t="str">
         <x:v>2026-10-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="41" t="str">
+        <x:v>OBS-002</x:v>
+      </x:c>
+      <x:c r="B31" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/112</x:v>
+      </x:c>
+      <x:c r="C31" s="41" t="str">
+        <x:v>codex/obs-002-client-errors</x:v>
+      </x:c>
+      <x:c r="D31" s="41" t="str">
+        <x:v>962e661</x:v>
+      </x:c>
+      <x:c r="E31" s="41" t="str">
+        <x:v>a78273a</x:v>
+      </x:c>
+      <x:c r="F31" s="41" t="str">
+        <x:v>WOW-MD PR 65 merged as c3ce5e5</x:v>
+      </x:c>
+      <x:c r="G31" s="41" t="str">
+        <x:v>Backend 1091 tests focused client-error E2E 3 frontend 267 mobile 4 lint typecheck builds and source protected CI passed</x:v>
+      </x:c>
+      <x:c r="H31" s="41" t="str">
+        <x:v>Deploy backend before clients; verify a forced browser and mobile failure reaches Loki with the same request ID and no query string or secret</x:v>
+      </x:c>
+      <x:c r="I31" s="41" t="str">
+        <x:v>Revert PR 112 and redeploy previous backend web and mobile builds; no database rollback</x:v>
+      </x:c>
+      <x:c r="J31" s="41" t="str">
+        <x:v>Frontend has no lint script; Expo production advisory exceptions remain tracked by the dependency gate</x:v>
+      </x:c>
+      <x:c r="K31" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L31" s="41" t="str">
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7755,7 +7864,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc22975456d554272"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9e100c2934645ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore: avoid vulnerable mobile test runner
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4b63f089cf524947"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R26ced0bf5739405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rca7126e8845546b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Racf4f5d051914a3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Ra37c02e643fa4ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R240a39bfabd54e49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R9b1516ee4c804224"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R981246c147d74b15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rf50d7c4ec23e4d04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Re06fb954d6fc4010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R32819d8b776c42e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6077accf1df54b78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Ra2e916555b454fa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rfc91663315ed4748"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb2701a45acbb4b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R9f141e375a6f48f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re5e2c08d6a3844f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R29710f4c92454be7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R08cc80592e5d4d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R71e2a5e9dcd74259"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -177,7 +182,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="62">
+  <x:cellXfs count="66">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -330,6 +335,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -949,7 +966,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R98ad0f7cfd0647f6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0a1dfc35f9284c21"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -959,7 +976,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M47"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -981,7 +998,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -997,7 +1014,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1013,7 +1030,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1031,7 +1048,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1049,7 +1066,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1066,7 +1083,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:K24"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
@@ -1086,7 +1103,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="62" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:L31"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
@@ -1107,7 +1124,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="63" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="72" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1567,7 +1584,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c81c0e3942941e0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05103e0bf2bc4d9a"/>
 </x:worksheet>
 </file>
 
@@ -1599,28 +1616,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="61" t="str">
+      <x:c r="H5" s="65" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2105,7 +2122,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb79d70f459224f34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1657957f4cc64502"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2143,43 +2160,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="61" t="str">
+      <x:c r="H5" s="65" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="61" t="str">
+      <x:c r="I5" s="65" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="61" t="str">
+      <x:c r="J5" s="65" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="61" t="str">
+      <x:c r="K5" s="65" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="61" t="str">
+      <x:c r="L5" s="65" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="61" t="str">
+      <x:c r="M5" s="65" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3873,7 +3890,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4700ec39734e492e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591ae5e7fec44212"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3905,25 +3922,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4449,7 +4466,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc51254b049d8442e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17aa52a5240a4823"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4481,25 +4498,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4900,7 +4917,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raef5210916e042a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5820dc5f69e4a3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4934,31 +4951,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="61" t="str">
+      <x:c r="H5" s="65" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="61" t="str">
+      <x:c r="I5" s="65" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5368,7 +5385,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2de6bd9834e24194"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44e4560d5fed4251"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5402,31 +5419,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="61" t="str">
+      <x:c r="H5" s="65" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="61" t="str">
+      <x:c r="I5" s="65" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5717,7 +5734,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7b34230bb0047a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a3e6873534f4dd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5750,28 +5767,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="61" t="str">
+      <x:c r="H5" s="65" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6058,7 +6075,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d5fe34652c44ca9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra97030b69223484e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6094,37 +6111,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="61" t="str">
+      <x:c r="H5" s="65" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="61" t="str">
+      <x:c r="I5" s="65" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="61" t="str">
+      <x:c r="J5" s="65" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="61" t="str">
+      <x:c r="K5" s="65" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6791,7 +6808,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8007ed52cc694b0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b9b0a33b12e4ae2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6828,40 +6845,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="61" t="str">
+      <x:c r="A5" s="65" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="61" t="str">
+      <x:c r="B5" s="65" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="61" t="str">
+      <x:c r="C5" s="65" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="61" t="str">
+      <x:c r="D5" s="65" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="str">
+      <x:c r="E5" s="65" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="str">
+      <x:c r="F5" s="65" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="61" t="str">
+      <x:c r="G5" s="65" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="61" t="str">
+      <x:c r="H5" s="65" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="61" t="str">
+      <x:c r="I5" s="65" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="61" t="str">
+      <x:c r="J5" s="65" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="61" t="str">
+      <x:c r="K5" s="65" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="61" t="str">
+      <x:c r="L5" s="65" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7830,10 +7847,10 @@
         <x:v>a78273a</x:v>
       </x:c>
       <x:c r="F31" s="41" t="str">
-        <x:v>WOW-MD PR 65 merged as c3ce5e5</x:v>
+        <x:v>WOW-MD PR 65 merged as c3ce5e5; follow-up dependency cleanup pending</x:v>
       </x:c>
       <x:c r="G31" s="41" t="str">
-        <x:v>Backend 1091 tests focused client-error E2E 3 frontend 267 mobile 4 lint typecheck builds and source protected CI passed</x:v>
+        <x:v>Backend 1091 tests focused client-error E2E 3 frontend 267 tests builds and mobile typecheck passed; source protected CI passed before test-runner cleanup</x:v>
       </x:c>
       <x:c r="H31" s="41" t="str">
         <x:v>Deploy backend before clients; verify a forced browser and mobile failure reaches Loki with the same request ID and no query string or secret</x:v>
@@ -7842,7 +7859,7 @@
         <x:v>Revert PR 112 and redeploy previous backend web and mobile builds; no database rollback</x:v>
       </x:c>
       <x:c r="J31" s="41" t="str">
-        <x:v>Frontend has no lint script; Expo production advisory exceptions remain tracked by the dependency gate</x:v>
+        <x:v>Frontend has no lint script; no new Jest Expo dependency alerts are accepted</x:v>
       </x:c>
       <x:c r="K31" s="41" t="str">
         <x:v>PR Open</x:v>
@@ -7864,7 +7881,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9e100c2934645ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82c421c8ef97469c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record OBS-002 dependency cleanup
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R32819d8b776c42e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6077accf1df54b78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Ra2e916555b454fa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rfc91663315ed4748"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb2701a45acbb4b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R9f141e375a6f48f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re5e2c08d6a3844f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R29710f4c92454be7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R08cc80592e5d4d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R71e2a5e9dcd74259"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc0252a819dcd416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R7f700be198654753"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R36e26a9e44ec41c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rf7b3691aaa364a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R91a7696f41c54a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R2f2658dca05f44f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rc0a5ec7b6ed24394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rf188b364cca74a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R685bae03cbda4abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R6d300d645e924a12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -182,7 +187,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -347,6 +352,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -966,7 +983,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0a1dfc35f9284c21"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4b4364e324d43c4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -976,7 +993,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="64" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="73" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M47"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -998,7 +1015,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="65" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="74" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1014,7 +1031,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="66" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="75" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1030,7 +1047,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="67" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="76" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1048,7 +1065,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="68" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="77" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1066,7 +1083,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="69" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="78" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1083,7 +1100,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="70" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="79" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:K24"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
@@ -1103,7 +1120,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="71" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="80" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:L31"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
@@ -1124,7 +1141,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="72" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="81" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1584,7 +1601,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05103e0bf2bc4d9a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2caba3ac874fc2"/>
 </x:worksheet>
 </file>
 
@@ -1616,28 +1633,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="65" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2122,7 +2139,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1657957f4cc64502"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafcfe9d924e14a34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2160,43 +2177,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="65" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="65" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="65" t="str">
+      <x:c r="J5" s="69" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="65" t="str">
+      <x:c r="K5" s="69" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="65" t="str">
+      <x:c r="L5" s="69" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="65" t="str">
+      <x:c r="M5" s="69" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2467,7 +2484,7 @@
         <x:v>Sanitized browser/mobile failures correlate with backend requests</x:v>
       </x:c>
       <x:c r="J12" s="41" t="str">
-        <x:v>client-error-observability plan; WOW-MD PR 65 merged as c3ce5e5</x:v>
+        <x:v>client-error-observability plan; WOW-MD PRs 65 and 69 merged as c3ce5e5 and 2c56a49</x:v>
       </x:c>
       <x:c r="K12" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/12</x:v>
@@ -3890,7 +3907,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R591ae5e7fec44212"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9a45b3d4714e91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3922,25 +3939,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4466,7 +4483,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17aa52a5240a4823"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeee5bfa07624a89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4498,25 +4515,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4917,7 +4934,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5820dc5f69e4a3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d74948cc3e4002"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4951,31 +4968,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="65" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="65" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5385,7 +5402,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44e4560d5fed4251"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab74984ac9e48a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5419,31 +5436,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="65" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="65" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5734,7 +5751,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a3e6873534f4dd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2f71c730c4649b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5767,28 +5784,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="65" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6075,7 +6092,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra97030b69223484e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37bc82d8285643f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6111,37 +6128,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="65" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="65" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="65" t="str">
+      <x:c r="J5" s="69" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="65" t="str">
+      <x:c r="K5" s="69" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6775,10 +6792,10 @@
         <x:v>RohithTadiparti/WOW-MD</x:v>
       </x:c>
       <x:c r="C24" s="41" t="str">
-        <x:v>c3ce5e554a5357a042a8187df5547b006afe5c69</x:v>
+        <x:v>c3ce5e554a5357a042a8187df5547b006afe5c69; 2c56a495c8b3dddcb8e558034cdf52fd549fec73</x:v>
       </x:c>
       <x:c r="D24" s="41" t="str">
-        <x:v>backend client error intake; frontend and mobile error instrumentation</x:v>
+        <x:v>backend client error intake; frontend and mobile error instrumentation; mobile test-only dependency cleanup</x:v>
       </x:c>
       <x:c r="E24" s="41" t="str">
         <x:v>Sanitized client error observability</x:v>
@@ -6799,7 +6816,7 @@
         <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="K24" s="41" t="str">
-        <x:v>WOW-MD PR 65; protected backend frontend mobile Docker and CodeQL checks passed</x:v>
+        <x:v>WOW-MD PRs 65 and 69; protected backend frontend mobile Docker and CodeQL checks passed without the rejected Jest Expo chain</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6808,7 +6825,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b9b0a33b12e4ae2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d005c97691e4dd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6845,40 +6862,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="65" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="65" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="65" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="65" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="65" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="65" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="65" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="65" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="65" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="65" t="str">
+      <x:c r="J5" s="69" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="65" t="str">
+      <x:c r="K5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="65" t="str">
+      <x:c r="L5" s="69" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7844,13 +7861,13 @@
         <x:v>962e661</x:v>
       </x:c>
       <x:c r="E31" s="41" t="str">
-        <x:v>a78273a</x:v>
+        <x:v>b37bc2f</x:v>
       </x:c>
       <x:c r="F31" s="41" t="str">
-        <x:v>WOW-MD PR 65 merged as c3ce5e5; follow-up dependency cleanup pending</x:v>
+        <x:v>WOW-MD PR 65 merged as c3ce5e5; cleanup PR 69 merged as 2c56a49</x:v>
       </x:c>
       <x:c r="G31" s="41" t="str">
-        <x:v>Backend 1091 tests focused client-error E2E 3 frontend 267 tests builds and mobile typecheck passed; source protected CI passed before test-runner cleanup</x:v>
+        <x:v>Backend 1091 tests focused client-error E2E 3 frontend 267 tests builds and mobile typecheck passed; both source PRs passed protected backend frontend mobile Docker and CodeQL checks</x:v>
       </x:c>
       <x:c r="H31" s="41" t="str">
         <x:v>Deploy backend before clients; verify a forced browser and mobile failure reaches Loki with the same request ID and no query string or secret</x:v>
@@ -7859,7 +7876,7 @@
         <x:v>Revert PR 112 and redeploy previous backend web and mobile builds; no database rollback</x:v>
       </x:c>
       <x:c r="J31" s="41" t="str">
-        <x:v>Frontend has no lint script; no new Jest Expo dependency alerts are accepted</x:v>
+        <x:v>Frontend has no lint script; no new Jest Expo dependency alerts were accepted</x:v>
       </x:c>
       <x:c r="K31" s="41" t="str">
         <x:v>PR Open</x:v>
@@ -7881,7 +7898,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82c421c8ef97469c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R556b7c5a1a334920"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: track OPS-003 alert delivery PR
Record PR 113, WOW-MD mirror PR 70, test evidence, risk and gate evidence, and regenerate the tracking workbook.
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf7479dbe6891426e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R20a74cb2670545fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R8991c4b587f94d62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R950d147c9d854bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb1d1a810bc724160"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R0983492983184893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R6dc43b77fe4a4e44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rc4f76861903a4ab3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R489a18fd1be348e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rce06ee81a6ff48b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R96f85f96403b41fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Raa5113fb748c4be9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rdac9c11eec704cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R148881b4d2764b3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rd9cc661c767642c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Refeeda49dcb44112"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R02fbcf10decc4d9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R8f18281de7bc47c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rc7c4079e9e754e91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rd5d5c7e5b5f74e8d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -202,7 +207,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="86">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -415,6 +420,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1034,7 +1051,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5e7ebf774a74471"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ea430a0fff3459f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1044,7 +1061,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="100" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="109" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -1066,7 +1083,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="101" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="110" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1082,8 +1099,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="102" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:G22"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="111" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G23"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Layer"/>
@@ -1098,7 +1115,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="103" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="112" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1116,7 +1133,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="104" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="113" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1134,7 +1151,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="105" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="114" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1151,8 +1168,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="106" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K27"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="115" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K28"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1171,8 +1188,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="107" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L34"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="116" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L35"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1192,8 +1209,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="108" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:H23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="117" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:H24"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Document"/>
@@ -1461,7 +1478,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1469,7 +1486,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1545,7 +1562,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1553,7 +1570,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1652,7 +1669,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d7acc17661d445e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e32cc8a45274a1e"/>
 </x:worksheet>
 </file>
 
@@ -1684,28 +1701,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="str">
+      <x:c r="H5" s="85" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2175,6 +2192,32 @@
       </x:c>
       <x:c r="H23" s="41" t="str">
         <x:v>QA-001 GATE-006</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="41" t="str">
+        <x:v>DOC-019</x:v>
+      </x:c>
+      <x:c r="B24" s="41" t="str">
+        <x:v>Platform configuration guide</x:v>
+      </x:c>
+      <x:c r="C24" s="41" t="str">
+        <x:v>docs/operations/platform-configuration.md</x:v>
+      </x:c>
+      <x:c r="D24" s="41" t="str">
+        <x:v>Engineering and operations</x:v>
+      </x:c>
+      <x:c r="E24" s="41" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="F24" s="41" t="str">
+        <x:v>Each configuration change</x:v>
+      </x:c>
+      <x:c r="G24" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="H24" s="41" t="str">
+        <x:v>CFG-001 OPS-003</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2190,7 +2233,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e6608c2ff244cda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab6dbb708c2b472c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2228,43 +2271,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="str">
+      <x:c r="H5" s="85" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="81" t="str">
+      <x:c r="I5" s="85" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="81" t="str">
+      <x:c r="J5" s="85" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="81" t="str">
+      <x:c r="K5" s="85" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="81" t="str">
+      <x:c r="L5" s="85" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="81" t="str">
+      <x:c r="M5" s="85" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2728,7 +2771,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F17" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G17" s="41" t="str">
         <x:v>Codex</x:v>
@@ -2740,7 +2783,7 @@
         <x:v>Exact account DAU request latency error resource database and cost measurements persist</x:v>
       </x:c>
       <x:c r="J17" s="41" t="str">
-        <x:v>WOW-MD PR 74 merged as cf50bb7; production PR 118</x:v>
+        <x:v>WOW-MD PR 74 and production PR 118 merged</x:v>
       </x:c>
       <x:c r="K17" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/17</x:v>
@@ -2769,10 +2812,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F18" s="41" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G18" s="41" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H18" s="41" t="str">
         <x:v>OPS-002</x:v>
@@ -2781,14 +2824,16 @@
         <x:v>Warnings and critical alerts reach portal email audit and logs without flooding</x:v>
       </x:c>
       <x:c r="J18" s="41" t="str">
-        <x:v>Production plan Task 7</x:v>
+        <x:v>WOW-MD PR 70 merged as daae790; production PR 113 rebased on OPS-002</x:v>
       </x:c>
       <x:c r="K18" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/18</x:v>
       </x:c>
-      <x:c r="L18" s="41" t="str"/>
+      <x:c r="L18" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/113</x:v>
+      </x:c>
       <x:c r="M18" s="41" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
@@ -4040,7 +4085,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8299128b7ccc48b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc03dd2b64e9d4f8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4072,25 +4117,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4616,7 +4661,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd43cf042f8074834"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36c1b7a12fb04b01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4648,25 +4693,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -5059,6 +5104,29 @@
       </x:c>
       <x:c r="G22" s="41" t="str">
         <x:v>OBS-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="41" t="str">
+        <x:v>QA-OPS-003</x:v>
+      </x:c>
+      <x:c r="B23" s="41" t="str">
+        <x:v>Operational alert delivery</x:v>
+      </x:c>
+      <x:c r="C23" s="41" t="str">
+        <x:v>Eligible admin fan-out configured-recipient email simulated mock mail deduplication promotion reminder acknowledgement resolution redaction and channel failures</x:v>
+      </x:c>
+      <x:c r="D23" s="41" t="str">
+        <x:v>OPS-003 PR 113 and WOW-MD PR 70</x:v>
+      </x:c>
+      <x:c r="E23" s="41" t="str">
+        <x:v>Focused 112 passed; backend 1149 passed 9 skipped; E2E 71 passed; frontend 273 passed</x:v>
+      </x:c>
+      <x:c r="F23" s="41" t="str">
+        <x:v>Protected CI on the rebased PR; controlled SMTP delivery at the final mail gate; live hourly alert observed on the Railway candidate</x:v>
+      </x:c>
+      <x:c r="G23" s="41" t="str">
+        <x:v>OPS-003</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5067,7 +5135,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09351394130d4266"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b280ce5dc4941d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5101,31 +5169,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="str">
+      <x:c r="H5" s="85" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="81" t="str">
+      <x:c r="I5" s="85" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5372,7 +5440,9 @@
       <x:c r="H14" s="41" t="str">
         <x:v>Open</x:v>
       </x:c>
-      <x:c r="I14" s="41" t="str"/>
+      <x:c r="I14" s="41" t="str">
+        <x:v>OPS-003 PR 113 records log-provider operational mail as simulated and never sent; production provider validation remains in CFG-001 and SEC-001</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="41" t="str">
@@ -5535,7 +5605,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f753e51048f417c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b16ecf4c6642fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5569,31 +5639,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="str">
+      <x:c r="H5" s="85" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="81" t="str">
+      <x:c r="I5" s="85" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5884,7 +5954,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77d866181e114513"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7ad7426f9e4968"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5917,28 +5987,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="str">
+      <x:c r="H5" s="85" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6031,7 +6101,9 @@
       <x:c r="F9" s="41" t="str">
         <x:v>Unassigned</x:v>
       </x:c>
-      <x:c r="G9" s="41" t="str"/>
+      <x:c r="G9" s="41" t="str">
+        <x:v>OPS-003 PR 113 adds deduplicated portal email audit and log operational alerts (stacked on OPS-002); backup restore evidence pending</x:v>
+      </x:c>
       <x:c r="H9" s="41" t="str"/>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -6225,7 +6297,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23b6139cdf044f1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a64f91a9f484a46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6261,37 +6333,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="str">
+      <x:c r="H5" s="85" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="81" t="str">
+      <x:c r="I5" s="85" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="81" t="str">
+      <x:c r="J5" s="85" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="81" t="str">
+      <x:c r="K5" s="85" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -7055,6 +7127,41 @@
       </x:c>
       <x:c r="K27" s="41" t="str">
         <x:v>WOW-MD PR 74; exact measurements, retention, replica lock, sustained/consecutive alert evaluation and telemetry failure isolation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="41" t="str">
+        <x:v>CHG-023</x:v>
+      </x:c>
+      <x:c r="B28" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C28" s="41" t="str">
+        <x:v>daae7902cc8d669b3b73cfeab4d47ae055aac4eb</x:v>
+      </x:c>
+      <x:c r="D28" s="41" t="str">
+        <x:v>backend operations alert delivery notifications mail audit authz and config; frontend notification copy and permission; config/platform.yaml; operations documentation</x:v>
+      </x:c>
+      <x:c r="E28" s="41" t="str">
+        <x:v>Operational alert delivery mirror</x:v>
+      </x:c>
+      <x:c r="F28" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G28" s="41" t="str">
+        <x:v>OPS-003</x:v>
+      </x:c>
+      <x:c r="H28" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/113</x:v>
+      </x:c>
+      <x:c r="I28" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J28" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K28" s="41" t="str">
+        <x:v>WOW-MD PR 70; reviewed deduplication, bounded retries, portal/email/audit/log delivery and redaction</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7063,7 +7170,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd25a199b1e3405e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R799e133a8d0b4838"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7100,40 +7207,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="81" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="81" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="81" t="str">
+      <x:c r="C5" s="85" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="81" t="str">
+      <x:c r="D5" s="85" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="81" t="str">
+      <x:c r="E5" s="85" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="81" t="str">
+      <x:c r="F5" s="85" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="81" t="str">
+      <x:c r="G5" s="85" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="81" t="str">
+      <x:c r="H5" s="85" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="81" t="str">
+      <x:c r="I5" s="85" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="81" t="str">
+      <x:c r="J5" s="85" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="81" t="str">
+      <x:c r="K5" s="85" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="81" t="str">
+      <x:c r="L5" s="85" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8234,6 +8341,44 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L34" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="41" t="str">
+        <x:v>OPS-003</x:v>
+      </x:c>
+      <x:c r="B35" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/113</x:v>
+      </x:c>
+      <x:c r="C35" s="41" t="str">
+        <x:v>claude/ops-003-alert-delivery</x:v>
+      </x:c>
+      <x:c r="D35" s="41" t="str">
+        <x:v>be5b81d</x:v>
+      </x:c>
+      <x:c r="E35" s="41" t="str">
+        <x:v>48d1ce6</x:v>
+      </x:c>
+      <x:c r="F35" s="41" t="str">
+        <x:v>WOW-MD PR 70 merged as daae790</x:v>
+      </x:c>
+      <x:c r="G35" s="41" t="str">
+        <x:v>Focused delivery 31 tests plus lint and typecheck passed; original full backend 1149 passed 9 skipped and frontend 273 passed; protected CI reruns after rebase</x:v>
+      </x:c>
+      <x:c r="H35" s="41" t="str">
+        <x:v>Back up PostgreSQL; deploy backend migration 1710000115000 then frontend; optionally set OPERATIONS_ALERT_RECIPIENTS; mail remains simulated until final mail gate</x:v>
+      </x:c>
+      <x:c r="I35" s="41" t="str">
+        <x:v>Redeploy prior images; keep additive delivery metadata and enum value</x:v>
+      </x:c>
+      <x:c r="J35" s="41" t="str">
+        <x:v>A delivery-state save failure after sending can repeat one send; live SMTP remains unproven until final Zoho mail gate</x:v>
+      </x:c>
+      <x:c r="K35" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L35" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -8250,7 +8395,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc1a895416f453b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ac43d1cf5704643"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: track UI-001 infrastructure dashboard PR
Record PR 114, WOW-MD mirror PR 71 (change intake CHG-021), test evidence and the config-boundary CI risk, and regenerate the tracking workbook.
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -816,7 +816,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -892,7 +892,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -931,7 +931,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -954,7 +954,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -1044,8 +1044,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A5:G23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A5:G24"/>
   <tableColumns count="7">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Layer"/>
@@ -1060,8 +1060,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A5:I19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RisksTable" displayName="RisksTable" ref="A5:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A5:I20"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Risk"/>
@@ -1113,8 +1113,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A5:K24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A5:K25"/>
   <tableColumns count="11">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="SourceRepository"/>
@@ -1133,8 +1133,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A5:L31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A5:L32"/>
   <tableColumns count="12">
     <tableColumn id="1" name="WorkItem"/>
     <tableColumn id="2" name="PR"/>
@@ -1458,7 +1458,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="E8" s="54" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G8" s="39" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="B9" s="54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="33" t="inlineStr">
         <is>
@@ -3590,12 +3590,12 @@
       </c>
       <c r="F19" s="41" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>PR Open</t>
         </is>
       </c>
       <c r="G19" s="41" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="H19" s="41" t="inlineStr">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="J19" s="41" t="inlineStr">
         <is>
-          <t>Production plan Task 8</t>
+          <t>Production plan Task 8; WOW-MD mirror PR 71; stacked on OPS-003 PR 113 and unmerged OPS-002 commit 8dc3412; merge only after OPS-003</t>
         </is>
       </c>
       <c r="K19" s="41" t="inlineStr">
@@ -3618,10 +3618,14 @@
           <t>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/19</t>
         </is>
       </c>
-      <c r="L19" s="41" t="n"/>
+      <c r="L19" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</t>
+        </is>
+      </c>
       <c r="M19" s="41" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G23"/>
+  <dimension ref="A2:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7092,6 +7096,43 @@
       <c r="G23" s="41" t="inlineStr">
         <is>
           <t>OPS-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>QA-UI-001</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="inlineStr">
+        <is>
+          <t>Administrator Infrastructure dashboard</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>Permission matrix guards exact persisted values and units stale missing and placeholder metrics as unknown alert ordering idempotent acknowledgement redacted delivery state disabled migration readiness and all UI states</t>
+        </is>
+      </c>
+      <c r="D24" s="41" t="inlineStr">
+        <is>
+          <t>UI-001 PR 114 and WOW-MD PR 71</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>Backend 1219 passed 9 skipped; E2E 79 passed; frontend 296 passed; Playwright 4 passed</t>
+        </is>
+      </c>
+      <c r="F24" s="41" t="inlineStr">
+        <is>
+          <t>Protected CI on the rebased PR; admin walk on the Railway candidate with live hourly snapshots</t>
+        </is>
+      </c>
+      <c r="G24" s="41" t="inlineStr">
+        <is>
+          <t>UI-001</t>
         </is>
       </c>
     </row>
@@ -7113,7 +7154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:I19"/>
+  <dimension ref="A2:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7818,14 +7859,61 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>RISK-015</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>The CI configuration-boundary check runs from backend/ where it scans zero files so new direct process.env reads could pass CI</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D20" s="41" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F20" s="41" t="inlineStr">
+        <is>
+          <t>Run scripts/verify-config-boundary.mjs from the repository root in CI and assert a non-zero scanned-file count</t>
+        </is>
+      </c>
+      <c r="G20" s="41" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H20" s="41" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I20" s="41" t="inlineStr">
+        <is>
+          <t>Found during UI-001 PR 114 verification: 0 files from backend/ and 582 files from the repository root</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A3:I3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:E19">
+  <conditionalFormatting sqref="E6:E20">
     <cfRule type="containsText" priority="1" operator="containsText" dxfId="0" text="P0"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H6:H19">
+  <conditionalFormatting sqref="H6:H20">
     <cfRule type="containsText" priority="2" operator="containsText" dxfId="1" text="Open"/>
     <cfRule type="containsText" priority="3" operator="containsText" dxfId="2" text="In Progress"/>
     <cfRule type="containsText" priority="4" operator="containsText" dxfId="0" text="Blocked"/>
@@ -8902,7 +8990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K24"/>
+  <dimension ref="A2:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10053,6 +10141,63 @@
       <c r="K24" s="41" t="inlineStr">
         <is>
           <t>WOW-MD PR 70 is stacked on the OPS-002 source mirror 4092a52; same patch-id as production 48d1ce6; accept only after OPS-002 merges in both repositories</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>CHG-021</t>
+        </is>
+      </c>
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t>RohithTadiparti/WOW-MD</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>08d1b63</t>
+        </is>
+      </c>
+      <c r="D25" s="41" t="inlineStr">
+        <is>
+          <t>backend/src/modules/operations/ (controller dashboard service dto redaction module capacity types); backend/src/common/authz/permissions.ts; backend/test/operations-dashboard.e2e-spec.ts; frontend/src/pages/admin/; frontend/src/components/admin/infrastructure/; frontend/src/lib/; frontend/src/App.tsx; frontend/e2e/admin-infrastructure.e2e.ts</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="inlineStr">
+        <is>
+          <t>Administrator Infrastructure dashboard mirror</t>
+        </is>
+      </c>
+      <c r="F25" s="41" t="inlineStr">
+        <is>
+          <t>Pending review</t>
+        </is>
+      </c>
+      <c r="G25" s="41" t="inlineStr">
+        <is>
+          <t>UI-001</t>
+        </is>
+      </c>
+      <c r="H25" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</t>
+        </is>
+      </c>
+      <c r="I25" s="41" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="J25" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="K25" s="41" t="inlineStr">
+        <is>
+          <t>WOW-MD PR 71 is stacked on OPS-003 PR 70; same patch-id as production c04cde9; accept only after OPS-003 merges in both repositories</t>
         </is>
       </c>
     </row>
@@ -10074,7 +10219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L31"/>
+  <dimension ref="A2:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11775,11 +11920,73 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>UI-001</t>
+        </is>
+      </c>
+      <c r="B32" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</t>
+        </is>
+      </c>
+      <c r="C32" s="41" t="inlineStr">
+        <is>
+          <t>claude/ui-001-infrastructure-dashboard</t>
+        </is>
+      </c>
+      <c r="D32" s="41" t="inlineStr">
+        <is>
+          <t>19d93e9</t>
+        </is>
+      </c>
+      <c r="E32" s="41" t="inlineStr">
+        <is>
+          <t>c04cde9</t>
+        </is>
+      </c>
+      <c r="F32" s="41" t="inlineStr">
+        <is>
+          <t>WOW-MD PR 71 head 08d1b63 (stacked on OPS-003 PR 70)</t>
+        </is>
+      </c>
+      <c r="G32" s="41" t="inlineStr">
+        <is>
+          <t>Backend focused 126 passed; backend 1219 passed 9 skipped; lint typecheck build pass; production audits no high or critical; migration order 98 files and config boundary 582 files OK; backend E2E 10 suites 79 passed; frontend typecheck 296 tests build pass; Playwright 4 passed including non-admin refusal and 390px</t>
+        </is>
+      </c>
+      <c r="H32" s="41" t="inlineStr">
+        <is>
+          <t>After OPS-003: deploy backend then frontend; no migration or configuration change</t>
+        </is>
+      </c>
+      <c r="I32" s="41" t="inlineStr">
+        <is>
+          <t>Redeploy previous images; acknowledgement fields are ignored by the previous release</t>
+        </is>
+      </c>
+      <c r="J32" s="41" t="inlineStr">
+        <is>
+          <t>Stacked on OPS-003 and unmerged OPS-002 so rebase and workbook regeneration are required before merge; acknowledgement shows actor id not name; AUTH-001 MIG-001 and GATE-009 to 011 prerequisites are hard-coded unmet until those items land; revenue unknown until a net revenue source exists</t>
+        </is>
+      </c>
+      <c r="K32" s="41" t="inlineStr">
+        <is>
+          <t>Open - stacked on OPS-003</t>
+        </is>
+      </c>
+      <c r="L32" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A3:L3"/>
   </mergeCells>
-  <conditionalFormatting sqref="K6:K31">
+  <conditionalFormatting sqref="K6:K32">
     <cfRule type="containsText" priority="1" operator="containsText" dxfId="1" text="Open"/>
     <cfRule type="containsText" priority="2" operator="containsText" dxfId="2" text="In Progress"/>
     <cfRule type="containsText" priority="3" operator="containsText" dxfId="0" text="Blocked"/>

</xml_diff>

<commit_message>
docs: register SYNC-008 intake and review handoff
Records CHG-019, the SYNC-008 open item and the PR handoff for the
officer QA sheet mirror. The reviewed source baseline stays at 2bd8eaa
because source commits c3ce5e5 and 2c56a49 remain unclassified.
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc0252a819dcd416f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R7f700be198654753"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R36e26a9e44ec41c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rf7b3691aaa364a54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R91a7696f41c54a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R2f2658dca05f44f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rc0a5ec7b6ed24394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rf188b364cca74a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R685bae03cbda4abf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R6d300d645e924a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdadfb1bbefa24d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R53733130a20c450f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Re9518ec89e9e47f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R59c0eb4864ed48ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb0314245f4084619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rc24c988b78fb499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rda5d85a43f49420f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R5ac14ff73955477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re6a6e4efd66c4d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rdf937ed671204371"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -187,7 +192,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="70">
+  <x:cellXfs count="74">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -364,6 +369,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -983,7 +1000,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4b4364e324d43c4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5e35a1a47fe24629"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -993,8 +1010,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="73" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:M47"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="82" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:M48"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1015,7 +1032,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="74" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="83" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1031,7 +1048,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="75" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="84" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1047,7 +1064,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="76" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="85" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1065,7 +1082,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="77" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="86" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1083,7 +1100,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="78" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1100,8 +1117,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="79" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K24"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K25"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1120,8 +1137,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="80" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L31"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="89" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L32"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1141,7 +1158,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="81" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="90" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1397,13 +1414,13 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1452,7 +1469,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1460,7 +1477,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1601,7 +1618,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2caba3ac874fc2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1adc7a65c9df449a"/>
 </x:worksheet>
 </file>
 
@@ -1633,28 +1650,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2139,7 +2156,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafcfe9d924e14a34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22872b2ed3c240b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2177,43 +2194,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="69" t="str">
+      <x:c r="J5" s="73" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="69" t="str">
+      <x:c r="K5" s="73" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="69" t="str">
+      <x:c r="L5" s="73" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="69" t="str">
+      <x:c r="M5" s="73" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3889,6 +3906,47 @@
       </x:c>
       <x:c r="M47" s="41" t="str">
         <x:v>2026-10-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="41" t="str">
+        <x:v>SYNC-008</x:v>
+      </x:c>
+      <x:c r="B48" s="41" t="str">
+        <x:v>Mirror reviewed officer QA sheet fixes</x:v>
+      </x:c>
+      <x:c r="C48" s="41" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D48" s="41" t="str">
+        <x:v>Change intake</x:v>
+      </x:c>
+      <x:c r="E48" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F48" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G48" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H48" s="41" t="str">
+        <x:v>SYNC-007</x:v>
+      </x:c>
+      <x:c r="I48" s="41" t="str">
+        <x:v>Production exactly mirrors WOW-MD PR 73 officer Support scoping settlement-notes phone-sync roster and mobile gate fixes with green local suites and updated source baseline</x:v>
+      </x:c>
+      <x:c r="J48" s="41" t="str">
+        <x:v>WOW-MD PR 73 pending merge</x:v>
+      </x:c>
+      <x:c r="K48" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/115</x:v>
+      </x:c>
+      <x:c r="L48" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/116</x:v>
+      </x:c>
+      <x:c r="M48" s="41" t="str">
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3907,7 +3965,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9a45b3d4714e91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73af2198434e4566"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3939,25 +3997,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4483,7 +4541,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeee5bfa07624a89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f4d36ddbe724a41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4515,25 +4573,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4934,7 +4992,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d74948cc3e4002"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R077d3eb852c846f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4968,31 +5026,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5402,7 +5460,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab74984ac9e48a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb0c7c7dd4ef4e7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5436,31 +5494,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5751,7 +5809,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2f71c730c4649b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15a3b933fd1e414b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5784,28 +5842,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6092,7 +6150,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37bc82d8285643f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b9b04e4df7543f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6128,37 +6186,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="69" t="str">
+      <x:c r="J5" s="73" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="69" t="str">
+      <x:c r="K5" s="73" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6817,6 +6875,41 @@
       </x:c>
       <x:c r="K24" s="41" t="str">
         <x:v>WOW-MD PRs 65 and 69; protected backend frontend mobile Docker and CodeQL checks passed without the rejected Jest Expo chain</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="41" t="str">
+        <x:v>CHG-020</x:v>
+      </x:c>
+      <x:c r="B25" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C25" s="41" t="str">
+        <x:v>a4a8f18982c242a5611b82a7960dd1bac3db6a0e</x:v>
+      </x:c>
+      <x:c r="D25" s="41" t="str">
+        <x:v>backend/; frontend/; mobile/ (23 reviewed paths)</x:v>
+      </x:c>
+      <x:c r="E25" s="41" t="str">
+        <x:v>Officer QA sheet functional fixes</x:v>
+      </x:c>
+      <x:c r="F25" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G25" s="41" t="str">
+        <x:v>SYNC-008</x:v>
+      </x:c>
+      <x:c r="H25" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/116</x:v>
+      </x:c>
+      <x:c r="I25" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J25" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K25" s="41" t="str">
+        <x:v>WOW-MD PR 73; officer Support scoping mandatory settlement notes planner case context account-phone sync roster not-set display nav dedupe password patterns and mobile set-password gate plus phone verification</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6825,7 +6918,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d005c97691e4dd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c299564289f41a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6862,40 +6955,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="69" t="str">
+      <x:c r="J5" s="73" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="69" t="str">
+      <x:c r="K5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="69" t="str">
+      <x:c r="L5" s="73" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7882,6 +7975,44 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L31" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="41" t="str">
+        <x:v>SYNC-008</x:v>
+      </x:c>
+      <x:c r="B32" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/116</x:v>
+      </x:c>
+      <x:c r="C32" s="41" t="str">
+        <x:v>codex/sync-008-officer-qa-fixes</x:v>
+      </x:c>
+      <x:c r="D32" s="41" t="str">
+        <x:v>f0373ec</x:v>
+      </x:c>
+      <x:c r="E32" s="41" t="str">
+        <x:v>12afb25</x:v>
+      </x:c>
+      <x:c r="F32" s="41" t="str">
+        <x:v>WOW-MD PR 73 merged as a4a8f18</x:v>
+      </x:c>
+      <x:c r="G32" s="41" t="str">
+        <x:v>Local backend typecheck and 1101 tests frontend typecheck 268 tests and build mobile typecheck all passed; register validation passed; protected CI passed before rebase and will rerun</x:v>
+      </x:c>
+      <x:c r="H32" s="41" t="str">
+        <x:v>Rebuild backend frontend and mobile artifacts from the mirrored commit; no migration or environment change</x:v>
+      </x:c>
+      <x:c r="I32" s="41" t="str">
+        <x:v>Revert PR 116 and redeploy the prior images; no schema or data boundary</x:v>
+      </x:c>
+      <x:c r="J32" s="41" t="str">
+        <x:v>Existing officers with diverged account phones keep the old number until re-saving the profile; live sheet re-run after deployment is tracked separately</x:v>
+      </x:c>
+      <x:c r="K32" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L32" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -7898,7 +8029,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R556b7c5a1a334920"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b2f2c4fa4f84574"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
OBS-002: capture sanitized client failures (#112)
* feat(observability): capture sanitized client errors

* docs: track OBS-002 source intake

* docs: register OBS-002 pull request

* chore: avoid vulnerable mobile test runner

* docs: record OBS-002 dependency cleanup

* ci: refresh OBS-002 governance context

* ci: refresh OBS-002 mirror metadata

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6e56b5f07d8d4a7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R98bfb4ac07f64004"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb97312d6f75c464f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R040e79bcff6148dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Re8150c62f4784f28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R57ae3e8362e24e52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rfd992a56a0314ec6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R6c744d63506b461c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rdaa38fecef194fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb10cc6f2ee954f4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc0252a819dcd416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R7f700be198654753"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R36e26a9e44ec41c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rf7b3691aaa364a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R91a7696f41c54a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R2f2658dca05f44f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rc0a5ec7b6ed24394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rf188b364cca74a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R685bae03cbda4abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R6d300d645e924a12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -167,7 +187,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -296,6 +316,54 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -915,7 +983,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33f7ed370fe048f7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4b4364e324d43c4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -925,7 +993,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="73" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M47"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -947,7 +1015,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="74" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -963,7 +1031,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="75" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -979,7 +1047,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="76" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -997,7 +1065,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="77" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1015,7 +1083,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="78" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1032,8 +1100,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="79" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K24"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1052,8 +1120,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="80" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L31"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1073,7 +1141,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="81" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1301,7 +1369,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-08. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-09. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1342,7 +1410,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1350,7 +1418,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1384,7 +1452,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1392,7 +1460,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1533,7 +1601,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re750c8b8437c4db7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2caba3ac874fc2"/>
 </x:worksheet>
 </file>
 
@@ -1565,28 +1633,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2071,7 +2139,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32bcd9a369054268"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafcfe9d924e14a34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2109,43 +2177,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="53" t="str">
+      <x:c r="J5" s="69" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="53" t="str">
+      <x:c r="K5" s="69" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="53" t="str">
+      <x:c r="L5" s="69" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="53" t="str">
+      <x:c r="M5" s="69" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2404,10 +2472,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F12" s="41" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G12" s="41" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H12" s="41" t="str">
         <x:v>OBS-001</x:v>
@@ -2416,14 +2484,16 @@
         <x:v>Sanitized browser/mobile failures correlate with backend requests</x:v>
       </x:c>
       <x:c r="J12" s="41" t="str">
-        <x:v>client-error-observability plan</x:v>
+        <x:v>client-error-observability plan; WOW-MD PRs 65 and 69 merged as c3ce5e5 and 2c56a49</x:v>
       </x:c>
       <x:c r="K12" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/12</x:v>
       </x:c>
-      <x:c r="L12" s="41" t="str"/>
+      <x:c r="L12" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/112</x:v>
+      </x:c>
       <x:c r="M12" s="41" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -3837,7 +3907,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebe211c52d154a6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9a45b3d4714e91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3869,25 +3939,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4413,7 +4483,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R270cdbb4c7824feb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeee5bfa07624a89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4445,25 +4515,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4864,7 +4934,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra91d5514fc0b4611"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d74948cc3e4002"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4898,31 +4968,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5332,7 +5402,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57685158522b41e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab74984ac9e48a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5366,31 +5436,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5681,7 +5751,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79dc3050deee40ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2f71c730c4649b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5714,28 +5784,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6022,7 +6092,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c57c6d2ee264a11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37bc82d8285643f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6058,37 +6128,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="53" t="str">
+      <x:c r="J5" s="69" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="53" t="str">
+      <x:c r="K5" s="69" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6712,6 +6782,41 @@
       </x:c>
       <x:c r="K23" s="41" t="str">
         <x:v>WOW-MD PR 63; reviewed session rotation PII masking media-origin gates matchmaking readiness admin verification boundaries maintenance tools and two migrations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="41" t="str">
+        <x:v>CHG-019</x:v>
+      </x:c>
+      <x:c r="B24" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C24" s="41" t="str">
+        <x:v>c3ce5e554a5357a042a8187df5547b006afe5c69; 2c56a495c8b3dddcb8e558034cdf52fd549fec73</x:v>
+      </x:c>
+      <x:c r="D24" s="41" t="str">
+        <x:v>backend client error intake; frontend and mobile error instrumentation; mobile test-only dependency cleanup</x:v>
+      </x:c>
+      <x:c r="E24" s="41" t="str">
+        <x:v>Sanitized client error observability</x:v>
+      </x:c>
+      <x:c r="F24" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G24" s="41" t="str">
+        <x:v>OBS-002</x:v>
+      </x:c>
+      <x:c r="H24" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/112</x:v>
+      </x:c>
+      <x:c r="I24" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J24" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K24" s="41" t="str">
+        <x:v>WOW-MD PRs 65 and 69; protected backend frontend mobile Docker and CodeQL checks passed without the rejected Jest Expo chain</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6720,7 +6825,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6318755a7df64f89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d005c97691e4dd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6757,40 +6862,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="69" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="53" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="53" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="53" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="53" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="53" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="53" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="53" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="53" t="str">
+      <x:c r="I5" s="69" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="53" t="str">
+      <x:c r="J5" s="69" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="53" t="str">
+      <x:c r="K5" s="69" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="53" t="str">
+      <x:c r="L5" s="69" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7740,6 +7845,44 @@
       </x:c>
       <x:c r="L30" s="41" t="str">
         <x:v>2026-10-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="41" t="str">
+        <x:v>OBS-002</x:v>
+      </x:c>
+      <x:c r="B31" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/112</x:v>
+      </x:c>
+      <x:c r="C31" s="41" t="str">
+        <x:v>codex/obs-002-client-errors</x:v>
+      </x:c>
+      <x:c r="D31" s="41" t="str">
+        <x:v>962e661</x:v>
+      </x:c>
+      <x:c r="E31" s="41" t="str">
+        <x:v>b37bc2f</x:v>
+      </x:c>
+      <x:c r="F31" s="41" t="str">
+        <x:v>WOW-MD PR 65 merged as c3ce5e5; cleanup PR 69 merged as 2c56a49</x:v>
+      </x:c>
+      <x:c r="G31" s="41" t="str">
+        <x:v>Backend 1091 tests focused client-error E2E 3 frontend 267 tests builds and mobile typecheck passed; both source PRs passed protected backend frontend mobile Docker and CodeQL checks</x:v>
+      </x:c>
+      <x:c r="H31" s="41" t="str">
+        <x:v>Deploy backend before clients; verify a forced browser and mobile failure reaches Loki with the same request ID and no query string or secret</x:v>
+      </x:c>
+      <x:c r="I31" s="41" t="str">
+        <x:v>Revert PR 112 and redeploy previous backend web and mobile builds; no database rollback</x:v>
+      </x:c>
+      <x:c r="J31" s="41" t="str">
+        <x:v>Frontend has no lint script; no new Jest Expo dependency alerts were accepted</x:v>
+      </x:c>
+      <x:c r="K31" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L31" s="41" t="str">
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7755,7 +7898,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc22975456d554272"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R556b7c5a1a334920"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
SYNC-008: mirror reviewed officer QA sheet fixes (#116)
* SYNC-008: mirror reviewed officer QA sheet fixes

Mirrors WOW-MD PR 73 (commit 05724c8): officer Support scoping,
mandatory settlement notes, planner case context, account-phone sync,
roster not-set availability, nav dedupe, password patterns and the
mobile set-password gate plus phone verification.

* docs: register SYNC-008 intake and review handoff

Records CHG-019, the SYNC-008 open item and the PR handoff for the
officer QA sheet mirror. The reviewed source baseline stays at 2bd8eaa
because source commits c3ce5e5 and 2c56a49 remain unclassified.

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc0252a819dcd416f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R7f700be198654753"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R36e26a9e44ec41c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Rf7b3691aaa364a54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R91a7696f41c54a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R2f2658dca05f44f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rc0a5ec7b6ed24394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rf188b364cca74a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R685bae03cbda4abf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R6d300d645e924a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdadfb1bbefa24d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R53733130a20c450f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Re9518ec89e9e47f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R59c0eb4864ed48ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb0314245f4084619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rc24c988b78fb499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rda5d85a43f49420f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R5ac14ff73955477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re6a6e4efd66c4d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rdf937ed671204371"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -187,7 +192,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="70">
+  <x:cellXfs count="74">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -364,6 +369,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -983,7 +1000,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4b4364e324d43c4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5e35a1a47fe24629"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -993,8 +1010,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="73" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:M47"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="82" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:M48"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1015,7 +1032,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="74" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="83" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1031,7 +1048,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="75" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="84" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1047,7 +1064,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="76" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="85" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1065,7 +1082,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="77" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="86" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1083,7 +1100,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="78" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1100,8 +1117,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="79" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K24"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K25"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1120,8 +1137,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="80" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L31"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="89" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L32"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1141,7 +1158,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="81" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="90" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1397,13 +1414,13 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1452,7 +1469,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1460,7 +1477,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1601,7 +1618,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2caba3ac874fc2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1adc7a65c9df449a"/>
 </x:worksheet>
 </file>
 
@@ -1633,28 +1650,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2139,7 +2156,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafcfe9d924e14a34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22872b2ed3c240b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2177,43 +2194,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="69" t="str">
+      <x:c r="J5" s="73" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="69" t="str">
+      <x:c r="K5" s="73" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="69" t="str">
+      <x:c r="L5" s="73" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="69" t="str">
+      <x:c r="M5" s="73" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3889,6 +3906,47 @@
       </x:c>
       <x:c r="M47" s="41" t="str">
         <x:v>2026-10-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="41" t="str">
+        <x:v>SYNC-008</x:v>
+      </x:c>
+      <x:c r="B48" s="41" t="str">
+        <x:v>Mirror reviewed officer QA sheet fixes</x:v>
+      </x:c>
+      <x:c r="C48" s="41" t="str">
+        <x:v>Source intake</x:v>
+      </x:c>
+      <x:c r="D48" s="41" t="str">
+        <x:v>Change intake</x:v>
+      </x:c>
+      <x:c r="E48" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F48" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G48" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H48" s="41" t="str">
+        <x:v>SYNC-007</x:v>
+      </x:c>
+      <x:c r="I48" s="41" t="str">
+        <x:v>Production exactly mirrors WOW-MD PR 73 officer Support scoping settlement-notes phone-sync roster and mobile gate fixes with green local suites and updated source baseline</x:v>
+      </x:c>
+      <x:c r="J48" s="41" t="str">
+        <x:v>WOW-MD PR 73 pending merge</x:v>
+      </x:c>
+      <x:c r="K48" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/115</x:v>
+      </x:c>
+      <x:c r="L48" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/116</x:v>
+      </x:c>
+      <x:c r="M48" s="41" t="str">
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3907,7 +3965,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9a45b3d4714e91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73af2198434e4566"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3939,25 +3997,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4483,7 +4541,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeee5bfa07624a89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f4d36ddbe724a41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4515,25 +4573,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4934,7 +4992,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d74948cc3e4002"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R077d3eb852c846f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4968,31 +5026,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5402,7 +5460,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab74984ac9e48a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb0c7c7dd4ef4e7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5436,31 +5494,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5751,7 +5809,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2f71c730c4649b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15a3b933fd1e414b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5784,28 +5842,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6092,7 +6150,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37bc82d8285643f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b9b04e4df7543f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6128,37 +6186,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="69" t="str">
+      <x:c r="J5" s="73" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="69" t="str">
+      <x:c r="K5" s="73" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6817,6 +6875,41 @@
       </x:c>
       <x:c r="K24" s="41" t="str">
         <x:v>WOW-MD PRs 65 and 69; protected backend frontend mobile Docker and CodeQL checks passed without the rejected Jest Expo chain</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="41" t="str">
+        <x:v>CHG-020</x:v>
+      </x:c>
+      <x:c r="B25" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C25" s="41" t="str">
+        <x:v>a4a8f18982c242a5611b82a7960dd1bac3db6a0e</x:v>
+      </x:c>
+      <x:c r="D25" s="41" t="str">
+        <x:v>backend/; frontend/; mobile/ (23 reviewed paths)</x:v>
+      </x:c>
+      <x:c r="E25" s="41" t="str">
+        <x:v>Officer QA sheet functional fixes</x:v>
+      </x:c>
+      <x:c r="F25" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G25" s="41" t="str">
+        <x:v>SYNC-008</x:v>
+      </x:c>
+      <x:c r="H25" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/116</x:v>
+      </x:c>
+      <x:c r="I25" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J25" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K25" s="41" t="str">
+        <x:v>WOW-MD PR 73; officer Support scoping mandatory settlement notes planner case context account-phone sync roster not-set display nav dedupe password patterns and mobile set-password gate plus phone verification</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6825,7 +6918,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d005c97691e4dd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c299564289f41a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6862,40 +6955,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="69" t="str">
+      <x:c r="A5" s="73" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="69" t="str">
+      <x:c r="B5" s="73" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="69" t="str">
+      <x:c r="C5" s="73" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="69" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="69" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="69" t="str">
+      <x:c r="F5" s="73" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="69" t="str">
+      <x:c r="G5" s="73" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="69" t="str">
+      <x:c r="H5" s="73" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="69" t="str">
+      <x:c r="I5" s="73" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="69" t="str">
+      <x:c r="J5" s="73" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="69" t="str">
+      <x:c r="K5" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="69" t="str">
+      <x:c r="L5" s="73" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -7882,6 +7975,44 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L31" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="41" t="str">
+        <x:v>SYNC-008</x:v>
+      </x:c>
+      <x:c r="B32" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/116</x:v>
+      </x:c>
+      <x:c r="C32" s="41" t="str">
+        <x:v>codex/sync-008-officer-qa-fixes</x:v>
+      </x:c>
+      <x:c r="D32" s="41" t="str">
+        <x:v>f0373ec</x:v>
+      </x:c>
+      <x:c r="E32" s="41" t="str">
+        <x:v>12afb25</x:v>
+      </x:c>
+      <x:c r="F32" s="41" t="str">
+        <x:v>WOW-MD PR 73 merged as a4a8f18</x:v>
+      </x:c>
+      <x:c r="G32" s="41" t="str">
+        <x:v>Local backend typecheck and 1101 tests frontend typecheck 268 tests and build mobile typecheck all passed; register validation passed; protected CI passed before rebase and will rerun</x:v>
+      </x:c>
+      <x:c r="H32" s="41" t="str">
+        <x:v>Rebuild backend frontend and mobile artifacts from the mirrored commit; no migration or environment change</x:v>
+      </x:c>
+      <x:c r="I32" s="41" t="str">
+        <x:v>Revert PR 116 and redeploy the prior images; no schema or data boundary</x:v>
+      </x:c>
+      <x:c r="J32" s="41" t="str">
+        <x:v>Existing officers with diverged account phones keep the old number until re-saving the profile; live sheet re-run after deployment is tracked separately</x:v>
+      </x:c>
+      <x:c r="K32" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L32" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -7898,7 +8029,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R556b7c5a1a334920"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b2f2c4fa4f84574"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: register DEP-005 source mirror
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdadfb1bbefa24d39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R53733130a20c450f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Re9518ec89e9e47f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R59c0eb4864ed48ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb0314245f4084619"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rc24c988b78fb499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rda5d85a43f49420f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R5ac14ff73955477b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re6a6e4efd66c4d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rdf937ed671204371"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c4a89865ef945fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R197417dd42494b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf07063130ae14466"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R540a1bf3a09c4951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R857539a5cea840ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R5b5d770048ff4ef2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R4399d3ff9c544dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re4b398e4c75e4d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R2c16e8ada9464404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7b82584a78964305"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -192,7 +197,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="74">
+  <x:cellXfs count="78">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -381,6 +386,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1000,7 +1017,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5e35a1a47fe24629"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra5cb08d8553646f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1010,8 +1027,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="82" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:M48"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="91" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1032,7 +1049,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="83" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="92" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1048,7 +1065,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="84" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="93" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1064,7 +1081,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="85" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="94" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1082,7 +1099,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="86" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="95" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1100,7 +1117,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="96" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1117,8 +1134,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="97" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K26"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1137,8 +1154,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="89" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L32"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="98" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L33"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1158,7 +1175,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="90" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="99" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1414,13 +1431,13 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1469,7 +1486,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1477,7 +1494,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1618,7 +1635,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1adc7a65c9df449a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2610b6b399634af0"/>
 </x:worksheet>
 </file>
 
@@ -1650,28 +1667,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2156,7 +2173,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22872b2ed3c240b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd00aaa0c67a8425f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2194,43 +2211,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="73" t="str">
+      <x:c r="J5" s="77" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="73" t="str">
+      <x:c r="K5" s="77" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="73" t="str">
+      <x:c r="L5" s="77" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="73" t="str">
+      <x:c r="M5" s="77" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3946,6 +3963,45 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/116</x:v>
       </x:c>
       <x:c r="M48" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="41" t="str">
+        <x:v>DEP-005</x:v>
+      </x:c>
+      <x:c r="B49" s="41" t="str">
+        <x:v>Mirror body-parser and Handlebars security fixes</x:v>
+      </x:c>
+      <x:c r="C49" s="41" t="str">
+        <x:v>Public beta safety</x:v>
+      </x:c>
+      <x:c r="D49" s="41" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E49" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F49" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G49" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H49" s="41" t="str">
+        <x:v>DEP-004</x:v>
+      </x:c>
+      <x:c r="I49" s="41" t="str">
+        <x:v>Production backend lockfile resolves body-parser 1.20.8 and Handlebars 4.7.10 exactly as reviewed in source</x:v>
+      </x:c>
+      <x:c r="J49" s="41" t="str">
+        <x:v>WOW-MD PRs 66 and 67</x:v>
+      </x:c>
+      <x:c r="K49" s="41" t="str"/>
+      <x:c r="L49" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/117</x:v>
+      </x:c>
+      <x:c r="M49" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -3965,7 +4021,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73af2198434e4566"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c8885ce78a64210"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3997,25 +4053,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4541,7 +4597,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f4d36ddbe724a41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R069f0f19c73649dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4573,25 +4629,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4992,7 +5048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R077d3eb852c846f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a80d0a37ac4ceb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5026,31 +5082,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5460,7 +5516,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb0c7c7dd4ef4e7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7d7bf4884ab4be8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5494,31 +5550,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5809,7 +5865,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15a3b933fd1e414b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R809985a19a024a92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5842,28 +5898,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6150,7 +6206,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b9b04e4df7543f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff61da0be1ba4ab7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6186,37 +6242,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="73" t="str">
+      <x:c r="J5" s="77" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="73" t="str">
+      <x:c r="K5" s="77" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6910,6 +6966,41 @@
       </x:c>
       <x:c r="K25" s="41" t="str">
         <x:v>WOW-MD PR 73; officer Support scoping mandatory settlement notes planner case context account-phone sync roster not-set display nav dedupe password patterns and mobile set-password gate plus phone verification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="41" t="str">
+        <x:v>CHG-021</x:v>
+      </x:c>
+      <x:c r="B26" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C26" s="41" t="str">
+        <x:v>4d618f897b6dab21270022b056de46a2a18d6288; 779e39624993a6ea739848aeba4b5819d7309568</x:v>
+      </x:c>
+      <x:c r="D26" s="41" t="str">
+        <x:v>backend/package-lock.json</x:v>
+      </x:c>
+      <x:c r="E26" s="41" t="str">
+        <x:v>Body-parser and Handlebars security lock resolutions</x:v>
+      </x:c>
+      <x:c r="F26" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G26" s="41" t="str">
+        <x:v>DEP-005</x:v>
+      </x:c>
+      <x:c r="H26" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/117</x:v>
+      </x:c>
+      <x:c r="I26" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J26" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K26" s="41" t="str">
+        <x:v>WOW-MD PRs 66 and 67; only resolved dependency metadata changed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6918,7 +7009,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c299564289f41a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e7320488c6e4269"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6955,40 +7046,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="73" t="str">
+      <x:c r="J5" s="77" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="73" t="str">
+      <x:c r="K5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="73" t="str">
+      <x:c r="L5" s="77" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8013,6 +8104,44 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L32" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="41" t="str">
+        <x:v>DEP-005</x:v>
+      </x:c>
+      <x:c r="B33" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/117</x:v>
+      </x:c>
+      <x:c r="C33" s="41" t="str">
+        <x:v>codex/dep-005-source-locks</x:v>
+      </x:c>
+      <x:c r="D33" s="41" t="str">
+        <x:v>7a56690</x:v>
+      </x:c>
+      <x:c r="E33" s="41" t="str">
+        <x:v>f2c2a59</x:v>
+      </x:c>
+      <x:c r="F33" s="41" t="str">
+        <x:v>WOW-MD PR 66 merged as 4d618f8; PR 67 merged as 779e396</x:v>
+      </x:c>
+      <x:c r="G33" s="41" t="str">
+        <x:v>Production lock resolution matches source semantically; protected CI runs on PR 117</x:v>
+      </x:c>
+      <x:c r="H33" s="41" t="str">
+        <x:v>Rebuild backend image from the reviewed lockfile</x:v>
+      </x:c>
+      <x:c r="I33" s="41" t="str">
+        <x:v>Revert PR 117 and rebuild prior image; no schema or data rollback</x:v>
+      </x:c>
+      <x:c r="J33" s="41" t="str">
+        <x:v>Remaining advisories require separate review; this PR only mirrors the two reviewed source changes</x:v>
+      </x:c>
+      <x:c r="K33" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L33" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -8029,7 +8158,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b2f2c4fa4f84574"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54cfd12ee9a9447e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
DEP-005: mirror body-parser and Handlebars fixes (#117)
* build(deps): mirror body-parser and handlebars fixes

* docs: register DEP-005 source mirror

* ci: refresh DEP-005 mirror declaration

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdadfb1bbefa24d39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R53733130a20c450f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Re9518ec89e9e47f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R59c0eb4864ed48ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb0314245f4084619"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rc24c988b78fb499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rda5d85a43f49420f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R5ac14ff73955477b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Re6a6e4efd66c4d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rdf937ed671204371"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c4a89865ef945fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R197417dd42494b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf07063130ae14466"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R540a1bf3a09c4951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R857539a5cea840ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R5b5d770048ff4ef2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R4399d3ff9c544dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re4b398e4c75e4d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R2c16e8ada9464404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7b82584a78964305"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -192,7 +197,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="74">
+  <x:cellXfs count="78">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -381,6 +386,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1000,7 +1017,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5e35a1a47fe24629"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra5cb08d8553646f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1010,8 +1027,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="82" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:M48"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="91" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1032,7 +1049,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="83" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="92" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1048,7 +1065,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="84" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="93" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1064,7 +1081,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="85" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="94" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1082,7 +1099,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="86" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="95" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1100,7 +1117,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="96" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1117,8 +1134,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="97" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K26"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1137,8 +1154,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="89" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L32"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="98" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L33"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1158,7 +1175,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="90" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="99" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1414,13 +1431,13 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B6" s="34" t="n">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1469,7 +1486,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1477,7 +1494,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1618,7 +1635,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1adc7a65c9df449a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2610b6b399634af0"/>
 </x:worksheet>
 </file>
 
@@ -1650,28 +1667,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2156,7 +2173,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22872b2ed3c240b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd00aaa0c67a8425f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2194,43 +2211,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="73" t="str">
+      <x:c r="J5" s="77" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="73" t="str">
+      <x:c r="K5" s="77" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="73" t="str">
+      <x:c r="L5" s="77" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="73" t="str">
+      <x:c r="M5" s="77" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -3946,6 +3963,45 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/116</x:v>
       </x:c>
       <x:c r="M48" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="41" t="str">
+        <x:v>DEP-005</x:v>
+      </x:c>
+      <x:c r="B49" s="41" t="str">
+        <x:v>Mirror body-parser and Handlebars security fixes</x:v>
+      </x:c>
+      <x:c r="C49" s="41" t="str">
+        <x:v>Public beta safety</x:v>
+      </x:c>
+      <x:c r="D49" s="41" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E49" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="F49" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="G49" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H49" s="41" t="str">
+        <x:v>DEP-004</x:v>
+      </x:c>
+      <x:c r="I49" s="41" t="str">
+        <x:v>Production backend lockfile resolves body-parser 1.20.8 and Handlebars 4.7.10 exactly as reviewed in source</x:v>
+      </x:c>
+      <x:c r="J49" s="41" t="str">
+        <x:v>WOW-MD PRs 66 and 67</x:v>
+      </x:c>
+      <x:c r="K49" s="41" t="str"/>
+      <x:c r="L49" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/117</x:v>
+      </x:c>
+      <x:c r="M49" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -3965,7 +4021,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73af2198434e4566"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c8885ce78a64210"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3997,25 +4053,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4541,7 +4597,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f4d36ddbe724a41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R069f0f19c73649dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4573,25 +4629,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -4992,7 +5048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R077d3eb852c846f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a80d0a37ac4ceb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5026,31 +5082,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5460,7 +5516,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb0c7c7dd4ef4e7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7d7bf4884ab4be8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5494,31 +5550,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5809,7 +5865,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15a3b933fd1e414b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R809985a19a024a92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5842,28 +5898,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6150,7 +6206,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b9b04e4df7543f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff61da0be1ba4ab7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6186,37 +6242,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="73" t="str">
+      <x:c r="J5" s="77" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="73" t="str">
+      <x:c r="K5" s="77" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6910,6 +6966,41 @@
       </x:c>
       <x:c r="K25" s="41" t="str">
         <x:v>WOW-MD PR 73; officer Support scoping mandatory settlement notes planner case context account-phone sync roster not-set display nav dedupe password patterns and mobile set-password gate plus phone verification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="41" t="str">
+        <x:v>CHG-021</x:v>
+      </x:c>
+      <x:c r="B26" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C26" s="41" t="str">
+        <x:v>4d618f897b6dab21270022b056de46a2a18d6288; 779e39624993a6ea739848aeba4b5819d7309568</x:v>
+      </x:c>
+      <x:c r="D26" s="41" t="str">
+        <x:v>backend/package-lock.json</x:v>
+      </x:c>
+      <x:c r="E26" s="41" t="str">
+        <x:v>Body-parser and Handlebars security lock resolutions</x:v>
+      </x:c>
+      <x:c r="F26" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G26" s="41" t="str">
+        <x:v>DEP-005</x:v>
+      </x:c>
+      <x:c r="H26" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/117</x:v>
+      </x:c>
+      <x:c r="I26" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J26" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K26" s="41" t="str">
+        <x:v>WOW-MD PRs 66 and 67; only resolved dependency metadata changed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6918,7 +7009,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c299564289f41a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e7320488c6e4269"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6955,40 +7046,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="73" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="73" t="str">
+      <x:c r="B5" s="77" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="73" t="str">
+      <x:c r="C5" s="77" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="73" t="str">
+      <x:c r="D5" s="77" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="73" t="str">
+      <x:c r="E5" s="77" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="73" t="str">
+      <x:c r="F5" s="77" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="73" t="str">
+      <x:c r="G5" s="77" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="73" t="str">
+      <x:c r="H5" s="77" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="73" t="str">
+      <x:c r="I5" s="77" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="73" t="str">
+      <x:c r="J5" s="77" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="73" t="str">
+      <x:c r="K5" s="77" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="73" t="str">
+      <x:c r="L5" s="77" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8013,6 +8104,44 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L32" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="41" t="str">
+        <x:v>DEP-005</x:v>
+      </x:c>
+      <x:c r="B33" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/117</x:v>
+      </x:c>
+      <x:c r="C33" s="41" t="str">
+        <x:v>codex/dep-005-source-locks</x:v>
+      </x:c>
+      <x:c r="D33" s="41" t="str">
+        <x:v>7a56690</x:v>
+      </x:c>
+      <x:c r="E33" s="41" t="str">
+        <x:v>f2c2a59</x:v>
+      </x:c>
+      <x:c r="F33" s="41" t="str">
+        <x:v>WOW-MD PR 66 merged as 4d618f8; PR 67 merged as 779e396</x:v>
+      </x:c>
+      <x:c r="G33" s="41" t="str">
+        <x:v>Production lock resolution matches source semantically; protected CI runs on PR 117</x:v>
+      </x:c>
+      <x:c r="H33" s="41" t="str">
+        <x:v>Rebuild backend image from the reviewed lockfile</x:v>
+      </x:c>
+      <x:c r="I33" s="41" t="str">
+        <x:v>Revert PR 117 and rebuild prior image; no schema or data rollback</x:v>
+      </x:c>
+      <x:c r="J33" s="41" t="str">
+        <x:v>Remaining advisories require separate review; this PR only mirrors the two reviewed source changes</x:v>
+      </x:c>
+      <x:c r="K33" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L33" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -8029,7 +8158,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b2f2c4fa4f84574"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54cfd12ee9a9447e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
OPS-002: collect capacity and cost snapshots
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c4a89865ef945fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R197417dd42494b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf07063130ae14466"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R540a1bf3a09c4951"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R857539a5cea840ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R5b5d770048ff4ef2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R4399d3ff9c544dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re4b398e4c75e4d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R2c16e8ada9464404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7b82584a78964305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf7479dbe6891426e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R20a74cb2670545fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R8991c4b587f94d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R950d147c9d854bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb1d1a810bc724160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R0983492983184893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R6dc43b77fe4a4e44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rc4f76861903a4ab3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R489a18fd1be348e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rce06ee81a6ff48b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -197,7 +202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="78">
+  <x:cellXfs count="82">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -398,6 +403,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1017,7 +1034,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra5cb08d8553646f7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5e7ebf774a74471"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1027,7 +1044,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="91" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="100" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -1049,7 +1066,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="92" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="101" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1065,7 +1082,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="93" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="102" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1081,7 +1098,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="94" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="103" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1099,7 +1116,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="95" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="104" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1117,7 +1134,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="96" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="105" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1134,8 +1151,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="97" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K26"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="106" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K27"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1154,8 +1171,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="98" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L33"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="107" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L34"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1175,7 +1192,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="99" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="108" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1444,7 +1461,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1452,7 +1469,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1486,7 +1503,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1494,7 +1511,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1635,7 +1652,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2610b6b399634af0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d7acc17661d445e"/>
 </x:worksheet>
 </file>
 
@@ -1667,28 +1684,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2173,7 +2190,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd00aaa0c67a8425f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e6608c2ff244cda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2211,43 +2228,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="77" t="str">
+      <x:c r="J5" s="81" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="77" t="str">
+      <x:c r="K5" s="81" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="77" t="str">
+      <x:c r="L5" s="81" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="77" t="str">
+      <x:c r="M5" s="81" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2711,10 +2728,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F17" s="41" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G17" s="41" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H17" s="41" t="str">
         <x:v>CFG-001,OBS-001</x:v>
@@ -2723,14 +2740,16 @@
         <x:v>Exact account DAU request latency error resource database and cost measurements persist</x:v>
       </x:c>
       <x:c r="J17" s="41" t="str">
-        <x:v>Production plan Task 6</x:v>
+        <x:v>WOW-MD PR 74 merged as cf50bb7; production PR 118</x:v>
       </x:c>
       <x:c r="K17" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/17</x:v>
       </x:c>
-      <x:c r="L17" s="41" t="str"/>
+      <x:c r="L17" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/118</x:v>
+      </x:c>
       <x:c r="M17" s="41" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
@@ -4021,7 +4040,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c8885ce78a64210"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8299128b7ccc48b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4053,25 +4072,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4597,7 +4616,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R069f0f19c73649dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd43cf042f8074834"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4629,25 +4648,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -5048,7 +5067,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a80d0a37ac4ceb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09351394130d4266"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5082,31 +5101,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5516,7 +5535,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7d7bf4884ab4be8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f753e51048f417c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5550,31 +5569,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5865,7 +5884,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R809985a19a024a92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77d866181e114513"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5898,28 +5917,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6206,7 +6225,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff61da0be1ba4ab7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23b6139cdf044f1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6242,37 +6261,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="77" t="str">
+      <x:c r="J5" s="81" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="77" t="str">
+      <x:c r="K5" s="81" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -7001,6 +7020,41 @@
       </x:c>
       <x:c r="K26" s="41" t="str">
         <x:v>WOW-MD PRs 66 and 67; only resolved dependency metadata changed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="41" t="str">
+        <x:v>CHG-022</x:v>
+      </x:c>
+      <x:c r="B27" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C27" s="41" t="str">
+        <x:v>cf50bb7395bb0f8b2613161e9d008d3c74c73593</x:v>
+      </x:c>
+      <x:c r="D27" s="41" t="str">
+        <x:v>backend operations capacity collector evaluator scheduler entities and migration; config/platform.yaml</x:v>
+      </x:c>
+      <x:c r="E27" s="41" t="str">
+        <x:v>Capacity and cost snapshot collection</x:v>
+      </x:c>
+      <x:c r="F27" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G27" s="41" t="str">
+        <x:v>OPS-002</x:v>
+      </x:c>
+      <x:c r="H27" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/118</x:v>
+      </x:c>
+      <x:c r="I27" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J27" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K27" s="41" t="str">
+        <x:v>WOW-MD PR 74; exact measurements, retention, replica lock, sustained/consecutive alert evaluation and telemetry failure isolation</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7009,7 +7063,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e7320488c6e4269"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd25a199b1e3405e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7046,40 +7100,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="77" t="str">
+      <x:c r="J5" s="81" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="77" t="str">
+      <x:c r="K5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="77" t="str">
+      <x:c r="L5" s="81" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8142,6 +8196,44 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L33" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="41" t="str">
+        <x:v>OPS-002</x:v>
+      </x:c>
+      <x:c r="B34" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/118</x:v>
+      </x:c>
+      <x:c r="C34" s="41" t="str">
+        <x:v>codex/ops-002-capacity</x:v>
+      </x:c>
+      <x:c r="D34" s="41" t="str">
+        <x:v>20ac88c</x:v>
+      </x:c>
+      <x:c r="E34" s="41" t="str">
+        <x:v>240cddb</x:v>
+      </x:c>
+      <x:c r="F34" s="41" t="str">
+        <x:v>WOW-MD PR 74 merged as cf50bb7</x:v>
+      </x:c>
+      <x:c r="G34" s="41" t="str">
+        <x:v>Backend 113 suites and 1109 tests passed with 9 skipped; typecheck lint focused tests and disposable migration apply/no-op passed; protected CI runs on PR 118</x:v>
+      </x:c>
+      <x:c r="H34" s="41" t="str">
+        <x:v>Back up PostgreSQL; deploy backend and run migration 1710000114000 before relying on hourly snapshots</x:v>
+      </x:c>
+      <x:c r="I34" s="41" t="str">
+        <x:v>Revert application release; retain additive evidence tables unless export and deletion are explicitly approved</x:v>
+      </x:c>
+      <x:c r="J34" s="41" t="str">
+        <x:v>Railway cost remains a configured estimate until a billing adapter supplies measured cost; live capacity evidence awaits the Railway candidate</x:v>
+      </x:c>
+      <x:c r="K34" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L34" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -8158,7 +8250,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54cfd12ee9a9447e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc1a895416f453b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
OPS-002: collect capacity and cost snapshots (#118)
Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4c4a89865ef945fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R197417dd42494b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf07063130ae14466"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R540a1bf3a09c4951"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R857539a5cea840ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R5b5d770048ff4ef2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R4399d3ff9c544dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re4b398e4c75e4d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R2c16e8ada9464404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R7b82584a78964305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf7479dbe6891426e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R20a74cb2670545fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R8991c4b587f94d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R950d147c9d854bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb1d1a810bc724160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R0983492983184893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R6dc43b77fe4a4e44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rc4f76861903a4ab3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R489a18fd1be348e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rce06ee81a6ff48b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -197,7 +202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="78">
+  <x:cellXfs count="82">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -398,6 +403,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1017,7 +1034,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra5cb08d8553646f7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5e7ebf774a74471"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1027,7 +1044,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="91" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="100" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -1049,7 +1066,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="92" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="101" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1065,7 +1082,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="93" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="102" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G22"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1081,7 +1098,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="94" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="103" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1099,7 +1116,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="95" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="104" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1117,7 +1134,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="96" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="105" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1134,8 +1151,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="97" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K26"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="106" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K27"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1154,8 +1171,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="98" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L33"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="107" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L34"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1175,7 +1192,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="99" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="108" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H23"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1444,7 +1461,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1452,7 +1469,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1486,7 +1503,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1494,7 +1511,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1635,7 +1652,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2610b6b399634af0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d7acc17661d445e"/>
 </x:worksheet>
 </file>
 
@@ -1667,28 +1684,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2173,7 +2190,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd00aaa0c67a8425f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e6608c2ff244cda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2211,43 +2228,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="77" t="str">
+      <x:c r="J5" s="81" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="77" t="str">
+      <x:c r="K5" s="81" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="77" t="str">
+      <x:c r="L5" s="81" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="77" t="str">
+      <x:c r="M5" s="81" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2711,10 +2728,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F17" s="41" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G17" s="41" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H17" s="41" t="str">
         <x:v>CFG-001,OBS-001</x:v>
@@ -2723,14 +2740,16 @@
         <x:v>Exact account DAU request latency error resource database and cost measurements persist</x:v>
       </x:c>
       <x:c r="J17" s="41" t="str">
-        <x:v>Production plan Task 6</x:v>
+        <x:v>WOW-MD PR 74 merged as cf50bb7; production PR 118</x:v>
       </x:c>
       <x:c r="K17" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/17</x:v>
       </x:c>
-      <x:c r="L17" s="41" t="str"/>
+      <x:c r="L17" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/118</x:v>
+      </x:c>
       <x:c r="M17" s="41" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
@@ -4021,7 +4040,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c8885ce78a64210"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8299128b7ccc48b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4053,25 +4072,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4597,7 +4616,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R069f0f19c73649dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd43cf042f8074834"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4629,25 +4648,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -5048,7 +5067,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a80d0a37ac4ceb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09351394130d4266"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5082,31 +5101,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5516,7 +5535,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7d7bf4884ab4be8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f753e51048f417c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5550,31 +5569,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5865,7 +5884,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R809985a19a024a92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77d866181e114513"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5898,28 +5917,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6206,7 +6225,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff61da0be1ba4ab7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23b6139cdf044f1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6242,37 +6261,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="77" t="str">
+      <x:c r="J5" s="81" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="77" t="str">
+      <x:c r="K5" s="81" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -7001,6 +7020,41 @@
       </x:c>
       <x:c r="K26" s="41" t="str">
         <x:v>WOW-MD PRs 66 and 67; only resolved dependency metadata changed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="41" t="str">
+        <x:v>CHG-022</x:v>
+      </x:c>
+      <x:c r="B27" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C27" s="41" t="str">
+        <x:v>cf50bb7395bb0f8b2613161e9d008d3c74c73593</x:v>
+      </x:c>
+      <x:c r="D27" s="41" t="str">
+        <x:v>backend operations capacity collector evaluator scheduler entities and migration; config/platform.yaml</x:v>
+      </x:c>
+      <x:c r="E27" s="41" t="str">
+        <x:v>Capacity and cost snapshot collection</x:v>
+      </x:c>
+      <x:c r="F27" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G27" s="41" t="str">
+        <x:v>OPS-002</x:v>
+      </x:c>
+      <x:c r="H27" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/118</x:v>
+      </x:c>
+      <x:c r="I27" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J27" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K27" s="41" t="str">
+        <x:v>WOW-MD PR 74; exact measurements, retention, replica lock, sustained/consecutive alert evaluation and telemetry failure isolation</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7009,7 +7063,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e7320488c6e4269"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd25a199b1e3405e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7046,40 +7100,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="77" t="str">
+      <x:c r="A5" s="81" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="77" t="str">
+      <x:c r="B5" s="81" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="77" t="str">
+      <x:c r="C5" s="81" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="77" t="str">
+      <x:c r="D5" s="81" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="77" t="str">
+      <x:c r="E5" s="81" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="77" t="str">
+      <x:c r="F5" s="81" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="str">
+      <x:c r="G5" s="81" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="77" t="str">
+      <x:c r="H5" s="81" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="77" t="str">
+      <x:c r="I5" s="81" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="77" t="str">
+      <x:c r="J5" s="81" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="77" t="str">
+      <x:c r="K5" s="81" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="77" t="str">
+      <x:c r="L5" s="81" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8142,6 +8196,44 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L33" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="41" t="str">
+        <x:v>OPS-002</x:v>
+      </x:c>
+      <x:c r="B34" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/118</x:v>
+      </x:c>
+      <x:c r="C34" s="41" t="str">
+        <x:v>codex/ops-002-capacity</x:v>
+      </x:c>
+      <x:c r="D34" s="41" t="str">
+        <x:v>20ac88c</x:v>
+      </x:c>
+      <x:c r="E34" s="41" t="str">
+        <x:v>240cddb</x:v>
+      </x:c>
+      <x:c r="F34" s="41" t="str">
+        <x:v>WOW-MD PR 74 merged as cf50bb7</x:v>
+      </x:c>
+      <x:c r="G34" s="41" t="str">
+        <x:v>Backend 113 suites and 1109 tests passed with 9 skipped; typecheck lint focused tests and disposable migration apply/no-op passed; protected CI runs on PR 118</x:v>
+      </x:c>
+      <x:c r="H34" s="41" t="str">
+        <x:v>Back up PostgreSQL; deploy backend and run migration 1710000114000 before relying on hourly snapshots</x:v>
+      </x:c>
+      <x:c r="I34" s="41" t="str">
+        <x:v>Revert application release; retain additive evidence tables unless export and deletion are explicitly approved</x:v>
+      </x:c>
+      <x:c r="J34" s="41" t="str">
+        <x:v>Railway cost remains a configured estimate until a billing adapter supplies measured cost; live capacity evidence awaits the Railway candidate</x:v>
+      </x:c>
+      <x:c r="K34" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L34" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -8158,7 +8250,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54cfd12ee9a9447e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc1a895416f453b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: regenerate UI-001 tracking workbook
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R96f85f96403b41fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Raa5113fb748c4be9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rdac9c11eec704cdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R148881b4d2764b3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rd9cc661c767642c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Refeeda49dcb44112"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R02fbcf10decc4d9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R8f18281de7bc47c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rc7c4079e9e754e91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rd5d5c7e5b5f74e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0e4106f37f9043d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R9852e7b8e7d74d28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R48c30abff1dd44b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Racaab772ab5a429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Re2c5671dc23545ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R7fa590f71e54469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R519c322ee8af4023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rcf785155abf549de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8f9be5321daa401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rbf605a880640403d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="14">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -207,7 +212,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="86">
+  <x:cellXfs count="90">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -432,6 +437,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1051,7 +1068,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ea430a0fff3459f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc98c4a87726448ab"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1061,7 +1078,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="109" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="118" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -1083,7 +1100,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="110" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="119" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1099,8 +1116,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="111" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:G23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="120" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G24"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Layer"/>
@@ -1115,8 +1132,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="112" name="RisksTable" displayName="RisksTable" ref="A5:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:I19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="121" name="RisksTable" displayName="RisksTable" ref="A5:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:I20"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risk"/>
@@ -1133,7 +1150,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="113" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="122" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1151,7 +1168,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="114" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="123" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1168,8 +1185,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="115" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:K28"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="124" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:K29"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="SourceRepository"/>
@@ -1188,8 +1205,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="116" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:L35"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="125" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:L36"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
     <x:tableColumn id="2" name="PR"/>
@@ -1209,7 +1226,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="117" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="126" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H24"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1478,7 +1495,7 @@
       </x:c>
       <x:c r="H6" s="39" t="n">
         <x:f>B7</x:f>
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1486,7 +1503,7 @@
         <x:v>Open</x:v>
       </x:c>
       <x:c r="B7" s="34" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
         <x:v>Open release gates</x:v>
@@ -1513,7 +1530,7 @@
         <x:v>Open risks</x:v>
       </x:c>
       <x:c r="E8" s="34" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G8" s="39" t="str">
         <x:v>PR Open</x:v>
@@ -1562,7 +1579,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1570,7 +1587,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1669,7 +1686,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e32cc8a45274a1e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb850042d782413d"/>
 </x:worksheet>
 </file>
 
@@ -1701,28 +1718,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="85" t="str">
+      <x:c r="H5" s="89" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2233,7 +2250,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab6dbb708c2b472c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc62557d20df946ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2271,43 +2288,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="85" t="str">
+      <x:c r="H5" s="89" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="85" t="str">
+      <x:c r="I5" s="89" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="85" t="str">
+      <x:c r="J5" s="89" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="85" t="str">
+      <x:c r="K5" s="89" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="85" t="str">
+      <x:c r="L5" s="89" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="85" t="str">
+      <x:c r="M5" s="89" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2812,7 +2829,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F18" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G18" s="41" t="str">
         <x:v>Codex</x:v>
@@ -2824,7 +2841,7 @@
         <x:v>Warnings and critical alerts reach portal email audit and logs without flooding</x:v>
       </x:c>
       <x:c r="J18" s="41" t="str">
-        <x:v>WOW-MD PR 70 merged as daae790; production PR 113 rebased on OPS-002</x:v>
+        <x:v>WOW-MD PR 70 and production PR 113 merged</x:v>
       </x:c>
       <x:c r="K18" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/18</x:v>
@@ -2853,10 +2870,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F19" s="41" t="str">
-        <x:v>Open</x:v>
+        <x:v>PR Open</x:v>
       </x:c>
       <x:c r="G19" s="41" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H19" s="41" t="str">
         <x:v>OPS-003</x:v>
@@ -2865,14 +2882,16 @@
         <x:v>Admin sees exact values thresholds evidence alert status and migration readiness</x:v>
       </x:c>
       <x:c r="J19" s="41" t="str">
-        <x:v>Production plan Task 8</x:v>
+        <x:v>WOW-MD PR 75 merged as 0d23fa2; production PR 114 rebased on OPS-003</x:v>
       </x:c>
       <x:c r="K19" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/19</x:v>
       </x:c>
-      <x:c r="L19" s="41" t="str"/>
+      <x:c r="L19" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</x:v>
+      </x:c>
       <x:c r="M19" s="41" t="str">
-        <x:v>2026-10-04</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
@@ -4085,7 +4104,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc03dd2b64e9d4f8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad7baf4e49a24326"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4117,25 +4136,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4661,7 +4680,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36c1b7a12fb04b01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6fd738240c34e4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4693,25 +4712,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -5127,6 +5146,29 @@
       </x:c>
       <x:c r="G23" s="41" t="str">
         <x:v>OPS-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="41" t="str">
+        <x:v>QA-UI-001</x:v>
+      </x:c>
+      <x:c r="B24" s="41" t="str">
+        <x:v>Administrator Infrastructure dashboard</x:v>
+      </x:c>
+      <x:c r="C24" s="41" t="str">
+        <x:v>Permission matrix guards exact persisted values and units stale missing and placeholder metrics as unknown alert ordering idempotent acknowledgement redacted delivery state disabled migration readiness and all UI states</x:v>
+      </x:c>
+      <x:c r="D24" s="41" t="str">
+        <x:v>UI-001 PR 114 and WOW-MD PR 71</x:v>
+      </x:c>
+      <x:c r="E24" s="41" t="str">
+        <x:v>Backend 1219 passed 9 skipped; E2E 79 passed; frontend 296 passed; Playwright 4 passed</x:v>
+      </x:c>
+      <x:c r="F24" s="41" t="str">
+        <x:v>Protected CI on the rebased PR; admin walk on the Railway candidate with live hourly snapshots</x:v>
+      </x:c>
+      <x:c r="G24" s="41" t="str">
+        <x:v>UI-001</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5135,7 +5177,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b280ce5dc4941d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743a011aec234f6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5169,31 +5211,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="85" t="str">
+      <x:c r="H5" s="89" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="85" t="str">
+      <x:c r="I5" s="89" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5587,6 +5629,35 @@
       </x:c>
       <x:c r="I19" s="41" t="str">
         <x:v>DEP-001 PR 59 records zero critical/high backend runtime advisories zero frontend advisories and the exact mobile exception set</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="41" t="str">
+        <x:v>RISK-015</x:v>
+      </x:c>
+      <x:c r="B20" s="41" t="str">
+        <x:v>The CI configuration-boundary check runs from backend/ where it scans zero files so new direct process.env reads could pass CI</x:v>
+      </x:c>
+      <x:c r="C20" s="41" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D20" s="41" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="E20" s="41" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="F20" s="41" t="str">
+        <x:v>Run scripts/verify-config-boundary.mjs from the repository root in CI and assert a non-zero scanned-file count</x:v>
+      </x:c>
+      <x:c r="G20" s="41" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="H20" s="41" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I20" s="41" t="str">
+        <x:v>Found during UI-001 PR 114 verification: 0 files from backend/ and 582 files from the repository root</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5605,7 +5676,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b16ecf4c6642fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67c9f6db6d234cd2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5639,31 +5710,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="85" t="str">
+      <x:c r="H5" s="89" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="85" t="str">
+      <x:c r="I5" s="89" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -5954,7 +6025,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7ad7426f9e4968"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5607db8b695349a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5987,28 +6058,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="85" t="str">
+      <x:c r="H5" s="89" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6297,7 +6368,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a64f91a9f484a46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racb54887a2484c25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6333,37 +6404,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="85" t="str">
+      <x:c r="H5" s="89" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="85" t="str">
+      <x:c r="I5" s="89" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="85" t="str">
+      <x:c r="J5" s="89" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="85" t="str">
+      <x:c r="K5" s="89" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -7162,6 +7233,41 @@
       </x:c>
       <x:c r="K28" s="41" t="str">
         <x:v>WOW-MD PR 70; reviewed deduplication, bounded retries, portal/email/audit/log delivery and redaction</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="41" t="str">
+        <x:v>CHG-024</x:v>
+      </x:c>
+      <x:c r="B29" s="41" t="str">
+        <x:v>RohithTadiparti/WOW-MD</x:v>
+      </x:c>
+      <x:c r="C29" s="41" t="str">
+        <x:v>0d23fa25f166b61dae654b44c7b3b818102ad2e6</x:v>
+      </x:c>
+      <x:c r="D29" s="41" t="str">
+        <x:v>backend operations dashboard controller service DTO redaction authz and E2E; frontend admin infrastructure page components library route and E2E</x:v>
+      </x:c>
+      <x:c r="E29" s="41" t="str">
+        <x:v>Administrator Infrastructure dashboard mirror</x:v>
+      </x:c>
+      <x:c r="F29" s="41" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="G29" s="41" t="str">
+        <x:v>UI-001</x:v>
+      </x:c>
+      <x:c r="H29" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</x:v>
+      </x:c>
+      <x:c r="I29" s="41" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J29" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="K29" s="41" t="str">
+        <x:v>WOW-MD replacement PR 75; PR 71 closed automatically when its stacked base was deleted</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7170,7 +7276,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R799e133a8d0b4838"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R294094c8554f434b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7207,40 +7313,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="89" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="85" t="str">
+      <x:c r="C5" s="89" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="85" t="str">
+      <x:c r="D5" s="89" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="85" t="str">
+      <x:c r="E5" s="89" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="85" t="str">
+      <x:c r="F5" s="89" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="85" t="str">
+      <x:c r="G5" s="89" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="85" t="str">
+      <x:c r="H5" s="89" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="85" t="str">
+      <x:c r="I5" s="89" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="85" t="str">
+      <x:c r="J5" s="89" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="85" t="str">
+      <x:c r="K5" s="89" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="85" t="str">
+      <x:c r="L5" s="89" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8379,6 +8485,44 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="L35" s="41" t="str">
+        <x:v>2026-10-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="41" t="str">
+        <x:v>UI-001</x:v>
+      </x:c>
+      <x:c r="B36" s="41" t="str">
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</x:v>
+      </x:c>
+      <x:c r="C36" s="41" t="str">
+        <x:v>claude/ui-001-infrastructure-dashboard</x:v>
+      </x:c>
+      <x:c r="D36" s="41" t="str">
+        <x:v>8f648fa</x:v>
+      </x:c>
+      <x:c r="E36" s="41" t="str">
+        <x:v>c04cde9</x:v>
+      </x:c>
+      <x:c r="F36" s="41" t="str">
+        <x:v>WOW-MD PR 75 merged as 0d23fa2; PR 71 was replaced after stacked-base deletion</x:v>
+      </x:c>
+      <x:c r="G36" s="41" t="str">
+        <x:v>Backend focused 126 passed; backend 1219 passed 9 skipped; lint typecheck build passed; E2E 79 passed; frontend 296 tests build and Playwright 4 passed; exact-digit formatter review added 23 focused frontend tests</x:v>
+      </x:c>
+      <x:c r="H36" s="41" t="str">
+        <x:v>Deploy backend then frontend; no additional migration or configuration beyond OPS-003</x:v>
+      </x:c>
+      <x:c r="I36" s="41" t="str">
+        <x:v>Redeploy previous images; acknowledgement fields remain harmless</x:v>
+      </x:c>
+      <x:c r="J36" s="41" t="str">
+        <x:v>Acknowledgement shows actor ID not name; AUTH-001 MIG-001 and GATE-009 to GATE-011 remain unmet by design; revenue stays unknown until a net revenue source exists</x:v>
+      </x:c>
+      <x:c r="K36" s="41" t="str">
+        <x:v>PR Open</x:v>
+      </x:c>
+      <x:c r="L36" s="41" t="str">
         <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
@@ -8395,7 +8539,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ac43d1cf5704643"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9da800edcab44719"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: register replacement UI-001 PR
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0e4106f37f9043d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R9852e7b8e7d74d28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R48c30abff1dd44b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="Racaab772ab5a429d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Re2c5671dc23545ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R7fa590f71e54469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R519c322ee8af4023"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Rcf785155abf549de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R8f9be5321daa401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rbf605a880640403d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb6616c3478f540c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Re3a6d20631904ca9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R61d69bff82fd46da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R4330efaf8fe24d1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R3648d17b45a94966"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R40ef62c353884730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R1029743b7e93411e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R197f5aca6ff644c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ref036850fcc54271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Ra892f1c70ea84b1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -212,7 +217,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="90">
+  <x:cellXfs count="94">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -449,6 +454,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1068,7 +1085,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc98c4a87726448ab"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9e510fc592904642"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1078,7 +1095,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="118" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="127" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -1100,7 +1117,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="119" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="128" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1116,7 +1133,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="120" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="129" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G24"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1132,7 +1149,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="121" name="RisksTable" displayName="RisksTable" ref="A5:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="130" name="RisksTable" displayName="RisksTable" ref="A5:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I20"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1150,7 +1167,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="122" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="131" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1168,7 +1185,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="123" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="132" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1185,7 +1202,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="124" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="133" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:K29"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
@@ -1205,7 +1222,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="125" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="134" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:L36"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
@@ -1226,7 +1243,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="126" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="135" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H24"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1686,7 +1703,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb850042d782413d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb565007c95214c62"/>
 </x:worksheet>
 </file>
 
@@ -1718,28 +1735,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="89" t="str">
+      <x:c r="H5" s="93" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2250,7 +2267,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc62557d20df946ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21b5434d68c24197"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2288,43 +2305,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="89" t="str">
+      <x:c r="H5" s="93" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="89" t="str">
+      <x:c r="I5" s="93" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="89" t="str">
+      <x:c r="J5" s="93" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="89" t="str">
+      <x:c r="K5" s="93" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="89" t="str">
+      <x:c r="L5" s="93" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="89" t="str">
+      <x:c r="M5" s="93" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2882,13 +2899,13 @@
         <x:v>Admin sees exact values thresholds evidence alert status and migration readiness</x:v>
       </x:c>
       <x:c r="J19" s="41" t="str">
-        <x:v>WOW-MD PR 75 merged as 0d23fa2; production PR 114 rebased on OPS-003</x:v>
+        <x:v>WOW-MD PR 75 merged as 0d23fa2; production replacement PR 119 rebased on OPS-003</x:v>
       </x:c>
       <x:c r="K19" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/19</x:v>
       </x:c>
       <x:c r="L19" s="41" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/119</x:v>
       </x:c>
       <x:c r="M19" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -4104,7 +4121,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad7baf4e49a24326"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ad93776740b4b8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4136,25 +4153,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4680,7 +4697,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6fd738240c34e4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf3d58e51bc94ef8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4712,25 +4729,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -5177,7 +5194,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743a011aec234f6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fd864dcd1cc4bd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5211,31 +5228,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="89" t="str">
+      <x:c r="H5" s="93" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="89" t="str">
+      <x:c r="I5" s="93" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5676,7 +5693,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67c9f6db6d234cd2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfe7f5e78a84d51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5710,31 +5727,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="89" t="str">
+      <x:c r="H5" s="93" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="89" t="str">
+      <x:c r="I5" s="93" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6025,7 +6042,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5607db8b695349a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a4768ac602b422c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6058,28 +6075,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="89" t="str">
+      <x:c r="H5" s="93" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6368,7 +6385,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racb54887a2484c25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bf0841cfafa4565"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6404,37 +6421,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="89" t="str">
+      <x:c r="H5" s="93" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="89" t="str">
+      <x:c r="I5" s="93" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="89" t="str">
+      <x:c r="J5" s="93" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="89" t="str">
+      <x:c r="K5" s="93" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -7258,7 +7275,7 @@
         <x:v>UI-001</x:v>
       </x:c>
       <x:c r="H29" s="41" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/119</x:v>
       </x:c>
       <x:c r="I29" s="41" t="str">
         <x:v>Codex</x:v>
@@ -7267,7 +7284,7 @@
         <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="K29" s="41" t="str">
-        <x:v>WOW-MD replacement PR 75; PR 71 closed automatically when its stacked base was deleted</x:v>
+        <x:v>WOW-MD replacement PR 75; source PR 71 and production PR 114 closed automatically when their stacked bases were deleted</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7276,7 +7293,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R294094c8554f434b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra147ae714d144a27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7313,40 +7330,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="93" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="93" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="93" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="93" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="89" t="str">
+      <x:c r="E5" s="93" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="93" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="89" t="str">
+      <x:c r="G5" s="93" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="89" t="str">
+      <x:c r="H5" s="93" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="89" t="str">
+      <x:c r="I5" s="93" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="89" t="str">
+      <x:c r="J5" s="93" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="89" t="str">
+      <x:c r="K5" s="93" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="89" t="str">
+      <x:c r="L5" s="93" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8493,7 +8510,7 @@
         <x:v>UI-001</x:v>
       </x:c>
       <x:c r="B36" s="41" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/114</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/119</x:v>
       </x:c>
       <x:c r="C36" s="41" t="str">
         <x:v>claude/ui-001-infrastructure-dashboard</x:v>
@@ -8505,7 +8522,7 @@
         <x:v>c04cde9</x:v>
       </x:c>
       <x:c r="F36" s="41" t="str">
-        <x:v>WOW-MD PR 75 merged as 0d23fa2; PR 71 was replaced after stacked-base deletion</x:v>
+        <x:v>WOW-MD PR 75 merged as 0d23fa2; source PR 71 and production PR 114 were replaced after stacked-base deletion</x:v>
       </x:c>
       <x:c r="G36" s="41" t="str">
         <x:v>Backend focused 126 passed; backend 1219 passed 9 skipped; lint typecheck build passed; E2E 79 passed; frontend 296 tests build and Playwright 4 passed; exact-digit formatter review added 23 focused frontend tests</x:v>
@@ -8539,7 +8556,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9da800edcab44719"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10505c326a314fee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close OBS and operations delivery tracking
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb6616c3478f540c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Re3a6d20631904ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R61d69bff82fd46da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R4330efaf8fe24d1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R3648d17b45a94966"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R40ef62c353884730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R1029743b7e93411e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R197f5aca6ff644c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ref036850fcc54271"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Ra892f1c70ea84b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a9184afdfd84d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R786334ba3b584f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb017360dcba94192"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R4228fbcc203646bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R54fed5612bb646ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rc0f95789c0574fb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R83a6ca2f446d49b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R0f5a1906575f43b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra12ecc6399d54c7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb1c1001243334d4a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -217,7 +222,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="94">
+  <x:cellXfs count="98">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -466,6 +471,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1085,7 +1102,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9e510fc592904642"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39f5df5413eb460c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1095,7 +1112,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="127" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="136" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -1117,7 +1134,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="128" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="137" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1133,7 +1150,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="129" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="138" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G24"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1149,7 +1166,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="130" name="RisksTable" displayName="RisksTable" ref="A5:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="139" name="RisksTable" displayName="RisksTable" ref="A5:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I20"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1167,7 +1184,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="131" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="140" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1185,7 +1202,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="132" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="141" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1202,7 +1219,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="133" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="142" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:K29"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
@@ -1222,7 +1239,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="134" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="143" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:L36"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
@@ -1243,7 +1260,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="135" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="144" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H24"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1505,7 +1522,7 @@
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1554,7 +1571,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1562,7 +1579,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1596,7 +1613,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>23</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1604,7 +1621,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>23</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1703,7 +1720,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb565007c95214c62"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3b96049e8ff46b0"/>
 </x:worksheet>
 </file>
 
@@ -1735,28 +1752,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2267,7 +2284,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21b5434d68c24197"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdafacf08f59e4d53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2305,43 +2322,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="93" t="str">
+      <x:c r="J5" s="97" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="93" t="str">
+      <x:c r="K5" s="97" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="93" t="str">
+      <x:c r="L5" s="97" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="93" t="str">
+      <x:c r="M5" s="97" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2600,7 +2617,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F12" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G12" s="41" t="str">
         <x:v>Codex</x:v>
@@ -2612,7 +2629,7 @@
         <x:v>Sanitized browser/mobile failures correlate with backend requests</x:v>
       </x:c>
       <x:c r="J12" s="41" t="str">
-        <x:v>client-error-observability plan; WOW-MD PRs 65 and 69 merged as c3ce5e5 and 2c56a49</x:v>
+        <x:v>WOW-MD PRs 65 and 69 plus production PR 112 merged</x:v>
       </x:c>
       <x:c r="K12" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/12</x:v>
@@ -2887,7 +2904,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F19" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G19" s="41" t="str">
         <x:v>Codex</x:v>
@@ -2899,7 +2916,7 @@
         <x:v>Admin sees exact values thresholds evidence alert status and migration readiness</x:v>
       </x:c>
       <x:c r="J19" s="41" t="str">
-        <x:v>WOW-MD PR 75 merged as 0d23fa2; production replacement PR 119 rebased on OPS-003</x:v>
+        <x:v>WOW-MD PR 75 and production replacement PR 119 merged</x:v>
       </x:c>
       <x:c r="K19" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/19</x:v>
@@ -4042,7 +4059,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F48" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G48" s="41" t="str">
         <x:v>Codex</x:v>
@@ -4054,7 +4071,7 @@
         <x:v>Production exactly mirrors WOW-MD PR 73 officer Support scoping settlement-notes phone-sync roster and mobile gate fixes with green local suites and updated source baseline</x:v>
       </x:c>
       <x:c r="J48" s="41" t="str">
-        <x:v>WOW-MD PR 73 pending merge</x:v>
+        <x:v>WOW-MD PR 73 and production PR 116 merged</x:v>
       </x:c>
       <x:c r="K48" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/115</x:v>
@@ -4083,7 +4100,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F49" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G49" s="41" t="str">
         <x:v>Codex</x:v>
@@ -4095,7 +4112,7 @@
         <x:v>Production backend lockfile resolves body-parser 1.20.8 and Handlebars 4.7.10 exactly as reviewed in source</x:v>
       </x:c>
       <x:c r="J49" s="41" t="str">
-        <x:v>WOW-MD PRs 66 and 67</x:v>
+        <x:v>WOW-MD PRs 66 and 67; production PR 117 merged</x:v>
       </x:c>
       <x:c r="K49" s="41" t="str"/>
       <x:c r="L49" s="41" t="str">
@@ -4121,7 +4138,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ad93776740b4b8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ebd0616483b4bbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4153,25 +4170,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4697,7 +4714,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf3d58e51bc94ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7844399862b499e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4729,25 +4746,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -5194,7 +5211,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fd864dcd1cc4bd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d4f2a494e7248e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5228,31 +5245,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5693,7 +5710,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfe7f5e78a84d51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0265d852e1364cf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5727,31 +5744,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6042,7 +6059,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a4768ac602b422c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fee00e5887f4b01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6075,28 +6092,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6385,7 +6402,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bf0841cfafa4565"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3b5affce5f48e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6421,37 +6438,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="93" t="str">
+      <x:c r="J5" s="97" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="93" t="str">
+      <x:c r="K5" s="97" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -7293,7 +7310,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra147ae714d144a27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3b1f260e25e403c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7330,40 +7347,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="93" t="str">
+      <x:c r="J5" s="97" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="93" t="str">
+      <x:c r="K5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="93" t="str">
+      <x:c r="L5" s="97" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8347,7 +8364,7 @@
         <x:v>Frontend has no lint script; no new Jest Expo dependency alerts were accepted</x:v>
       </x:c>
       <x:c r="K31" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L31" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8373,7 +8390,7 @@
         <x:v>WOW-MD PR 73 merged as a4a8f18</x:v>
       </x:c>
       <x:c r="G32" s="41" t="str">
-        <x:v>Local backend typecheck and 1101 tests frontend typecheck 268 tests and build mobile typecheck all passed; register validation passed; protected CI passed before rebase and will rerun</x:v>
+        <x:v>Local backend typecheck and 1101 tests frontend typecheck 268 tests and build mobile typecheck all passed; register validation and all protected CI passed</x:v>
       </x:c>
       <x:c r="H32" s="41" t="str">
         <x:v>Rebuild backend frontend and mobile artifacts from the mirrored commit; no migration or environment change</x:v>
@@ -8385,7 +8402,7 @@
         <x:v>Existing officers with diverged account phones keep the old number until re-saving the profile; live sheet re-run after deployment is tracked separately</x:v>
       </x:c>
       <x:c r="K32" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L32" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8411,7 +8428,7 @@
         <x:v>WOW-MD PR 66 merged as 4d618f8; PR 67 merged as 779e396</x:v>
       </x:c>
       <x:c r="G33" s="41" t="str">
-        <x:v>Production lock resolution matches source semantically; protected CI runs on PR 117</x:v>
+        <x:v>Production lock resolution matches source semantically; all protected CI passed</x:v>
       </x:c>
       <x:c r="H33" s="41" t="str">
         <x:v>Rebuild backend image from the reviewed lockfile</x:v>
@@ -8423,7 +8440,7 @@
         <x:v>Remaining advisories require separate review; this PR only mirrors the two reviewed source changes</x:v>
       </x:c>
       <x:c r="K33" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L33" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8449,7 +8466,7 @@
         <x:v>WOW-MD PR 74 merged as cf50bb7</x:v>
       </x:c>
       <x:c r="G34" s="41" t="str">
-        <x:v>Backend 113 suites and 1109 tests passed with 9 skipped; typecheck lint focused tests and disposable migration apply/no-op passed; protected CI runs on PR 118</x:v>
+        <x:v>Backend 113 suites and 1109 tests passed with 9 skipped; typecheck lint focused tests disposable migration apply/no-op and all protected CI passed</x:v>
       </x:c>
       <x:c r="H34" s="41" t="str">
         <x:v>Back up PostgreSQL; deploy backend and run migration 1710000114000 before relying on hourly snapshots</x:v>
@@ -8461,7 +8478,7 @@
         <x:v>Railway cost remains a configured estimate until a billing adapter supplies measured cost; live capacity evidence awaits the Railway candidate</x:v>
       </x:c>
       <x:c r="K34" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L34" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8487,7 +8504,7 @@
         <x:v>WOW-MD PR 70 merged as daae790</x:v>
       </x:c>
       <x:c r="G35" s="41" t="str">
-        <x:v>Focused delivery 31 tests plus lint and typecheck passed; original full backend 1149 passed 9 skipped and frontend 273 passed; protected CI reruns after rebase</x:v>
+        <x:v>Focused delivery 31 tests plus lint and typecheck passed; original full backend 1149 passed 9 skipped and frontend 273 passed; all protected CI passed after rebase</x:v>
       </x:c>
       <x:c r="H35" s="41" t="str">
         <x:v>Back up PostgreSQL; deploy backend migration 1710000115000 then frontend; optionally set OPERATIONS_ALERT_RECIPIENTS; mail remains simulated until final mail gate</x:v>
@@ -8499,7 +8516,7 @@
         <x:v>A delivery-state save failure after sending can repeat one send; live SMTP remains unproven until final Zoho mail gate</x:v>
       </x:c>
       <x:c r="K35" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L35" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8525,7 +8542,7 @@
         <x:v>WOW-MD PR 75 merged as 0d23fa2; source PR 71 and production PR 114 were replaced after stacked-base deletion</x:v>
       </x:c>
       <x:c r="G36" s="41" t="str">
-        <x:v>Backend focused 126 passed; backend 1219 passed 9 skipped; lint typecheck build passed; E2E 79 passed; frontend 296 tests build and Playwright 4 passed; exact-digit formatter review added 23 focused frontend tests</x:v>
+        <x:v>Backend focused 126 passed; backend 1219 passed 9 skipped; lint typecheck build E2E 79 frontend 296 tests Playwright 4 exact-digit 23 tests and all protected CI passed</x:v>
       </x:c>
       <x:c r="H36" s="41" t="str">
         <x:v>Deploy backend then frontend; no additional migration or configuration beyond OPS-003</x:v>
@@ -8537,7 +8554,7 @@
         <x:v>Acknowledgement shows actor ID not name; AUTH-001 MIG-001 and GATE-009 to GATE-011 remain unmet by design; revenue stays unknown until a net revenue source exists</x:v>
       </x:c>
       <x:c r="K36" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L36" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8556,7 +8573,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10505c326a314fee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7cd5158be5c4c17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Tracking: close observability and operations delivery (#120)
* docs: close OBS and operations delivery tracking

* docs: advance reviewed source baseline

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb6616c3478f540c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="Re3a6d20631904ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R61d69bff82fd46da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R4330efaf8fe24d1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R3648d17b45a94966"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R40ef62c353884730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R1029743b7e93411e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R197f5aca6ff644c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ref036850fcc54271"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Ra892f1c70ea84b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a9184afdfd84d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R786334ba3b584f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb017360dcba94192"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R4228fbcc203646bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R54fed5612bb646ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rc0f95789c0574fb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R83a6ca2f446d49b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R0f5a1906575f43b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra12ecc6399d54c7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb1c1001243334d4a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF6E1026"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6E0B2B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -217,7 +222,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="94">
+  <x:cellXfs count="98">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -466,6 +471,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1085,7 +1102,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9e510fc592904642"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39f5df5413eb460c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1095,7 +1112,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="127" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="136" name="OpenItemsTable" displayName="OpenItemsTable" ref="A5:M49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:M49"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="ID"/>
@@ -1117,7 +1134,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="128" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="137" name="RequirementsTable" displayName="RequirementsTable" ref="A5:G27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1133,7 +1150,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="129" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="138" name="TestInventoryTable" displayName="TestInventoryTable" ref="A5:G24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G24"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
@@ -1149,7 +1166,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="130" name="RisksTable" displayName="RisksTable" ref="A5:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="139" name="RisksTable" displayName="RisksTable" ref="A5:I20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I20"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1167,7 +1184,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="131" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="140" name="AccessTable" displayName="AccessTable" ref="A5:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
@@ -1185,7 +1202,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="132" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="141" name="ReleaseGatesTable" displayName="ReleaseGatesTable" ref="A5:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H17"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1202,7 +1219,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="133" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="142" name="ChangeIntakeTable" displayName="ChangeIntakeTable" ref="A5:K29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:K29"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
@@ -1222,7 +1239,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="134" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="143" name="PrHandoffsTable" displayName="PrHandoffsTable" ref="A5:L36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:L36"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="WorkItem"/>
@@ -1243,7 +1260,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="135" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="144" name="DocumentsTable" displayName="DocumentsTable" ref="A5:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H24"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
@@ -1505,7 +1522,7 @@
         <x:v>P0 items not done</x:v>
       </x:c>
       <x:c r="E6" s="34" t="n">
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G6" s="39" t="str">
         <x:v>Open</x:v>
@@ -1554,7 +1571,7 @@
       </x:c>
       <x:c r="H8" s="39" t="n">
         <x:f>B9</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1562,7 +1579,7 @@
         <x:v>PR Open</x:v>
       </x:c>
       <x:c r="B9" s="34" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
         <x:v>P0 open risks</x:v>
@@ -1596,7 +1613,7 @@
       </x:c>
       <x:c r="H10" s="39" t="n">
         <x:f>B11</x:f>
-        <x:v>23</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1604,7 +1621,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>23</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G11" t="str"/>
       <x:c r="H11"/>
@@ -1703,7 +1720,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb565007c95214c62"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3b96049e8ff46b0"/>
 </x:worksheet>
 </file>
 
@@ -1735,28 +1752,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Path</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>ReviewCadence</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>LastReviewed</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>RelatedItems</x:v>
       </x:c>
     </x:row>
@@ -2267,7 +2284,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21b5434d68c24197"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdafacf08f59e4d53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2305,43 +2322,43 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Phase</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>DependsOn</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Acceptance</x:v>
       </x:c>
-      <x:c r="J5" s="93" t="str">
+      <x:c r="J5" s="97" t="str">
         <x:v>SourceRef</x:v>
       </x:c>
-      <x:c r="K5" s="93" t="str">
+      <x:c r="K5" s="97" t="str">
         <x:v>GitHubIssue</x:v>
       </x:c>
-      <x:c r="L5" s="93" t="str">
+      <x:c r="L5" s="97" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="M5" s="93" t="str">
+      <x:c r="M5" s="97" t="str">
         <x:v>LastUpdated</x:v>
       </x:c>
     </x:row>
@@ -2600,7 +2617,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F12" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G12" s="41" t="str">
         <x:v>Codex</x:v>
@@ -2612,7 +2629,7 @@
         <x:v>Sanitized browser/mobile failures correlate with backend requests</x:v>
       </x:c>
       <x:c r="J12" s="41" t="str">
-        <x:v>client-error-observability plan; WOW-MD PRs 65 and 69 merged as c3ce5e5 and 2c56a49</x:v>
+        <x:v>WOW-MD PRs 65 and 69 plus production PR 112 merged</x:v>
       </x:c>
       <x:c r="K12" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/12</x:v>
@@ -2887,7 +2904,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F19" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G19" s="41" t="str">
         <x:v>Codex</x:v>
@@ -2899,7 +2916,7 @@
         <x:v>Admin sees exact values thresholds evidence alert status and migration readiness</x:v>
       </x:c>
       <x:c r="J19" s="41" t="str">
-        <x:v>WOW-MD PR 75 merged as 0d23fa2; production replacement PR 119 rebased on OPS-003</x:v>
+        <x:v>WOW-MD PR 75 and production replacement PR 119 merged</x:v>
       </x:c>
       <x:c r="K19" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/19</x:v>
@@ -4042,7 +4059,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F48" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G48" s="41" t="str">
         <x:v>Codex</x:v>
@@ -4054,7 +4071,7 @@
         <x:v>Production exactly mirrors WOW-MD PR 73 officer Support scoping settlement-notes phone-sync roster and mobile gate fixes with green local suites and updated source baseline</x:v>
       </x:c>
       <x:c r="J48" s="41" t="str">
-        <x:v>WOW-MD PR 73 pending merge</x:v>
+        <x:v>WOW-MD PR 73 and production PR 116 merged</x:v>
       </x:c>
       <x:c r="K48" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/115</x:v>
@@ -4083,7 +4100,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F49" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G49" s="41" t="str">
         <x:v>Codex</x:v>
@@ -4095,7 +4112,7 @@
         <x:v>Production backend lockfile resolves body-parser 1.20.8 and Handlebars 4.7.10 exactly as reviewed in source</x:v>
       </x:c>
       <x:c r="J49" s="41" t="str">
-        <x:v>WOW-MD PRs 66 and 67</x:v>
+        <x:v>WOW-MD PRs 66 and 67; production PR 117 merged</x:v>
       </x:c>
       <x:c r="K49" s="41" t="str"/>
       <x:c r="L49" s="41" t="str">
@@ -4121,7 +4138,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ad93776740b4b8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ebd0616483b4bbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4153,25 +4170,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Requirement</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Verification</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -4697,7 +4714,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf3d58e51bc94ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7844399862b499e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4729,25 +4746,25 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Layer</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Scope</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>CurrentEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>CurrentResult</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>RequiredNextEvidence</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>WorkItems</x:v>
       </x:c>
     </x:row>
@@ -5194,7 +5211,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fd864dcd1cc4bd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d4f2a494e7248e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5228,31 +5245,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Risk</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Impact</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>Likelihood</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Mitigation</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Evidence</x:v>
       </x:c>
     </x:row>
@@ -5693,7 +5710,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfe7f5e78a84d51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0265d852e1364cf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5727,31 +5744,31 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>System</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>AccessNeeded</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>HumanOwner</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>MachineIdentity</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>SecretLocation</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>VerifiedDate</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -6042,7 +6059,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a4768ac602b422c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fee00e5887f4b01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6075,28 +6092,28 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>RequiredEvidence</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>ApprovedDate</x:v>
       </x:c>
     </x:row>
@@ -6385,7 +6402,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bf0841cfafa4565"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3b5affce5f48e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6421,37 +6438,37 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>SourceRepository</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>SourceCommit</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>SourcePath</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>Classification</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>ProductionItem</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>ProductionPR</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>ReviewedBy</x:v>
       </x:c>
-      <x:c r="J5" s="93" t="str">
+      <x:c r="J5" s="97" t="str">
         <x:v>ReviewedDate</x:v>
       </x:c>
-      <x:c r="K5" s="93" t="str">
+      <x:c r="K5" s="97" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -7293,7 +7310,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra147ae714d144a27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3b1f260e25e403c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7330,40 +7347,40 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="93" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>WorkItem</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="97" t="str">
         <x:v>PR</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="97" t="str">
         <x:v>Branch</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="str">
+      <x:c r="D5" s="97" t="str">
         <x:v>BaseCommit</x:v>
       </x:c>
-      <x:c r="E5" s="93" t="str">
+      <x:c r="E5" s="97" t="str">
         <x:v>HeadCommit</x:v>
       </x:c>
-      <x:c r="F5" s="93" t="str">
+      <x:c r="F5" s="97" t="str">
         <x:v>SourceCommits</x:v>
       </x:c>
-      <x:c r="G5" s="93" t="str">
+      <x:c r="G5" s="97" t="str">
         <x:v>Tests</x:v>
       </x:c>
-      <x:c r="H5" s="93" t="str">
+      <x:c r="H5" s="97" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I5" s="93" t="str">
+      <x:c r="I5" s="97" t="str">
         <x:v>Rollback</x:v>
       </x:c>
-      <x:c r="J5" s="93" t="str">
+      <x:c r="J5" s="97" t="str">
         <x:v>ResidualRisks</x:v>
       </x:c>
-      <x:c r="K5" s="93" t="str">
+      <x:c r="K5" s="97" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="L5" s="93" t="str">
+      <x:c r="L5" s="97" t="str">
         <x:v>Updated</x:v>
       </x:c>
     </x:row>
@@ -8347,7 +8364,7 @@
         <x:v>Frontend has no lint script; no new Jest Expo dependency alerts were accepted</x:v>
       </x:c>
       <x:c r="K31" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L31" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8373,7 +8390,7 @@
         <x:v>WOW-MD PR 73 merged as a4a8f18</x:v>
       </x:c>
       <x:c r="G32" s="41" t="str">
-        <x:v>Local backend typecheck and 1101 tests frontend typecheck 268 tests and build mobile typecheck all passed; register validation passed; protected CI passed before rebase and will rerun</x:v>
+        <x:v>Local backend typecheck and 1101 tests frontend typecheck 268 tests and build mobile typecheck all passed; register validation and all protected CI passed</x:v>
       </x:c>
       <x:c r="H32" s="41" t="str">
         <x:v>Rebuild backend frontend and mobile artifacts from the mirrored commit; no migration or environment change</x:v>
@@ -8385,7 +8402,7 @@
         <x:v>Existing officers with diverged account phones keep the old number until re-saving the profile; live sheet re-run after deployment is tracked separately</x:v>
       </x:c>
       <x:c r="K32" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L32" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8411,7 +8428,7 @@
         <x:v>WOW-MD PR 66 merged as 4d618f8; PR 67 merged as 779e396</x:v>
       </x:c>
       <x:c r="G33" s="41" t="str">
-        <x:v>Production lock resolution matches source semantically; protected CI runs on PR 117</x:v>
+        <x:v>Production lock resolution matches source semantically; all protected CI passed</x:v>
       </x:c>
       <x:c r="H33" s="41" t="str">
         <x:v>Rebuild backend image from the reviewed lockfile</x:v>
@@ -8423,7 +8440,7 @@
         <x:v>Remaining advisories require separate review; this PR only mirrors the two reviewed source changes</x:v>
       </x:c>
       <x:c r="K33" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L33" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8449,7 +8466,7 @@
         <x:v>WOW-MD PR 74 merged as cf50bb7</x:v>
       </x:c>
       <x:c r="G34" s="41" t="str">
-        <x:v>Backend 113 suites and 1109 tests passed with 9 skipped; typecheck lint focused tests and disposable migration apply/no-op passed; protected CI runs on PR 118</x:v>
+        <x:v>Backend 113 suites and 1109 tests passed with 9 skipped; typecheck lint focused tests disposable migration apply/no-op and all protected CI passed</x:v>
       </x:c>
       <x:c r="H34" s="41" t="str">
         <x:v>Back up PostgreSQL; deploy backend and run migration 1710000114000 before relying on hourly snapshots</x:v>
@@ -8461,7 +8478,7 @@
         <x:v>Railway cost remains a configured estimate until a billing adapter supplies measured cost; live capacity evidence awaits the Railway candidate</x:v>
       </x:c>
       <x:c r="K34" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L34" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8487,7 +8504,7 @@
         <x:v>WOW-MD PR 70 merged as daae790</x:v>
       </x:c>
       <x:c r="G35" s="41" t="str">
-        <x:v>Focused delivery 31 tests plus lint and typecheck passed; original full backend 1149 passed 9 skipped and frontend 273 passed; protected CI reruns after rebase</x:v>
+        <x:v>Focused delivery 31 tests plus lint and typecheck passed; original full backend 1149 passed 9 skipped and frontend 273 passed; all protected CI passed after rebase</x:v>
       </x:c>
       <x:c r="H35" s="41" t="str">
         <x:v>Back up PostgreSQL; deploy backend migration 1710000115000 then frontend; optionally set OPERATIONS_ALERT_RECIPIENTS; mail remains simulated until final mail gate</x:v>
@@ -8499,7 +8516,7 @@
         <x:v>A delivery-state save failure after sending can repeat one send; live SMTP remains unproven until final Zoho mail gate</x:v>
       </x:c>
       <x:c r="K35" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L35" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8525,7 +8542,7 @@
         <x:v>WOW-MD PR 75 merged as 0d23fa2; source PR 71 and production PR 114 were replaced after stacked-base deletion</x:v>
       </x:c>
       <x:c r="G36" s="41" t="str">
-        <x:v>Backend focused 126 passed; backend 1219 passed 9 skipped; lint typecheck build passed; E2E 79 passed; frontend 296 tests build and Playwright 4 passed; exact-digit formatter review added 23 focused frontend tests</x:v>
+        <x:v>Backend focused 126 passed; backend 1219 passed 9 skipped; lint typecheck build E2E 79 frontend 296 tests Playwright 4 exact-digit 23 tests and all protected CI passed</x:v>
       </x:c>
       <x:c r="H36" s="41" t="str">
         <x:v>Deploy backend then frontend; no additional migration or configuration beyond OPS-003</x:v>
@@ -8537,7 +8554,7 @@
         <x:v>Acknowledgement shows actor ID not name; AUTH-001 MIG-001 and GATE-009 to GATE-011 remain unmet by design; revenue stays unknown until a net revenue source exists</x:v>
       </x:c>
       <x:c r="K36" s="41" t="str">
-        <x:v>PR Open</x:v>
+        <x:v>Merged</x:v>
       </x:c>
       <x:c r="L36" s="41" t="str">
         <x:v>2026-10-09</x:v>
@@ -8556,7 +8573,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10505c326a314fee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7cd5158be5c4c17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record Railway staging validation
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a9184afdfd84d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R786334ba3b584f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb017360dcba94192"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R4228fbcc203646bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R54fed5612bb646ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rc0f95789c0574fb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R83a6ca2f446d49b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R0f5a1906575f43b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra12ecc6399d54c7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb1c1001243334d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd2635863090f4a27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6399e51b18e04cdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rd80a163f05b045b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R7647f26c523443f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rdc39569c9fc74ce6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R04efb2c0bea04dae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R132498f8a28941ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re07fe24b092c44a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R158a761a9d2946f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R23eba6e6b13a41d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1102,7 +1102,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39f5df5413eb460c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f450787776f4b2c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1488,7 +1488,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-09. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-10. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1550,7 +1550,7 @@
       </x:c>
       <x:c r="H7" s="39" t="n">
         <x:f>B8</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1558,7 +1558,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
@@ -1592,7 +1592,7 @@
       </x:c>
       <x:c r="H9" s="39" t="n">
         <x:f>B10</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1600,7 +1600,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
@@ -1665,13 +1665,13 @@
         <x:v>Railway candidate</x:v>
       </x:c>
       <x:c r="B15" s="26" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="C15" s="26" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="D15" s="26" t="str">
-        <x:v>Create the disposable Railway project, apply private S3, then run live smoke and capacity evidence</x:v>
+        <x:v>Add the project-scoped Railway token and run the protected staging workflow; retain live service IDs, smoke output and cost/resource evidence</x:v>
       </x:c>
       <x:c r="E15" s="26" t="str">
         <x:v>Keep the production domain detached</x:v>
@@ -1720,7 +1720,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3b96049e8ff46b0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d4a98c3f4534070"/>
 </x:worksheet>
 </file>
 
@@ -2284,7 +2284,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdafacf08f59e4d53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04066106ac5d4b95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2740,10 +2740,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F15" s="41" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G15" s="41" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="H15" s="41" t="str">
         <x:v>CFG-001</x:v>
@@ -2752,7 +2752,7 @@
         <x:v>Frontend API PostgreSQL and Redis pass cross-origin auth and WebSocket smoke tests</x:v>
       </x:c>
       <x:c r="J15" s="41" t="str">
-        <x:v>Production plan Task 4; repository contract merged in PR 103; create the disposable Railway project and protected token without attaching the production domain</x:v>
+        <x:v>Live four-service Railway staging candidate online; direct and proxied health 200; local protected-equivalent Playwright smoke passed 1 of 1 on 2026-10-10; configure the project-scoped Railway token and exercise the protected workflow before closure</x:v>
       </x:c>
       <x:c r="K15" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/15</x:v>
@@ -2761,8 +2761,21 @@
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/103</x:v>
       </x:c>
       <x:c r="M15" s="41" t="str">
-        <x:v>2026-10-08</x:v>
-      </x:c>
+        <x:v>2026-10-10</x:v>
+      </x:c>
+      <x:c r="N15"/>
+      <x:c r="O15"/>
+      <x:c r="P15"/>
+      <x:c r="Q15"/>
+      <x:c r="R15"/>
+      <x:c r="S15"/>
+      <x:c r="T15"/>
+      <x:c r="U15"/>
+      <x:c r="V15"/>
+      <x:c r="W15"/>
+      <x:c r="X15"/>
+      <x:c r="Y15"/>
+      <x:c r="Z15"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="41" t="str">
@@ -4138,7 +4151,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ebd0616483b4bbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4b506a014a94d51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4714,7 +4727,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7844399862b499e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf8954b1b1644c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4986,17 +4999,36 @@
         <x:v>Four services health CORS registration refresh-cookie authenticated navigation and WebSocket reconnect</x:v>
       </x:c>
       <x:c r="D15" s="41" t="str">
-        <x:v>RLY-001 PR 103</x:v>
+        <x:v>RLY-001 PR 103; live Railway staging run 2026-10-10</x:v>
       </x:c>
       <x:c r="E15" s="41" t="str">
-        <x:v>Contract tests 3 of 3; root-context image build nginx injection and Compose validation passed; live smoke pending</x:v>
+        <x:v>Contract tests 4 of 4; live Playwright smoke 1 of 1 passed in 21.9 seconds; frontend direct backend PostgreSQL and Redis online; direct and proxied health 200</x:v>
       </x:c>
       <x:c r="F15" s="41" t="str">
-        <x:v>Run the protected smoke suite on the disposable Railway project</x:v>
+        <x:v>Configure the project-scoped Railway token and repeat through the protected railway-staging workflow</x:v>
       </x:c>
       <x:c r="G15" s="41" t="str">
         <x:v>RLY-001</x:v>
       </x:c>
+      <x:c r="H15"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
+      <x:c r="K15"/>
+      <x:c r="L15"/>
+      <x:c r="M15"/>
+      <x:c r="N15"/>
+      <x:c r="O15"/>
+      <x:c r="P15"/>
+      <x:c r="Q15"/>
+      <x:c r="R15"/>
+      <x:c r="S15"/>
+      <x:c r="T15"/>
+      <x:c r="U15"/>
+      <x:c r="V15"/>
+      <x:c r="W15"/>
+      <x:c r="X15"/>
+      <x:c r="Y15"/>
+      <x:c r="Z15"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="41" t="str">
@@ -5211,7 +5243,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d4f2a494e7248e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03deec45fae0461e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5710,7 +5742,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0265d852e1364cf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra303cd7304ed4031"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6059,7 +6091,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fee00e5887f4b01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4015531ec114138"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6402,7 +6434,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3b5affce5f48e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re35f791943164171"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7310,7 +7342,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3b1f260e25e403c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33777b33838b4b80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8573,7 +8605,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7cd5158be5c4c17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb5b467e101749b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: defer paid Railway automation
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd2635863090f4a27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R6399e51b18e04cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rd80a163f05b045b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R7647f26c523443f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rdc39569c9fc74ce6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="R04efb2c0bea04dae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R132498f8a28941ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re07fe24b092c44a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="R158a761a9d2946f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="R23eba6e6b13a41d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfd404593fc9f4a36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R2d7dab8993a443ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb2c7c2267b68462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R36b8e475a0b94fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb4f30701aa9845b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Ree3b7087a5104da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R10b025df4dc14ff7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re439214db26545ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rd1fe419431824729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Re762995b9dc343f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1102,7 +1102,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f450787776f4b2c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4ddf72cafaf4b47"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1671,7 +1671,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="D15" s="26" t="str">
-        <x:v>Add the project-scoped Railway token and run the protected staging workflow; retain live service IDs, smoke output and cost/resource evidence</x:v>
+        <x:v>Trial candidate and live smoke are verified; paid project-token automation is deferred until Hobby or public-beta approval, then capture protected workflow and cost/resource evidence</x:v>
       </x:c>
       <x:c r="E15" s="26" t="str">
         <x:v>Keep the production domain detached</x:v>
@@ -1720,7 +1720,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d4a98c3f4534070"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3731981821e244bd"/>
 </x:worksheet>
 </file>
 
@@ -2284,7 +2284,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04066106ac5d4b95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcec36a9de04c4d7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2752,13 +2752,13 @@
         <x:v>Frontend API PostgreSQL and Redis pass cross-origin auth and WebSocket smoke tests</x:v>
       </x:c>
       <x:c r="J15" s="41" t="str">
-        <x:v>Live four-service Railway staging candidate online; direct and proxied health 200; local protected-equivalent Playwright smoke passed 1 of 1 on 2026-10-10; configure the project-scoped Railway token and exercise the protected workflow before closure</x:v>
+        <x:v>Repository contract merged in PR 103; live four-service Trial candidate and smoke evidence recorded in PR 121; protected runs 37987169744 and 37987323813 safely stopped before deployment because the supplied token belonged to another project; correct project-token creation is plan-gated, so paid automation is deferred until Hobby or public-beta approval</x:v>
       </x:c>
       <x:c r="K15" s="41" t="str">
         <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/issues/15</x:v>
       </x:c>
       <x:c r="L15" s="41" t="str">
-        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/103</x:v>
+        <x:v>https://github.com/RohithTadiparti/world-of-weddingz-production/pull/121</x:v>
       </x:c>
       <x:c r="M15" s="41" t="str">
         <x:v>2026-10-10</x:v>
@@ -4151,7 +4151,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4b506a014a94d51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b934751394c48d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4727,7 +4727,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf8954b1b1644c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cdb271fa1614274"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4999,13 +4999,13 @@
         <x:v>Four services health CORS registration refresh-cookie authenticated navigation and WebSocket reconnect</x:v>
       </x:c>
       <x:c r="D15" s="41" t="str">
-        <x:v>RLY-001 PR 103; live Railway staging run 2026-10-10</x:v>
+        <x:v>RLY-001 PRs 103 and 121; live Railway staging run 2026-10-10; protected runs 37987169744 and 37987323813</x:v>
       </x:c>
       <x:c r="E15" s="41" t="str">
-        <x:v>Contract tests 4 of 4; live Playwright smoke 1 of 1 passed in 21.9 seconds; frontend direct backend PostgreSQL and Redis online; direct and proxied health 200</x:v>
+        <x:v>Contract tests 5 of 5; live Playwright smoke 1 of 1 passed in 21.9 seconds; frontend backend PostgreSQL and Redis online; direct and proxied health 200; token-scope preflight prevented a cross-project deployment</x:v>
       </x:c>
       <x:c r="F15" s="41" t="str">
-        <x:v>Configure the project-scoped Railway token and repeat through the protected railway-staging workflow</x:v>
+        <x:v>At Hobby or public-beta approval create a project token for confident-vibrancy staging, replace the environment secret, run the protected workflow and capture resource and cost evidence</x:v>
       </x:c>
       <x:c r="G15" s="41" t="str">
         <x:v>RLY-001</x:v>
@@ -5243,7 +5243,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03deec45fae0461e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bbc50f670e644b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5742,7 +5742,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra303cd7304ed4031"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1f605cf3be4436c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6091,7 +6091,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4015531ec114138"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ce12b2b78f046fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6434,7 +6434,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re35f791943164171"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b631f0a8124222"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7342,7 +7342,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33777b33838b4b80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccbf57dee0e64d08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8605,7 +8605,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb5b467e101749b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb02d662a43d74a4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record Railway staging live validation (#121)
* docs: record Railway staging validation

* ci: validate Railway token scope

* docs: defer paid Railway automation

---------

Co-authored-by: RohithTadiparti <326478345+RohithTadiparti@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/production-readiness-tracker.xlsx
+++ b/docs/tracking/production-readiness-tracker.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a9184afdfd84d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R786334ba3b584f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb017360dcba94192"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R4228fbcc203646bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="R54fed5612bb646ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Rc0f95789c0574fb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R83a6ca2f446d49b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="R0f5a1906575f43b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Ra12ecc6399d54c7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Rb1c1001243334d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfd404593fc9f4a36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" r:id="R2d7dab8993a443ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb2c7c2267b68462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Inventory" sheetId="4" r:id="R36b8e475a0b94fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="5" r:id="Rb4f30701aa9845b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="6" r:id="Ree3b7087a5104da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R10b025df4dc14ff7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Intake" sheetId="8" r:id="Re439214db26545ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PR Handoffs" sheetId="9" r:id="Rd1fe419431824729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="10" r:id="Re762995b9dc343f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1102,7 +1102,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39f5df5413eb460c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4ddf72cafaf4b47"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1488,7 +1488,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>As of 2026-10-09. Counts link to the canonical CSV registers included in the production repository.</x:v>
+        <x:v>As of 2026-10-10. Counts link to the canonical CSV registers included in the production repository.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1550,7 +1550,7 @@
       </x:c>
       <x:c r="H7" s="39" t="n">
         <x:f>B8</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1558,7 +1558,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B8" s="34" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
         <x:v>Open risks</x:v>
@@ -1592,7 +1592,7 @@
       </x:c>
       <x:c r="H9" s="39" t="n">
         <x:f>B10</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1600,7 +1600,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="34" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="33" t="str">
         <x:v>Approved requirements</x:v>
@@ -1665,13 +1665,13 @@
         <x:v>Railway candidate</x:v>
       </x:c>
       <x:c r="B15" s="26" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="C15" s="26" t="str">
-        <x:v>Product owner</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="D15" s="26" t="str">
-        <x:v>Create the disposable Railway project, apply private S3, then run live smoke and capacity evidence</x:v>
+        <x:v>Trial candidate and live smoke are verified; paid project-token automation is deferred until Hobby or public-beta approval, then capture protected workflow and cost/resource evidence</x:v>
       </x:c>
       <x:c r="E15" s="26" t="str">
         <x:v>Keep the production domain detached</x:v>
@@ -1720,7 +1720,7 @@
     <x:cfRule type="containsText" dxfId="39" priority="2" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" head